<commit_message>
chore(plan): note that InitialCreate.sql is kept in legacy-trash
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -595,7 +595,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -603,7 +602,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -618,7 +616,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -633,7 +630,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -648,7 +644,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -663,7 +658,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -678,7 +672,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -693,7 +686,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
@@ -747,7 +739,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -7098,7 +7089,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -9392,7 +9382,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -9556,7 +9545,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
@@ -9792,7 +9780,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
@@ -9848,7 +9835,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
@@ -9916,7 +9902,6 @@
         </is>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
@@ -10293,7 +10278,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -37510,7 +37494,7 @@
       </c>
       <c r="H312" s="8" t="inlineStr">
         <is>
-          <t>Moved with git mv to legacy-trash/manual-sql/ (same relative paths, README maps each to its replacement): PEMS.Persistence/Scripts/EnableFullTextSearch.sql (now migration FullTextSearch), docs/procurement/*.migration.sql and P4_P5_delta/PREFLIGHT, docs/task manager/TaskManagerCore_migration.sql, plus the root InitialCreate.sql removed earlier. References in docs and code comments updated. Operator tools that are not schema setup (scripts/cmms, scripts/rcm data repairs and read-only reports, docs/sql checks, deploy/ reviewed-script flow) were deliberately left in place; see #313.</t>
+          <t>Moved with git mv to legacy-trash/manual-sql/ (same relative paths, README maps each to its replacement): PEMS.Persistence/Scripts/EnableFullTextSearch.sql (now migration FullTextSearch), docs/procurement/*.migration.sql and P4_P5_delta/PREFLIGHT, docs/task manager/TaskManagerCore_migration.sql, plus the root InitialCreate.sql (full-schema script). References in docs and code comments updated. Operator tools that are not schema setup (scripts/cmms, scripts/rcm data repairs and read-only reports, docs/sql checks, deploy/ reviewed-script flow) were deliberately left in place; see #313.</t>
         </is>
       </c>
       <c r="I312" s="8" t="inlineStr">
@@ -39156,7 +39140,6 @@
         <v/>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
@@ -39250,7 +39233,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -39427,7 +39409,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
@@ -41221,8 +41202,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>
@@ -41264,7 +41243,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -41337,7 +41315,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(plan): record test evidence for the code-first database work (#309, #310)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -37320,7 +37320,7 @@
       </c>
       <c r="H310" s="8" t="inlineStr">
         <is>
-          <t>Was: EF Core code-first model + migration history, but nothing applied them at startup (Program.cs only ran seeders) and the full-text script was a manual SSMS step with a hardcoded 'USE PEMSDB'. Now: DatabaseInitializer (create database if missing before Hangfire connects) + IDatabaseUpdateService (see #310) run before the seeders; settings Database:CreateIfMissing / MigrateOnStartup; full-text search is the migration FullTextSearch; the manual schema SQL is moved to legacy-trash/ (#311); CI 'Model drift gate'; docs/deployment/CODE_FIRST_DATABASE.md. VERIFIED 2026-10-22 on SQL Server LocalDB: the real app started against a database that did not exist, created it, installed 116 migrations (Startup/FirstRun recorded), seeders ran with 0 errors, /health/database = 200; integration tests prove install -&gt; up to date -&gt; update and that an unmanaged schema is untouched. NOT yet verified: the CI drift gate on GitHub, a restart no-op in the full app, hosting on the real demo server (Plesk/IIS, SQL Server Full-Text feature, startup time limit).</t>
+          <t>Was: EF Core code-first model + migration history, but nothing applied them at startup (Program.cs only ran seeders) and the full-text script was a manual SSMS step with a hardcoded 'USE PEMSDB'. Now: DatabaseInitializer (create database if missing before Hangfire connects) + IDatabaseUpdateService (see #310) run before the seeders; settings Database:CreateIfMissing / MigrateOnStartup; full-text search is the migration FullTextSearch; the manual schema SQL is moved to legacy-trash/ (#311); CI 'Model drift gate'; docs/deployment/CODE_FIRST_DATABASE.md. VERIFIED 2026-10-22 on SQL Server LocalDB: the real app started against a database that did not exist, created it, installed 116 migrations (Startup/FirstRun recorded), seeders ran with 0 errors, /health/database = 200; integration tests prove install -&gt; up to date -&gt; update and that an unmanaged schema is untouched. NOT yet verified: the CI drift gate on GitHub, a restart no-op in the full app, hosting on the real demo server (Plesk/IIS, SQL Server Full-Text feature, startup time limit). TESTS 2026-10-23 on LocalDB: Authorization 73/73, Search 16/16, Setup 12/12, MyWork 42/42, Web 232/235 (2 were missing localization keys for the new page - fixed; 1 needs SQLEXPRESS by design), Deployment 19/21 (2 failures in deploy/ artifact tests that this work does not touch: LF-only assertion on a Windows autocrlf checkout and the bash mock harness), new code-first tests 57/57 after fixes, Admin page driven in a browser (install shown, update available, backup confirmation enforced, update applied and recorded). The full 1,400-test suite was not completed on this machine (hours; LocalDB wedged by killed runs).</t>
         </is>
       </c>
       <c r="I310" s="8" t="inlineStr">
@@ -37397,7 +37397,7 @@
       </c>
       <c r="F311" s="10" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G311" s="10" t="inlineStr">
@@ -37407,7 +37407,7 @@
       </c>
       <c r="H311" s="8" t="inlineStr">
         <is>
-          <t>IDatabaseUpdateService (PEMS.Application) + DatabaseUpdateService (PEMS.Persistence) with the pure DatabaseSetupClassifier: FirstRun, UpdateAvailable, UpToDate, UnmanagedSchema, DatabaseNewerThanApplication, Unreachable. Entity DatabaseUpdateRun + migration DatabaseUpdateRuns (audit of every attempt). Admin &gt; System Monitoring &gt; Database Update (/Admin/DatabaseUpdate, SystemAdmin, backup confirmation, antiforgery). GET /health/database (anonymous, state only). Verified 2026-10-22: 9 tests (classifier + real SQL Server install/update/unmanaged on throw-away LocalDB databases); page compiled and anonymous access redirects to login. Not yet viewed in a browser as the admin.</t>
+          <t>IDatabaseUpdateService (PEMS.Application) + DatabaseUpdateService (PEMS.Persistence) with the pure DatabaseSetupClassifier: FirstRun, UpdateAvailable, UpToDate, UnmanagedSchema, DatabaseNewerThanApplication, Unreachable. Entity DatabaseUpdateRun + migration DatabaseUpdateRuns (audit of every attempt). Admin &gt; System Monitoring &gt; Database Update (/Admin/DatabaseUpdate, SystemAdmin, backup confirmation, antiforgery). GET /health/database (anonymous, state only). Verified 2026-10-22: 9 tests (classifier + real SQL Server install/update/unmanaged on throw-away LocalDB databases); page compiled and anonymous access redirects to login. Driven in a browser as the seeded dev admin on 2026-10-23: state card, pending list, backup confirmation refused/accepted, update applied, run recorded as Admin/Update.</t>
         </is>
       </c>
       <c r="I311" s="8" t="inlineStr">

</xml_diff>

<commit_message>
chore(plan): add backlog #314 - "What's new" panel on the login page
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -21,12 +21,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$S$314</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Plan'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$S$315</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Plan'!$A$1:$H$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Roadmap'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Capability Checklist'!$A$1:$H$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Lessons'!$A$10:$E$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Supportability Matrix'!$A$4:$I$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Supportability Matrix'!$A$4:$I$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Old to New Map'!$A$1:$H$131</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -595,6 +595,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -602,6 +603,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -616,6 +618,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -630,6 +633,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -644,6 +648,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -658,6 +663,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -672,6 +678,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -686,6 +693,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
@@ -711,7 +719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -739,6 +747,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -2042,8 +2051,55 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>SM-29</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Branding</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Release notes on the login page</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Core / login</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Planned: bilingual, offline release notes of the installed release shown to anonymous visitors.</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="H33" s="10" t="inlineStr">
+        <is>
+          <t>#314</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>Not started.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I32"/>
+  <autoFilter ref="A4:I33"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
@@ -7089,6 +7145,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -7096,7 +7153,7 @@
         </is>
       </c>
       <c r="B3" s="12">
-        <f>COUNTA(Backlog!$D$2:$D$314)</f>
+        <f>COUNTA(Backlog!$D$2:$D$315)</f>
         <v/>
       </c>
       <c r="C3" s="12" t="n"/>
@@ -7113,7 +7170,7 @@
         </is>
       </c>
       <c r="B4" s="12">
-        <f>COUNTIF(Backlog!$B$2:$B$314,"User")</f>
+        <f>COUNTIF(Backlog!$B$2:$B$315,"User")</f>
         <v/>
       </c>
       <c r="C4" s="12" t="n"/>
@@ -7187,19 +7244,19 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A8,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A8,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A8,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A8,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A8,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A8,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A8,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A8,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="F8" s="12">
@@ -7216,19 +7273,19 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A9,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A9,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A9,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A9,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A9,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A9,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A9,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A9,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="F9" s="12">
@@ -7245,19 +7302,19 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A10,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A10,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A10,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A10,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A10,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A10,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A10,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A10,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="F10" s="12">
@@ -7274,19 +7331,19 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A11,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A11,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A11,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A11,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A11,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A11,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A11,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A11,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="F11" s="12">
@@ -7303,19 +7360,19 @@
         </is>
       </c>
       <c r="B12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A12,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A12,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="C12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A12,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A12,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A12,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A12,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="E12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A12,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A12,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="F12" s="12">
@@ -7332,19 +7389,19 @@
         </is>
       </c>
       <c r="B13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A13,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A13,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="C13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A13,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A13,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A13,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A13,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="E13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A13,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A13,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="F13" s="12">
@@ -7361,19 +7418,19 @@
         </is>
       </c>
       <c r="B14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A14,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A14,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="C14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A14,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A14,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="D14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A14,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A14,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="E14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A14,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A14,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="F14" s="12">
@@ -7390,19 +7447,19 @@
         </is>
       </c>
       <c r="B15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A15,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A15,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="C15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A15,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A15,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="D15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A15,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A15,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="E15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$314,$A15,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$315,$A15,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="F15" s="12">
@@ -7513,31 +7570,31 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A20)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A20,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A20,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A20,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A20,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G20" s="12">
-        <f>B20-H20-COUNTIFS(Backlog!$C$2:$C$314,$A20,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A20,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A20,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B20-H20-COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A20,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7548,31 +7605,31 @@
         </is>
       </c>
       <c r="B21" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A21)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A21,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A21,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A21,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A21,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G21" s="12">
-        <f>B21-H21-COUNTIFS(Backlog!$C$2:$C$314,$A21,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A21,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A21,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B21-H21-COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A21,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7583,31 +7640,31 @@
         </is>
       </c>
       <c r="B22" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A22)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A22,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A22,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A22,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A22,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G22" s="12">
-        <f>B22-H22-COUNTIFS(Backlog!$C$2:$C$314,$A22,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A22,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A22,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B22-H22-COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A22,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7618,31 +7675,31 @@
         </is>
       </c>
       <c r="B23" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A23)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A23)</f>
         <v/>
       </c>
       <c r="C23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A23,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A23,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A23,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A23,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G23" s="12">
-        <f>B23-H23-COUNTIFS(Backlog!$C$2:$C$314,$A23,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A23,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A23,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B23-H23-COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A23,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7653,31 +7710,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A24)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A24,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A24,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A24,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A24,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>B24-H24-COUNTIFS(Backlog!$C$2:$C$314,$A24,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A24,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A24,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B24-H24-COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A24,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7688,31 +7745,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A25)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A25,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A25,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A25,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A25,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>B25-H25-COUNTIFS(Backlog!$C$2:$C$314,$A25,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A25,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A25,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B25-H25-COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A25,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7723,31 +7780,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A26)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A26,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A26,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A26,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A26,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>B26-H26-COUNTIFS(Backlog!$C$2:$C$314,$A26,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A26,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A26,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B26-H26-COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A26,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7758,31 +7815,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A27)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A27,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A27,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A27,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A27,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>B27-H27-COUNTIFS(Backlog!$C$2:$C$314,$A27,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A27,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A27,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B27-H27-COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A27,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7793,31 +7850,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A28)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A28,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A28,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A28,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A28,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>B28-H28-COUNTIFS(Backlog!$C$2:$C$314,$A28,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A28,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A28,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B28-H28-COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A28,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7828,31 +7885,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A29)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A29,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A29,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A29,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A29,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>B29-H29-COUNTIFS(Backlog!$C$2:$C$314,$A29,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A29,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A29,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B29-H29-COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A29,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7863,31 +7920,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A30)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A30,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A30,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A30,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A30,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>B30-H30-COUNTIFS(Backlog!$C$2:$C$314,$A30,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A30,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A30,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B30-H30-COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A30,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7898,31 +7955,31 @@
         </is>
       </c>
       <c r="B31" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A31)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A31,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A31,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A31,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A31,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G31" s="12">
-        <f>B31-H31-COUNTIFS(Backlog!$C$2:$C$314,$A31,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A31,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A31,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B31-H31-COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A31,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7933,31 +7990,31 @@
         </is>
       </c>
       <c r="B32" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A32)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A32,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A32,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A32,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A32,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G32" s="12">
-        <f>B32-H32-COUNTIFS(Backlog!$C$2:$C$314,$A32,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A32,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A32,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B32-H32-COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A32,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7968,31 +8025,31 @@
         </is>
       </c>
       <c r="B33" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A33)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A33)</f>
         <v/>
       </c>
       <c r="C33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A33,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A33,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A33,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A33,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G33" s="12">
-        <f>B33-H33-COUNTIFS(Backlog!$C$2:$C$314,$A33,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A33,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A33,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B33-H33-COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A33,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8003,31 +8060,31 @@
         </is>
       </c>
       <c r="B34" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A34)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A34)</f>
         <v/>
       </c>
       <c r="C34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A34,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A34,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A34,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A34,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G34" s="12">
-        <f>B34-H34-COUNTIFS(Backlog!$C$2:$C$314,$A34,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A34,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A34,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B34-H34-COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A34,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8038,31 +8095,31 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A35)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A35)</f>
         <v/>
       </c>
       <c r="C35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A35,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A35,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A35,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A35,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G35" s="12">
-        <f>B35-H35-COUNTIFS(Backlog!$C$2:$C$314,$A35,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A35,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A35,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B35-H35-COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A35,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8073,31 +8130,31 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A36)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A36)</f>
         <v/>
       </c>
       <c r="C36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A36,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A36,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A36,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A36,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G36" s="12">
-        <f>B36-H36-COUNTIFS(Backlog!$C$2:$C$314,$A36,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A36,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A36,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B36-H36-COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A36,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8108,31 +8165,31 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A37)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A37,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A37,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A37,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A37,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G37" s="12">
-        <f>B37-H37-COUNTIFS(Backlog!$C$2:$C$314,$A37,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A37,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A37,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B37-H37-COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A37,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8143,31 +8200,31 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A38)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A38,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A38,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A38,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A38,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G38" s="12">
-        <f>B38-H38-COUNTIFS(Backlog!$C$2:$C$314,$A38,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A38,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A38,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B38-H38-COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A38,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8178,31 +8235,31 @@
         </is>
       </c>
       <c r="B39" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A39)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A39,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A39,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A39,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A39,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G39" s="12">
-        <f>B39-H39-COUNTIFS(Backlog!$C$2:$C$314,$A39,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A39,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A39,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B39-H39-COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A39,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8213,31 +8270,31 @@
         </is>
       </c>
       <c r="B40" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A40)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A40,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A40,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A40,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A40,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G40" s="12">
-        <f>B40-H40-COUNTIFS(Backlog!$C$2:$C$314,$A40,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A40,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A40,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B40-H40-COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A40,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8248,31 +8305,31 @@
         </is>
       </c>
       <c r="B41" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A41)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A41,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A41,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A41,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A41,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G41" s="12">
-        <f>B41-H41-COUNTIFS(Backlog!$C$2:$C$314,$A41,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A41,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A41,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B41-H41-COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A41,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8283,31 +8340,31 @@
         </is>
       </c>
       <c r="B42" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A42)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A42,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A42,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A42,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A42,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G42" s="12">
-        <f>B42-H42-COUNTIFS(Backlog!$C$2:$C$314,$A42,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A42,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A42,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B42-H42-COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A42,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8318,31 +8375,31 @@
         </is>
       </c>
       <c r="B43" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A43)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A43,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A43,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A43,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A43,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G43" s="12">
-        <f>B43-H43-COUNTIFS(Backlog!$C$2:$C$314,$A43,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A43,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A43,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B43-H43-COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A43,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8353,31 +8410,31 @@
         </is>
       </c>
       <c r="B44" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A44)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A44,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A44,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A44,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A44,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G44" s="12">
-        <f>B44-H44-COUNTIFS(Backlog!$C$2:$C$314,$A44,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A44,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A44,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B44-H44-COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A44,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8388,31 +8445,31 @@
         </is>
       </c>
       <c r="B45" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A45)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A45,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A45,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A45,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A45,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G45" s="12">
-        <f>B45-H45-COUNTIFS(Backlog!$C$2:$C$314,$A45,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A45,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A45,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B45-H45-COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A45,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8423,31 +8480,31 @@
         </is>
       </c>
       <c r="B46" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$314,$A46)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$315,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A46,Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="D46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A46,Backlog!$G$2:$G$314,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$G$2:$G$315,"P1")</f>
         <v/>
       </c>
       <c r="E46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A46,Backlog!$G$2:$G$314,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$G$2:$G$315,"P2")</f>
         <v/>
       </c>
       <c r="F46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A46,Backlog!$G$2:$G$314,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$G$2:$G$315,"P3")</f>
         <v/>
       </c>
       <c r="G46" s="12">
-        <f>B46-H46-COUNTIFS(Backlog!$C$2:$C$314,$A46,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$314,$A46,Backlog!$F$2:$F$314,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$314,$A46,Backlog!$F$2:$F$314,"Later")</f>
+        <f>B46-H46-COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="H46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$314,$A46,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8515,23 +8572,23 @@
         </is>
       </c>
       <c r="B50" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A50)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A50,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A50,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A50,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A50,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E50" s="12">
-        <f>B50-C50-D50-COUNTIFS(Backlog!$R$2:$R$314,$A50,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A50,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B50-C50-D50-COUNTIFS(Backlog!$R$2:$R$315,$A50,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A50,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A50,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A50,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G50" s="12" t="n"/>
@@ -8544,23 +8601,23 @@
         </is>
       </c>
       <c r="B51" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A51)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A51)</f>
         <v/>
       </c>
       <c r="C51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A51,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A51,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A51,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A51,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E51" s="12">
-        <f>B51-C51-D51-COUNTIFS(Backlog!$R$2:$R$314,$A51,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A51,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B51-C51-D51-COUNTIFS(Backlog!$R$2:$R$315,$A51,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A51,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A51,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A51,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G51" s="12" t="n"/>
@@ -8573,23 +8630,23 @@
         </is>
       </c>
       <c r="B52" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A52)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A52)</f>
         <v/>
       </c>
       <c r="C52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A52,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A52,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A52,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A52,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E52" s="12">
-        <f>B52-C52-D52-COUNTIFS(Backlog!$R$2:$R$314,$A52,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A52,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B52-C52-D52-COUNTIFS(Backlog!$R$2:$R$315,$A52,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A52,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A52,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A52,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G52" s="12" t="n"/>
@@ -8602,23 +8659,23 @@
         </is>
       </c>
       <c r="B53" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A53)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A53)</f>
         <v/>
       </c>
       <c r="C53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A53,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A53,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A53,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A53,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E53" s="12">
-        <f>B53-C53-D53-COUNTIFS(Backlog!$R$2:$R$314,$A53,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A53,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B53-C53-D53-COUNTIFS(Backlog!$R$2:$R$315,$A53,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A53,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A53,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A53,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G53" s="12" t="n"/>
@@ -8631,23 +8688,23 @@
         </is>
       </c>
       <c r="B54" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A54)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A54)</f>
         <v/>
       </c>
       <c r="C54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A54,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A54,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A54,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A54,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E54" s="12">
-        <f>B54-C54-D54-COUNTIFS(Backlog!$R$2:$R$314,$A54,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A54,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B54-C54-D54-COUNTIFS(Backlog!$R$2:$R$315,$A54,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A54,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A54,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A54,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G54" s="12" t="n"/>
@@ -8660,23 +8717,23 @@
         </is>
       </c>
       <c r="B55" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A55)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A55,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A55,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A55,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A55,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E55" s="12">
-        <f>B55-C55-D55-COUNTIFS(Backlog!$R$2:$R$314,$A55,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A55,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B55-C55-D55-COUNTIFS(Backlog!$R$2:$R$315,$A55,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A55,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A55,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A55,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G55" s="12" t="n"/>
@@ -8689,23 +8746,23 @@
         </is>
       </c>
       <c r="B56" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A56)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A56,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A56,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A56,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A56,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E56" s="12">
-        <f>B56-C56-D56-COUNTIFS(Backlog!$R$2:$R$314,$A56,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A56,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B56-C56-D56-COUNTIFS(Backlog!$R$2:$R$315,$A56,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A56,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A56,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A56,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G56" s="12" t="n"/>
@@ -8718,23 +8775,23 @@
         </is>
       </c>
       <c r="B57" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A57)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A57,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A57,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A57,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A57,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E57" s="12">
-        <f>B57-C57-D57-COUNTIFS(Backlog!$R$2:$R$314,$A57,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A57,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B57-C57-D57-COUNTIFS(Backlog!$R$2:$R$315,$A57,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A57,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A57,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A57,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G57" s="12" t="n"/>
@@ -8747,23 +8804,23 @@
         </is>
       </c>
       <c r="B58" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A58)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A58,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A58,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A58,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A58,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E58" s="12">
-        <f>B58-C58-D58-COUNTIFS(Backlog!$R$2:$R$314,$A58,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A58,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B58-C58-D58-COUNTIFS(Backlog!$R$2:$R$315,$A58,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A58,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A58,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A58,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G58" s="12" t="n"/>
@@ -8776,23 +8833,23 @@
         </is>
       </c>
       <c r="B59" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A59)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A59,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A59,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A59,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A59,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E59" s="12">
-        <f>B59-C59-D59-COUNTIFS(Backlog!$R$2:$R$314,$A59,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A59,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B59-C59-D59-COUNTIFS(Backlog!$R$2:$R$315,$A59,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A59,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A59,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A59,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G59" s="12" t="n"/>
@@ -8805,23 +8862,23 @@
         </is>
       </c>
       <c r="B60" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A60)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A60,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A60,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A60,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A60,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E60" s="12">
-        <f>B60-C60-D60-COUNTIFS(Backlog!$R$2:$R$314,$A60,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A60,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B60-C60-D60-COUNTIFS(Backlog!$R$2:$R$315,$A60,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A60,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A60,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A60,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G60" s="12" t="n"/>
@@ -8834,23 +8891,23 @@
         </is>
       </c>
       <c r="B61" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A61)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A61,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A61,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A61,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A61,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E61" s="12">
-        <f>B61-C61-D61-COUNTIFS(Backlog!$R$2:$R$314,$A61,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A61,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B61-C61-D61-COUNTIFS(Backlog!$R$2:$R$315,$A61,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A61,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A61,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A61,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G61" s="12" t="n"/>
@@ -8863,23 +8920,23 @@
         </is>
       </c>
       <c r="B62" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A62)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A62,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A62,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A62,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A62,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E62" s="12">
-        <f>B62-C62-D62-COUNTIFS(Backlog!$R$2:$R$314,$A62,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A62,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B62-C62-D62-COUNTIFS(Backlog!$R$2:$R$315,$A62,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A62,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A62,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A62,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G62" s="12" t="n"/>
@@ -8892,23 +8949,23 @@
         </is>
       </c>
       <c r="B63" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A63)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A63,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A63,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A63,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A63,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E63" s="12">
-        <f>B63-C63-D63-COUNTIFS(Backlog!$R$2:$R$314,$A63,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A63,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B63-C63-D63-COUNTIFS(Backlog!$R$2:$R$315,$A63,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A63,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A63,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A63,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G63" s="12" t="n"/>
@@ -8921,23 +8978,23 @@
         </is>
       </c>
       <c r="B64" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A64)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A64,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A64,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A64,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A64,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E64" s="12">
-        <f>B64-C64-D64-COUNTIFS(Backlog!$R$2:$R$314,$A64,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A64,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B64-C64-D64-COUNTIFS(Backlog!$R$2:$R$315,$A64,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A64,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A64,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A64,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G64" s="12" t="n"/>
@@ -8950,23 +9007,23 @@
         </is>
       </c>
       <c r="B65" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A65)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A65,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A65,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A65,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A65,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E65" s="12">
-        <f>B65-C65-D65-COUNTIFS(Backlog!$R$2:$R$314,$A65,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A65,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B65-C65-D65-COUNTIFS(Backlog!$R$2:$R$315,$A65,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A65,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A65,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A65,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G65" s="12" t="n"/>
@@ -8979,23 +9036,23 @@
         </is>
       </c>
       <c r="B66" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A66)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A66,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A66,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A66,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A66,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E66" s="12">
-        <f>B66-C66-D66-COUNTIFS(Backlog!$R$2:$R$314,$A66,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A66,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B66-C66-D66-COUNTIFS(Backlog!$R$2:$R$315,$A66,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A66,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A66,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A66,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G66" s="12" t="n"/>
@@ -9008,23 +9065,23 @@
         </is>
       </c>
       <c r="B67" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A67)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A67,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A67,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A67,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A67,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E67" s="12">
-        <f>B67-C67-D67-COUNTIFS(Backlog!$R$2:$R$314,$A67,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A67,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B67-C67-D67-COUNTIFS(Backlog!$R$2:$R$315,$A67,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A67,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A67,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A67,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G67" s="12" t="n"/>
@@ -9037,23 +9094,23 @@
         </is>
       </c>
       <c r="B68" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A68)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A68,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A68,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A68,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A68,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E68" s="12">
-        <f>B68-C68-D68-COUNTIFS(Backlog!$R$2:$R$314,$A68,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A68,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B68-C68-D68-COUNTIFS(Backlog!$R$2:$R$315,$A68,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A68,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A68,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A68,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G68" s="12" t="n"/>
@@ -9066,23 +9123,23 @@
         </is>
       </c>
       <c r="B69" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A69)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A69,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A69,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A69,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A69,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E69" s="12">
-        <f>B69-C69-D69-COUNTIFS(Backlog!$R$2:$R$314,$A69,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A69,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B69-C69-D69-COUNTIFS(Backlog!$R$2:$R$315,$A69,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A69,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A69,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A69,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G69" s="12" t="n"/>
@@ -9095,23 +9152,23 @@
         </is>
       </c>
       <c r="B70" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A70)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A70,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A70,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A70,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A70,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E70" s="12">
-        <f>B70-C70-D70-COUNTIFS(Backlog!$R$2:$R$314,$A70,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A70,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B70-C70-D70-COUNTIFS(Backlog!$R$2:$R$315,$A70,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A70,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A70,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A70,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G70" s="12" t="n"/>
@@ -9124,23 +9181,23 @@
         </is>
       </c>
       <c r="B71" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A71)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A71,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A71,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A71,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A71,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E71" s="12">
-        <f>B71-C71-D71-COUNTIFS(Backlog!$R$2:$R$314,$A71,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A71,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B71-C71-D71-COUNTIFS(Backlog!$R$2:$R$315,$A71,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A71,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A71,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A71,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G71" s="12" t="n"/>
@@ -9153,23 +9210,23 @@
         </is>
       </c>
       <c r="B72" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A72)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A72,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A72,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A72,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A72,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E72" s="12">
-        <f>B72-C72-D72-COUNTIFS(Backlog!$R$2:$R$314,$A72,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A72,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B72-C72-D72-COUNTIFS(Backlog!$R$2:$R$315,$A72,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A72,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A72,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A72,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G72" s="12" t="n"/>
@@ -9182,23 +9239,23 @@
         </is>
       </c>
       <c r="B73" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$314,$A73)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$315,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A73,Backlog!$F$2:$F$314,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A73,Backlog!$F$2:$F$315,"Done")</f>
         <v/>
       </c>
       <c r="D73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A73,Backlog!$F$2:$F$314,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A73,Backlog!$F$2:$F$315,"Later")</f>
         <v/>
       </c>
       <c r="E73" s="12">
-        <f>B73-C73-D73-COUNTIFS(Backlog!$R$2:$R$314,$A73,Backlog!$F$2:$F$314,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$314,$A73,Backlog!$F$2:$F$314,"Obsolete")</f>
+        <f>B73-C73-D73-COUNTIFS(Backlog!$R$2:$R$315,$A73,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A73,Backlog!$F$2:$F$315,"Obsolete")</f>
         <v/>
       </c>
       <c r="F73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$314,$A73,Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$315,$A73,Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="G73" s="12" t="n"/>
@@ -9220,7 +9277,7 @@
         </is>
       </c>
       <c r="B75" s="12">
-        <f>COUNTIF(Backlog!$S$2:$S$314,"Yes")</f>
+        <f>COUNTIF(Backlog!$S$2:$S$315,"Yes")</f>
         <v/>
       </c>
       <c r="C75" s="12" t="n"/>
@@ -9237,7 +9294,7 @@
         </is>
       </c>
       <c r="B76" s="12">
-        <f>COUNTIFS(Backlog!$S$2:$S$314,"Yes",Backlog!$G$2:$G$314,"P0")</f>
+        <f>COUNTIFS(Backlog!$S$2:$S$315,"Yes",Backlog!$G$2:$G$315,"P0")</f>
         <v/>
       </c>
       <c r="C76" s="12" t="n"/>
@@ -9254,7 +9311,7 @@
         </is>
       </c>
       <c r="B77" s="12">
-        <f>COUNTIFS(Backlog!$S$2:$S$314,"No",Backlog!$G$2:$G$314,"P0",Backlog!$F$2:$F$314,"&lt;&gt;Done",Backlog!$F$2:$F$314,"&lt;&gt;Later",Backlog!$F$2:$F$314,"&lt;&gt;Cancelled",Backlog!$F$2:$F$314,"&lt;&gt;Obsolete")</f>
+        <f>COUNTIFS(Backlog!$S$2:$S$315,"No",Backlog!$G$2:$G$315,"P0",Backlog!$F$2:$F$315,"&lt;&gt;Done",Backlog!$F$2:$F$315,"&lt;&gt;Later",Backlog!$F$2:$F$315,"&lt;&gt;Cancelled",Backlog!$F$2:$F$315,"&lt;&gt;Obsolete")</f>
         <v/>
       </c>
       <c r="C77" s="12" t="n"/>
@@ -9271,7 +9328,7 @@
         </is>
       </c>
       <c r="B78" s="12">
-        <f>COUNTIF(Backlog!$F$2:$F$314,"Hold")</f>
+        <f>COUNTIF(Backlog!$F$2:$F$315,"Hold")</f>
         <v/>
       </c>
       <c r="C78" s="12" t="n"/>
@@ -9297,7 +9354,7 @@
         </is>
       </c>
       <c r="B80" s="12">
-        <f>COUNTIFS(Backlog!$G$2:$G$314,"P0",Backlog!$F$2:$F$314,"&lt;&gt;Done",Backlog!$F$2:$F$314,"&lt;&gt;Cancelled",Backlog!$F$2:$F$314,"&lt;&gt;Obsolete",Backlog!$F$2:$F$314,"&lt;&gt;Later")</f>
+        <f>COUNTIFS(Backlog!$G$2:$G$315,"P0",Backlog!$F$2:$F$315,"&lt;&gt;Done",Backlog!$F$2:$F$315,"&lt;&gt;Cancelled",Backlog!$F$2:$F$315,"&lt;&gt;Obsolete",Backlog!$F$2:$F$315,"&lt;&gt;Later")</f>
         <v/>
       </c>
       <c r="C80" s="12" t="n"/>
@@ -9314,7 +9371,7 @@
         </is>
       </c>
       <c r="B81" s="12">
-        <f>COUNTIFS(Backlog!$N$2:$N$314,"Sales blocker",Backlog!$F$2:$F$314,"&lt;&gt;Done")</f>
+        <f>COUNTIFS(Backlog!$N$2:$N$315,"Sales blocker",Backlog!$F$2:$F$315,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="C81" s="12" t="n"/>
@@ -9331,7 +9388,7 @@
         </is>
       </c>
       <c r="B82" s="12">
-        <f>COUNTIFS(Backlog!$E$2:$E$314,"Decision Needed",Backlog!$F$2:$F$314,"&lt;&gt;Done")</f>
+        <f>COUNTIFS(Backlog!$E$2:$E$315,"Decision Needed",Backlog!$F$2:$F$315,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="C82" s="12" t="n"/>
@@ -9382,6 +9439,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -9545,6 +9603,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
@@ -9780,6 +9839,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
@@ -9835,6 +9895,7 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
@@ -9902,6 +9963,7 @@
         </is>
       </c>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
@@ -10278,6 +10340,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -10651,7 +10714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S314"/>
+  <dimension ref="A1:S315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -37715,9 +37778,92 @@
         </is>
       </c>
     </row>
+    <row r="315">
+      <c r="A315" s="10" t="n">
+        <v>314</v>
+      </c>
+      <c r="B315" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C315" s="8" t="inlineStr">
+        <is>
+          <t>Company, Brand &amp; Commercial Packaging</t>
+        </is>
+      </c>
+      <c r="D315" s="8" t="inlineStr">
+        <is>
+          <t>"What's new" panel on the login page: the latest release notes shown to visitors before sign-in, in Persian and English, fully offline</t>
+        </is>
+      </c>
+      <c r="E315" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F315" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G315" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H315" s="8" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-23. Today the login page has no release information and the repository only has a developer CHANGELOG.md. Customers installing or updating (#309/#310, #167) cannot see what changed. The login page is the one surface every user sees; the brand profile already comes from the database for the same page (see Lessons: live brand profile).</t>
+        </is>
+      </c>
+      <c r="I315" s="8" t="inlineStr">
+        <is>
+          <t>Design first: one source of truth for release notes (a curated, bilingual 'release notes' data file or table maintained per release - NOT the raw developer CHANGELOG), shipped inside the package and loaded from the database/disk with no external call. Then add a compact panel to the login page: latest release title and date, 3-5 highlights, 'older releases' expander, anonymous-safe (no internal ids, user names or unreleased work). Entries are written in the release task; the pipeline fails the release if the notes for the tagged version are missing.</t>
+        </is>
+      </c>
+      <c r="J315" s="8" t="inlineStr">
+        <is>
+          <t>The login page shows the notes of the installed release in the active language without any internet access; only features that are Done with evidence are listed (Instructions rule 13); the panel works for an anonymous visitor, is accessible (keyboard, contrast, RTL) and collapses on small screens.</t>
+        </is>
+      </c>
+      <c r="K315" s="8" t="n"/>
+      <c r="L315" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M315" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N315" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O315" s="10" t="inlineStr">
+        <is>
+          <t>#129 #170 #269</t>
+        </is>
+      </c>
+      <c r="P315" s="10" t="n"/>
+      <c r="Q315" s="10" t="n"/>
+      <c r="R315" s="8" t="inlineStr">
+        <is>
+          <t>Company, brand &amp; legal</t>
+        </is>
+      </c>
+      <c r="S315" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S314"/>
-  <conditionalFormatting sqref="F2:F314">
+  <autoFilter ref="A1:S315"/>
+  <conditionalFormatting sqref="F2:F315">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
@@ -37740,7 +37886,7 @@
       <formula>"Obsolete"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G314">
+  <conditionalFormatting sqref="G2:G315">
     <cfRule type="cellIs" priority="8" operator="equal" dxfId="6">
       <formula>"P0"</formula>
     </cfRule>
@@ -37748,27 +37894,27 @@
       <formula>"P1"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S314">
+  <conditionalFormatting sqref="S2:S315">
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N314">
+  <conditionalFormatting sqref="N2:N315">
     <cfRule type="cellIs" priority="11" operator="equal" dxfId="6">
       <formula>"Sales blocker"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="F2:F314" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F315" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Partial,Done,Hold,Later,Cancelled,Obsolete"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G314" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G315" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B314" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B2:B315" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Claude,User,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S314" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="S2:S315" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -37782,7 +37928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -38863,10 +39009,48 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="10" t="n">
+        <v>314</v>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Company, Brand &amp; Commercial Packaging</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>What's new panel on the login page</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>An installed release with notes in Persian and English; no internet access.</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>1) Open the login page signed out, in Persian and in English. 2) Disconnect the network and reload. 3) Check keyboard navigation, RTL layout and a phone-width screen. Expected: the installed release's notes show, nothing is fetched externally, no internal data is exposed.</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Risk if it fails: Customers cannot see what changed, or the page leaks internal information.</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>Needs QA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H28"/>
+  <autoFilter ref="A1:H29"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H2:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Needs QA,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -38950,7 +39134,7 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$314,"M0")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$315,"M0")</f>
         <v/>
       </c>
     </row>
@@ -38981,7 +39165,7 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$314,"M1")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$315,"M1")</f>
         <v/>
       </c>
     </row>
@@ -39012,7 +39196,7 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$314,"M2")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$315,"M2")</f>
         <v/>
       </c>
     </row>
@@ -39043,7 +39227,7 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$314,"M3")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$315,"M3")</f>
         <v/>
       </c>
     </row>
@@ -39074,7 +39258,7 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$314,"M4")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$315,"M4")</f>
         <v/>
       </c>
     </row>
@@ -39105,7 +39289,7 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$314,"M5")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$315,"M5")</f>
         <v/>
       </c>
     </row>
@@ -39136,10 +39320,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$314,"M6")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$315,"M6")</f>
         <v/>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
@@ -39233,6 +39418,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -39409,6 +39595,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
@@ -41202,6 +41389,8 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>
@@ -41243,6 +41432,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -41315,6 +41505,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(plan): record environment files work (#315) and follow-ups #316-#318
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -21,12 +21,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$S$315</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Plan'!$A$1:$H$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$S$319</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Plan'!$A$1:$H$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Roadmap'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Capability Checklist'!$A$1:$H$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Lessons'!$A$10:$E$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Supportability Matrix'!$A$4:$I$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Lessons'!$A$10:$E$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Supportability Matrix'!$A$4:$I$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Old to New Map'!$A$1:$H$131</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -719,7 +719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2098,8 +2098,55 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>SM-30</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Configuration and secrets</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Settings in env/&lt;name&gt;.env and secrets in env/&lt;name&gt;.secrets.env for local, docker, demo, uat and production-kangan; PEMS_ENV selects the environment; real environment variables override; required settings fail fast; appsettings.json is empty.</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>Supported (unverified)</t>
+        </is>
+      </c>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>#315 #316</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>Verified on a developer machine (LocalDB). Demo pipeline, Docker and the Linux VM kit not yet exercised.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I33"/>
+  <autoFilter ref="A4:I34"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
@@ -7153,7 +7200,7 @@
         </is>
       </c>
       <c r="B3" s="12">
-        <f>COUNTA(Backlog!$D$2:$D$315)</f>
+        <f>COUNTA(Backlog!$D$2:$D$319)</f>
         <v/>
       </c>
       <c r="C3" s="12" t="n"/>
@@ -7170,7 +7217,7 @@
         </is>
       </c>
       <c r="B4" s="12">
-        <f>COUNTIF(Backlog!$B$2:$B$315,"User")</f>
+        <f>COUNTIF(Backlog!$B$2:$B$319,"User")</f>
         <v/>
       </c>
       <c r="C4" s="12" t="n"/>
@@ -7244,19 +7291,19 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A8,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A8,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A8,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A8,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A8,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A8,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A8,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A8,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="F8" s="12">
@@ -7273,19 +7320,19 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A9,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A9,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A9,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A9,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A9,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A9,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A9,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A9,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="F9" s="12">
@@ -7302,19 +7349,19 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A10,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A10,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A10,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A10,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A10,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A10,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A10,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A10,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="F10" s="12">
@@ -7331,19 +7378,19 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A11,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A11,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A11,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A11,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A11,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A11,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A11,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A11,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="F11" s="12">
@@ -7360,19 +7407,19 @@
         </is>
       </c>
       <c r="B12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A12,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A12,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="C12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A12,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A12,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A12,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A12,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="E12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A12,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A12,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="F12" s="12">
@@ -7389,19 +7436,19 @@
         </is>
       </c>
       <c r="B13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A13,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A13,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="C13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A13,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A13,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A13,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A13,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="E13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A13,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A13,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="F13" s="12">
@@ -7418,19 +7465,19 @@
         </is>
       </c>
       <c r="B14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A14,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A14,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="C14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A14,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A14,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="D14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A14,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A14,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="E14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A14,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A14,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="F14" s="12">
@@ -7447,19 +7494,19 @@
         </is>
       </c>
       <c r="B15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A15,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A15,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="C15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A15,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A15,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="D15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A15,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A15,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="E15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$315,$A15,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$319,$A15,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="F15" s="12">
@@ -7570,31 +7617,31 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A20)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A20,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A20,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A20,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A20,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G20" s="12">
-        <f>B20-H20-COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B20-H20-COUNTIFS(Backlog!$C$2:$C$319,$A20,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A20,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A20,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A20,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A20,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7605,31 +7652,31 @@
         </is>
       </c>
       <c r="B21" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A21)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A21,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A21,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A21,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A21,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G21" s="12">
-        <f>B21-H21-COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B21-H21-COUNTIFS(Backlog!$C$2:$C$319,$A21,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A21,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A21,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A21,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A21,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7640,31 +7687,31 @@
         </is>
       </c>
       <c r="B22" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A22)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A22,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A22,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A22,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A22,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G22" s="12">
-        <f>B22-H22-COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B22-H22-COUNTIFS(Backlog!$C$2:$C$319,$A22,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A22,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A22,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A22,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A22,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7675,31 +7722,31 @@
         </is>
       </c>
       <c r="B23" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A23)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A23)</f>
         <v/>
       </c>
       <c r="C23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A23,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A23,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A23,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A23,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G23" s="12">
-        <f>B23-H23-COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B23-H23-COUNTIFS(Backlog!$C$2:$C$319,$A23,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A23,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A23,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A23,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A23,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7710,31 +7757,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A24)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A24,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A24,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A24,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A24,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>B24-H24-COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B24-H24-COUNTIFS(Backlog!$C$2:$C$319,$A24,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A24,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A24,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A24,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A24,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7745,31 +7792,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A25)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A25,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A25,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A25,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A25,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>B25-H25-COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B25-H25-COUNTIFS(Backlog!$C$2:$C$319,$A25,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A25,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A25,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A25,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A25,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7780,31 +7827,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A26)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A26,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A26,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A26,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A26,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>B26-H26-COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B26-H26-COUNTIFS(Backlog!$C$2:$C$319,$A26,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A26,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A26,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A26,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A26,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7815,31 +7862,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A27)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A27,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A27,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A27,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A27,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>B27-H27-COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B27-H27-COUNTIFS(Backlog!$C$2:$C$319,$A27,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A27,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A27,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A27,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A27,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7850,31 +7897,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A28)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A28,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A28,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A28,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A28,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>B28-H28-COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B28-H28-COUNTIFS(Backlog!$C$2:$C$319,$A28,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A28,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A28,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A28,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A28,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7885,31 +7932,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A29)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A29,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A29,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A29,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A29,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>B29-H29-COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B29-H29-COUNTIFS(Backlog!$C$2:$C$319,$A29,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A29,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A29,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A29,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A29,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7920,31 +7967,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A30)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A30,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A30,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A30,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A30,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>B30-H30-COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B30-H30-COUNTIFS(Backlog!$C$2:$C$319,$A30,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A30,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A30,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A30,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A30,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7955,31 +8002,31 @@
         </is>
       </c>
       <c r="B31" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A31)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A31,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A31,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A31,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A31,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G31" s="12">
-        <f>B31-H31-COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B31-H31-COUNTIFS(Backlog!$C$2:$C$319,$A31,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A31,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A31,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A31,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A31,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -7990,31 +8037,31 @@
         </is>
       </c>
       <c r="B32" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A32)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A32,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A32,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A32,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A32,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G32" s="12">
-        <f>B32-H32-COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B32-H32-COUNTIFS(Backlog!$C$2:$C$319,$A32,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A32,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A32,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A32,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A32,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8025,31 +8072,31 @@
         </is>
       </c>
       <c r="B33" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A33)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A33)</f>
         <v/>
       </c>
       <c r="C33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A33,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A33,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A33,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A33,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G33" s="12">
-        <f>B33-H33-COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B33-H33-COUNTIFS(Backlog!$C$2:$C$319,$A33,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A33,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A33,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A33,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A33,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8060,31 +8107,31 @@
         </is>
       </c>
       <c r="B34" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A34)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A34)</f>
         <v/>
       </c>
       <c r="C34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A34,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A34,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A34,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A34,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G34" s="12">
-        <f>B34-H34-COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B34-H34-COUNTIFS(Backlog!$C$2:$C$319,$A34,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A34,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A34,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A34,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A34,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8095,31 +8142,31 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A35)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A35)</f>
         <v/>
       </c>
       <c r="C35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A35,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A35,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A35,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A35,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G35" s="12">
-        <f>B35-H35-COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B35-H35-COUNTIFS(Backlog!$C$2:$C$319,$A35,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A35,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A35,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A35,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A35,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8130,31 +8177,31 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A36)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A36)</f>
         <v/>
       </c>
       <c r="C36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A36,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A36,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A36,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A36,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G36" s="12">
-        <f>B36-H36-COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B36-H36-COUNTIFS(Backlog!$C$2:$C$319,$A36,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A36,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A36,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A36,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A36,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8165,31 +8212,31 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A37)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A37,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A37,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A37,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A37,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G37" s="12">
-        <f>B37-H37-COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B37-H37-COUNTIFS(Backlog!$C$2:$C$319,$A37,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A37,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A37,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A37,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A37,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8200,31 +8247,31 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A38)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A38,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A38,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A38,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A38,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G38" s="12">
-        <f>B38-H38-COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B38-H38-COUNTIFS(Backlog!$C$2:$C$319,$A38,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A38,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A38,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A38,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A38,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8235,31 +8282,31 @@
         </is>
       </c>
       <c r="B39" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A39)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A39,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A39,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A39,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A39,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G39" s="12">
-        <f>B39-H39-COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B39-H39-COUNTIFS(Backlog!$C$2:$C$319,$A39,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A39,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A39,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A39,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A39,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8270,31 +8317,31 @@
         </is>
       </c>
       <c r="B40" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A40)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A40,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A40,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A40,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A40,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G40" s="12">
-        <f>B40-H40-COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B40-H40-COUNTIFS(Backlog!$C$2:$C$319,$A40,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A40,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A40,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A40,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A40,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8305,31 +8352,31 @@
         </is>
       </c>
       <c r="B41" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A41)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A41,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A41,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A41,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A41,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G41" s="12">
-        <f>B41-H41-COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B41-H41-COUNTIFS(Backlog!$C$2:$C$319,$A41,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A41,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A41,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A41,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A41,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8340,31 +8387,31 @@
         </is>
       </c>
       <c r="B42" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A42)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A42,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A42,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A42,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A42,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G42" s="12">
-        <f>B42-H42-COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B42-H42-COUNTIFS(Backlog!$C$2:$C$319,$A42,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A42,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A42,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A42,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A42,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8375,31 +8422,31 @@
         </is>
       </c>
       <c r="B43" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A43)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A43,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A43,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A43,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A43,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G43" s="12">
-        <f>B43-H43-COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B43-H43-COUNTIFS(Backlog!$C$2:$C$319,$A43,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A43,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A43,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A43,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A43,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8410,31 +8457,31 @@
         </is>
       </c>
       <c r="B44" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A44)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A44,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A44,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A44,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A44,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G44" s="12">
-        <f>B44-H44-COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B44-H44-COUNTIFS(Backlog!$C$2:$C$319,$A44,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A44,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A44,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A44,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A44,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8445,31 +8492,31 @@
         </is>
       </c>
       <c r="B45" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A45)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A45,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A45,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A45,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A45,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G45" s="12">
-        <f>B45-H45-COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B45-H45-COUNTIFS(Backlog!$C$2:$C$319,$A45,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A45,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A45,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A45,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A45,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8480,31 +8527,31 @@
         </is>
       </c>
       <c r="B46" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$315,$A46)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$319,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A46,Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="D46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$G$2:$G$315,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A46,Backlog!$G$2:$G$319,"P1")</f>
         <v/>
       </c>
       <c r="E46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$G$2:$G$315,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A46,Backlog!$G$2:$G$319,"P2")</f>
         <v/>
       </c>
       <c r="F46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$G$2:$G$315,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A46,Backlog!$G$2:$G$319,"P3")</f>
         <v/>
       </c>
       <c r="G46" s="12">
-        <f>B46-H46-COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$F$2:$F$315,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$F$2:$F$315,"Later")</f>
+        <f>B46-H46-COUNTIFS(Backlog!$C$2:$C$319,$A46,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$319,$A46,Backlog!$F$2:$F$319,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$319,$A46,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="H46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$315,$A46,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$319,$A46,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8572,23 +8619,23 @@
         </is>
       </c>
       <c r="B50" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A50)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A50,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A50,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A50,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A50,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E50" s="12">
-        <f>B50-C50-D50-COUNTIFS(Backlog!$R$2:$R$315,$A50,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A50,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B50-C50-D50-COUNTIFS(Backlog!$R$2:$R$319,$A50,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A50,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A50,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A50,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G50" s="12" t="n"/>
@@ -8601,23 +8648,23 @@
         </is>
       </c>
       <c r="B51" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A51)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A51)</f>
         <v/>
       </c>
       <c r="C51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A51,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A51,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A51,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A51,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E51" s="12">
-        <f>B51-C51-D51-COUNTIFS(Backlog!$R$2:$R$315,$A51,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A51,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B51-C51-D51-COUNTIFS(Backlog!$R$2:$R$319,$A51,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A51,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A51,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A51,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G51" s="12" t="n"/>
@@ -8630,23 +8677,23 @@
         </is>
       </c>
       <c r="B52" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A52)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A52)</f>
         <v/>
       </c>
       <c r="C52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A52,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A52,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A52,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A52,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E52" s="12">
-        <f>B52-C52-D52-COUNTIFS(Backlog!$R$2:$R$315,$A52,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A52,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B52-C52-D52-COUNTIFS(Backlog!$R$2:$R$319,$A52,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A52,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A52,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A52,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G52" s="12" t="n"/>
@@ -8659,23 +8706,23 @@
         </is>
       </c>
       <c r="B53" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A53)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A53)</f>
         <v/>
       </c>
       <c r="C53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A53,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A53,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A53,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A53,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E53" s="12">
-        <f>B53-C53-D53-COUNTIFS(Backlog!$R$2:$R$315,$A53,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A53,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B53-C53-D53-COUNTIFS(Backlog!$R$2:$R$319,$A53,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A53,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A53,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A53,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G53" s="12" t="n"/>
@@ -8688,23 +8735,23 @@
         </is>
       </c>
       <c r="B54" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A54)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A54)</f>
         <v/>
       </c>
       <c r="C54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A54,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A54,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A54,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A54,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E54" s="12">
-        <f>B54-C54-D54-COUNTIFS(Backlog!$R$2:$R$315,$A54,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A54,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B54-C54-D54-COUNTIFS(Backlog!$R$2:$R$319,$A54,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A54,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A54,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A54,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G54" s="12" t="n"/>
@@ -8717,23 +8764,23 @@
         </is>
       </c>
       <c r="B55" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A55)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A55,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A55,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A55,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A55,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E55" s="12">
-        <f>B55-C55-D55-COUNTIFS(Backlog!$R$2:$R$315,$A55,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A55,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B55-C55-D55-COUNTIFS(Backlog!$R$2:$R$319,$A55,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A55,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A55,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A55,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G55" s="12" t="n"/>
@@ -8746,23 +8793,23 @@
         </is>
       </c>
       <c r="B56" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A56)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A56,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A56,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A56,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A56,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E56" s="12">
-        <f>B56-C56-D56-COUNTIFS(Backlog!$R$2:$R$315,$A56,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A56,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B56-C56-D56-COUNTIFS(Backlog!$R$2:$R$319,$A56,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A56,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A56,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A56,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G56" s="12" t="n"/>
@@ -8775,23 +8822,23 @@
         </is>
       </c>
       <c r="B57" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A57)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A57,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A57,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A57,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A57,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E57" s="12">
-        <f>B57-C57-D57-COUNTIFS(Backlog!$R$2:$R$315,$A57,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A57,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B57-C57-D57-COUNTIFS(Backlog!$R$2:$R$319,$A57,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A57,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A57,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A57,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G57" s="12" t="n"/>
@@ -8804,23 +8851,23 @@
         </is>
       </c>
       <c r="B58" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A58)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A58,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A58,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A58,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A58,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E58" s="12">
-        <f>B58-C58-D58-COUNTIFS(Backlog!$R$2:$R$315,$A58,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A58,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B58-C58-D58-COUNTIFS(Backlog!$R$2:$R$319,$A58,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A58,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A58,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A58,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G58" s="12" t="n"/>
@@ -8833,23 +8880,23 @@
         </is>
       </c>
       <c r="B59" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A59)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A59,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A59,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A59,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A59,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E59" s="12">
-        <f>B59-C59-D59-COUNTIFS(Backlog!$R$2:$R$315,$A59,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A59,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B59-C59-D59-COUNTIFS(Backlog!$R$2:$R$319,$A59,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A59,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A59,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A59,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G59" s="12" t="n"/>
@@ -8862,23 +8909,23 @@
         </is>
       </c>
       <c r="B60" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A60)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A60,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A60,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A60,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A60,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E60" s="12">
-        <f>B60-C60-D60-COUNTIFS(Backlog!$R$2:$R$315,$A60,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A60,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B60-C60-D60-COUNTIFS(Backlog!$R$2:$R$319,$A60,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A60,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A60,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A60,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G60" s="12" t="n"/>
@@ -8891,23 +8938,23 @@
         </is>
       </c>
       <c r="B61" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A61)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A61,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A61,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A61,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A61,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E61" s="12">
-        <f>B61-C61-D61-COUNTIFS(Backlog!$R$2:$R$315,$A61,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A61,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B61-C61-D61-COUNTIFS(Backlog!$R$2:$R$319,$A61,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A61,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A61,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A61,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G61" s="12" t="n"/>
@@ -8920,23 +8967,23 @@
         </is>
       </c>
       <c r="B62" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A62)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A62,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A62,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A62,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A62,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E62" s="12">
-        <f>B62-C62-D62-COUNTIFS(Backlog!$R$2:$R$315,$A62,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A62,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B62-C62-D62-COUNTIFS(Backlog!$R$2:$R$319,$A62,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A62,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A62,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A62,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G62" s="12" t="n"/>
@@ -8949,23 +8996,23 @@
         </is>
       </c>
       <c r="B63" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A63)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A63,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A63,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A63,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A63,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E63" s="12">
-        <f>B63-C63-D63-COUNTIFS(Backlog!$R$2:$R$315,$A63,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A63,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B63-C63-D63-COUNTIFS(Backlog!$R$2:$R$319,$A63,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A63,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A63,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A63,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G63" s="12" t="n"/>
@@ -8978,23 +9025,23 @@
         </is>
       </c>
       <c r="B64" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A64)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A64,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A64,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A64,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A64,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E64" s="12">
-        <f>B64-C64-D64-COUNTIFS(Backlog!$R$2:$R$315,$A64,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A64,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B64-C64-D64-COUNTIFS(Backlog!$R$2:$R$319,$A64,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A64,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A64,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A64,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G64" s="12" t="n"/>
@@ -9007,23 +9054,23 @@
         </is>
       </c>
       <c r="B65" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A65)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A65,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A65,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A65,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A65,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E65" s="12">
-        <f>B65-C65-D65-COUNTIFS(Backlog!$R$2:$R$315,$A65,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A65,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B65-C65-D65-COUNTIFS(Backlog!$R$2:$R$319,$A65,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A65,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A65,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A65,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G65" s="12" t="n"/>
@@ -9036,23 +9083,23 @@
         </is>
       </c>
       <c r="B66" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A66)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A66,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A66,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A66,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A66,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E66" s="12">
-        <f>B66-C66-D66-COUNTIFS(Backlog!$R$2:$R$315,$A66,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A66,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B66-C66-D66-COUNTIFS(Backlog!$R$2:$R$319,$A66,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A66,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A66,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A66,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G66" s="12" t="n"/>
@@ -9065,23 +9112,23 @@
         </is>
       </c>
       <c r="B67" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A67)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A67,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A67,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A67,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A67,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E67" s="12">
-        <f>B67-C67-D67-COUNTIFS(Backlog!$R$2:$R$315,$A67,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A67,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B67-C67-D67-COUNTIFS(Backlog!$R$2:$R$319,$A67,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A67,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A67,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A67,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G67" s="12" t="n"/>
@@ -9094,23 +9141,23 @@
         </is>
       </c>
       <c r="B68" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A68)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A68,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A68,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A68,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A68,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E68" s="12">
-        <f>B68-C68-D68-COUNTIFS(Backlog!$R$2:$R$315,$A68,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A68,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B68-C68-D68-COUNTIFS(Backlog!$R$2:$R$319,$A68,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A68,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A68,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A68,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G68" s="12" t="n"/>
@@ -9123,23 +9170,23 @@
         </is>
       </c>
       <c r="B69" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A69)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A69,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A69,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A69,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A69,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E69" s="12">
-        <f>B69-C69-D69-COUNTIFS(Backlog!$R$2:$R$315,$A69,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A69,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B69-C69-D69-COUNTIFS(Backlog!$R$2:$R$319,$A69,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A69,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A69,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A69,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G69" s="12" t="n"/>
@@ -9152,23 +9199,23 @@
         </is>
       </c>
       <c r="B70" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A70)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A70,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A70,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A70,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A70,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E70" s="12">
-        <f>B70-C70-D70-COUNTIFS(Backlog!$R$2:$R$315,$A70,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A70,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B70-C70-D70-COUNTIFS(Backlog!$R$2:$R$319,$A70,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A70,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A70,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A70,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G70" s="12" t="n"/>
@@ -9181,23 +9228,23 @@
         </is>
       </c>
       <c r="B71" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A71)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A71,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A71,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A71,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A71,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E71" s="12">
-        <f>B71-C71-D71-COUNTIFS(Backlog!$R$2:$R$315,$A71,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A71,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B71-C71-D71-COUNTIFS(Backlog!$R$2:$R$319,$A71,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A71,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A71,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A71,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G71" s="12" t="n"/>
@@ -9210,23 +9257,23 @@
         </is>
       </c>
       <c r="B72" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A72)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A72,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A72,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A72,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A72,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E72" s="12">
-        <f>B72-C72-D72-COUNTIFS(Backlog!$R$2:$R$315,$A72,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A72,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B72-C72-D72-COUNTIFS(Backlog!$R$2:$R$319,$A72,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A72,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A72,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A72,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G72" s="12" t="n"/>
@@ -9239,23 +9286,23 @@
         </is>
       </c>
       <c r="B73" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$315,$A73)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$319,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A73,Backlog!$F$2:$F$315,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A73,Backlog!$F$2:$F$319,"Done")</f>
         <v/>
       </c>
       <c r="D73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A73,Backlog!$F$2:$F$315,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A73,Backlog!$F$2:$F$319,"Later")</f>
         <v/>
       </c>
       <c r="E73" s="12">
-        <f>B73-C73-D73-COUNTIFS(Backlog!$R$2:$R$315,$A73,Backlog!$F$2:$F$315,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$315,$A73,Backlog!$F$2:$F$315,"Obsolete")</f>
+        <f>B73-C73-D73-COUNTIFS(Backlog!$R$2:$R$319,$A73,Backlog!$F$2:$F$319,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$319,$A73,Backlog!$F$2:$F$319,"Obsolete")</f>
         <v/>
       </c>
       <c r="F73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$315,$A73,Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$319,$A73,Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="G73" s="12" t="n"/>
@@ -9277,7 +9324,7 @@
         </is>
       </c>
       <c r="B75" s="12">
-        <f>COUNTIF(Backlog!$S$2:$S$315,"Yes")</f>
+        <f>COUNTIF(Backlog!$S$2:$S$319,"Yes")</f>
         <v/>
       </c>
       <c r="C75" s="12" t="n"/>
@@ -9294,7 +9341,7 @@
         </is>
       </c>
       <c r="B76" s="12">
-        <f>COUNTIFS(Backlog!$S$2:$S$315,"Yes",Backlog!$G$2:$G$315,"P0")</f>
+        <f>COUNTIFS(Backlog!$S$2:$S$319,"Yes",Backlog!$G$2:$G$319,"P0")</f>
         <v/>
       </c>
       <c r="C76" s="12" t="n"/>
@@ -9311,7 +9358,7 @@
         </is>
       </c>
       <c r="B77" s="12">
-        <f>COUNTIFS(Backlog!$S$2:$S$315,"No",Backlog!$G$2:$G$315,"P0",Backlog!$F$2:$F$315,"&lt;&gt;Done",Backlog!$F$2:$F$315,"&lt;&gt;Later",Backlog!$F$2:$F$315,"&lt;&gt;Cancelled",Backlog!$F$2:$F$315,"&lt;&gt;Obsolete")</f>
+        <f>COUNTIFS(Backlog!$S$2:$S$319,"No",Backlog!$G$2:$G$319,"P0",Backlog!$F$2:$F$319,"&lt;&gt;Done",Backlog!$F$2:$F$319,"&lt;&gt;Later",Backlog!$F$2:$F$319,"&lt;&gt;Cancelled",Backlog!$F$2:$F$319,"&lt;&gt;Obsolete")</f>
         <v/>
       </c>
       <c r="C77" s="12" t="n"/>
@@ -9328,7 +9375,7 @@
         </is>
       </c>
       <c r="B78" s="12">
-        <f>COUNTIF(Backlog!$F$2:$F$315,"Hold")</f>
+        <f>COUNTIF(Backlog!$F$2:$F$319,"Hold")</f>
         <v/>
       </c>
       <c r="C78" s="12" t="n"/>
@@ -9354,7 +9401,7 @@
         </is>
       </c>
       <c r="B80" s="12">
-        <f>COUNTIFS(Backlog!$G$2:$G$315,"P0",Backlog!$F$2:$F$315,"&lt;&gt;Done",Backlog!$F$2:$F$315,"&lt;&gt;Cancelled",Backlog!$F$2:$F$315,"&lt;&gt;Obsolete",Backlog!$F$2:$F$315,"&lt;&gt;Later")</f>
+        <f>COUNTIFS(Backlog!$G$2:$G$319,"P0",Backlog!$F$2:$F$319,"&lt;&gt;Done",Backlog!$F$2:$F$319,"&lt;&gt;Cancelled",Backlog!$F$2:$F$319,"&lt;&gt;Obsolete",Backlog!$F$2:$F$319,"&lt;&gt;Later")</f>
         <v/>
       </c>
       <c r="C80" s="12" t="n"/>
@@ -9371,7 +9418,7 @@
         </is>
       </c>
       <c r="B81" s="12">
-        <f>COUNTIFS(Backlog!$N$2:$N$315,"Sales blocker",Backlog!$F$2:$F$315,"&lt;&gt;Done")</f>
+        <f>COUNTIFS(Backlog!$N$2:$N$319,"Sales blocker",Backlog!$F$2:$F$319,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="C81" s="12" t="n"/>
@@ -9388,7 +9435,7 @@
         </is>
       </c>
       <c r="B82" s="12">
-        <f>COUNTIFS(Backlog!$E$2:$E$315,"Decision Needed",Backlog!$F$2:$F$315,"&lt;&gt;Done")</f>
+        <f>COUNTIFS(Backlog!$E$2:$E$319,"Decision Needed",Backlog!$F$2:$F$319,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="C82" s="12" t="n"/>
@@ -10318,7 +10365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10700,6 +10747,21 @@
       <c r="C27" s="8" t="inlineStr">
         <is>
           <t>Owner decision 2026-10-22: the database is fully code-first. A new environment is installed and every release updated by the migrator (startup or Admin &gt; Database Update); no hand-run SQL for schema setup or updates. Needed DDL that EF cannot model goes into a migration (migrationBuilder.Sql); superseded SQL moves to legacy-trash/, it is not deleted until the owner agrees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Settings in env files, secrets apart, nothing hard-coded</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Owner decision 2026-10-23: every setting lives in env/&lt;name&gt;.env, every secret only in env/&lt;name&gt;.secrets.env (git-ignored) or an environment variable, for local, docker, demo, uat and production-&lt;customer&gt;. No environment-dependent value (URL, host, credential, port, lifetime, culture, policy flag) is hard-coded in code; a new setting is added to every env file and read with Required*. Customer differences are the production-&lt;customer&gt;.env file and the licence (rule 17).</t>
         </is>
       </c>
     </row>
@@ -10714,7 +10776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S315"/>
+  <dimension ref="A1:S319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -37861,9 +37923,345 @@
         </is>
       </c>
     </row>
+    <row r="316">
+      <c r="A316" s="10" t="n">
+        <v>315</v>
+      </c>
+      <c r="B316" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C316" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D316" s="8" t="inlineStr">
+        <is>
+          <t>Environment settings and secrets files for local, docker, demo, uat and production-kangan; no hard-coded settings in code</t>
+        </is>
+      </c>
+      <c r="E316" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F316" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G316" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H316" s="8" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-23. Before: settings in appsettings.json/.Development/.UAT plus literals in code (Fido2, Ollama URL, password policy, cookie, log retention, culture, built-in admin account and password, design-time connection string, docker-compose defaults). Now: env/&lt;name&gt;.env (settings, committed) and env/&lt;name&gt;.secrets.env (secrets, git-ignored, templates *.secrets.env.example); PEMS_ENV selects the file; loader PEMS.Shared EnvFiles + AddPemsEnvFiles (precedence: env file &lt; secrets file &lt; environment variables &lt; command line); required settings fail fast; appsettings.json is empty; the first administrator comes from Seed:Admin:*; the dotnet ef factory reads the env files; docker-compose, Dockerfile, Build-Package and the demo pipeline use them. VERIFIED 2026-10-23: the real app booted on LocalDB from env/local.env + env/local.secrets.env alone (no environment variables), created and installed the database and seeded the admin, whose secret password signs in (a wrong one is refused); a missing env file and a missing required setting stop startup with a clear message; the web.config transformation yields well-formed XML. TESTS 2026-10-23: new env tests 10/10; Help 110/110, Letters 261/261, HTTP security host 9/9 (boots Program from the env files), Deployment 29/30 and Web 240/241 and Authorization 19/20 - the three remaining failures are pre-existing and unrelated (LF-only assertion on a Windows autocrlf checkout; a test that refuses non-SQLEXPRESS; ImportCenterNavigationTests flags LetterCompose and fails identically on a clean origin/main).</t>
+        </is>
+      </c>
+      <c r="I316" s="8" t="inlineStr">
+        <is>
+          <t>Run the demo pipeline once with the new secrets (#317); install on the Linux VM with PEMS_ENV set (#316).</t>
+        </is>
+      </c>
+      <c r="J316" s="8" t="inlineStr">
+        <is>
+          <t>Every setting is in an env file, every secret only in a secrets file or an environment variable, the committed files contain no secrets (test), all environments define the same keys (test), and the app starts from the files alone.</t>
+        </is>
+      </c>
+      <c r="K316" s="8" t="inlineStr">
+        <is>
+          <t>Local commits on branch temp/code-first-database ('feat(config): environment settings and secrets files ...'). Not pushed.</t>
+        </is>
+      </c>
+      <c r="L316" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M316" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N316" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O316" s="10" t="inlineStr">
+        <is>
+          <t>#309 #295 #167</t>
+        </is>
+      </c>
+      <c r="P316" s="10" t="n"/>
+      <c r="Q316" s="10" t="n"/>
+      <c r="R316" s="8" t="inlineStr">
+        <is>
+          <t>Install &amp; update</t>
+        </is>
+      </c>
+      <c r="S316" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="10" t="n">
+        <v>316</v>
+      </c>
+      <c r="B317" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C317" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D317" s="8" t="inlineStr">
+        <is>
+          <t>Linux VM kit: set PEMS_ENV and ship the matching env file; adapt pems-docker.sh adopt-env and the VM env file to the new settings</t>
+        </is>
+      </c>
+      <c r="E317" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F317" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G317" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H317" s="8" t="inlineStr">
+        <is>
+          <t>The VM kit's pems-web container env file (generated by adopt-env, VM-only) relied on appsettings.json defaults that no longer exist. Build-Package now ships env/*.env but the VM environment must add PEMS_ENV (for example production-kangan) and the secret keys, otherwise startup stops on the first missing required setting.</t>
+        </is>
+      </c>
+      <c r="I317" s="8" t="inlineStr">
+        <is>
+          <t>Update deploy/remote/pems-docker.sh (adopt-env) and the runbook so the VM env file contains PEMS_ENV and the secret keys, extend the mock harness test; do not touch the live VM without the owner.</t>
+        </is>
+      </c>
+      <c r="J317" s="8" t="inlineStr">
+        <is>
+          <t>A release package starts on the VM with PEMS_ENV set; adopt-env writes the new keys; the kit tests pass.</t>
+        </is>
+      </c>
+      <c r="K317" s="8" t="n"/>
+      <c r="L317" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M317" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N317" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O317" s="10" t="inlineStr">
+        <is>
+          <t>#315</t>
+        </is>
+      </c>
+      <c r="P317" s="10" t="n"/>
+      <c r="Q317" s="10" t="n"/>
+      <c r="R317" s="8" t="inlineStr">
+        <is>
+          <t>Install &amp; update</t>
+        </is>
+      </c>
+      <c r="S317" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="10" t="n">
+        <v>317</v>
+      </c>
+      <c r="B318" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C318" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D318" s="8" t="inlineStr">
+        <is>
+          <t>Provide and protect the real secrets: GitHub secrets for the demo, fill the REPLACE values in env/production-kangan.env, create the production secrets file on the server, rotate every secret pasted into chat</t>
+        </is>
+      </c>
+      <c r="E318" s="10" t="inlineStr">
+        <is>
+          <t>Ops Process</t>
+        </is>
+      </c>
+      <c r="F318" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G318" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H318" s="8" t="inlineStr">
+        <is>
+          <t>The demo FTP password and the demo database password were pasted into a chat session, and the public repository exposed a default admin password in code (now removed). Secrets must exist only in GitHub secrets, env/*.secrets.env on servers, or a vault.</t>
+        </is>
+      </c>
+      <c r="I318" s="8" t="inlineStr">
+        <is>
+          <t>Rotate the demo FTP and demo database passwords; add DEMO_FTP_*, DEMO_SQL_CONNECTION_STRING, DEMO_ADMIN_PASSWORD and DEMO_SITE_URL as GitHub secrets; set the Kangan domain and name in env/production-kangan.env; create env/production-kangan.secrets.env (mode 600) on the server; change the default admin password on every existing database.</t>
+        </is>
+      </c>
+      <c r="J318" s="8" t="inlineStr">
+        <is>
+          <t>No still-valid secret remains in the repository, its history or chat; the demo pipeline runs with GitHub secrets only.</t>
+        </is>
+      </c>
+      <c r="K318" s="8" t="n"/>
+      <c r="L318" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M318" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N318" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O318" s="10" t="inlineStr">
+        <is>
+          <t>#315 #295</t>
+        </is>
+      </c>
+      <c r="P318" s="10" t="n"/>
+      <c r="Q318" s="10" t="n"/>
+      <c r="R318" s="8" t="inlineStr">
+        <is>
+          <t>Install &amp; update</t>
+        </is>
+      </c>
+      <c r="S318" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="10" t="n">
+        <v>318</v>
+      </c>
+      <c r="B319" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C319" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D319" s="8" t="inlineStr">
+        <is>
+          <t>Second pass over remaining in-code constants: classify each as a setting (move to env files), a policy constant (document) or a domain rule</t>
+        </is>
+      </c>
+      <c r="E319" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F319" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G319" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H319" s="8" t="inlineStr">
+        <is>
+          <t>The first pass moved environment-dependent values (URLs, credentials, ports, lifetimes, culture, password policy, log retention). Other literals remain, for example HSTS/redirect behaviour, cookie SameSite, upload size limits, page sizes, SignalR and Hangfire options, default pagination, timeouts in services.</t>
+        </is>
+      </c>
+      <c r="I319" s="8" t="inlineStr">
+        <is>
+          <t>Search Program.cs and the services for numeric/string literals, decide per item, move the settings into every env file with Required* and a test, and record the policy constants in a short document.</t>
+        </is>
+      </c>
+      <c r="J319" s="8" t="inlineStr">
+        <is>
+          <t>A list of each remaining literal with its classification; settings moved; tests keep the key sets identical.</t>
+        </is>
+      </c>
+      <c r="K319" s="8" t="n"/>
+      <c r="L319" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M319" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N319" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O319" s="10" t="inlineStr">
+        <is>
+          <t>#315</t>
+        </is>
+      </c>
+      <c r="P319" s="10" t="n"/>
+      <c r="Q319" s="10" t="n"/>
+      <c r="R319" s="8" t="inlineStr">
+        <is>
+          <t>Install &amp; update</t>
+        </is>
+      </c>
+      <c r="S319" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S315"/>
-  <conditionalFormatting sqref="F2:F315">
+  <autoFilter ref="A1:S319"/>
+  <conditionalFormatting sqref="F2:F319">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
@@ -37886,7 +38284,7 @@
       <formula>"Obsolete"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G315">
+  <conditionalFormatting sqref="G2:G319">
     <cfRule type="cellIs" priority="8" operator="equal" dxfId="6">
       <formula>"P0"</formula>
     </cfRule>
@@ -37894,27 +38292,27 @@
       <formula>"P1"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S315">
+  <conditionalFormatting sqref="S2:S319">
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N315">
+  <conditionalFormatting sqref="N2:N319">
     <cfRule type="cellIs" priority="11" operator="equal" dxfId="6">
       <formula>"Sales blocker"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="F2:F315" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F319" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Partial,Done,Hold,Later,Cancelled,Obsolete"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G315" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G319" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B315" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B2:B319" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Claude,User,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S315" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="S2:S319" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -37928,7 +38326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -39047,10 +39445,124 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="10" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>315</v>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>App starts from the env files alone</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>env/local.env and env/local.secrets.env; no environment variables; an empty database.</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Start the app. Expected: 'Settings loaded for environment local' in the log, database installed, the administrator from Seed:Admin:* signs in with the secrets-file password.</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Risk if it fails: Developers and customers cannot start the product.</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>Needs QA</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="10" t="n">
+        <v>315</v>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Missing settings fail fast</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Remove one required key (for example Fido2__ServerDomain) or set PEMS_ENV to an unknown name.</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Start the app. Expected: it stops with a message naming the missing key or file, never with a silent default.</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Risk if it fails: A mis-configured server runs with wrong defaults.</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>Needs QA</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="10" t="n">
+        <v>315</v>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Secrets never ship</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>A release package, a docker image and the demo upload.</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Inspect each: only env/&lt;name&gt;.env is present; env/*.secrets.env appears only where the pipeline or operator placed it; the repository has no secrets file.</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Risk if it fails: Credentials leak through a package or the repository.</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>Needs QA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H29"/>
+  <autoFilter ref="A1:H32"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H2:H32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Needs QA,Pass,Fail,Blocked"</formula1>
     </dataValidation>
   </dataValidations>
@@ -39134,7 +39646,7 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$315,"M0")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$319,"M0")</f>
         <v/>
       </c>
     </row>
@@ -39165,7 +39677,7 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$315,"M1")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$319,"M1")</f>
         <v/>
       </c>
     </row>
@@ -39196,7 +39708,7 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$315,"M2")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$319,"M2")</f>
         <v/>
       </c>
     </row>
@@ -39227,7 +39739,7 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$315,"M3")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$319,"M3")</f>
         <v/>
       </c>
     </row>
@@ -39258,7 +39770,7 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$315,"M4")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$319,"M4")</f>
         <v/>
       </c>
     </row>
@@ -39289,7 +39801,7 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$315,"M5")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$319,"M5")</f>
         <v/>
       </c>
     </row>
@@ -39320,7 +39832,7 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$315,"M6")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$319,"M6")</f>
         <v/>
       </c>
     </row>
@@ -41415,7 +41927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -42158,8 +42670,33 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>One settings contract: files for settings, files for secrets, nothing in code</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>PEMS (2026-10-23)</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Settings were spread over appsettings.*.json, in-code '?? default' values and a built-in administrator password in a public repository. Keep one key set per environment in committed env files, secrets only in git-ignored files or environment variables, required keys that fail fast, and tests that keep key sets identical and scan the committed files for secrets. A dependency-free reader is needed where the configuration packages cannot be referenced (design-time EF factory).</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>#315 #316 #317</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A10:E35"/>
+  <autoFilter ref="A10:E36"/>
   <mergeCells count="6">
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="B4:E4"/>

</xml_diff>

<commit_message>
chore(plan): #340 make the demo site start (TLS certificate, startup diagnosis) added to Sprint 1; demo evidence on #295/#312
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$340</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$341</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Plan'!$A$1:$H$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Roadmap'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Capability Checklist'!$A$1:$H$37</definedName>
@@ -599,6 +599,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -606,6 +607,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -620,6 +622,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -634,6 +637,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -648,6 +652,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -662,6 +667,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -676,6 +682,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -690,6 +697,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
@@ -732,6 +740,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -804,6 +813,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
@@ -1604,6 +1614,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -8142,6 +8153,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -8149,7 +8161,7 @@
         </is>
       </c>
       <c r="B3" s="12">
-        <f>COUNTA(Backlog!$D$2:$D$340)</f>
+        <f>COUNTA(Backlog!$D$2:$D$341)</f>
         <v/>
       </c>
       <c r="C3" s="12" t="n"/>
@@ -8166,7 +8178,7 @@
         </is>
       </c>
       <c r="B4" s="12">
-        <f>COUNTIF(Backlog!$B$2:$B$340,"User")</f>
+        <f>COUNTIF(Backlog!$B$2:$B$341,"User")</f>
         <v/>
       </c>
       <c r="C4" s="12" t="n"/>
@@ -8240,19 +8252,19 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A8,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A8,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A8,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A8,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A8,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A8,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A8,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A8,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="F8" s="12">
@@ -8269,19 +8281,19 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A9,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A9,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A9,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A9,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A9,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A9,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A9,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A9,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="F9" s="12">
@@ -8298,19 +8310,19 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A10,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A10,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A10,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A10,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A10,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A10,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A10,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A10,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="F10" s="12">
@@ -8327,19 +8339,19 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A11,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A11,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A11,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A11,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A11,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A11,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A11,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A11,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="F11" s="12">
@@ -8356,19 +8368,19 @@
         </is>
       </c>
       <c r="B12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A12,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A12,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="C12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A12,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A12,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A12,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A12,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="E12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A12,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A12,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="F12" s="12">
@@ -8385,19 +8397,19 @@
         </is>
       </c>
       <c r="B13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A13,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A13,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="C13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A13,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A13,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A13,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A13,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="E13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A13,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A13,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="F13" s="12">
@@ -8414,19 +8426,19 @@
         </is>
       </c>
       <c r="B14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A14,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A14,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="C14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A14,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A14,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="D14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A14,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A14,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="E14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A14,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A14,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="F14" s="12">
@@ -8443,19 +8455,19 @@
         </is>
       </c>
       <c r="B15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A15,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A15,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="C15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A15,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A15,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="D15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A15,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A15,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="E15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$340,$A15,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$341,$A15,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="F15" s="12">
@@ -8566,31 +8578,31 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A20)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A20,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A20,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A20,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A20,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G20" s="12">
-        <f>B20-H20-COUNTIFS(Backlog!$C$2:$C$340,$A20,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A20,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A20,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B20-H20-COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A20,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8601,31 +8613,31 @@
         </is>
       </c>
       <c r="B21" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A21)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A21,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A21,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A21,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A21,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G21" s="12">
-        <f>B21-H21-COUNTIFS(Backlog!$C$2:$C$340,$A21,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A21,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A21,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B21-H21-COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A21,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8636,31 +8648,31 @@
         </is>
       </c>
       <c r="B22" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A22)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A22,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A22,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A22,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A22,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G22" s="12">
-        <f>B22-H22-COUNTIFS(Backlog!$C$2:$C$340,$A22,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A22,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A22,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B22-H22-COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A22,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8671,31 +8683,31 @@
         </is>
       </c>
       <c r="B23" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A23)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A23)</f>
         <v/>
       </c>
       <c r="C23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A23,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A23,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A23,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A23,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G23" s="12">
-        <f>B23-H23-COUNTIFS(Backlog!$C$2:$C$340,$A23,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A23,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A23,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B23-H23-COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A23,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8706,31 +8718,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A24)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A24,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A24,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A24,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A24,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>B24-H24-COUNTIFS(Backlog!$C$2:$C$340,$A24,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A24,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A24,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B24-H24-COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A24,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8741,31 +8753,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A25)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A25,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A25,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A25,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A25,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>B25-H25-COUNTIFS(Backlog!$C$2:$C$340,$A25,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A25,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A25,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B25-H25-COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A25,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8776,31 +8788,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A26)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A26,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A26,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A26,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A26,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>B26-H26-COUNTIFS(Backlog!$C$2:$C$340,$A26,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A26,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A26,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B26-H26-COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A26,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8811,31 +8823,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A27)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A27,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A27,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A27,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A27,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>B27-H27-COUNTIFS(Backlog!$C$2:$C$340,$A27,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A27,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A27,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B27-H27-COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A27,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8846,31 +8858,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A28)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A28,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A28,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A28,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A28,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>B28-H28-COUNTIFS(Backlog!$C$2:$C$340,$A28,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A28,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A28,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B28-H28-COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A28,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8881,31 +8893,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A29)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A29,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A29,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A29,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A29,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>B29-H29-COUNTIFS(Backlog!$C$2:$C$340,$A29,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A29,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A29,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B29-H29-COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A29,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8916,31 +8928,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A30)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A30,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A30,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A30,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A30,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>B30-H30-COUNTIFS(Backlog!$C$2:$C$340,$A30,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A30,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A30,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B30-H30-COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A30,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8951,31 +8963,31 @@
         </is>
       </c>
       <c r="B31" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A31)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A31,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A31,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A31,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A31,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G31" s="12">
-        <f>B31-H31-COUNTIFS(Backlog!$C$2:$C$340,$A31,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A31,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A31,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B31-H31-COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A31,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8986,31 +8998,31 @@
         </is>
       </c>
       <c r="B32" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A32)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A32,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A32,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A32,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A32,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G32" s="12">
-        <f>B32-H32-COUNTIFS(Backlog!$C$2:$C$340,$A32,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A32,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A32,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B32-H32-COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A32,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9021,31 +9033,31 @@
         </is>
       </c>
       <c r="B33" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A33)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A33)</f>
         <v/>
       </c>
       <c r="C33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A33,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A33,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A33,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A33,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G33" s="12">
-        <f>B33-H33-COUNTIFS(Backlog!$C$2:$C$340,$A33,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A33,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A33,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B33-H33-COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A33,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9056,31 +9068,31 @@
         </is>
       </c>
       <c r="B34" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A34)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A34)</f>
         <v/>
       </c>
       <c r="C34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A34,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A34,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A34,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A34,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G34" s="12">
-        <f>B34-H34-COUNTIFS(Backlog!$C$2:$C$340,$A34,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A34,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A34,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B34-H34-COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A34,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9091,31 +9103,31 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A35)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A35)</f>
         <v/>
       </c>
       <c r="C35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A35,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A35,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A35,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A35,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G35" s="12">
-        <f>B35-H35-COUNTIFS(Backlog!$C$2:$C$340,$A35,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A35,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A35,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B35-H35-COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A35,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9126,31 +9138,31 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A36)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A36)</f>
         <v/>
       </c>
       <c r="C36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A36,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A36,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A36,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A36,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G36" s="12">
-        <f>B36-H36-COUNTIFS(Backlog!$C$2:$C$340,$A36,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A36,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A36,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B36-H36-COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A36,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9161,31 +9173,31 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A37)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A37,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A37,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A37,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A37,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G37" s="12">
-        <f>B37-H37-COUNTIFS(Backlog!$C$2:$C$340,$A37,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A37,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A37,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B37-H37-COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A37,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9196,31 +9208,31 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A38)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A38,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A38,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A38,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A38,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G38" s="12">
-        <f>B38-H38-COUNTIFS(Backlog!$C$2:$C$340,$A38,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A38,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A38,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B38-H38-COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A38,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9231,31 +9243,31 @@
         </is>
       </c>
       <c r="B39" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A39)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A39,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A39,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A39,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A39,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G39" s="12">
-        <f>B39-H39-COUNTIFS(Backlog!$C$2:$C$340,$A39,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A39,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A39,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B39-H39-COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A39,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9266,31 +9278,31 @@
         </is>
       </c>
       <c r="B40" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A40)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A40,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A40,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A40,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A40,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G40" s="12">
-        <f>B40-H40-COUNTIFS(Backlog!$C$2:$C$340,$A40,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A40,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A40,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B40-H40-COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A40,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9301,31 +9313,31 @@
         </is>
       </c>
       <c r="B41" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A41)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A41,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A41,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A41,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A41,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G41" s="12">
-        <f>B41-H41-COUNTIFS(Backlog!$C$2:$C$340,$A41,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A41,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A41,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B41-H41-COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A41,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9336,31 +9348,31 @@
         </is>
       </c>
       <c r="B42" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A42)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A42,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A42,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A42,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A42,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G42" s="12">
-        <f>B42-H42-COUNTIFS(Backlog!$C$2:$C$340,$A42,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A42,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A42,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B42-H42-COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A42,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9371,31 +9383,31 @@
         </is>
       </c>
       <c r="B43" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A43)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A43,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A43,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A43,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A43,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G43" s="12">
-        <f>B43-H43-COUNTIFS(Backlog!$C$2:$C$340,$A43,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A43,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A43,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B43-H43-COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A43,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9406,31 +9418,31 @@
         </is>
       </c>
       <c r="B44" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A44)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A44,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A44,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A44,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A44,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G44" s="12">
-        <f>B44-H44-COUNTIFS(Backlog!$C$2:$C$340,$A44,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A44,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A44,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B44-H44-COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A44,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9441,31 +9453,31 @@
         </is>
       </c>
       <c r="B45" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A45)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A45,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A45,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A45,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A45,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G45" s="12">
-        <f>B45-H45-COUNTIFS(Backlog!$C$2:$C$340,$A45,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A45,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A45,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B45-H45-COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A45,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9476,31 +9488,31 @@
         </is>
       </c>
       <c r="B46" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$340,$A46)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$341,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A46,Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="D46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A46,Backlog!$G$2:$G$340,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$G$2:$G$341,"P1")</f>
         <v/>
       </c>
       <c r="E46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A46,Backlog!$G$2:$G$340,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$G$2:$G$341,"P2")</f>
         <v/>
       </c>
       <c r="F46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A46,Backlog!$G$2:$G$340,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$G$2:$G$341,"P3")</f>
         <v/>
       </c>
       <c r="G46" s="12">
-        <f>B46-H46-COUNTIFS(Backlog!$C$2:$C$340,$A46,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$340,$A46,Backlog!$F$2:$F$340,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$340,$A46,Backlog!$F$2:$F$340,"Later")</f>
+        <f>B46-H46-COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="H46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$340,$A46,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9568,23 +9580,23 @@
         </is>
       </c>
       <c r="B50" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A50)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A50,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A50,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A50,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A50,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E50" s="12">
-        <f>B50-C50-D50-COUNTIFS(Backlog!$R$2:$R$340,$A50,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A50,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B50-C50-D50-COUNTIFS(Backlog!$R$2:$R$341,$A50,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A50,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A50,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A50,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G50" s="12" t="n"/>
@@ -9597,23 +9609,23 @@
         </is>
       </c>
       <c r="B51" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A51)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A51)</f>
         <v/>
       </c>
       <c r="C51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A51,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A51,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A51,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A51,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E51" s="12">
-        <f>B51-C51-D51-COUNTIFS(Backlog!$R$2:$R$340,$A51,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A51,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B51-C51-D51-COUNTIFS(Backlog!$R$2:$R$341,$A51,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A51,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A51,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A51,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G51" s="12" t="n"/>
@@ -9626,23 +9638,23 @@
         </is>
       </c>
       <c r="B52" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A52)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A52)</f>
         <v/>
       </c>
       <c r="C52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A52,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A52,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A52,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A52,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E52" s="12">
-        <f>B52-C52-D52-COUNTIFS(Backlog!$R$2:$R$340,$A52,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A52,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B52-C52-D52-COUNTIFS(Backlog!$R$2:$R$341,$A52,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A52,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A52,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A52,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G52" s="12" t="n"/>
@@ -9655,23 +9667,23 @@
         </is>
       </c>
       <c r="B53" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A53)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A53)</f>
         <v/>
       </c>
       <c r="C53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A53,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A53,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A53,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A53,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E53" s="12">
-        <f>B53-C53-D53-COUNTIFS(Backlog!$R$2:$R$340,$A53,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A53,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B53-C53-D53-COUNTIFS(Backlog!$R$2:$R$341,$A53,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A53,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A53,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A53,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G53" s="12" t="n"/>
@@ -9684,23 +9696,23 @@
         </is>
       </c>
       <c r="B54" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A54)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A54)</f>
         <v/>
       </c>
       <c r="C54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A54,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A54,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A54,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A54,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E54" s="12">
-        <f>B54-C54-D54-COUNTIFS(Backlog!$R$2:$R$340,$A54,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A54,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B54-C54-D54-COUNTIFS(Backlog!$R$2:$R$341,$A54,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A54,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A54,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A54,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G54" s="12" t="n"/>
@@ -9713,23 +9725,23 @@
         </is>
       </c>
       <c r="B55" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A55)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A55,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A55,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A55,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A55,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E55" s="12">
-        <f>B55-C55-D55-COUNTIFS(Backlog!$R$2:$R$340,$A55,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A55,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B55-C55-D55-COUNTIFS(Backlog!$R$2:$R$341,$A55,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A55,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A55,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A55,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G55" s="12" t="n"/>
@@ -9742,23 +9754,23 @@
         </is>
       </c>
       <c r="B56" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A56)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A56,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A56,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A56,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A56,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E56" s="12">
-        <f>B56-C56-D56-COUNTIFS(Backlog!$R$2:$R$340,$A56,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A56,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B56-C56-D56-COUNTIFS(Backlog!$R$2:$R$341,$A56,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A56,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A56,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A56,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G56" s="12" t="n"/>
@@ -9771,23 +9783,23 @@
         </is>
       </c>
       <c r="B57" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A57)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A57,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A57,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A57,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A57,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E57" s="12">
-        <f>B57-C57-D57-COUNTIFS(Backlog!$R$2:$R$340,$A57,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A57,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B57-C57-D57-COUNTIFS(Backlog!$R$2:$R$341,$A57,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A57,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A57,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A57,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G57" s="12" t="n"/>
@@ -9800,23 +9812,23 @@
         </is>
       </c>
       <c r="B58" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A58)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A58,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A58,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A58,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A58,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E58" s="12">
-        <f>B58-C58-D58-COUNTIFS(Backlog!$R$2:$R$340,$A58,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A58,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B58-C58-D58-COUNTIFS(Backlog!$R$2:$R$341,$A58,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A58,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A58,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A58,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G58" s="12" t="n"/>
@@ -9829,23 +9841,23 @@
         </is>
       </c>
       <c r="B59" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A59)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A59,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A59,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A59,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A59,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E59" s="12">
-        <f>B59-C59-D59-COUNTIFS(Backlog!$R$2:$R$340,$A59,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A59,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B59-C59-D59-COUNTIFS(Backlog!$R$2:$R$341,$A59,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A59,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A59,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A59,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G59" s="12" t="n"/>
@@ -9858,23 +9870,23 @@
         </is>
       </c>
       <c r="B60" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A60)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A60,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A60,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A60,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A60,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E60" s="12">
-        <f>B60-C60-D60-COUNTIFS(Backlog!$R$2:$R$340,$A60,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A60,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B60-C60-D60-COUNTIFS(Backlog!$R$2:$R$341,$A60,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A60,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A60,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A60,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G60" s="12" t="n"/>
@@ -9887,23 +9899,23 @@
         </is>
       </c>
       <c r="B61" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A61)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A61,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A61,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A61,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A61,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E61" s="12">
-        <f>B61-C61-D61-COUNTIFS(Backlog!$R$2:$R$340,$A61,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A61,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B61-C61-D61-COUNTIFS(Backlog!$R$2:$R$341,$A61,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A61,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A61,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A61,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G61" s="12" t="n"/>
@@ -9916,23 +9928,23 @@
         </is>
       </c>
       <c r="B62" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A62)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A62,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A62,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A62,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A62,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E62" s="12">
-        <f>B62-C62-D62-COUNTIFS(Backlog!$R$2:$R$340,$A62,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A62,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B62-C62-D62-COUNTIFS(Backlog!$R$2:$R$341,$A62,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A62,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A62,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A62,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G62" s="12" t="n"/>
@@ -9945,23 +9957,23 @@
         </is>
       </c>
       <c r="B63" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A63)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A63,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A63,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A63,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A63,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E63" s="12">
-        <f>B63-C63-D63-COUNTIFS(Backlog!$R$2:$R$340,$A63,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A63,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B63-C63-D63-COUNTIFS(Backlog!$R$2:$R$341,$A63,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A63,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A63,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A63,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G63" s="12" t="n"/>
@@ -9974,23 +9986,23 @@
         </is>
       </c>
       <c r="B64" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A64)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A64,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A64,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A64,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A64,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E64" s="12">
-        <f>B64-C64-D64-COUNTIFS(Backlog!$R$2:$R$340,$A64,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A64,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B64-C64-D64-COUNTIFS(Backlog!$R$2:$R$341,$A64,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A64,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A64,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A64,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G64" s="12" t="n"/>
@@ -10003,23 +10015,23 @@
         </is>
       </c>
       <c r="B65" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A65)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A65,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A65,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A65,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A65,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E65" s="12">
-        <f>B65-C65-D65-COUNTIFS(Backlog!$R$2:$R$340,$A65,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A65,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B65-C65-D65-COUNTIFS(Backlog!$R$2:$R$341,$A65,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A65,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A65,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A65,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G65" s="12" t="n"/>
@@ -10032,23 +10044,23 @@
         </is>
       </c>
       <c r="B66" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A66)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A66,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A66,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A66,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A66,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E66" s="12">
-        <f>B66-C66-D66-COUNTIFS(Backlog!$R$2:$R$340,$A66,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A66,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B66-C66-D66-COUNTIFS(Backlog!$R$2:$R$341,$A66,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A66,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A66,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A66,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G66" s="12" t="n"/>
@@ -10061,23 +10073,23 @@
         </is>
       </c>
       <c r="B67" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A67)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A67,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A67,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A67,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A67,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E67" s="12">
-        <f>B67-C67-D67-COUNTIFS(Backlog!$R$2:$R$340,$A67,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A67,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B67-C67-D67-COUNTIFS(Backlog!$R$2:$R$341,$A67,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A67,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A67,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A67,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G67" s="12" t="n"/>
@@ -10090,23 +10102,23 @@
         </is>
       </c>
       <c r="B68" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A68)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A68,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A68,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A68,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A68,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E68" s="12">
-        <f>B68-C68-D68-COUNTIFS(Backlog!$R$2:$R$340,$A68,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A68,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B68-C68-D68-COUNTIFS(Backlog!$R$2:$R$341,$A68,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A68,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A68,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A68,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G68" s="12" t="n"/>
@@ -10119,23 +10131,23 @@
         </is>
       </c>
       <c r="B69" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A69)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A69,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A69,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A69,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A69,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E69" s="12">
-        <f>B69-C69-D69-COUNTIFS(Backlog!$R$2:$R$340,$A69,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A69,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B69-C69-D69-COUNTIFS(Backlog!$R$2:$R$341,$A69,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A69,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A69,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A69,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G69" s="12" t="n"/>
@@ -10148,23 +10160,23 @@
         </is>
       </c>
       <c r="B70" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A70)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A70,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A70,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A70,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A70,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E70" s="12">
-        <f>B70-C70-D70-COUNTIFS(Backlog!$R$2:$R$340,$A70,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A70,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B70-C70-D70-COUNTIFS(Backlog!$R$2:$R$341,$A70,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A70,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A70,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A70,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G70" s="12" t="n"/>
@@ -10177,23 +10189,23 @@
         </is>
       </c>
       <c r="B71" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A71)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A71,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A71,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A71,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A71,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E71" s="12">
-        <f>B71-C71-D71-COUNTIFS(Backlog!$R$2:$R$340,$A71,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A71,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B71-C71-D71-COUNTIFS(Backlog!$R$2:$R$341,$A71,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A71,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A71,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A71,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G71" s="12" t="n"/>
@@ -10206,23 +10218,23 @@
         </is>
       </c>
       <c r="B72" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A72)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A72,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A72,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A72,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A72,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E72" s="12">
-        <f>B72-C72-D72-COUNTIFS(Backlog!$R$2:$R$340,$A72,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A72,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B72-C72-D72-COUNTIFS(Backlog!$R$2:$R$341,$A72,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A72,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A72,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A72,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G72" s="12" t="n"/>
@@ -10235,23 +10247,23 @@
         </is>
       </c>
       <c r="B73" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$340,$A73)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$341,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A73,Backlog!$F$2:$F$340,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A73,Backlog!$F$2:$F$341,"Done")</f>
         <v/>
       </c>
       <c r="D73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A73,Backlog!$F$2:$F$340,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A73,Backlog!$F$2:$F$341,"Later")</f>
         <v/>
       </c>
       <c r="E73" s="12">
-        <f>B73-C73-D73-COUNTIFS(Backlog!$R$2:$R$340,$A73,Backlog!$F$2:$F$340,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$340,$A73,Backlog!$F$2:$F$340,"Obsolete")</f>
+        <f>B73-C73-D73-COUNTIFS(Backlog!$R$2:$R$341,$A73,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A73,Backlog!$F$2:$F$341,"Obsolete")</f>
         <v/>
       </c>
       <c r="F73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$340,$A73,Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$341,$A73,Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="G73" s="12" t="n"/>
@@ -10273,7 +10285,7 @@
         </is>
       </c>
       <c r="B75" s="12">
-        <f>COUNTIF(Backlog!$S$2:$S$340,"Yes")</f>
+        <f>COUNTIF(Backlog!$S$2:$S$341,"Yes")</f>
         <v/>
       </c>
       <c r="C75" s="12" t="n"/>
@@ -10290,7 +10302,7 @@
         </is>
       </c>
       <c r="B76" s="12">
-        <f>COUNTIFS(Backlog!$S$2:$S$340,"Yes",Backlog!$G$2:$G$340,"P0")</f>
+        <f>COUNTIFS(Backlog!$S$2:$S$341,"Yes",Backlog!$G$2:$G$341,"P0")</f>
         <v/>
       </c>
       <c r="C76" s="12" t="n"/>
@@ -10307,7 +10319,7 @@
         </is>
       </c>
       <c r="B77" s="12">
-        <f>COUNTIFS(Backlog!$S$2:$S$340,"No",Backlog!$G$2:$G$340,"P0",Backlog!$F$2:$F$340,"&lt;&gt;Done",Backlog!$F$2:$F$340,"&lt;&gt;Later",Backlog!$F$2:$F$340,"&lt;&gt;Cancelled",Backlog!$F$2:$F$340,"&lt;&gt;Obsolete")</f>
+        <f>COUNTIFS(Backlog!$S$2:$S$341,"No",Backlog!$G$2:$G$341,"P0",Backlog!$F$2:$F$341,"&lt;&gt;Done",Backlog!$F$2:$F$341,"&lt;&gt;Later",Backlog!$F$2:$F$341,"&lt;&gt;Cancelled",Backlog!$F$2:$F$341,"&lt;&gt;Obsolete")</f>
         <v/>
       </c>
       <c r="C77" s="12" t="n"/>
@@ -10324,7 +10336,7 @@
         </is>
       </c>
       <c r="B78" s="12">
-        <f>COUNTIF(Backlog!$F$2:$F$340,"Hold")</f>
+        <f>COUNTIF(Backlog!$F$2:$F$341,"Hold")</f>
         <v/>
       </c>
       <c r="C78" s="12" t="n"/>
@@ -10350,7 +10362,7 @@
         </is>
       </c>
       <c r="B80" s="12">
-        <f>COUNTIFS(Backlog!$G$2:$G$340,"P0",Backlog!$F$2:$F$340,"&lt;&gt;Done",Backlog!$F$2:$F$340,"&lt;&gt;Cancelled",Backlog!$F$2:$F$340,"&lt;&gt;Obsolete",Backlog!$F$2:$F$340,"&lt;&gt;Later")</f>
+        <f>COUNTIFS(Backlog!$G$2:$G$341,"P0",Backlog!$F$2:$F$341,"&lt;&gt;Done",Backlog!$F$2:$F$341,"&lt;&gt;Cancelled",Backlog!$F$2:$F$341,"&lt;&gt;Obsolete",Backlog!$F$2:$F$341,"&lt;&gt;Later")</f>
         <v/>
       </c>
       <c r="C80" s="12" t="n"/>
@@ -10367,7 +10379,7 @@
         </is>
       </c>
       <c r="B81" s="12">
-        <f>COUNTIFS(Backlog!$N$2:$N$340,"Sales blocker",Backlog!$F$2:$F$340,"&lt;&gt;Done")</f>
+        <f>COUNTIFS(Backlog!$N$2:$N$341,"Sales blocker",Backlog!$F$2:$F$341,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="C81" s="12" t="n"/>
@@ -10384,7 +10396,7 @@
         </is>
       </c>
       <c r="B82" s="12">
-        <f>COUNTIFS(Backlog!$E$2:$E$340,"Decision Needed",Backlog!$F$2:$F$340,"&lt;&gt;Done")</f>
+        <f>COUNTIFS(Backlog!$E$2:$E$341,"Decision Needed",Backlog!$F$2:$F$341,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="C82" s="12" t="n"/>
@@ -10435,6 +10447,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -10598,6 +10611,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
@@ -10857,6 +10871,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
@@ -10912,6 +10927,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
@@ -10979,6 +10995,7 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
@@ -11355,6 +11372,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -11773,7 +11791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U340"/>
+  <dimension ref="A1:U341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -37972,7 +37990,7 @@
       </c>
       <c r="H296" s="8" t="inlineStr">
         <is>
-          <t>Owner requirement 2026-10-18: the demo is a branch of the main repository, deployed to the main host by GitHub Actions and completely separate from the landing website's deployment. 2026-10-22: .github/workflows/deploy-demo.yml now builds, runs the model-drift gate and tests, publishes self-contained win-x64, injects the demo connection string and Database settings, uploads by FTP and waits for /health/database = UpToDate (install on the first deploy, update afterwards) - see #312. Not yet run on GitHub; sample-data pack, demo licence, rollback and backup steps are still open.</t>
+          <t>Owner requirement 2026-10-18: the demo is a branch of the main repository, deployed to the main host by GitHub Actions and completely separate from the landing website's deployment. 2026-10-22: .github/workflows/deploy-demo.yml now builds, runs the model-drift gate and tests, publishes self-contained win-x64, injects the demo connection string and Database settings, uploads by FTP and waits for /health/database = UpToDate (install on the first deploy, update afterwards) - see #312. Not yet run on GitHub; sample-data pack, demo licence, rollback and backup steps are still open. 2026-10-24 first runs on the demo branch: build, drift gate, database-free tests, publish and the FTP upload from the GitHub runner PASS; the post-deploy health check failed - the demo site has no valid TLS certificate and the application does not answer on first start (details and steps: docs/deployment/DEMO_DEPLOYMENT.md, row #340).</t>
         </is>
       </c>
       <c r="I296" s="8" t="inlineStr">
@@ -39429,7 +39447,7 @@
       </c>
       <c r="H313" s="8" t="inlineStr">
         <is>
-          <t>deploy-demo.yml: model-drift gate (dotnet ef migrations has-pending-model-changes), jq injects the demo connection string and Database={CreateIfMissing:false,MigrateOnStartup:true}, sed raises the IIS startupTimeLimit to 900 s (the first run installs the whole schema before serving), FTP upload, then polls DEMO_SITE_URL/health/database until UpToDate (fails the run after 30 minutes). YAML validated; web.config patch checked on a real publish. Not yet executed on GitHub.</t>
+          <t>deploy-demo.yml: model-drift gate (dotnet ef migrations has-pending-model-changes), jq injects the demo connection string and Database={CreateIfMissing:false,MigrateOnStartup:true}, sed raises the IIS startupTimeLimit to 900 s (the first run installs the whole schema before serving), FTP upload, then polls DEMO_SITE_URL/health/database until UpToDate (fails the run after 30 minutes). YAML validated; web.config patch checked on a real publish. Not yet executed on GitHub. 2026-10-24 first runs on the demo branch: build, drift gate, database-free tests, publish and the FTP upload from the GitHub runner PASS; the post-deploy health check failed - the demo site has no valid TLS certificate and the application does not answer on first start (details and steps: docs/deployment/DEMO_DEPLOYMENT.md, row #340).</t>
         </is>
       </c>
       <c r="I313" s="8" t="inlineStr">
@@ -41817,9 +41835,106 @@
         </is>
       </c>
     </row>
+    <row r="341">
+      <c r="A341" s="10" t="n">
+        <v>340</v>
+      </c>
+      <c r="B341" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C341" s="8" t="inlineStr">
+        <is>
+          <t>Online Demo</t>
+        </is>
+      </c>
+      <c r="D341" s="8" t="inlineStr">
+        <is>
+          <t>Make the demo site start: issue the TLS certificate and diagnose why the application does not answer after the first deploy</t>
+        </is>
+      </c>
+      <c r="E341" s="10" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="F341" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G341" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H341" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-24 findings: the pipeline now reaches the host (upload passes) but https://demo.parmisata.ir fails certificate verification (Plesk shows 'Domain not secured') and, with verification off, a request hangs and is reset after about 60 seconds. The first start installs about 116 migrations and the seeders, or it fails on startup (database unreachable from the web host, ASP.NET Core Module missing, app pool stopped).</t>
+        </is>
+      </c>
+      <c r="I341" s="8" t="inlineStr">
+        <is>
+          <t>1) In Plesk open the subdomain, SSL/TLS Certificates, and get a free Let's Encrypt certificate for demo.parmisata.ir. 2) Re-run the demo workflow (it now writes logs/stdout* on the server and the health probe tolerates the certificate). 3) Open Plesk &gt; Files &gt; logs and read logs/stdout* and logs/pems-*.log. 4) Fix the cause shown there: check the connection string in DEMO_SQL_CONNECTION_STRING (Server=10.45.12.3, no ':0'; try ',1433'), the ASP.NET Core Module and the app pool, and SQL Full-Text only if the log asks. 5) Confirm with curl -sSk https://demo.parmisata.ir/health/database.</t>
+        </is>
+      </c>
+      <c r="J341" s="8" t="inlineStr">
+        <is>
+          <t>Done when: https://demo.parmisata.ir opens with a valid certificate; /health/database returns UpToDate; the demo workflow run is green end to end; the cause and fix are written in docs/deployment/DEMO_DEPLOYMENT.md.</t>
+        </is>
+      </c>
+      <c r="K341" s="8" t="inlineStr">
+        <is>
+          <t>Pipeline hardening committed (insecure health probe, TLS report, stdout logs, 60-minute upload limit); server-side steps need the hosting panel.</t>
+        </is>
+      </c>
+      <c r="L341" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M341" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N341" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O341" s="10" t="inlineStr">
+        <is>
+          <t>#312 #295</t>
+        </is>
+      </c>
+      <c r="P341" s="10" t="n"/>
+      <c r="Q341" s="10" t="n"/>
+      <c r="R341" s="8" t="inlineStr">
+        <is>
+          <t>Online demo</t>
+        </is>
+      </c>
+      <c r="S341" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T341" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="U341" s="10" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U340"/>
-  <conditionalFormatting sqref="F2:F340">
+  <autoFilter ref="A1:U341"/>
+  <conditionalFormatting sqref="F2:F341">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
@@ -41842,7 +41957,7 @@
       <formula>"Obsolete"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G340">
+  <conditionalFormatting sqref="G2:G341">
     <cfRule type="cellIs" priority="8" operator="equal" dxfId="6">
       <formula>"P0"</formula>
     </cfRule>
@@ -41850,27 +41965,27 @@
       <formula>"P1"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S340">
+  <conditionalFormatting sqref="S2:S341">
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N340">
+  <conditionalFormatting sqref="N2:N341">
     <cfRule type="cellIs" priority="11" operator="equal" dxfId="6">
       <formula>"Sales blocker"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="F2:F340" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F341" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Partial,Done,Hold,Later,Cancelled,Obsolete"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G340" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G341" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B340" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B2:B341" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Claude,User,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S340" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="S2:S341" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -43280,7 +43395,7 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$340,"M0")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$341,"M0")</f>
         <v/>
       </c>
     </row>
@@ -43311,7 +43426,7 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$340,"M1")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$341,"M1")</f>
         <v/>
       </c>
     </row>
@@ -43342,7 +43457,7 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$340,"M2")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$341,"M2")</f>
         <v/>
       </c>
     </row>
@@ -43373,7 +43488,7 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$340,"M3")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$341,"M3")</f>
         <v/>
       </c>
     </row>
@@ -43404,7 +43519,7 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$340,"M4")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$341,"M4")</f>
         <v/>
       </c>
     </row>
@@ -43435,7 +43550,7 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$340,"M5")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$341,"M5")</f>
         <v/>
       </c>
     </row>
@@ -43466,10 +43581,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$340,"M6")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$341,"M6")</f>
         <v/>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
@@ -43539,7 +43655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -44323,6 +44439,46 @@
       <c r="H26" s="15" t="inlineStr">
         <is>
           <t>Done when: the solution builds and the tests pass; the HTTP smoke tests still pass; PEMS.Web renders the same pages with its assets served from PEMS.UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="n">
+        <v>340</v>
+      </c>
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>Make the demo site start: issue the TLS certificate and diagnose why the application does not answer after the first deploy</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>Member B</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="H27" s="15" t="inlineStr">
+        <is>
+          <t>Done when: https://demo.parmisata.ir opens with a valid certificate; /health/database returns UpToDate; the demo workflow run is green end to end; the cause and fix are written in docs/deployment/DEMO_DEPLOYMENT.md.</t>
         </is>
       </c>
     </row>
@@ -44361,6 +44517,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -44537,6 +44694,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
@@ -46330,6 +46488,8 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs+ci: demo pipeline green end to end; record causes and fixes; docs-only pushes do not redeploy; plan #312 done, #340 revised
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -599,7 +599,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -607,7 +606,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -622,7 +620,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -637,7 +634,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -652,7 +648,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -667,7 +662,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -682,7 +676,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -697,7 +690,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
@@ -740,7 +732,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -813,7 +804,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
@@ -1614,7 +1604,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -8153,7 +8142,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -10447,7 +10435,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -10611,7 +10598,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
@@ -10871,7 +10857,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
@@ -10927,7 +10912,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
@@ -10995,7 +10979,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
@@ -11372,7 +11355,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -37990,7 +37972,7 @@
       </c>
       <c r="H296" s="8" t="inlineStr">
         <is>
-          <t>Owner requirement 2026-10-18: the demo is a branch of the main repository, deployed to the main host by GitHub Actions and completely separate from the landing website's deployment. 2026-10-22: .github/workflows/deploy-demo.yml now builds, runs the model-drift gate and tests, publishes self-contained win-x64, injects the demo connection string and Database settings, uploads by FTP and waits for /health/database = UpToDate (install on the first deploy, update afterwards) - see #312. Not yet run on GitHub; sample-data pack, demo licence, rollback and backup steps are still open. 2026-10-24 first runs on the demo branch: build, drift gate, database-free tests, publish and the FTP upload from the GitHub runner PASS; the post-deploy health check failed - the demo site has no valid TLS certificate and the application does not answer on first start (details and steps: docs/deployment/DEMO_DEPLOYMENT.md, row #340).</t>
+          <t>Owner requirement 2026-10-18: the demo is a branch of the main repository, deployed to the main host by GitHub Actions and completely separate from the landing website's deployment. 2026-10-22: .github/workflows/deploy-demo.yml now builds, runs the model-drift gate and tests, publishes self-contained win-x64, injects the demo connection string and Database settings, uploads by FTP and waits for /health/database = UpToDate (install on the first deploy, update afterwards) - see #312. Not yet run on GitHub; sample-data pack, demo licence, rollback and backup steps are still open. 2026-10-24 first runs on the demo branch: build, drift gate, database-free tests, publish and the FTP upload from the GitHub runner PASS; the post-deploy health check failed - the demo site has no valid TLS certificate and the application does not answer on first start (details and steps: docs/deployment/DEMO_DEPLOYMENT.md, row #340). 2026-10-24 update: the pipeline now deploys and installs the database (see #312); sample data, licence install, backup and rollback steps remain.</t>
         </is>
       </c>
       <c r="I296" s="8" t="inlineStr">
@@ -39437,7 +39419,7 @@
       </c>
       <c r="F313" s="10" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G313" s="10" t="inlineStr">
@@ -39462,7 +39444,7 @@
       </c>
       <c r="K313" s="8" t="inlineStr">
         <is>
-          <t>See #309 report.</t>
+          <t>2026-10-24 run 5 on the demo branch is green end to end: drift gate, database-free tests, publish, app_offline, FTP upload, health check 'attempt 1: HTTP 200 UpToDate' (the demo database was installed by the first start). Fixes needed on the way: dummy connection string for the drift gate, app_offline.htm (IIS file locks, FTP 550), 180 s FTP timeout plus one retry. Open: valid TLS certificate (#340).</t>
         </is>
       </c>
       <c r="L313" s="10" t="inlineStr">
@@ -41861,7 +41843,7 @@
       </c>
       <c r="F341" s="10" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="G341" s="10" t="inlineStr">
@@ -41871,17 +41853,17 @@
       </c>
       <c r="H341" s="8" t="inlineStr">
         <is>
-          <t>2026-10-24 findings: the pipeline now reaches the host (upload passes) but https://demo.parmisata.ir fails certificate verification (Plesk shows 'Domain not secured') and, with verification off, a request hangs and is reset after about 60 seconds. The first start installs about 116 migrations and the seeders, or it fails on startup (database unreachable from the web host, ASP.NET Core Module missing, app pool stopped).</t>
+          <t>2026-10-24 revised findings: the application DOES start and install its database when deployed (health check from the GitHub runner: HTTP 200 UpToDate). The earlier failures were pipeline issues (fixed in #312). Still open: (1) no valid TLS certificate on demo.parmisata.ir (Plesk shows 'Domain not secured'; the runner reports a verification failure); (2) the site does not answer from the developer machine's network (requests time out after 30-60 s) while it answers from GitHub - check the local route/ISP, or test from another network, before assuming a server fault.</t>
         </is>
       </c>
       <c r="I341" s="8" t="inlineStr">
         <is>
-          <t>1) In Plesk open the subdomain, SSL/TLS Certificates, and get a free Let's Encrypt certificate for demo.parmisata.ir. 2) Re-run the demo workflow (it now writes logs/stdout* on the server and the health probe tolerates the certificate). 3) Open Plesk &gt; Files &gt; logs and read logs/stdout* and logs/pems-*.log. 4) Fix the cause shown there: check the connection string in DEMO_SQL_CONNECTION_STRING (Server=10.45.12.3, no ':0'; try ',1433'), the ASP.NET Core Module and the app pool, and SQL Full-Text only if the log asks. 5) Confirm with curl -sSk https://demo.parmisata.ir/health/database.</t>
+          <t>1) In Plesk open the subdomain, SSL/TLS Certificates, get a free Let's Encrypt certificate for demo.parmisata.ir. 2) Open https://demo.parmisata.ir/health/database from a phone network and from the office network; compare with the result from GitHub (UpToDate). 3) If only the office network fails, ask the network owner to allow 185.10.74.207:443; if everywhere fails, read logs/stdout* and logs/pems-*.log in Plesk &gt; Files. 4) Sign in as the seeded administrator and open Admin &gt; Database Update to confirm 116 migrations.</t>
         </is>
       </c>
       <c r="J341" s="8" t="inlineStr">
         <is>
-          <t>Done when: https://demo.parmisata.ir opens with a valid certificate; /health/database returns UpToDate; the demo workflow run is green end to end; the cause and fix are written in docs/deployment/DEMO_DEPLOYMENT.md.</t>
+          <t>Done when: https://demo.parmisata.ir opens with a valid certificate from the team's networks; the administrator signs in; Admin &gt; Database Update shows the database up to date.</t>
         </is>
       </c>
       <c r="K341" s="8" t="inlineStr">
@@ -43585,7 +43567,6 @@
         <v/>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
@@ -43759,7 +43740,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
@@ -44517,7 +44497,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -44694,7 +44673,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
@@ -46488,8 +46466,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(plan): add issued-licence ledger, licence flow gate and owner-initiated admin reset rows (#341-#348)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$341</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$349</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Plan'!$A$1:$H$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Roadmap'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Capability Checklist'!$A$1:$H$37</definedName>
@@ -599,6 +599,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -606,6 +607,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -620,6 +622,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -634,6 +637,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -648,6 +652,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -662,6 +667,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -676,6 +682,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -690,6 +697,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
@@ -732,6 +740,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -804,6 +813,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
@@ -1604,6 +1614,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -8142,6 +8153,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -8149,7 +8161,7 @@
         </is>
       </c>
       <c r="B3" s="12">
-        <f>COUNTA(Backlog!$D$2:$D$341)</f>
+        <f>COUNTA(Backlog!$D$2:$D$349)</f>
         <v/>
       </c>
       <c r="C3" s="12" t="n"/>
@@ -8166,7 +8178,7 @@
         </is>
       </c>
       <c r="B4" s="12">
-        <f>COUNTIF(Backlog!$B$2:$B$341,"User")</f>
+        <f>COUNTIF(Backlog!$B$2:$B$349,"User")</f>
         <v/>
       </c>
       <c r="C4" s="12" t="n"/>
@@ -8240,19 +8252,19 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A8,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A8,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A8,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A8,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A8,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A8,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A8,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A8,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="F8" s="12">
@@ -8269,19 +8281,19 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A9,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A9,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A9,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A9,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A9,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A9,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A9,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A9,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="F9" s="12">
@@ -8298,19 +8310,19 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A10,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A10,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A10,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A10,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A10,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A10,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A10,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A10,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="F10" s="12">
@@ -8327,19 +8339,19 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A11,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A11,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A11,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A11,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A11,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A11,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A11,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A11,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="F11" s="12">
@@ -8356,19 +8368,19 @@
         </is>
       </c>
       <c r="B12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A12,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A12,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="C12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A12,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A12,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A12,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A12,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="E12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A12,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A12,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="F12" s="12">
@@ -8385,19 +8397,19 @@
         </is>
       </c>
       <c r="B13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A13,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A13,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="C13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A13,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A13,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A13,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A13,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="E13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A13,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A13,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="F13" s="12">
@@ -8414,19 +8426,19 @@
         </is>
       </c>
       <c r="B14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A14,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A14,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="C14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A14,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A14,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="D14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A14,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A14,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="E14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A14,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A14,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="F14" s="12">
@@ -8443,19 +8455,19 @@
         </is>
       </c>
       <c r="B15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A15,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A15,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="C15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A15,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A15,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="D15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A15,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A15,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="E15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$341,$A15,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$349,$A15,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="F15" s="12">
@@ -8566,31 +8578,31 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A20)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G20" s="12">
-        <f>B20-H20-COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B20-H20-COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A20,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8601,31 +8613,31 @@
         </is>
       </c>
       <c r="B21" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A21)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G21" s="12">
-        <f>B21-H21-COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B21-H21-COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A21,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8636,31 +8648,31 @@
         </is>
       </c>
       <c r="B22" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A22)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G22" s="12">
-        <f>B22-H22-COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B22-H22-COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A22,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8671,31 +8683,31 @@
         </is>
       </c>
       <c r="B23" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A23)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A23)</f>
         <v/>
       </c>
       <c r="C23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G23" s="12">
-        <f>B23-H23-COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B23-H23-COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A23,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8706,31 +8718,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A24)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>B24-H24-COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B24-H24-COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A24,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8741,31 +8753,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A25)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>B25-H25-COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B25-H25-COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A25,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8776,31 +8788,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A26)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>B26-H26-COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B26-H26-COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A26,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8811,31 +8823,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A27)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>B27-H27-COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B27-H27-COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A27,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8846,31 +8858,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A28)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>B28-H28-COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B28-H28-COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A28,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8881,31 +8893,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A29)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>B29-H29-COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B29-H29-COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A29,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8916,31 +8928,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A30)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>B30-H30-COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B30-H30-COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A30,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8951,31 +8963,31 @@
         </is>
       </c>
       <c r="B31" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A31)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G31" s="12">
-        <f>B31-H31-COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B31-H31-COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A31,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8986,31 +8998,31 @@
         </is>
       </c>
       <c r="B32" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A32)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G32" s="12">
-        <f>B32-H32-COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B32-H32-COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A32,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9021,31 +9033,31 @@
         </is>
       </c>
       <c r="B33" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A33)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A33)</f>
         <v/>
       </c>
       <c r="C33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G33" s="12">
-        <f>B33-H33-COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B33-H33-COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A33,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9056,31 +9068,31 @@
         </is>
       </c>
       <c r="B34" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A34)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A34)</f>
         <v/>
       </c>
       <c r="C34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G34" s="12">
-        <f>B34-H34-COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B34-H34-COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A34,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9091,31 +9103,31 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A35)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A35)</f>
         <v/>
       </c>
       <c r="C35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G35" s="12">
-        <f>B35-H35-COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B35-H35-COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A35,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9126,31 +9138,31 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A36)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A36)</f>
         <v/>
       </c>
       <c r="C36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G36" s="12">
-        <f>B36-H36-COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B36-H36-COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A36,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9161,31 +9173,31 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A37)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G37" s="12">
-        <f>B37-H37-COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B37-H37-COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A37,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9196,31 +9208,31 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A38)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G38" s="12">
-        <f>B38-H38-COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B38-H38-COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A38,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9231,31 +9243,31 @@
         </is>
       </c>
       <c r="B39" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A39)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G39" s="12">
-        <f>B39-H39-COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B39-H39-COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A39,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9266,31 +9278,31 @@
         </is>
       </c>
       <c r="B40" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A40)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G40" s="12">
-        <f>B40-H40-COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B40-H40-COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A40,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9301,31 +9313,31 @@
         </is>
       </c>
       <c r="B41" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A41)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G41" s="12">
-        <f>B41-H41-COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B41-H41-COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A41,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9336,31 +9348,31 @@
         </is>
       </c>
       <c r="B42" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A42)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G42" s="12">
-        <f>B42-H42-COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B42-H42-COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A42,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9371,31 +9383,31 @@
         </is>
       </c>
       <c r="B43" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A43)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G43" s="12">
-        <f>B43-H43-COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B43-H43-COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A43,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9406,31 +9418,31 @@
         </is>
       </c>
       <c r="B44" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A44)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G44" s="12">
-        <f>B44-H44-COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B44-H44-COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A44,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9441,31 +9453,31 @@
         </is>
       </c>
       <c r="B45" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A45)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G45" s="12">
-        <f>B45-H45-COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B45-H45-COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A45,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9476,31 +9488,31 @@
         </is>
       </c>
       <c r="B46" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$341,$A46)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$349,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="D46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$G$2:$G$341,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$G$2:$G$349,"P1")</f>
         <v/>
       </c>
       <c r="E46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$G$2:$G$341,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$G$2:$G$349,"P2")</f>
         <v/>
       </c>
       <c r="F46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$G$2:$G$341,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$G$2:$G$349,"P3")</f>
         <v/>
       </c>
       <c r="G46" s="12">
-        <f>B46-H46-COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$F$2:$F$341,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$F$2:$F$341,"Later")</f>
+        <f>B46-H46-COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="H46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$341,$A46,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9568,23 +9580,23 @@
         </is>
       </c>
       <c r="B50" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A50)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A50,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A50,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A50,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A50,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E50" s="12">
-        <f>B50-C50-D50-COUNTIFS(Backlog!$R$2:$R$341,$A50,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A50,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B50-C50-D50-COUNTIFS(Backlog!$R$2:$R$349,$A50,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A50,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A50,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A50,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G50" s="12" t="n"/>
@@ -9597,23 +9609,23 @@
         </is>
       </c>
       <c r="B51" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A51)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A51)</f>
         <v/>
       </c>
       <c r="C51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A51,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A51,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A51,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A51,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E51" s="12">
-        <f>B51-C51-D51-COUNTIFS(Backlog!$R$2:$R$341,$A51,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A51,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B51-C51-D51-COUNTIFS(Backlog!$R$2:$R$349,$A51,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A51,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A51,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A51,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G51" s="12" t="n"/>
@@ -9626,23 +9638,23 @@
         </is>
       </c>
       <c r="B52" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A52)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A52)</f>
         <v/>
       </c>
       <c r="C52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A52,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A52,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A52,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A52,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E52" s="12">
-        <f>B52-C52-D52-COUNTIFS(Backlog!$R$2:$R$341,$A52,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A52,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B52-C52-D52-COUNTIFS(Backlog!$R$2:$R$349,$A52,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A52,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A52,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A52,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G52" s="12" t="n"/>
@@ -9655,23 +9667,23 @@
         </is>
       </c>
       <c r="B53" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A53)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A53)</f>
         <v/>
       </c>
       <c r="C53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A53,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A53,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A53,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A53,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E53" s="12">
-        <f>B53-C53-D53-COUNTIFS(Backlog!$R$2:$R$341,$A53,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A53,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B53-C53-D53-COUNTIFS(Backlog!$R$2:$R$349,$A53,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A53,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A53,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A53,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G53" s="12" t="n"/>
@@ -9684,23 +9696,23 @@
         </is>
       </c>
       <c r="B54" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A54)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A54)</f>
         <v/>
       </c>
       <c r="C54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A54,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A54,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A54,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A54,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E54" s="12">
-        <f>B54-C54-D54-COUNTIFS(Backlog!$R$2:$R$341,$A54,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A54,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B54-C54-D54-COUNTIFS(Backlog!$R$2:$R$349,$A54,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A54,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A54,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A54,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G54" s="12" t="n"/>
@@ -9713,23 +9725,23 @@
         </is>
       </c>
       <c r="B55" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A55)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A55,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A55,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A55,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A55,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E55" s="12">
-        <f>B55-C55-D55-COUNTIFS(Backlog!$R$2:$R$341,$A55,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A55,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B55-C55-D55-COUNTIFS(Backlog!$R$2:$R$349,$A55,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A55,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A55,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A55,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G55" s="12" t="n"/>
@@ -9742,23 +9754,23 @@
         </is>
       </c>
       <c r="B56" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A56)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A56,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A56,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A56,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A56,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E56" s="12">
-        <f>B56-C56-D56-COUNTIFS(Backlog!$R$2:$R$341,$A56,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A56,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B56-C56-D56-COUNTIFS(Backlog!$R$2:$R$349,$A56,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A56,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A56,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A56,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G56" s="12" t="n"/>
@@ -9771,23 +9783,23 @@
         </is>
       </c>
       <c r="B57" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A57)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A57,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A57,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A57,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A57,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E57" s="12">
-        <f>B57-C57-D57-COUNTIFS(Backlog!$R$2:$R$341,$A57,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A57,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B57-C57-D57-COUNTIFS(Backlog!$R$2:$R$349,$A57,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A57,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A57,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A57,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G57" s="12" t="n"/>
@@ -9800,23 +9812,23 @@
         </is>
       </c>
       <c r="B58" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A58)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A58,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A58,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A58,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A58,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E58" s="12">
-        <f>B58-C58-D58-COUNTIFS(Backlog!$R$2:$R$341,$A58,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A58,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B58-C58-D58-COUNTIFS(Backlog!$R$2:$R$349,$A58,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A58,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A58,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A58,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G58" s="12" t="n"/>
@@ -9829,23 +9841,23 @@
         </is>
       </c>
       <c r="B59" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A59)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A59,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A59,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A59,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A59,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E59" s="12">
-        <f>B59-C59-D59-COUNTIFS(Backlog!$R$2:$R$341,$A59,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A59,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B59-C59-D59-COUNTIFS(Backlog!$R$2:$R$349,$A59,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A59,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A59,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A59,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G59" s="12" t="n"/>
@@ -9858,23 +9870,23 @@
         </is>
       </c>
       <c r="B60" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A60)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A60,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A60,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A60,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A60,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E60" s="12">
-        <f>B60-C60-D60-COUNTIFS(Backlog!$R$2:$R$341,$A60,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A60,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B60-C60-D60-COUNTIFS(Backlog!$R$2:$R$349,$A60,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A60,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A60,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A60,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G60" s="12" t="n"/>
@@ -9887,23 +9899,23 @@
         </is>
       </c>
       <c r="B61" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A61)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A61,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A61,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A61,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A61,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E61" s="12">
-        <f>B61-C61-D61-COUNTIFS(Backlog!$R$2:$R$341,$A61,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A61,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B61-C61-D61-COUNTIFS(Backlog!$R$2:$R$349,$A61,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A61,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A61,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A61,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G61" s="12" t="n"/>
@@ -9916,23 +9928,23 @@
         </is>
       </c>
       <c r="B62" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A62)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A62,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A62,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A62,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A62,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E62" s="12">
-        <f>B62-C62-D62-COUNTIFS(Backlog!$R$2:$R$341,$A62,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A62,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B62-C62-D62-COUNTIFS(Backlog!$R$2:$R$349,$A62,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A62,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A62,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A62,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G62" s="12" t="n"/>
@@ -9945,23 +9957,23 @@
         </is>
       </c>
       <c r="B63" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A63)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A63,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A63,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A63,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A63,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E63" s="12">
-        <f>B63-C63-D63-COUNTIFS(Backlog!$R$2:$R$341,$A63,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A63,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B63-C63-D63-COUNTIFS(Backlog!$R$2:$R$349,$A63,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A63,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A63,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A63,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G63" s="12" t="n"/>
@@ -9974,23 +9986,23 @@
         </is>
       </c>
       <c r="B64" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A64)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A64,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A64,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A64,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A64,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E64" s="12">
-        <f>B64-C64-D64-COUNTIFS(Backlog!$R$2:$R$341,$A64,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A64,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B64-C64-D64-COUNTIFS(Backlog!$R$2:$R$349,$A64,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A64,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A64,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A64,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G64" s="12" t="n"/>
@@ -10003,23 +10015,23 @@
         </is>
       </c>
       <c r="B65" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A65)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A65,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A65,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A65,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A65,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E65" s="12">
-        <f>B65-C65-D65-COUNTIFS(Backlog!$R$2:$R$341,$A65,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A65,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B65-C65-D65-COUNTIFS(Backlog!$R$2:$R$349,$A65,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A65,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A65,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A65,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G65" s="12" t="n"/>
@@ -10032,23 +10044,23 @@
         </is>
       </c>
       <c r="B66" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A66)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A66,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A66,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A66,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A66,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E66" s="12">
-        <f>B66-C66-D66-COUNTIFS(Backlog!$R$2:$R$341,$A66,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A66,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B66-C66-D66-COUNTIFS(Backlog!$R$2:$R$349,$A66,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A66,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A66,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A66,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G66" s="12" t="n"/>
@@ -10061,23 +10073,23 @@
         </is>
       </c>
       <c r="B67" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A67)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A67,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A67,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A67,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A67,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E67" s="12">
-        <f>B67-C67-D67-COUNTIFS(Backlog!$R$2:$R$341,$A67,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A67,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B67-C67-D67-COUNTIFS(Backlog!$R$2:$R$349,$A67,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A67,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A67,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A67,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G67" s="12" t="n"/>
@@ -10090,23 +10102,23 @@
         </is>
       </c>
       <c r="B68" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A68)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A68,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A68,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A68,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A68,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E68" s="12">
-        <f>B68-C68-D68-COUNTIFS(Backlog!$R$2:$R$341,$A68,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A68,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B68-C68-D68-COUNTIFS(Backlog!$R$2:$R$349,$A68,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A68,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A68,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A68,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G68" s="12" t="n"/>
@@ -10119,23 +10131,23 @@
         </is>
       </c>
       <c r="B69" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A69)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A69,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A69,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A69,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A69,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E69" s="12">
-        <f>B69-C69-D69-COUNTIFS(Backlog!$R$2:$R$341,$A69,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A69,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B69-C69-D69-COUNTIFS(Backlog!$R$2:$R$349,$A69,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A69,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A69,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A69,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G69" s="12" t="n"/>
@@ -10148,23 +10160,23 @@
         </is>
       </c>
       <c r="B70" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A70)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A70,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A70,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A70,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A70,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E70" s="12">
-        <f>B70-C70-D70-COUNTIFS(Backlog!$R$2:$R$341,$A70,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A70,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B70-C70-D70-COUNTIFS(Backlog!$R$2:$R$349,$A70,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A70,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A70,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A70,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G70" s="12" t="n"/>
@@ -10177,23 +10189,23 @@
         </is>
       </c>
       <c r="B71" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A71)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A71,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A71,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A71,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A71,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E71" s="12">
-        <f>B71-C71-D71-COUNTIFS(Backlog!$R$2:$R$341,$A71,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A71,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B71-C71-D71-COUNTIFS(Backlog!$R$2:$R$349,$A71,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A71,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A71,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A71,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G71" s="12" t="n"/>
@@ -10206,23 +10218,23 @@
         </is>
       </c>
       <c r="B72" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A72)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A72,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A72,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A72,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A72,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E72" s="12">
-        <f>B72-C72-D72-COUNTIFS(Backlog!$R$2:$R$341,$A72,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A72,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B72-C72-D72-COUNTIFS(Backlog!$R$2:$R$349,$A72,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A72,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A72,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A72,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G72" s="12" t="n"/>
@@ -10235,23 +10247,23 @@
         </is>
       </c>
       <c r="B73" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$341,$A73)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$349,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A73,Backlog!$F$2:$F$341,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A73,Backlog!$F$2:$F$349,"Done")</f>
         <v/>
       </c>
       <c r="D73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A73,Backlog!$F$2:$F$341,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A73,Backlog!$F$2:$F$349,"Later")</f>
         <v/>
       </c>
       <c r="E73" s="12">
-        <f>B73-C73-D73-COUNTIFS(Backlog!$R$2:$R$341,$A73,Backlog!$F$2:$F$341,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$341,$A73,Backlog!$F$2:$F$341,"Obsolete")</f>
+        <f>B73-C73-D73-COUNTIFS(Backlog!$R$2:$R$349,$A73,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A73,Backlog!$F$2:$F$349,"Obsolete")</f>
         <v/>
       </c>
       <c r="F73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$341,$A73,Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$349,$A73,Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="G73" s="12" t="n"/>
@@ -10273,7 +10285,7 @@
         </is>
       </c>
       <c r="B75" s="12">
-        <f>COUNTIF(Backlog!$S$2:$S$341,"Yes")</f>
+        <f>COUNTIF(Backlog!$S$2:$S$349,"Yes")</f>
         <v/>
       </c>
       <c r="C75" s="12" t="n"/>
@@ -10290,7 +10302,7 @@
         </is>
       </c>
       <c r="B76" s="12">
-        <f>COUNTIFS(Backlog!$S$2:$S$341,"Yes",Backlog!$G$2:$G$341,"P0")</f>
+        <f>COUNTIFS(Backlog!$S$2:$S$349,"Yes",Backlog!$G$2:$G$349,"P0")</f>
         <v/>
       </c>
       <c r="C76" s="12" t="n"/>
@@ -10307,7 +10319,7 @@
         </is>
       </c>
       <c r="B77" s="12">
-        <f>COUNTIFS(Backlog!$S$2:$S$341,"No",Backlog!$G$2:$G$341,"P0",Backlog!$F$2:$F$341,"&lt;&gt;Done",Backlog!$F$2:$F$341,"&lt;&gt;Later",Backlog!$F$2:$F$341,"&lt;&gt;Cancelled",Backlog!$F$2:$F$341,"&lt;&gt;Obsolete")</f>
+        <f>COUNTIFS(Backlog!$S$2:$S$349,"No",Backlog!$G$2:$G$349,"P0",Backlog!$F$2:$F$349,"&lt;&gt;Done",Backlog!$F$2:$F$349,"&lt;&gt;Later",Backlog!$F$2:$F$349,"&lt;&gt;Cancelled",Backlog!$F$2:$F$349,"&lt;&gt;Obsolete")</f>
         <v/>
       </c>
       <c r="C77" s="12" t="n"/>
@@ -10324,7 +10336,7 @@
         </is>
       </c>
       <c r="B78" s="12">
-        <f>COUNTIF(Backlog!$F$2:$F$341,"Hold")</f>
+        <f>COUNTIF(Backlog!$F$2:$F$349,"Hold")</f>
         <v/>
       </c>
       <c r="C78" s="12" t="n"/>
@@ -10350,7 +10362,7 @@
         </is>
       </c>
       <c r="B80" s="12">
-        <f>COUNTIFS(Backlog!$G$2:$G$341,"P0",Backlog!$F$2:$F$341,"&lt;&gt;Done",Backlog!$F$2:$F$341,"&lt;&gt;Cancelled",Backlog!$F$2:$F$341,"&lt;&gt;Obsolete",Backlog!$F$2:$F$341,"&lt;&gt;Later")</f>
+        <f>COUNTIFS(Backlog!$G$2:$G$349,"P0",Backlog!$F$2:$F$349,"&lt;&gt;Done",Backlog!$F$2:$F$349,"&lt;&gt;Cancelled",Backlog!$F$2:$F$349,"&lt;&gt;Obsolete",Backlog!$F$2:$F$349,"&lt;&gt;Later")</f>
         <v/>
       </c>
       <c r="C80" s="12" t="n"/>
@@ -10367,7 +10379,7 @@
         </is>
       </c>
       <c r="B81" s="12">
-        <f>COUNTIFS(Backlog!$N$2:$N$341,"Sales blocker",Backlog!$F$2:$F$341,"&lt;&gt;Done")</f>
+        <f>COUNTIFS(Backlog!$N$2:$N$349,"Sales blocker",Backlog!$F$2:$F$349,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="C81" s="12" t="n"/>
@@ -10384,7 +10396,7 @@
         </is>
       </c>
       <c r="B82" s="12">
-        <f>COUNTIFS(Backlog!$E$2:$E$341,"Decision Needed",Backlog!$F$2:$F$341,"&lt;&gt;Done")</f>
+        <f>COUNTIFS(Backlog!$E$2:$E$349,"Decision Needed",Backlog!$F$2:$F$349,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="C82" s="12" t="n"/>
@@ -10435,6 +10447,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -10598,6 +10611,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
@@ -10857,6 +10871,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
@@ -10912,6 +10927,7 @@
         </is>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
@@ -10979,6 +10995,7 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
@@ -11355,6 +11372,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -11773,7 +11791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U341"/>
+  <dimension ref="A1:U349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -21352,7 +21370,11 @@
           <t>The tool is absent from every customer release (package scan); every issue is recorded in the ledger with a sequence number; issuing, revoking and key operations need no terminal.</t>
         </is>
       </c>
-      <c r="K107" s="8" t="n"/>
+      <c r="K107" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-25: the issued-licence ledger (#341) and the licence flow gate (#342) feed the owner-initiated admin reset (#343-#348).</t>
+        </is>
+      </c>
       <c r="L107" s="10" t="inlineStr">
         <is>
           <t>M1</t>
@@ -22925,7 +22947,11 @@
           <t>Each request is answered within 2 business days.</t>
         </is>
       </c>
-      <c r="K124" s="8" t="n"/>
+      <c r="K124" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-25: the issued-licence ledger (#341) and the licence flow gate (#342) feed the owner-initiated admin reset (#343-#348).</t>
+        </is>
+      </c>
       <c r="L124" s="10" t="inlineStr">
         <is>
           <t>M3</t>
@@ -41914,9 +41940,689 @@
         </is>
       </c>
     </row>
+    <row r="342">
+      <c r="A342" s="10" t="n">
+        <v>341</v>
+      </c>
+      <c r="B342" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C342" s="8" t="inlineStr">
+        <is>
+          <t>Licensing &amp; Protection</t>
+        </is>
+      </c>
+      <c r="D342" s="8" t="inlineStr">
+        <is>
+          <t>Issued-licence ledger on the vendor side and import of licence files that were already issued to customers</t>
+        </is>
+      </c>
+      <c r="E342" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F342" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G342" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H342" s="8" t="inlineStr">
+        <is>
+          <t>Today there is no record that lets the owner pick a customer and find the licence that customer received. Licences issued before the ledger existed must stay usable for later owner actions such as the one-time admin reset (#343-#348).</t>
+        </is>
+      </c>
+      <c r="I342" s="8" t="inlineStr">
+        <is>
+          <t>In the vendor tool (#106) keep a ledger: customer, licence id, Install ID, fingerprint hash, signing key id, edition/modules, type and period, status (active/revoked/expired), issue date and the original request nonce. Add an import action: upload an already issued .pemslic (or zip); the tool verifies the signature with the public key, reads the bound fields and creates or updates the ledger row after the owner confirms the customer. Everything is done in the UI; no terminal or CLI step is required. Every change writes an audit entry. Export to CSV/Excel.</t>
+        </is>
+      </c>
+      <c r="J342" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the owner selects a customer in the vendor tool and sees every licence issued to it; a licence file issued before the ledger existed is imported with a valid signature and appears in the list; a tampered file is rejected; each import and edit is audited.</t>
+        </is>
+      </c>
+      <c r="K342" s="8" t="n"/>
+      <c r="L342" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M342" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N342" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O342" s="10" t="inlineStr">
+        <is>
+          <t>#101 #106 #107</t>
+        </is>
+      </c>
+      <c r="P342" s="10" t="n"/>
+      <c r="Q342" s="10" t="n"/>
+      <c r="R342" s="8" t="inlineStr">
+        <is>
+          <t>Licensing chain</t>
+        </is>
+      </c>
+      <c r="S342" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T342" s="10" t="n"/>
+      <c r="U342" s="10" t="n"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="10" t="n">
+        <v>342</v>
+      </c>
+      <c r="B343" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C343" s="8" t="inlineStr">
+        <is>
+          <t>Licensing &amp; Protection</t>
+        </is>
+      </c>
+      <c r="D343" s="8" t="inlineStr">
+        <is>
+          <t>Licence issuance flow verified end to end (request, issue, deliver, install, activate, ledger): the prerequisite for every admin-password-reset task</t>
+        </is>
+      </c>
+      <c r="E343" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F343" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G343" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H343" s="8" t="inlineStr">
+        <is>
+          <t>The owner-initiated admin reset (#343-#348) must work from the licence that a customer really holds, so the whole licence chain has to be proven first: customer request file, owner issues the licence, customer installs it, the product accepts it and the ledger shows it. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+        </is>
+      </c>
+      <c r="I343" s="8" t="inlineStr">
+        <is>
+          <t>On a clean installation: 1) the customer licence page (#108) generates the .pemsreq request; 2) the vendor tool (#106) validates it and issues the .pemslic signed with the key from #107; 3) the licence is uploaded in the UI (and in the first-run flow #109) and activated; 4) the issue is recorded in the ledger (#341); 5) repeat for a customer whose licence was issued earlier and imported (#341). Fix what breaks, and record the run in the licence acceptance checklist (#122). Everything in this flow is done in the UI; no terminal or CLI step is required.</t>
+        </is>
+      </c>
+      <c r="J343" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a clean install is activated with a licence issued by the vendor tool; the ledger lists that licence with its Install ID and fingerprint hash; an imported earlier licence behaves the same; the run is written in the acceptance checklist. Only then are #343-#348 unblocked.</t>
+        </is>
+      </c>
+      <c r="K343" s="8" t="n"/>
+      <c r="L343" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M343" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N343" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O343" s="10" t="inlineStr">
+        <is>
+          <t>#98 #99 #100 #101 #106 #107 #108 #109 #122 #339 #341</t>
+        </is>
+      </c>
+      <c r="P343" s="10" t="n"/>
+      <c r="Q343" s="10" t="n"/>
+      <c r="R343" s="8" t="inlineStr">
+        <is>
+          <t>Licensing chain</t>
+        </is>
+      </c>
+      <c r="S343" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T343" s="10" t="n"/>
+      <c r="U343" s="10" t="n"/>
+    </row>
+    <row r="344">
+      <c r="A344" s="10" t="n">
+        <v>343</v>
+      </c>
+      <c r="B344" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C344" s="8" t="inlineStr">
+        <is>
+          <t>Access, RLS, Sessions &amp; Security</t>
+        </is>
+      </c>
+      <c r="D344" s="8" t="inlineStr">
+        <is>
+          <t>Design and decision for an owner-initiated admin password reset by a one-time link tied to the customer's licence (threat model, binding, expiry, key custody)</t>
+        </is>
+      </c>
+      <c r="E344" s="10" t="inlineStr">
+        <is>
+          <t>Decision Needed</t>
+        </is>
+      </c>
+      <c r="F344" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G344" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H344" s="8" t="inlineStr">
+        <is>
+          <t>A customer who loses the administrator password must be recoverable by the system owner without a back door in the product and without internet access. The reset has to work only on the customer's own installation, once, and only if the owner chooses that customer. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+        </is>
+      </c>
+      <c r="I344" s="8" t="inlineStr">
+        <is>
+          <t>Write docs/design/ADMIN_RESET.md (no secrets): the reset ticket is signed by the owner, bound to licence id + Install ID + fingerprint hash + signing key id, has a short expiry, a random nonce stored on use so it works once, and is delivered as a link or file by any channel. Decide: which key signs it (the licence key stays offline per #107; a separate reset-only key may be allowed on the owner's local computer or the assistant's computer, never the licence key), what is reset (password only, or also MFA/passkeys and sessions), how the owner verifies the customer identity before issuing, rate limits, audit on both sides, and what happens on a cloned or re-hosted machine (#104, #116).</t>
+        </is>
+      </c>
+      <c r="J344" s="8" t="inlineStr">
+        <is>
+          <t>Done when: an approved ADR with the threat model (replay, wrong customer, tampered ticket, cloned machine, clock change, leaked link), the key-custody decision, and the exact ticket fields; the next rows #344-#348 are written against it.</t>
+        </is>
+      </c>
+      <c r="K344" s="8" t="n"/>
+      <c r="L344" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M344" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N344" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O344" s="10" t="inlineStr">
+        <is>
+          <t>#96 #107 #178 #182 #339 #342</t>
+        </is>
+      </c>
+      <c r="P344" s="10" t="n"/>
+      <c r="Q344" s="10" t="n"/>
+      <c r="R344" s="8" t="inlineStr">
+        <is>
+          <t>Security &amp; access</t>
+        </is>
+      </c>
+      <c r="S344" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T344" s="10" t="n"/>
+      <c r="U344" s="10" t="n"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="10" t="n">
+        <v>344</v>
+      </c>
+      <c r="B345" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C345" s="8" t="inlineStr">
+        <is>
+          <t>Access, RLS, Sessions &amp; Security</t>
+        </is>
+      </c>
+      <c r="D345" s="8" t="inlineStr">
+        <is>
+          <t>Reset ticket format and signing library: payload fields, signature, expiry, nonce, link and file encodings, verification used by both the owner tool and the product</t>
+        </is>
+      </c>
+      <c r="E345" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F345" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G345" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H345" s="8" t="inlineStr">
+        <is>
+          <t>One shared, tested implementation prevents the owner tool and the product from disagreeing about what a valid ticket is. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+        </is>
+      </c>
+      <c r="I345" s="8" t="inlineStr">
+        <is>
+          <t>Implement the ticket from the ADR (#343) in a shared library (PEMS.Shared or a licensing project): canonical encoding, Ed25519/ECDSA signature with domain separation from licence files, fields (customer, licence id, Install ID, fingerprint hash, key id, issued-at, expires-at, nonce, purpose), link form (short URL path with the ticket in the fragment so it is not logged) and file form. Unit tests with test vectors for valid, expired, tampered, wrong-binding and wrong-purpose tickets.</t>
+        </is>
+      </c>
+      <c r="J345" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the library signs and verifies tickets; every negative test vector is rejected with a distinct reason; the same code is referenced by #345 and #346.</t>
+        </is>
+      </c>
+      <c r="K345" s="8" t="n"/>
+      <c r="L345" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M345" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N345" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O345" s="10" t="inlineStr">
+        <is>
+          <t>#101 #107 #343</t>
+        </is>
+      </c>
+      <c r="P345" s="10" t="n"/>
+      <c r="Q345" s="10" t="n"/>
+      <c r="R345" s="8" t="inlineStr">
+        <is>
+          <t>Security &amp; access</t>
+        </is>
+      </c>
+      <c r="S345" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T345" s="10" t="n"/>
+      <c r="U345" s="10" t="n"/>
+    </row>
+    <row r="346">
+      <c r="A346" s="10" t="n">
+        <v>345</v>
+      </c>
+      <c r="B346" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C346" s="8" t="inlineStr">
+        <is>
+          <t>Access, RLS, Sessions &amp; Security</t>
+        </is>
+      </c>
+      <c r="D346" s="8" t="inlineStr">
+        <is>
+          <t>Owner reset tool on the owner's local computer: choose the customer and licence from the ledger, issue a one-time reset link or file, audit it</t>
+        </is>
+      </c>
+      <c r="E346" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F346" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G346" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H346" s="8" t="inlineStr">
+        <is>
+          <t>The owner (or the assistant acting for the owner) needs a safe place to issue reset links without internet and without exposing the licence signing key. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+        </is>
+      </c>
+      <c r="I346" s="8" t="inlineStr">
+        <is>
+          <t>Add a Reset admin action to the vendor tool (#106) that runs on the owner's local computer: pick the customer, pick one of its licences from the ledger (#341), enter the reason and the identity check performed, choose the expiry, then produce the one-time link and the .pemsreset file using #344. Show the link once, never write it to a log, and record the issue (who, when, customer, licence, expiry, reason) in the audit. Revoked or expired licences cannot be selected. Works fully offline. Everything is done in the UI; no terminal or CLI step is required.</t>
+        </is>
+      </c>
+      <c r="J346" s="8" t="inlineStr">
+        <is>
+          <t>Done when: from the ledger the owner issues a link for a chosen customer in under a minute with no network; the audit shows it; a revoked licence cannot get a link; the signing key custody follows #343.</t>
+        </is>
+      </c>
+      <c r="K346" s="8" t="n"/>
+      <c r="L346" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M346" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N346" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O346" s="10" t="inlineStr">
+        <is>
+          <t>#341 #343 #344</t>
+        </is>
+      </c>
+      <c r="P346" s="10" t="n"/>
+      <c r="Q346" s="10" t="n"/>
+      <c r="R346" s="8" t="inlineStr">
+        <is>
+          <t>Security &amp; access</t>
+        </is>
+      </c>
+      <c r="S346" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T346" s="10" t="n"/>
+      <c r="U346" s="10" t="n"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="10" t="n">
+        <v>346</v>
+      </c>
+      <c r="B347" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C347" s="8" t="inlineStr">
+        <is>
+          <t>Access, RLS, Sessions &amp; Security</t>
+        </is>
+      </c>
+      <c r="D347" s="8" t="inlineStr">
+        <is>
+          <t>Product side of the one-time admin reset: verify the ticket against the installed licence, consume the nonce once, set a new administrator password, revoke sessions, audit</t>
+        </is>
+      </c>
+      <c r="E347" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F347" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G347" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H347" s="8" t="inlineStr">
+        <is>
+          <t>The customer opens the link on their own installation; the product must accept it only if it matches this installation's licence, and only once. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+        </is>
+      </c>
+      <c r="I347" s="8" t="inlineStr">
+        <is>
+          <t>Add an anonymous-safe reset page and endpoint: verify signature and expiry with #344, check licence id, Install ID and fingerprint hash against the installed licence (#99, #98), record the nonce in a new table through an EF migration so a second use fails, then let the person set a new administrator password under the password policy, require a password change at next sign-in, re-enrol MFA/passkeys as decided in #343, revoke all sessions of that user (#182), write the audit and rate-limit failures. The page is added to the always-free surfaces list and is available even before the first sign-in.</t>
+        </is>
+      </c>
+      <c r="J347" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a valid link resets the administrator password once on the matching installation; the same link, an expired link, a link for another customer or machine, and a tampered link are all refused with the audit entry; existing sessions end.</t>
+        </is>
+      </c>
+      <c r="K347" s="8" t="n"/>
+      <c r="L347" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M347" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N347" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O347" s="10" t="inlineStr">
+        <is>
+          <t>#98 #99 #108 #182 #343 #344</t>
+        </is>
+      </c>
+      <c r="P347" s="10" t="n"/>
+      <c r="Q347" s="10" t="n"/>
+      <c r="R347" s="8" t="inlineStr">
+        <is>
+          <t>Security &amp; access</t>
+        </is>
+      </c>
+      <c r="S347" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T347" s="10" t="n"/>
+      <c r="U347" s="10" t="n"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="10" t="n">
+        <v>347</v>
+      </c>
+      <c r="B348" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C348" s="8" t="inlineStr">
+        <is>
+          <t>Access, RLS, Sessions &amp; Security</t>
+        </is>
+      </c>
+      <c r="D348" s="8" t="inlineStr">
+        <is>
+          <t>Automated security tests for the admin reset: replay, expiry, wrong customer or machine, tampering, clock change, brute force, session revocation</t>
+        </is>
+      </c>
+      <c r="E348" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F348" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G348" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H348" s="8" t="inlineStr">
+        <is>
+          <t>A recovery path is a favourite attack target; it must be covered by tests before it ships. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+        </is>
+      </c>
+      <c r="I348" s="8" t="inlineStr">
+        <is>
+          <t>Write integration tests against the real product endpoint and the owner tool library: replay of a used link, expired ticket, ticket issued for another licence or Install ID, modified payload, signature from a different key, cloned machine (fingerprint mismatch), clock rolled back, repeated failures hitting the rate limit, and confirmation that sessions and MFA state are changed as specified. Add them to the CI gate.</t>
+        </is>
+      </c>
+      <c r="J348" s="8" t="inlineStr">
+        <is>
+          <t>Done when: each scenario has a passing test that fails if the defence is removed; the tests run in CI; results are linked from the licence acceptance checklist.</t>
+        </is>
+      </c>
+      <c r="K348" s="8" t="n"/>
+      <c r="L348" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M348" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N348" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O348" s="10" t="inlineStr">
+        <is>
+          <t>#305 #346</t>
+        </is>
+      </c>
+      <c r="P348" s="10" t="n"/>
+      <c r="Q348" s="10" t="n"/>
+      <c r="R348" s="8" t="inlineStr">
+        <is>
+          <t>Security &amp; access</t>
+        </is>
+      </c>
+      <c r="S348" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T348" s="10" t="n"/>
+      <c r="U348" s="10" t="n"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="10" t="n">
+        <v>348</v>
+      </c>
+      <c r="B349" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C349" s="8" t="inlineStr">
+        <is>
+          <t>Access, RLS, Sessions &amp; Security</t>
+        </is>
+      </c>
+      <c r="D349" s="8" t="inlineStr">
+        <is>
+          <t>Owner procedure and customer-facing guide for the admin reset: identity verification, issuing, delivery, audit review</t>
+        </is>
+      </c>
+      <c r="E349" s="10" t="inlineStr">
+        <is>
+          <t>Ops Process</t>
+        </is>
+      </c>
+      <c r="F349" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G349" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H349" s="8" t="inlineStr">
+        <is>
+          <t>Technical safety is not enough: the owner needs a written rule for when a reset is allowed, and customers need to know how to ask. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+        </is>
+      </c>
+      <c r="I349" s="8" t="inlineStr">
+        <is>
+          <t>Write the procedure: how the customer asks, how the owner verifies identity (named contact on the contract, call-back), which customer and licence to select in the owner tool, how the link is delivered, how long it stays valid, how the audit is reviewed monthly, and what is said to the customer. Add a short help topic in the product and link it from the licence support procedure (#123).</t>
+        </is>
+      </c>
+      <c r="J349" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the owner approves the procedure; a rehearsed reset from request to new password follows it; the help topic exists in Persian and English.</t>
+        </is>
+      </c>
+      <c r="K349" s="8" t="n"/>
+      <c r="L349" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M349" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N349" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O349" s="10" t="inlineStr">
+        <is>
+          <t>#123 #346</t>
+        </is>
+      </c>
+      <c r="P349" s="10" t="n"/>
+      <c r="Q349" s="10" t="n"/>
+      <c r="R349" s="8" t="inlineStr">
+        <is>
+          <t>Security &amp; access</t>
+        </is>
+      </c>
+      <c r="S349" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T349" s="10" t="n"/>
+      <c r="U349" s="10" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U341"/>
-  <conditionalFormatting sqref="F2:F341">
+  <autoFilter ref="A1:U349"/>
+  <conditionalFormatting sqref="F2:F349">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
@@ -41939,7 +42645,7 @@
       <formula>"Obsolete"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G341">
+  <conditionalFormatting sqref="G2:G349">
     <cfRule type="cellIs" priority="8" operator="equal" dxfId="6">
       <formula>"P0"</formula>
     </cfRule>
@@ -41947,27 +42653,27 @@
       <formula>"P1"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S341">
+  <conditionalFormatting sqref="S2:S349">
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N341">
+  <conditionalFormatting sqref="N2:N349">
     <cfRule type="cellIs" priority="11" operator="equal" dxfId="6">
       <formula>"Sales blocker"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="F2:F341" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F349" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Partial,Done,Hold,Later,Cancelled,Obsolete"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G341" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G349" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B341" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B2:B349" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Claude,User,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S341" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="S2:S349" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -43377,7 +44083,7 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$341,"M0")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$349,"M0")</f>
         <v/>
       </c>
     </row>
@@ -43408,7 +44114,7 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$341,"M1")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$349,"M1")</f>
         <v/>
       </c>
     </row>
@@ -43439,7 +44145,7 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$341,"M2")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$349,"M2")</f>
         <v/>
       </c>
     </row>
@@ -43470,7 +44176,7 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$341,"M3")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$349,"M3")</f>
         <v/>
       </c>
     </row>
@@ -43501,7 +44207,7 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$341,"M4")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$349,"M4")</f>
         <v/>
       </c>
     </row>
@@ -43532,7 +44238,7 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$341,"M5")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$349,"M5")</f>
         <v/>
       </c>
     </row>
@@ -43563,10 +44269,11 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$341,"M6")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$349,"M6")</f>
         <v/>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
@@ -43740,6 +44447,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
@@ -44497,6 +45205,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -44673,6 +45382,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
@@ -46466,6 +47176,8 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(plan): admin reset by file exchange with a separate reset key; AFTA constraints; independence from the parallel admin-recovery work; add #349
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -22,7 +22,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$349</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$350</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Test Plan'!$A$1:$H$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Roadmap'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Capability Checklist'!$A$1:$H$37</definedName>
@@ -599,7 +599,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -607,7 +606,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -622,7 +620,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
@@ -637,7 +634,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -652,7 +648,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -667,7 +662,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -682,7 +676,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -697,7 +690,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
@@ -740,7 +732,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -813,7 +804,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
@@ -1614,7 +1604,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -8153,7 +8142,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -8161,7 +8149,7 @@
         </is>
       </c>
       <c r="B3" s="12">
-        <f>COUNTA(Backlog!$D$2:$D$349)</f>
+        <f>COUNTA(Backlog!$D$2:$D$350)</f>
         <v/>
       </c>
       <c r="C3" s="12" t="n"/>
@@ -8178,7 +8166,7 @@
         </is>
       </c>
       <c r="B4" s="12">
-        <f>COUNTIF(Backlog!$B$2:$B$349,"User")</f>
+        <f>COUNTIF(Backlog!$B$2:$B$350,"User")</f>
         <v/>
       </c>
       <c r="C4" s="12" t="n"/>
@@ -8252,19 +8240,19 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A8,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A8,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A8,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A8,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A8,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A8,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A8,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A8,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="F8" s="12">
@@ -8281,19 +8269,19 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A9,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A9,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A9,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A9,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A9,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A9,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A9,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A9,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="F9" s="12">
@@ -8310,19 +8298,19 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A10,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A10,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A10,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A10,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A10,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A10,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A10,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A10,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="F10" s="12">
@@ -8339,19 +8327,19 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A11,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A11,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A11,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A11,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A11,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A11,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A11,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A11,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="F11" s="12">
@@ -8368,19 +8356,19 @@
         </is>
       </c>
       <c r="B12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A12,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A12,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="C12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A12,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A12,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A12,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A12,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="E12" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A12,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A12,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="F12" s="12">
@@ -8397,19 +8385,19 @@
         </is>
       </c>
       <c r="B13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A13,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A13,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="C13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A13,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A13,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="D13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A13,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A13,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="E13" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A13,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A13,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="F13" s="12">
@@ -8426,19 +8414,19 @@
         </is>
       </c>
       <c r="B14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A14,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A14,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="C14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A14,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A14,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="D14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A14,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A14,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="E14" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A14,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A14,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="F14" s="12">
@@ -8455,19 +8443,19 @@
         </is>
       </c>
       <c r="B15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A15,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A15,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="C15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A15,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A15,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="D15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A15,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A15,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="E15" s="12">
-        <f>COUNTIFS(Backlog!$F$2:$F$349,$A15,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$F$2:$F$350,$A15,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="F15" s="12">
@@ -8578,31 +8566,31 @@
         </is>
       </c>
       <c r="B20" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A20)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A20)</f>
         <v/>
       </c>
       <c r="C20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A20,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A20,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A20,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A20,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G20" s="12">
-        <f>B20-H20-COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B20-H20-COUNTIFS(Backlog!$C$2:$C$350,$A20,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A20,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A20,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H20" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A20,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A20,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8613,31 +8601,31 @@
         </is>
       </c>
       <c r="B21" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A21)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A21)</f>
         <v/>
       </c>
       <c r="C21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A21,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A21,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A21,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A21,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G21" s="12">
-        <f>B21-H21-COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B21-H21-COUNTIFS(Backlog!$C$2:$C$350,$A21,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A21,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A21,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H21" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A21,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A21,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8648,31 +8636,31 @@
         </is>
       </c>
       <c r="B22" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A22)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A22)</f>
         <v/>
       </c>
       <c r="C22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A22,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A22,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A22,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A22,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G22" s="12">
-        <f>B22-H22-COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B22-H22-COUNTIFS(Backlog!$C$2:$C$350,$A22,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A22,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A22,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H22" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A22,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A22,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8683,31 +8671,31 @@
         </is>
       </c>
       <c r="B23" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A23)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A23)</f>
         <v/>
       </c>
       <c r="C23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A23,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A23,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A23,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A23,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G23" s="12">
-        <f>B23-H23-COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B23-H23-COUNTIFS(Backlog!$C$2:$C$350,$A23,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A23,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A23,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H23" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A23,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A23,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8718,31 +8706,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A24)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A24,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A24,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A24,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A24,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>B24-H24-COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B24-H24-COUNTIFS(Backlog!$C$2:$C$350,$A24,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A24,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A24,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A24,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A24,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8753,31 +8741,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A25)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A25,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A25,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A25,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A25,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>B25-H25-COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B25-H25-COUNTIFS(Backlog!$C$2:$C$350,$A25,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A25,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A25,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A25,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A25,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8788,31 +8776,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A26)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A26,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A26,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A26,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A26,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>B26-H26-COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B26-H26-COUNTIFS(Backlog!$C$2:$C$350,$A26,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A26,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A26,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A26,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A26,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8823,31 +8811,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A27)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A27,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A27,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A27,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A27,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>B27-H27-COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B27-H27-COUNTIFS(Backlog!$C$2:$C$350,$A27,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A27,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A27,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A27,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A27,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8858,31 +8846,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A28)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A28,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A28,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A28,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A28,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>B28-H28-COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B28-H28-COUNTIFS(Backlog!$C$2:$C$350,$A28,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A28,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A28,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A28,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A28,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8893,31 +8881,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A29)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A29,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A29,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A29,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A29,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>B29-H29-COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B29-H29-COUNTIFS(Backlog!$C$2:$C$350,$A29,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A29,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A29,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A29,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A29,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8928,31 +8916,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A30)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A30,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A30,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A30,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A30,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>B30-H30-COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B30-H30-COUNTIFS(Backlog!$C$2:$C$350,$A30,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A30,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A30,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A30,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A30,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8963,31 +8951,31 @@
         </is>
       </c>
       <c r="B31" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A31)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A31,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A31,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A31,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A31,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G31" s="12">
-        <f>B31-H31-COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B31-H31-COUNTIFS(Backlog!$C$2:$C$350,$A31,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A31,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A31,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H31" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A31,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A31,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -8998,31 +8986,31 @@
         </is>
       </c>
       <c r="B32" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A32)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A32,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A32,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A32,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A32,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G32" s="12">
-        <f>B32-H32-COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B32-H32-COUNTIFS(Backlog!$C$2:$C$350,$A32,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A32,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A32,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H32" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A32,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A32,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9033,31 +9021,31 @@
         </is>
       </c>
       <c r="B33" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A33)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A33)</f>
         <v/>
       </c>
       <c r="C33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A33,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A33,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A33,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A33,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G33" s="12">
-        <f>B33-H33-COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B33-H33-COUNTIFS(Backlog!$C$2:$C$350,$A33,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A33,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A33,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H33" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A33,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A33,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9068,31 +9056,31 @@
         </is>
       </c>
       <c r="B34" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A34)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A34)</f>
         <v/>
       </c>
       <c r="C34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A34,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A34,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A34,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A34,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G34" s="12">
-        <f>B34-H34-COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B34-H34-COUNTIFS(Backlog!$C$2:$C$350,$A34,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A34,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A34,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H34" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A34,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A34,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9103,31 +9091,31 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A35)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A35)</f>
         <v/>
       </c>
       <c r="C35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A35,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A35,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A35,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A35,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G35" s="12">
-        <f>B35-H35-COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B35-H35-COUNTIFS(Backlog!$C$2:$C$350,$A35,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A35,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A35,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H35" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A35,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A35,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9138,31 +9126,31 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A36)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A36)</f>
         <v/>
       </c>
       <c r="C36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A36,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A36,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A36,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A36,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G36" s="12">
-        <f>B36-H36-COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B36-H36-COUNTIFS(Backlog!$C$2:$C$350,$A36,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A36,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A36,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H36" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A36,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A36,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9173,31 +9161,31 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A37)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A37,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A37,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A37,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A37,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G37" s="12">
-        <f>B37-H37-COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B37-H37-COUNTIFS(Backlog!$C$2:$C$350,$A37,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A37,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A37,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H37" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A37,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A37,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9208,31 +9196,31 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A38)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A38,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A38,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A38,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A38,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G38" s="12">
-        <f>B38-H38-COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B38-H38-COUNTIFS(Backlog!$C$2:$C$350,$A38,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A38,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A38,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H38" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A38,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A38,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9243,31 +9231,31 @@
         </is>
       </c>
       <c r="B39" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A39)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A39,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A39,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A39,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A39,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G39" s="12">
-        <f>B39-H39-COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B39-H39-COUNTIFS(Backlog!$C$2:$C$350,$A39,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A39,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A39,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H39" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A39,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A39,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9278,31 +9266,31 @@
         </is>
       </c>
       <c r="B40" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A40)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A40,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A40,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A40,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A40,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G40" s="12">
-        <f>B40-H40-COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B40-H40-COUNTIFS(Backlog!$C$2:$C$350,$A40,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A40,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A40,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H40" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A40,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A40,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9313,31 +9301,31 @@
         </is>
       </c>
       <c r="B41" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A41)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A41,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A41,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A41,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A41,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G41" s="12">
-        <f>B41-H41-COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B41-H41-COUNTIFS(Backlog!$C$2:$C$350,$A41,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A41,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A41,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H41" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A41,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A41,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9348,31 +9336,31 @@
         </is>
       </c>
       <c r="B42" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A42)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A42,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A42,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A42,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A42,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G42" s="12">
-        <f>B42-H42-COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B42-H42-COUNTIFS(Backlog!$C$2:$C$350,$A42,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A42,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A42,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H42" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A42,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A42,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9383,31 +9371,31 @@
         </is>
       </c>
       <c r="B43" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A43)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A43,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A43,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A43,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A43,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G43" s="12">
-        <f>B43-H43-COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B43-H43-COUNTIFS(Backlog!$C$2:$C$350,$A43,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A43,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A43,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H43" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A43,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A43,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9418,31 +9406,31 @@
         </is>
       </c>
       <c r="B44" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A44)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A44,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A44,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A44,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A44,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G44" s="12">
-        <f>B44-H44-COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B44-H44-COUNTIFS(Backlog!$C$2:$C$350,$A44,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A44,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A44,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H44" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A44,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A44,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9453,31 +9441,31 @@
         </is>
       </c>
       <c r="B45" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A45)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A45,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A45,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A45,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A45,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G45" s="12">
-        <f>B45-H45-COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B45-H45-COUNTIFS(Backlog!$C$2:$C$350,$A45,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A45,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A45,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H45" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A45,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A45,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9488,31 +9476,31 @@
         </is>
       </c>
       <c r="B46" s="12">
-        <f>COUNTIF(Backlog!$C$2:$C$349,$A46)</f>
+        <f>COUNTIF(Backlog!$C$2:$C$350,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A46,Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="D46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$G$2:$G$349,"P1")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A46,Backlog!$G$2:$G$350,"P1")</f>
         <v/>
       </c>
       <c r="E46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$G$2:$G$349,"P2")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A46,Backlog!$G$2:$G$350,"P2")</f>
         <v/>
       </c>
       <c r="F46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$G$2:$G$349,"P3")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A46,Backlog!$G$2:$G$350,"P3")</f>
         <v/>
       </c>
       <c r="G46" s="12">
-        <f>B46-H46-COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$F$2:$F$349,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$F$2:$F$349,"Later")</f>
+        <f>B46-H46-COUNTIFS(Backlog!$C$2:$C$350,$A46,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$C$2:$C$350,$A46,Backlog!$F$2:$F$350,"Obsolete")-COUNTIFS(Backlog!$C$2:$C$350,$A46,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="H46" s="12">
-        <f>COUNTIFS(Backlog!$C$2:$C$349,$A46,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$C$2:$C$350,$A46,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
     </row>
@@ -9580,23 +9568,23 @@
         </is>
       </c>
       <c r="B50" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A50)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A50,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A50,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A50,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A50,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E50" s="12">
-        <f>B50-C50-D50-COUNTIFS(Backlog!$R$2:$R$349,$A50,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A50,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B50-C50-D50-COUNTIFS(Backlog!$R$2:$R$350,$A50,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A50,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F50" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A50,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A50,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G50" s="12" t="n"/>
@@ -9609,23 +9597,23 @@
         </is>
       </c>
       <c r="B51" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A51)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A51)</f>
         <v/>
       </c>
       <c r="C51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A51,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A51,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A51,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A51,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E51" s="12">
-        <f>B51-C51-D51-COUNTIFS(Backlog!$R$2:$R$349,$A51,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A51,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B51-C51-D51-COUNTIFS(Backlog!$R$2:$R$350,$A51,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A51,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F51" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A51,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A51,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G51" s="12" t="n"/>
@@ -9638,23 +9626,23 @@
         </is>
       </c>
       <c r="B52" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A52)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A52)</f>
         <v/>
       </c>
       <c r="C52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A52,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A52,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A52,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A52,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E52" s="12">
-        <f>B52-C52-D52-COUNTIFS(Backlog!$R$2:$R$349,$A52,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A52,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B52-C52-D52-COUNTIFS(Backlog!$R$2:$R$350,$A52,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A52,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F52" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A52,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A52,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G52" s="12" t="n"/>
@@ -9667,23 +9655,23 @@
         </is>
       </c>
       <c r="B53" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A53)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A53)</f>
         <v/>
       </c>
       <c r="C53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A53,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A53,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A53,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A53,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E53" s="12">
-        <f>B53-C53-D53-COUNTIFS(Backlog!$R$2:$R$349,$A53,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A53,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B53-C53-D53-COUNTIFS(Backlog!$R$2:$R$350,$A53,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A53,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F53" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A53,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A53,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G53" s="12" t="n"/>
@@ -9696,23 +9684,23 @@
         </is>
       </c>
       <c r="B54" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A54)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A54)</f>
         <v/>
       </c>
       <c r="C54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A54,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A54,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A54,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A54,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E54" s="12">
-        <f>B54-C54-D54-COUNTIFS(Backlog!$R$2:$R$349,$A54,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A54,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B54-C54-D54-COUNTIFS(Backlog!$R$2:$R$350,$A54,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A54,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F54" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A54,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A54,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G54" s="12" t="n"/>
@@ -9725,23 +9713,23 @@
         </is>
       </c>
       <c r="B55" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A55)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A55,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A55,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A55,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A55,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E55" s="12">
-        <f>B55-C55-D55-COUNTIFS(Backlog!$R$2:$R$349,$A55,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A55,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B55-C55-D55-COUNTIFS(Backlog!$R$2:$R$350,$A55,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A55,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F55" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A55,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A55,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G55" s="12" t="n"/>
@@ -9754,23 +9742,23 @@
         </is>
       </c>
       <c r="B56" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A56)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A56,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A56,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A56,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A56,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E56" s="12">
-        <f>B56-C56-D56-COUNTIFS(Backlog!$R$2:$R$349,$A56,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A56,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B56-C56-D56-COUNTIFS(Backlog!$R$2:$R$350,$A56,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A56,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F56" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A56,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A56,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G56" s="12" t="n"/>
@@ -9783,23 +9771,23 @@
         </is>
       </c>
       <c r="B57" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A57)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A57,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A57,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A57,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A57,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E57" s="12">
-        <f>B57-C57-D57-COUNTIFS(Backlog!$R$2:$R$349,$A57,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A57,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B57-C57-D57-COUNTIFS(Backlog!$R$2:$R$350,$A57,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A57,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F57" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A57,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A57,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G57" s="12" t="n"/>
@@ -9812,23 +9800,23 @@
         </is>
       </c>
       <c r="B58" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A58)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A58,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A58,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A58,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A58,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E58" s="12">
-        <f>B58-C58-D58-COUNTIFS(Backlog!$R$2:$R$349,$A58,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A58,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B58-C58-D58-COUNTIFS(Backlog!$R$2:$R$350,$A58,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A58,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F58" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A58,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A58,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G58" s="12" t="n"/>
@@ -9841,23 +9829,23 @@
         </is>
       </c>
       <c r="B59" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A59)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A59,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A59,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A59,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A59,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E59" s="12">
-        <f>B59-C59-D59-COUNTIFS(Backlog!$R$2:$R$349,$A59,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A59,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B59-C59-D59-COUNTIFS(Backlog!$R$2:$R$350,$A59,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A59,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F59" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A59,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A59,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G59" s="12" t="n"/>
@@ -9870,23 +9858,23 @@
         </is>
       </c>
       <c r="B60" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A60)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A60,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A60,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A60,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A60,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E60" s="12">
-        <f>B60-C60-D60-COUNTIFS(Backlog!$R$2:$R$349,$A60,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A60,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B60-C60-D60-COUNTIFS(Backlog!$R$2:$R$350,$A60,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A60,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F60" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A60,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A60,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G60" s="12" t="n"/>
@@ -9899,23 +9887,23 @@
         </is>
       </c>
       <c r="B61" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A61)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A61,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A61,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A61,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A61,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E61" s="12">
-        <f>B61-C61-D61-COUNTIFS(Backlog!$R$2:$R$349,$A61,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A61,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B61-C61-D61-COUNTIFS(Backlog!$R$2:$R$350,$A61,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A61,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F61" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A61,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A61,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G61" s="12" t="n"/>
@@ -9928,23 +9916,23 @@
         </is>
       </c>
       <c r="B62" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A62)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A62,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A62,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A62,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A62,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E62" s="12">
-        <f>B62-C62-D62-COUNTIFS(Backlog!$R$2:$R$349,$A62,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A62,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B62-C62-D62-COUNTIFS(Backlog!$R$2:$R$350,$A62,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A62,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F62" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A62,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A62,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G62" s="12" t="n"/>
@@ -9957,23 +9945,23 @@
         </is>
       </c>
       <c r="B63" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A63)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A63,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A63,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A63,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A63,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E63" s="12">
-        <f>B63-C63-D63-COUNTIFS(Backlog!$R$2:$R$349,$A63,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A63,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B63-C63-D63-COUNTIFS(Backlog!$R$2:$R$350,$A63,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A63,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F63" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A63,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A63,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G63" s="12" t="n"/>
@@ -9986,23 +9974,23 @@
         </is>
       </c>
       <c r="B64" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A64)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A64,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A64,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A64,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A64,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E64" s="12">
-        <f>B64-C64-D64-COUNTIFS(Backlog!$R$2:$R$349,$A64,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A64,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B64-C64-D64-COUNTIFS(Backlog!$R$2:$R$350,$A64,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A64,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F64" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A64,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A64,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G64" s="12" t="n"/>
@@ -10015,23 +10003,23 @@
         </is>
       </c>
       <c r="B65" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A65)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A65,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A65,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A65,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A65,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E65" s="12">
-        <f>B65-C65-D65-COUNTIFS(Backlog!$R$2:$R$349,$A65,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A65,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B65-C65-D65-COUNTIFS(Backlog!$R$2:$R$350,$A65,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A65,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F65" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A65,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A65,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G65" s="12" t="n"/>
@@ -10044,23 +10032,23 @@
         </is>
       </c>
       <c r="B66" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A66)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A66,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A66,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A66,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A66,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E66" s="12">
-        <f>B66-C66-D66-COUNTIFS(Backlog!$R$2:$R$349,$A66,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A66,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B66-C66-D66-COUNTIFS(Backlog!$R$2:$R$350,$A66,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A66,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F66" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A66,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A66,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G66" s="12" t="n"/>
@@ -10073,23 +10061,23 @@
         </is>
       </c>
       <c r="B67" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A67)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A67,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A67,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A67,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A67,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E67" s="12">
-        <f>B67-C67-D67-COUNTIFS(Backlog!$R$2:$R$349,$A67,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A67,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B67-C67-D67-COUNTIFS(Backlog!$R$2:$R$350,$A67,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A67,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F67" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A67,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A67,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G67" s="12" t="n"/>
@@ -10102,23 +10090,23 @@
         </is>
       </c>
       <c r="B68" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A68)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A68,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A68,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A68,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A68,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E68" s="12">
-        <f>B68-C68-D68-COUNTIFS(Backlog!$R$2:$R$349,$A68,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A68,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B68-C68-D68-COUNTIFS(Backlog!$R$2:$R$350,$A68,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A68,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F68" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A68,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A68,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G68" s="12" t="n"/>
@@ -10131,23 +10119,23 @@
         </is>
       </c>
       <c r="B69" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A69)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A69,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A69,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A69,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A69,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E69" s="12">
-        <f>B69-C69-D69-COUNTIFS(Backlog!$R$2:$R$349,$A69,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A69,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B69-C69-D69-COUNTIFS(Backlog!$R$2:$R$350,$A69,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A69,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F69" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A69,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A69,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G69" s="12" t="n"/>
@@ -10160,23 +10148,23 @@
         </is>
       </c>
       <c r="B70" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A70)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A70,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A70,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A70,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A70,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E70" s="12">
-        <f>B70-C70-D70-COUNTIFS(Backlog!$R$2:$R$349,$A70,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A70,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B70-C70-D70-COUNTIFS(Backlog!$R$2:$R$350,$A70,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A70,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F70" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A70,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A70,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G70" s="12" t="n"/>
@@ -10189,23 +10177,23 @@
         </is>
       </c>
       <c r="B71" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A71)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A71,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A71,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A71,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A71,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E71" s="12">
-        <f>B71-C71-D71-COUNTIFS(Backlog!$R$2:$R$349,$A71,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A71,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B71-C71-D71-COUNTIFS(Backlog!$R$2:$R$350,$A71,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A71,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F71" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A71,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A71,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G71" s="12" t="n"/>
@@ -10218,23 +10206,23 @@
         </is>
       </c>
       <c r="B72" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A72)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A72,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A72,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A72,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A72,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E72" s="12">
-        <f>B72-C72-D72-COUNTIFS(Backlog!$R$2:$R$349,$A72,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A72,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B72-C72-D72-COUNTIFS(Backlog!$R$2:$R$350,$A72,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A72,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F72" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A72,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A72,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G72" s="12" t="n"/>
@@ -10247,23 +10235,23 @@
         </is>
       </c>
       <c r="B73" s="12">
-        <f>COUNTIF(Backlog!$R$2:$R$349,$A73)</f>
+        <f>COUNTIF(Backlog!$R$2:$R$350,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A73,Backlog!$F$2:$F$349,"Done")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A73,Backlog!$F$2:$F$350,"Done")</f>
         <v/>
       </c>
       <c r="D73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A73,Backlog!$F$2:$F$349,"Later")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A73,Backlog!$F$2:$F$350,"Later")</f>
         <v/>
       </c>
       <c r="E73" s="12">
-        <f>B73-C73-D73-COUNTIFS(Backlog!$R$2:$R$349,$A73,Backlog!$F$2:$F$349,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$349,$A73,Backlog!$F$2:$F$349,"Obsolete")</f>
+        <f>B73-C73-D73-COUNTIFS(Backlog!$R$2:$R$350,$A73,Backlog!$F$2:$F$350,"Cancelled")-COUNTIFS(Backlog!$R$2:$R$350,$A73,Backlog!$F$2:$F$350,"Obsolete")</f>
         <v/>
       </c>
       <c r="F73" s="12">
-        <f>COUNTIFS(Backlog!$R$2:$R$349,$A73,Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIFS(Backlog!$R$2:$R$350,$A73,Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="G73" s="12" t="n"/>
@@ -10285,7 +10273,7 @@
         </is>
       </c>
       <c r="B75" s="12">
-        <f>COUNTIF(Backlog!$S$2:$S$349,"Yes")</f>
+        <f>COUNTIF(Backlog!$S$2:$S$350,"Yes")</f>
         <v/>
       </c>
       <c r="C75" s="12" t="n"/>
@@ -10302,7 +10290,7 @@
         </is>
       </c>
       <c r="B76" s="12">
-        <f>COUNTIFS(Backlog!$S$2:$S$349,"Yes",Backlog!$G$2:$G$349,"P0")</f>
+        <f>COUNTIFS(Backlog!$S$2:$S$350,"Yes",Backlog!$G$2:$G$350,"P0")</f>
         <v/>
       </c>
       <c r="C76" s="12" t="n"/>
@@ -10319,7 +10307,7 @@
         </is>
       </c>
       <c r="B77" s="12">
-        <f>COUNTIFS(Backlog!$S$2:$S$349,"No",Backlog!$G$2:$G$349,"P0",Backlog!$F$2:$F$349,"&lt;&gt;Done",Backlog!$F$2:$F$349,"&lt;&gt;Later",Backlog!$F$2:$F$349,"&lt;&gt;Cancelled",Backlog!$F$2:$F$349,"&lt;&gt;Obsolete")</f>
+        <f>COUNTIFS(Backlog!$S$2:$S$350,"No",Backlog!$G$2:$G$350,"P0",Backlog!$F$2:$F$350,"&lt;&gt;Done",Backlog!$F$2:$F$350,"&lt;&gt;Later",Backlog!$F$2:$F$350,"&lt;&gt;Cancelled",Backlog!$F$2:$F$350,"&lt;&gt;Obsolete")</f>
         <v/>
       </c>
       <c r="C77" s="12" t="n"/>
@@ -10336,7 +10324,7 @@
         </is>
       </c>
       <c r="B78" s="12">
-        <f>COUNTIF(Backlog!$F$2:$F$349,"Hold")</f>
+        <f>COUNTIF(Backlog!$F$2:$F$350,"Hold")</f>
         <v/>
       </c>
       <c r="C78" s="12" t="n"/>
@@ -10362,7 +10350,7 @@
         </is>
       </c>
       <c r="B80" s="12">
-        <f>COUNTIFS(Backlog!$G$2:$G$349,"P0",Backlog!$F$2:$F$349,"&lt;&gt;Done",Backlog!$F$2:$F$349,"&lt;&gt;Cancelled",Backlog!$F$2:$F$349,"&lt;&gt;Obsolete",Backlog!$F$2:$F$349,"&lt;&gt;Later")</f>
+        <f>COUNTIFS(Backlog!$G$2:$G$350,"P0",Backlog!$F$2:$F$350,"&lt;&gt;Done",Backlog!$F$2:$F$350,"&lt;&gt;Cancelled",Backlog!$F$2:$F$350,"&lt;&gt;Obsolete",Backlog!$F$2:$F$350,"&lt;&gt;Later")</f>
         <v/>
       </c>
       <c r="C80" s="12" t="n"/>
@@ -10379,7 +10367,7 @@
         </is>
       </c>
       <c r="B81" s="12">
-        <f>COUNTIFS(Backlog!$N$2:$N$349,"Sales blocker",Backlog!$F$2:$F$349,"&lt;&gt;Done")</f>
+        <f>COUNTIFS(Backlog!$N$2:$N$350,"Sales blocker",Backlog!$F$2:$F$350,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="C81" s="12" t="n"/>
@@ -10396,7 +10384,7 @@
         </is>
       </c>
       <c r="B82" s="12">
-        <f>COUNTIFS(Backlog!$E$2:$E$349,"Decision Needed",Backlog!$F$2:$F$349,"&lt;&gt;Done")</f>
+        <f>COUNTIFS(Backlog!$E$2:$E$350,"Decision Needed",Backlog!$F$2:$F$350,"&lt;&gt;Done")</f>
         <v/>
       </c>
       <c r="C82" s="12" t="n"/>
@@ -10447,7 +10435,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -10611,7 +10598,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
@@ -10871,7 +10857,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
@@ -10927,7 +10912,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
@@ -10995,7 +10979,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
@@ -11372,7 +11355,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -11791,7 +11773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U349"/>
+  <dimension ref="A1:U350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -21372,7 +21354,7 @@
       </c>
       <c r="K107" s="8" t="inlineStr">
         <is>
-          <t>2026-10-25: the issued-licence ledger (#341) and the licence flow gate (#342) feed the owner-initiated admin reset (#343-#348).</t>
+          <t>2026-10-25: the issued-licence ledger (#341) and the licence flow gate (#342) feed the owner-initiated admin reset (#343-#349).</t>
         </is>
       </c>
       <c r="L107" s="10" t="inlineStr">
@@ -22949,7 +22931,7 @@
       </c>
       <c r="K124" s="8" t="inlineStr">
         <is>
-          <t>2026-10-25: the issued-licence ledger (#341) and the licence flow gate (#342) feed the owner-initiated admin reset (#343-#348).</t>
+          <t>2026-10-25: the issued-licence ledger (#341) and the licence flow gate (#342) feed the owner-initiated admin reset (#343-#349).</t>
         </is>
       </c>
       <c r="L124" s="10" t="inlineStr">
@@ -41976,7 +41958,7 @@
       </c>
       <c r="H342" s="8" t="inlineStr">
         <is>
-          <t>Today there is no record that lets the owner pick a customer and find the licence that customer received. Licences issued before the ledger existed must stay usable for later owner actions such as the one-time admin reset (#343-#348).</t>
+          <t>Today there is no record that lets the owner pick a customer and find the licence that customer received. Licences issued before the ledger existed must stay usable for later owner actions such as the one-time admin reset (#343-#349). The separate administrator-recovery work done by Saber (second-admin reset, recovery codes, server-side break-glass) does not depend on this row and can proceed without it.</t>
         </is>
       </c>
       <c r="I342" s="8" t="inlineStr">
@@ -42061,7 +42043,7 @@
       </c>
       <c r="H343" s="8" t="inlineStr">
         <is>
-          <t>The owner-initiated admin reset (#343-#348) must work from the licence that a customer really holds, so the whole licence chain has to be proven first: customer request file, owner issues the licence, customer installs it, the product accepts it and the ledger shows it. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+          <t>The owner-initiated admin reset (#343-#349) must work from the licence that a customer really holds, so the whole licence chain has to be proven first: customer request file, owner issues the licence, customer installs it, the product accepts it and the ledger shows it. Gate: every admin-password-reset row (#343-#349) can start only after #342 is Done. The separate administrator-recovery work done by Saber (second-admin reset, recovery codes, server-side break-glass) does not depend on this row and can proceed without it.</t>
         </is>
       </c>
       <c r="I343" s="8" t="inlineStr">
@@ -42071,7 +42053,7 @@
       </c>
       <c r="J343" s="8" t="inlineStr">
         <is>
-          <t>Done when: a clean install is activated with a licence issued by the vendor tool; the ledger lists that licence with its Install ID and fingerprint hash; an imported earlier licence behaves the same; the run is written in the acceptance checklist. Only then are #343-#348 unblocked.</t>
+          <t>Done when: a clean install is activated with a licence issued by the vendor tool; the ledger lists that licence with its Install ID and fingerprint hash; an imported earlier licence behaves the same; the run is written in the acceptance checklist. Only then are #343-#349 unblocked.</t>
         </is>
       </c>
       <c r="K343" s="8" t="n"/>
@@ -42126,7 +42108,7 @@
       </c>
       <c r="D344" s="8" t="inlineStr">
         <is>
-          <t>Design and decision for an owner-initiated admin password reset by a one-time link tied to the customer's licence (threat model, binding, expiry, key custody)</t>
+          <t>Design and decision for the vendor-assisted admin password reset by file exchange (request file out, signed response file back), separate reset key, and AFTA compatibility check</t>
         </is>
       </c>
       <c r="E344" s="10" t="inlineStr">
@@ -42146,17 +42128,17 @@
       </c>
       <c r="H344" s="8" t="inlineStr">
         <is>
-          <t>A customer who loses the administrator password must be recoverable by the system owner without a back door in the product and without internet access. The reset has to work only on the customer's own installation, once, and only if the owner chooses that customer. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+          <t>A customer whose production server is offline must be able to recover a lost administrator password with the vendor's help, without a back door in the product and without any remote access. The licence flow already proves that file exchange works offline; the reset reuses its shape with its own key. Gate: this row can start only after #342 (licence flow end to end) is Done. Independent of the separate administrator-recovery work done by Saber (second-admin reset, one-time recovery codes, server-side break-glass, shared audit/notification/session revocation): that work does not wait for the licence flow and this row does not block it; this flow plugs into it as the optional vendor-assisted recovery path, which must stay off until the customer enables it.</t>
         </is>
       </c>
       <c r="I344" s="8" t="inlineStr">
         <is>
-          <t>Write docs/design/ADMIN_RESET.md (no secrets): the reset ticket is signed by the owner, bound to licence id + Install ID + fingerprint hash + signing key id, has a short expiry, a random nonce stored on use so it works once, and is delivered as a link or file by any channel. Decide: which key signs it (the licence key stays offline per #107; a separate reset-only key may be allowed on the owner's local computer or the assistant's computer, never the licence key), what is reset (password only, or also MFA/passkeys and sessions), how the owner verifies the customer identity before issuing, rate limits, audit on both sides, and what happens on a cloned or re-hosted machine (#104, #116).</t>
+          <t>Write docs/design/ADMIN_RESET.md (no secrets). Flow (same shape as licence activation, all in the browser UI; no terminal or CLI step): 1) the customer opens the administrator recovery page on their installation and downloads a reset request file (.pemsrstreq: Install ID, fingerprint hash, licence id, product version, account, random nonce kept server-side as a pending request, signed by the install key); 2) the customer sends the file to us; 3) in the developer/owner UI we upload it, the tool verifies the signature, matches it to the customer and licence in the ledger, we confirm the customer, enter the reason and the identity check, and download a reset response file (.pemsreset) signed with the separate reset key and bound to the request nonce, licence id, Install ID, purpose and expiry; 4) the customer uploads the response file on the same page and the password reset form opens; the pending request is consumed so the file works once. Decide: reset-key custody and where it may live (on the owner's local computer or the assistant's computer, never the licence key), what the reset changes (password; MFA/passkeys and sessions as in the shared recovery rules), expiry of the response file, rate limits, audit on both sides, behaviour on a cloned or re-hosted machine (#104, #116). AFTA check (to be confirmed with the testing lab through #184): no default, master or hard-coded password and no standing vendor credential; the vendor can act only on a request that the installation itself generated, for one installation, once and for a short time; the capability is off by default and enabled explicitly by the customer administrator; every use is audited, all administrators are notified, the account sessions are revoked and the event goes to the SIEM feed; the reset key is separate from the licence key and can be revoked through an update; everything works offline by file exchange, so no remote access to the customer server is ever needed.</t>
         </is>
       </c>
       <c r="J344" s="8" t="inlineStr">
         <is>
-          <t>Done when: an approved ADR with the threat model (replay, wrong customer, tampered ticket, cloned machine, clock change, leaked link), the key-custody decision, and the exact ticket fields; the next rows #344-#348 are written against it.</t>
+          <t>Done when: an approved ADR with the file formats' fields, the key-custody decision, the threat model (replay, wrong customer, tampered or forged file, cloned machine, clock change, leaked file) and a written AFTA compatibility assessment accepted by the security consultant; #344-#349 are written against it.</t>
         </is>
       </c>
       <c r="K344" s="8" t="n"/>
@@ -42177,7 +42159,7 @@
       </c>
       <c r="O344" s="10" t="inlineStr">
         <is>
-          <t>#96 #107 #178 #182 #339 #342</t>
+          <t>#96 #107 #178 #182 #184 #339 #342</t>
         </is>
       </c>
       <c r="P344" s="10" t="n"/>
@@ -42211,7 +42193,7 @@
       </c>
       <c r="D345" s="8" t="inlineStr">
         <is>
-          <t>Reset ticket format and signing library: payload fields, signature, expiry, nonce, link and file encodings, verification used by both the owner tool and the product</t>
+          <t>Reset request and reset response file formats (.pemsrstreq and .pemsreset) with a shared signing and verification library</t>
         </is>
       </c>
       <c r="E345" s="10" t="inlineStr">
@@ -42231,17 +42213,17 @@
       </c>
       <c r="H345" s="8" t="inlineStr">
         <is>
-          <t>One shared, tested implementation prevents the owner tool and the product from disagreeing about what a valid ticket is. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+          <t>One shared, tested implementation prevents the owner UI and the product from disagreeing about what a valid file is. Gate: this row can start only after #342 (licence flow end to end) is Done. Independent of the separate administrator-recovery work done by Saber (second-admin reset, one-time recovery codes, server-side break-glass, shared audit/notification/session revocation): that work does not wait for the licence flow and this row does not block it; this flow plugs into it as the optional vendor-assisted recovery path, which must stay off until the customer enables it.</t>
         </is>
       </c>
       <c r="I345" s="8" t="inlineStr">
         <is>
-          <t>Implement the ticket from the ADR (#343) in a shared library (PEMS.Shared or a licensing project): canonical encoding, Ed25519/ECDSA signature with domain separation from licence files, fields (customer, licence id, Install ID, fingerprint hash, key id, issued-at, expires-at, nonce, purpose), link form (short URL path with the ticket in the fragment so it is not logged) and file form. Unit tests with test vectors for valid, expired, tampered, wrong-binding and wrong-purpose tickets.</t>
+          <t>Implement the two formats from the ADR (#343) in a shared library: canonical encoding; request signed by the install key; response signed by the reset key with domain separation from licence files; response bound to the request nonce, licence id, Install ID, fingerprint hash, reset key id, issued-at, expires-at and purpose. Unit tests with vectors for valid, expired, tampered, wrong-nonce, wrong-installation, wrong-key and wrong-purpose files, each rejected with a distinct reason.</t>
         </is>
       </c>
       <c r="J345" s="8" t="inlineStr">
         <is>
-          <t>Done when: the library signs and verifies tickets; every negative test vector is rejected with a distinct reason; the same code is referenced by #345 and #346.</t>
+          <t>Done when: the library creates and verifies both files; every negative vector is rejected with its own reason; the owner UI (#345) and the product (#346) use the same code.</t>
         </is>
       </c>
       <c r="K345" s="8" t="n"/>
@@ -42262,7 +42244,7 @@
       </c>
       <c r="O345" s="10" t="inlineStr">
         <is>
-          <t>#101 #107 #343</t>
+          <t>#101 #343 #349</t>
         </is>
       </c>
       <c r="P345" s="10" t="n"/>
@@ -42296,7 +42278,7 @@
       </c>
       <c r="D346" s="8" t="inlineStr">
         <is>
-          <t>Owner reset tool on the owner's local computer: choose the customer and licence from the ledger, issue a one-time reset link or file, audit it</t>
+          <t>Developer/owner UI: upload the customer's reset request file, match it to the customer and licence in the ledger, issue the signed reset response file</t>
         </is>
       </c>
       <c r="E346" s="10" t="inlineStr">
@@ -42316,17 +42298,17 @@
       </c>
       <c r="H346" s="8" t="inlineStr">
         <is>
-          <t>The owner (or the assistant acting for the owner) needs a safe place to issue reset links without internet and without exposing the licence signing key. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+          <t>The owner needs a safe, offline place to answer a customer's reset request without exposing the licence signing key. Gate: this row can start only after #342 (licence flow end to end) is Done. Independent of the separate administrator-recovery work done by Saber (second-admin reset, one-time recovery codes, server-side break-glass, shared audit/notification/session revocation): that work does not wait for the licence flow and this row does not block it; this flow plugs into it as the optional vendor-assisted recovery path, which must stay off until the customer enables it.</t>
         </is>
       </c>
       <c r="I346" s="8" t="inlineStr">
         <is>
-          <t>Add a Reset admin action to the vendor tool (#106) that runs on the owner's local computer: pick the customer, pick one of its licences from the ledger (#341), enter the reason and the identity check performed, choose the expiry, then produce the one-time link and the .pemsreset file using #344. Show the link once, never write it to a log, and record the issue (who, when, customer, licence, expiry, reason) in the audit. Revoked or expired licences cannot be selected. Works fully offline. Everything is done in the UI; no terminal or CLI step is required.</t>
+          <t>Add a Reset admin page to the vendor tool (#106), run on the owner's local computer: upload the .pemsrstreq, verify its signature, find the matching licence in the ledger (#341) by licence id, Install ID and fingerprint hash, show the customer and let the owner confirm or pick the customer (a mismatch is a warning that blocks issuing), enter the reason and the identity check performed, choose the expiry, then download the .pemsreset built with #344 and signed with the reset key (#349). Revoked or expired licences cannot be answered. Write an audit entry (who, when, customer, licence, request nonce, expiry, reason). Works fully offline. All in the UI; no terminal or CLI step.</t>
         </is>
       </c>
       <c r="J346" s="8" t="inlineStr">
         <is>
-          <t>Done when: from the ledger the owner issues a link for a chosen customer in under a minute with no network; the audit shows it; a revoked licence cannot get a link; the signing key custody follows #343.</t>
+          <t>Done when: from an uploaded request file the owner issues a response file for the right customer in under a minute with no network; a request for a revoked licence or for an unknown installation is refused; the audit shows each issue.</t>
         </is>
       </c>
       <c r="K346" s="8" t="n"/>
@@ -42347,7 +42329,7 @@
       </c>
       <c r="O346" s="10" t="inlineStr">
         <is>
-          <t>#341 #343 #344</t>
+          <t>#341 #343 #344 #349</t>
         </is>
       </c>
       <c r="P346" s="10" t="n"/>
@@ -42381,7 +42363,7 @@
       </c>
       <c r="D347" s="8" t="inlineStr">
         <is>
-          <t>Product side of the one-time admin reset: verify the ticket against the installed licence, consume the nonce once, set a new administrator password, revoke sessions, audit</t>
+          <t>Customer UI: administrator recovery page (download reset request file, upload reset response file, open the reset form), one-time, licence-bound, off by default</t>
         </is>
       </c>
       <c r="E347" s="10" t="inlineStr">
@@ -42401,17 +42383,17 @@
       </c>
       <c r="H347" s="8" t="inlineStr">
         <is>
-          <t>The customer opens the link on their own installation; the product must accept it only if it matches this installation's licence, and only once. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+          <t>The customer must be able to start and finish the recovery from the product UI of their own installation, and the product must accept only an answer to its own request. Gate: this row can start only after #342 (licence flow end to end) is Done. Independent of the separate administrator-recovery work done by Saber (second-admin reset, one-time recovery codes, server-side break-glass, shared audit/notification/session revocation): that work does not wait for the licence flow and this row does not block it; this flow plugs into it as the optional vendor-assisted recovery path, which must stay off until the customer enables it.</t>
         </is>
       </c>
       <c r="I347" s="8" t="inlineStr">
         <is>
-          <t>Add an anonymous-safe reset page and endpoint: verify signature and expiry with #344, check licence id, Install ID and fingerprint hash against the installed licence (#99, #98), record the nonce in a new table through an EF migration so a second use fails, then let the person set a new administrator password under the password policy, require a password change at next sign-in, re-enrol MFA/passkeys as decided in #343, revoke all sessions of that user (#182), write the audit and rate-limit failures. The page is added to the always-free surfaces list and is available even before the first sign-in.</t>
+          <t>Add the recovery page (anonymous-safe, on the always-free surfaces list) with a setting that keeps it disabled until a customer administrator enables it. Generate the .pemsrstreq (#344) and store the pending request (nonce, time, requested account) through an EF migration. On upload of a .pemsreset verify signature and expiry, match the stored nonce, licence id, Install ID and fingerprint hash against the installed licence (#98, #99), consume the pending request, then open the form to set a new administrator password under the password policy, require a change at next sign-in, handle MFA/passkeys and revoke the account's sessions (#182) as decided in #343, write the audit, notify all administrators, send the event to the SIEM feed and rate-limit failures.</t>
         </is>
       </c>
       <c r="J347" s="8" t="inlineStr">
         <is>
-          <t>Done when: a valid link resets the administrator password once on the matching installation; the same link, an expired link, a link for another customer or machine, and a tampered link are all refused with the audit entry; existing sessions end.</t>
+          <t>Done when: a valid response file resets the administrator password once on the matching installation; the same file again, an expired file, a file for another installation or request, and a tampered file are refused with an audit entry; sessions end; with the setting off the page offers nothing.</t>
         </is>
       </c>
       <c r="K347" s="8" t="n"/>
@@ -42432,7 +42414,7 @@
       </c>
       <c r="O347" s="10" t="inlineStr">
         <is>
-          <t>#98 #99 #108 #182 #343 #344</t>
+          <t>#98 #99 #108 #182 #343 #344 #349</t>
         </is>
       </c>
       <c r="P347" s="10" t="n"/>
@@ -42466,7 +42448,7 @@
       </c>
       <c r="D348" s="8" t="inlineStr">
         <is>
-          <t>Automated security tests for the admin reset: replay, expiry, wrong customer or machine, tampering, clock change, brute force, session revocation</t>
+          <t>Automated security tests for the admin reset: replay, expiry, wrong customer or installation, forged or tampered files, clock change, brute force, setting off, session revocation</t>
         </is>
       </c>
       <c r="E348" s="10" t="inlineStr">
@@ -42486,17 +42468,17 @@
       </c>
       <c r="H348" s="8" t="inlineStr">
         <is>
-          <t>A recovery path is a favourite attack target; it must be covered by tests before it ships. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+          <t>A recovery path is a favourite attack target; it must be covered by tests before it ships. Gate: this row can start only after #342 (licence flow end to end) is Done. Independent of the separate administrator-recovery work done by Saber (second-admin reset, one-time recovery codes, server-side break-glass, shared audit/notification/session revocation): that work does not wait for the licence flow and this row does not block it; this flow plugs into it as the optional vendor-assisted recovery path, which must stay off until the customer enables it.</t>
         </is>
       </c>
       <c r="I348" s="8" t="inlineStr">
         <is>
-          <t>Write integration tests against the real product endpoint and the owner tool library: replay of a used link, expired ticket, ticket issued for another licence or Install ID, modified payload, signature from a different key, cloned machine (fingerprint mismatch), clock rolled back, repeated failures hitting the rate limit, and confirmation that sessions and MFA state are changed as specified. Add them to the CI gate.</t>
+          <t>Write integration tests against the real product endpoint and the owner UI library: replay of a used response, expired response, response for another request or installation, modified payload, signature by a different or revoked key, forged request file, cloned machine (fingerprint mismatch), clock rolled back, repeated failures reaching the rate limit, the feature switched off, and that sessions, MFA state, audit and administrator notifications are as specified. Add them to the CI gate.</t>
         </is>
       </c>
       <c r="J348" s="8" t="inlineStr">
         <is>
-          <t>Done when: each scenario has a passing test that fails if the defence is removed; the tests run in CI; results are linked from the licence acceptance checklist.</t>
+          <t>Done when: each scenario has a passing test that fails if its defence is removed; the tests run in CI; results are linked from the licence acceptance checklist.</t>
         </is>
       </c>
       <c r="K348" s="8" t="n"/>
@@ -42551,7 +42533,7 @@
       </c>
       <c r="D349" s="8" t="inlineStr">
         <is>
-          <t>Owner procedure and customer-facing guide for the admin reset: identity verification, issuing, delivery, audit review</t>
+          <t>Owner procedure and customer-facing guide for the admin reset by file exchange: identity verification, request and response handling, enabling the feature, audit review</t>
         </is>
       </c>
       <c r="E349" s="10" t="inlineStr">
@@ -42571,17 +42553,17 @@
       </c>
       <c r="H349" s="8" t="inlineStr">
         <is>
-          <t>Technical safety is not enough: the owner needs a written rule for when a reset is allowed, and customers need to know how to ask. Gate: every admin-password-reset row (#343-#348) can start only after #342 is Done.</t>
+          <t>Technical safety is not enough: the owner needs a written rule for when a reset is allowed, and customers need to know how to ask. Gate: this row can start only after #342 (licence flow end to end) is Done. Independent of the separate administrator-recovery work done by Saber (second-admin reset, one-time recovery codes, server-side break-glass, shared audit/notification/session revocation): that work does not wait for the licence flow and this row does not block it; this flow plugs into it as the optional vendor-assisted recovery path, which must stay off until the customer enables it.</t>
         </is>
       </c>
       <c r="I349" s="8" t="inlineStr">
         <is>
-          <t>Write the procedure: how the customer asks, how the owner verifies identity (named contact on the contract, call-back), which customer and licence to select in the owner tool, how the link is delivered, how long it stays valid, how the audit is reviewed monthly, and what is said to the customer. Add a short help topic in the product and link it from the licence support procedure (#123).</t>
+          <t>Write the procedure: how the customer enables the recovery page and generates the request file, how the owner verifies identity (named contact on the contract, call-back), which customer is confirmed in the owner UI, how the response file is delivered and how long it stays valid, how the audit is reviewed monthly, and what is said to the customer. Add a help topic in the product and link it from the licence support procedure (#123).</t>
         </is>
       </c>
       <c r="J349" s="8" t="inlineStr">
         <is>
-          <t>Done when: the owner approves the procedure; a rehearsed reset from request to new password follows it; the help topic exists in Persian and English.</t>
+          <t>Done when: the owner approves the procedure; a rehearsed reset from request file to new password follows it; the help topic exists in Persian and English.</t>
         </is>
       </c>
       <c r="K349" s="8" t="n"/>
@@ -42620,9 +42602,94 @@
       <c r="T349" s="10" t="n"/>
       <c r="U349" s="10" t="n"/>
     </row>
+    <row r="350">
+      <c r="A350" s="10" t="n">
+        <v>349</v>
+      </c>
+      <c r="B350" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C350" s="8" t="inlineStr">
+        <is>
+          <t>Access, RLS, Sessions &amp; Security</t>
+        </is>
+      </c>
+      <c r="D350" s="8" t="inlineStr">
+        <is>
+          <t>Reset signing key procedure: create the separate reset key offline, custody, backup, rotation, revocation list shipped in updates, compromise plan</t>
+        </is>
+      </c>
+      <c r="E350" s="10" t="inlineStr">
+        <is>
+          <t>Ops Process</t>
+        </is>
+      </c>
+      <c r="F350" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G350" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H350" s="8" t="inlineStr">
+        <is>
+          <t>The reset response file must be signed by a key that is not the licence key, so that a leak of one never opens the other; it follows the same custody rules as the licence key (#107). Gate: this row can start only after #342 (licence flow end to end) is Done. Independent of the separate administrator-recovery work done by Saber (second-admin reset, one-time recovery codes, server-side break-glass, shared audit/notification/session revocation): that work does not wait for the licence flow and this row does not block it; this flow plugs into it as the optional vendor-assisted recovery path, which must stay off until the customer enables it.</t>
+        </is>
+      </c>
+      <c r="I350" s="8" t="inlineStr">
+        <is>
+          <t>1) Generate a separate reset key pair offline (Ed25519 recommended) and record its key id; the public key is embedded in the product with the key id, the private key lives on the owner's offline or local machine, never in the repository or on a shared server. 2) Decide in the ADR (#343) whether the assistant's computer may hold it. 3) Write docs/process/RESET_KEY_MANAGEMENT.md without secrets: holders, encrypted backups, rotation, how a revoked key id is delivered to installations through an update (#117), and the compromise plan. 4) Perform the ceremony and record who attended.</t>
+        </is>
+      </c>
+      <c r="J350" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the reset key pair exists with a key id; the procedure document is approved; a test response signed with it verifies in the product and a response signed with a revoked key id is refused.</t>
+        </is>
+      </c>
+      <c r="K350" s="8" t="n"/>
+      <c r="L350" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M350" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N350" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O350" s="10" t="inlineStr">
+        <is>
+          <t>#107 #343</t>
+        </is>
+      </c>
+      <c r="P350" s="10" t="n"/>
+      <c r="Q350" s="10" t="n"/>
+      <c r="R350" s="8" t="inlineStr">
+        <is>
+          <t>Security &amp; access</t>
+        </is>
+      </c>
+      <c r="S350" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T350" s="10" t="n"/>
+      <c r="U350" s="10" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U349"/>
-  <conditionalFormatting sqref="F2:F349">
+  <autoFilter ref="A1:U350"/>
+  <conditionalFormatting sqref="F2:F350">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Done"</formula>
     </cfRule>
@@ -42645,7 +42712,7 @@
       <formula>"Obsolete"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G349">
+  <conditionalFormatting sqref="G2:G350">
     <cfRule type="cellIs" priority="8" operator="equal" dxfId="6">
       <formula>"P0"</formula>
     </cfRule>
@@ -42653,27 +42720,27 @@
       <formula>"P1"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S349">
+  <conditionalFormatting sqref="S2:S350">
     <cfRule type="cellIs" priority="10" operator="equal" dxfId="8">
       <formula>"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N349">
+  <conditionalFormatting sqref="N2:N350">
     <cfRule type="cellIs" priority="11" operator="equal" dxfId="6">
       <formula>"Sales blocker"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="F2:F349" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F350" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not Started,In Progress,Partial,Done,Hold,Later,Cancelled,Obsolete"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G349" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G350" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B349" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B2:B350" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Claude,User,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S349" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="S2:S350" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -44083,7 +44150,7 @@
         </is>
       </c>
       <c r="F2" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$349,"M0")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$350,"M0")</f>
         <v/>
       </c>
     </row>
@@ -44114,7 +44181,7 @@
         </is>
       </c>
       <c r="F3" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$349,"M1")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$350,"M1")</f>
         <v/>
       </c>
     </row>
@@ -44145,7 +44212,7 @@
         </is>
       </c>
       <c r="F4" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$349,"M2")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$350,"M2")</f>
         <v/>
       </c>
     </row>
@@ -44176,7 +44243,7 @@
         </is>
       </c>
       <c r="F5" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$349,"M3")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$350,"M3")</f>
         <v/>
       </c>
     </row>
@@ -44207,7 +44274,7 @@
         </is>
       </c>
       <c r="F6" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$349,"M4")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$350,"M4")</f>
         <v/>
       </c>
     </row>
@@ -44238,7 +44305,7 @@
         </is>
       </c>
       <c r="F7" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$349,"M5")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$350,"M5")</f>
         <v/>
       </c>
     </row>
@@ -44269,11 +44336,10 @@
         </is>
       </c>
       <c r="F8" s="10">
-        <f>COUNTIF(Backlog!$L$2:$L$349,"M6")</f>
+        <f>COUNTIF(Backlog!$L$2:$L$350,"M6")</f>
         <v/>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
@@ -44447,7 +44513,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
@@ -45205,7 +45270,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -45382,7 +45446,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
@@ -47176,8 +47239,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(plan): admin reset response validity default 1 day, range 1-7 days, no unlimited option (#343-#348)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -42133,12 +42133,12 @@
       </c>
       <c r="I344" s="8" t="inlineStr">
         <is>
-          <t>Write docs/design/ADMIN_RESET.md (no secrets). Flow (same shape as licence activation, all in the browser UI; no terminal or CLI step): 1) the customer opens the administrator recovery page on their installation and downloads a reset request file (.pemsrstreq: Install ID, fingerprint hash, licence id, product version, account, random nonce kept server-side as a pending request, signed by the install key); 2) the customer sends the file to us; 3) in the developer/owner UI we upload it, the tool verifies the signature, matches it to the customer and licence in the ledger, we confirm the customer, enter the reason and the identity check, and download a reset response file (.pemsreset) signed with the separate reset key and bound to the request nonce, licence id, Install ID, purpose and expiry; 4) the customer uploads the response file on the same page and the password reset form opens; the pending request is consumed so the file works once. Decide: reset-key custody and where it may live (on the owner's local computer or the assistant's computer, never the licence key), what the reset changes (password; MFA/passkeys and sessions as in the shared recovery rules), expiry of the response file, rate limits, audit on both sides, behaviour on a cloned or re-hosted machine (#104, #116). AFTA check (to be confirmed with the testing lab through #184): no default, master or hard-coded password and no standing vendor credential; the vendor can act only on a request that the installation itself generated, for one installation, once and for a short time; the capability is off by default and enabled explicitly by the customer administrator; every use is audited, all administrators are notified, the account sessions are revoked and the event goes to the SIEM feed; the reset key is separate from the licence key and can be revoked through an update; everything works offline by file exchange, so no remote access to the customer server is ever needed.</t>
+          <t>Write docs/design/ADMIN_RESET.md (no secrets). Flow (same shape as licence activation, all in the browser UI; no terminal or CLI step): 1) the customer opens the administrator recovery page on their installation and downloads a reset request file (.pemsrstreq: Install ID, fingerprint hash, licence id, product version, account, random nonce kept server-side as a pending request, signed by the install key); 2) the customer sends the file to us; 3) in the developer/owner UI we upload it, the tool verifies the signature, matches it to the customer and licence in the ledger, we confirm the customer, enter the reason and the identity check, and download a reset response file (.pemsreset) signed with the separate reset key and bound to the request nonce, licence id, Install ID, purpose and expiry; 4) the customer uploads the response file on the same page and the password reset form opens; the pending request is consumed so the file works once. Decide: reset-key custody and where it may live (on the owner's local computer or the assistant's computer, never the licence key), what the reset changes (password; MFA/passkeys and sessions as in the shared recovery rules), expiry of the response file, rate limits, audit on both sides, behaviour on a cloned or re-hosted machine (#104, #116). AFTA check (to be confirmed with the testing lab through #184): no default, master or hard-coded password and no standing vendor credential; the vendor can act only on a request that the installation itself generated, for one installation, once and for a short time; the capability is off by default and enabled explicitly by the customer administrator; every use is audited, all administrators are notified, the account sessions are revoked and the event goes to the SIEM feed; the reset key is separate from the licence key and can be revoked through an update; everything works offline by file exchange, so no remote access to the customer server is ever needed. Validity: the response file expires after a period the owner chooses in the developer UI when the file is issued: default 1 day, allowed range 1 to 7 days in whole days, and no unlimited or open-ended option (the tool refuses values outside the range and the product checks the limits again, so a correctly signed file with a longer validity is rejected). The pending reset request on the customer side expires on the same bounds. AFTA: a short, bounded, single-use validity fits the check recorded here; the 1-day default and the 7-day maximum are to be confirmed with the testing lab (#184), and if the lab wants a shorter maximum the limits change in one setting without changing the file format.</t>
         </is>
       </c>
       <c r="J344" s="8" t="inlineStr">
         <is>
-          <t>Done when: an approved ADR with the file formats' fields, the key-custody decision, the threat model (replay, wrong customer, tampered or forged file, cloned machine, clock change, leaked file) and a written AFTA compatibility assessment accepted by the security consultant; #344-#349 are written against it.</t>
+          <t>Done when: an approved ADR with the file formats' fields, the key-custody decision, the threat model (replay, wrong customer, tampered or forged file, cloned machine, clock change, leaked file) and a written AFTA compatibility assessment accepted by the security consultant; #344-#349 are written against it. The validity rule (default 1 day, range 1 to 7 days, no unlimited option) is confirmed by the AFTA assessment.</t>
         </is>
       </c>
       <c r="K344" s="8" t="n"/>
@@ -42218,12 +42218,12 @@
       </c>
       <c r="I345" s="8" t="inlineStr">
         <is>
-          <t>Implement the two formats from the ADR (#343) in a shared library: canonical encoding; request signed by the install key; response signed by the reset key with domain separation from licence files; response bound to the request nonce, licence id, Install ID, fingerprint hash, reset key id, issued-at, expires-at and purpose. Unit tests with vectors for valid, expired, tampered, wrong-nonce, wrong-installation, wrong-key and wrong-purpose files, each rejected with a distinct reason.</t>
+          <t>Implement the two formats from the ADR (#343) in a shared library: canonical encoding; request signed by the install key; response signed by the reset key with domain separation from licence files; response bound to the request nonce, licence id, Install ID, fingerprint hash, reset key id, issued-at, expires-at and purpose. Unit tests with vectors for valid, expired, tampered, wrong-nonce, wrong-installation, wrong-key and wrong-purpose files, each rejected with a distinct reason. The response carries issued-at and expires-at; the library enforces 1 to 7 whole days between them, with the limits as shared named settings used by both sides; add vectors for a validity of 0, 8 days, negative and missing.</t>
         </is>
       </c>
       <c r="J345" s="8" t="inlineStr">
         <is>
-          <t>Done when: the library creates and verifies both files; every negative vector is rejected with its own reason; the owner UI (#345) and the product (#346) use the same code.</t>
+          <t>Done when: the library creates and verifies both files; every negative vector is rejected with its own reason; the owner UI (#345) and the product (#346) use the same code. Validity outside 1 to 7 days is rejected.</t>
         </is>
       </c>
       <c r="K345" s="8" t="n"/>
@@ -42303,12 +42303,12 @@
       </c>
       <c r="I346" s="8" t="inlineStr">
         <is>
-          <t>Add a Reset admin page to the vendor tool (#106), run on the owner's local computer: upload the .pemsrstreq, verify its signature, find the matching licence in the ledger (#341) by licence id, Install ID and fingerprint hash, show the customer and let the owner confirm or pick the customer (a mismatch is a warning that blocks issuing), enter the reason and the identity check performed, choose the expiry, then download the .pemsreset built with #344 and signed with the reset key (#349). Revoked or expired licences cannot be answered. Write an audit entry (who, when, customer, licence, request nonce, expiry, reason). Works fully offline. All in the UI; no terminal or CLI step.</t>
+          <t>Add a Reset admin page to the vendor tool (#106), run on the owner's local computer: upload the .pemsrstreq, verify its signature, find the matching licence in the ledger (#341) by licence id, Install ID and fingerprint hash, show the customer and let the owner confirm or pick the customer (a mismatch is a warning that blocks issuing), enter the reason and the identity check performed, choose the validity in whole days (default 1, range 1 to 7, no unlimited option), then download the .pemsreset built with #344 and signed with the reset key (#349). Revoked or expired licences cannot be answered. Write an audit entry (who, when, customer, licence, request nonce, expiry, reason). Works fully offline. All in the UI; no terminal or CLI step.</t>
         </is>
       </c>
       <c r="J346" s="8" t="inlineStr">
         <is>
-          <t>Done when: from an uploaded request file the owner issues a response file for the right customer in under a minute with no network; a request for a revoked licence or for an unknown installation is refused; the audit shows each issue.</t>
+          <t>Done when: from an uploaded request file the owner issues a response file for the right customer in under a minute with no network; a request for a revoked licence or for an unknown installation is refused; the audit shows each issue. A validity outside 1 to 7 days cannot be chosen.</t>
         </is>
       </c>
       <c r="K346" s="8" t="n"/>
@@ -42388,12 +42388,12 @@
       </c>
       <c r="I347" s="8" t="inlineStr">
         <is>
-          <t>Add the recovery page (anonymous-safe, on the always-free surfaces list) with a setting that keeps it disabled until a customer administrator enables it. Generate the .pemsrstreq (#344) and store the pending request (nonce, time, requested account) through an EF migration. On upload of a .pemsreset verify signature and expiry, match the stored nonce, licence id, Install ID and fingerprint hash against the installed licence (#98, #99), consume the pending request, then open the form to set a new administrator password under the password policy, require a change at next sign-in, handle MFA/passkeys and revoke the account's sessions (#182) as decided in #343, write the audit, notify all administrators, send the event to the SIEM feed and rate-limit failures.</t>
+          <t>Add the recovery page (anonymous-safe, on the always-free surfaces list) with a setting that keeps it disabled until a customer administrator enables it. Generate the .pemsrstreq (#344) and store the pending request (nonce, time, requested account) through an EF migration. On upload of a .pemsreset verify signature and expiry, match the stored nonce, licence id, Install ID and fingerprint hash against the installed licence (#98, #99), consume the pending request, then open the form to set a new administrator password under the password policy, require a change at next sign-in, handle MFA/passkeys and revoke the account's sessions (#182) as decided in #343, write the audit, notify all administrators, send the event to the SIEM feed and rate-limit failures. Reject a response whose validity is outside 1 to 7 days or whose expiry has passed (use the clock guard #105), and expire the pending request on the same bounds.</t>
         </is>
       </c>
       <c r="J347" s="8" t="inlineStr">
         <is>
-          <t>Done when: a valid response file resets the administrator password once on the matching installation; the same file again, an expired file, a file for another installation or request, and a tampered file are refused with an audit entry; sessions end; with the setting off the page offers nothing.</t>
+          <t>Done when: a valid response file resets the administrator password once on the matching installation; the same file again, an expired file, a file for another installation or request, and a tampered file are refused with an audit entry; sessions end; with the setting off the page offers nothing. A response valid for more than 7 days is refused even when correctly signed.</t>
         </is>
       </c>
       <c r="K347" s="8" t="n"/>
@@ -42473,7 +42473,7 @@
       </c>
       <c r="I348" s="8" t="inlineStr">
         <is>
-          <t>Write integration tests against the real product endpoint and the owner UI library: replay of a used response, expired response, response for another request or installation, modified payload, signature by a different or revoked key, forged request file, cloned machine (fingerprint mismatch), clock rolled back, repeated failures reaching the rate limit, the feature switched off, and that sessions, MFA state, audit and administrator notifications are as specified. Add them to the CI gate.</t>
+          <t>Write integration tests against the real product endpoint and the owner UI library: replay of a used response, expired response, response for another request or installation, modified payload, signature by a different or revoked key, forged request file, cloned machine (fingerprint mismatch), clock rolled back, repeated failures reaching the rate limit, the feature switched off, and that sessions, MFA state, audit and administrator notifications are as specified. Add them to the CI gate. Include validity 0, 8 days and a missing expiry, and a response used exactly at and just after its expiry.</t>
         </is>
       </c>
       <c r="J348" s="8" t="inlineStr">
@@ -42558,7 +42558,7 @@
       </c>
       <c r="I349" s="8" t="inlineStr">
         <is>
-          <t>Write the procedure: how the customer enables the recovery page and generates the request file, how the owner verifies identity (named contact on the contract, call-back), which customer is confirmed in the owner UI, how the response file is delivered and how long it stays valid, how the audit is reviewed monthly, and what is said to the customer. Add a help topic in the product and link it from the licence support procedure (#123).</t>
+          <t>Write the procedure: how the customer enables the recovery page and generates the request file, how the owner verifies identity (named contact on the contract, call-back), which customer is confirmed in the owner UI, how the response file is delivered and how long it stays valid, how the audit is reviewed monthly, and what is said to the customer. Add a help topic in the product and link it from the licence support procedure (#123). State that a response is valid for 1 day by default and up to 7 days when the owner chooses a longer window, depending on how fast the customer can return the file.</t>
         </is>
       </c>
       <c r="J349" s="8" t="inlineStr">

</xml_diff>

<commit_message>
docs(plan): key custody decided - licence and reset keys live only on the owner computers (#107, #343, #345, #349, rule 10)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -11355,6 +11355,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -11518,7 +11519,7 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>No real secret, key or connection string in the repo or release package. The licence-signing private key is never on a development machine or in the repo (L_KEYS).</t>
+          <t>No real secret, key or connection string in the repo or release package. The licence-signing private key and the reset private key are created and used only on the owner computers (Hamid's and Saber's own) and are never in the repo, on a CI or shared server, or in the assistant's environment (L_KEYS).</t>
         </is>
       </c>
     </row>
@@ -21441,12 +21442,12 @@
       </c>
       <c r="I108" s="8" t="inlineStr">
         <is>
-          <t>1) Choose the algorithm (recommended Ed25519) and where the private key lives (offline machine or hardware token, never a development machine or the repository, rule 10). 2) Write docs/process/KEY_MANAGEMENT.md without any secret: who holds the key, two encrypted backups in separate places, rotation schedule, what to do if it leaks. 3) Create the key pair under that procedure and commit only the public key for the verifier (#101).</t>
+          <t>1) Choose the algorithm (recommended Ed25519) and where the private key lives (an owner computer, meaning the own computer of Hamid or Saber, kept offline between uses, or a hardware token; never a shared, CI or server machine, the assistant's environment or the repository, rule 10). 2) Write docs/process/KEY_MANAGEMENT.md without any secret: who holds the key, two encrypted backups in separate places, rotation schedule, what to do if it leaks. 3) Create the key pair under that procedure and commit only the public key for the verifier (#101).</t>
         </is>
       </c>
       <c r="J108" s="8" t="inlineStr">
         <is>
-          <t>Done when: the procedure is approved and followed; the public key is in the repository; a test signature verifies; the private key is not on any development machine.</t>
+          <t>Done when: the procedure is approved and followed; the public key is in the repository; a test signature verifies; the private key is only on the owner computers and nowhere else (not in the repository, CI, a shared server or the assistant's environment).</t>
         </is>
       </c>
       <c r="K108" s="8" t="n"/>
@@ -42133,12 +42134,12 @@
       </c>
       <c r="I344" s="8" t="inlineStr">
         <is>
-          <t>Write docs/design/ADMIN_RESET.md (no secrets). Flow (same shape as licence activation, all in the browser UI; no terminal or CLI step): 1) the customer opens the administrator recovery page on their installation and downloads a reset request file (.pemsrstreq: Install ID, fingerprint hash, licence id, product version, account, random nonce kept server-side as a pending request, signed by the install key); 2) the customer sends the file to us; 3) in the developer/owner UI we upload it, the tool verifies the signature, matches it to the customer and licence in the ledger, we confirm the customer, enter the reason and the identity check, and download a reset response file (.pemsreset) signed with the separate reset key and bound to the request nonce, licence id, Install ID, purpose and expiry; 4) the customer uploads the response file on the same page and the password reset form opens; the pending request is consumed so the file works once. Decide: reset-key custody and where it may live (on the owner's local computer or the assistant's computer, never the licence key), what the reset changes (password; MFA/passkeys and sessions as in the shared recovery rules), expiry of the response file, rate limits, audit on both sides, behaviour on a cloned or re-hosted machine (#104, #116). AFTA check (to be confirmed with the testing lab through #184): no default, master or hard-coded password and no standing vendor credential; the vendor can act only on a request that the installation itself generated, for one installation, once and for a short time; the capability is off by default and enabled explicitly by the customer administrator; every use is audited, all administrators are notified, the account sessions are revoked and the event goes to the SIEM feed; the reset key is separate from the licence key and can be revoked through an update; everything works offline by file exchange, so no remote access to the customer server is ever needed. Validity: the response file expires after a period the owner chooses in the developer UI when the file is issued: default 1 day, allowed range 1 to 7 days in whole days, and no unlimited or open-ended option (the tool refuses values outside the range and the product checks the limits again, so a correctly signed file with a longer validity is rejected). The pending reset request on the customer side expires on the same bounds. AFTA: a short, bounded, single-use validity fits the check recorded here; the 1-day default and the 7-day maximum are to be confirmed with the testing lab (#184), and if the lab wants a shorter maximum the limits change in one setting without changing the file format.</t>
+          <t>Write docs/design/ADMIN_RESET.md (no secrets). Flow (same shape as licence activation, all in the browser UI; no terminal or CLI step): 1) the customer opens the administrator recovery page on their installation and downloads a reset request file (.pemsrstreq: Install ID, fingerprint hash, licence id, product version, account, random nonce kept server-side as a pending request, signed by the install key); 2) the customer sends the file to us; 3) in the developer/owner UI we upload it, the tool verifies the signature, matches it to the customer and licence in the ledger, we confirm the customer, enter the reason and the identity check, and download a reset response file (.pemsreset) signed with the separate reset key and bound to the request nonce, licence id, Install ID, purpose and expiry; 4) the customer uploads the response file on the same page and the password reset form opens; the pending request is consumed so the file works once. Decide: reset-key custody. Decided 2026-10-25 by the owners: the licence key and the reset key are each created and used only on the owner computers (the own computers of Hamid and Saber, who are the owners and the developers; also called developer-local or owner machines), as the last step of the licence and reset flows. Neither key is ever in the assistant's environment, on a shared or CI server, or in the repository. The reset key is still a different key from the licence key. To settle in the ADR: whether the keys stay offline (encrypted external drive) between uses, where the backup copies are and who holds them, what the reset changes (password; MFA/passkeys and sessions as in the shared recovery rules), expiry of the response file, rate limits, audit on both sides, behaviour on a cloned or re-hosted machine (#104, #116). AFTA check (to be confirmed with the testing lab through #184): no default, master or hard-coded password and no standing vendor credential; the vendor can act only on a request that the installation itself generated, for one installation, once and for a short time; the capability is off by default and enabled explicitly by the customer administrator; every use is audited, all administrators are notified, the account sessions are revoked and the event goes to the SIEM feed; the reset key is separate from the licence key and can be revoked through an update; everything works offline by file exchange, so no remote access to the customer server is ever needed. Validity: the response file expires after a period the owner chooses in the developer UI when the file is issued: default 1 day, allowed range 1 to 7 days in whole days, and no unlimited or open-ended option (the tool refuses values outside the range and the product checks the limits again, so a correctly signed file with a longer validity is rejected). The pending reset request on the customer side expires on the same bounds. AFTA: a short, bounded, single-use validity fits the check recorded here; the 1-day default and the 7-day maximum are to be confirmed with the testing lab (#184), and if the lab wants a shorter maximum the limits change in one setting without changing the file format.</t>
         </is>
       </c>
       <c r="J344" s="8" t="inlineStr">
         <is>
-          <t>Done when: an approved ADR with the file formats' fields, the key-custody decision, the threat model (replay, wrong customer, tampered or forged file, cloned machine, clock change, leaked file) and a written AFTA compatibility assessment accepted by the security consultant; #344-#349 are written against it. The validity rule (default 1 day, range 1 to 7 days, no unlimited option) is confirmed by the AFTA assessment.</t>
+          <t>Done when: an approved ADR with the file formats' fields, the key-custody details on the owner computers, the threat model (replay, wrong customer, tampered or forged file, cloned machine, clock change, leaked file) and a written AFTA compatibility assessment accepted by the security consultant; #344-#349 are written against it. The validity rule (default 1 day, range 1 to 7 days, no unlimited option) is confirmed by the AFTA assessment.</t>
         </is>
       </c>
       <c r="K344" s="8" t="n"/>
@@ -42303,7 +42304,7 @@
       </c>
       <c r="I346" s="8" t="inlineStr">
         <is>
-          <t>Add a Reset admin page to the vendor tool (#106), run on the owner's local computer: upload the .pemsrstreq, verify its signature, find the matching licence in the ledger (#341) by licence id, Install ID and fingerprint hash, show the customer and let the owner confirm or pick the customer (a mismatch is a warning that blocks issuing), enter the reason and the identity check performed, choose the validity in whole days (default 1, range 1 to 7, no unlimited option), then download the .pemsreset built with #344 and signed with the reset key (#349). Revoked or expired licences cannot be answered. Write an audit entry (who, when, customer, licence, request nonce, expiry, reason). Works fully offline. All in the UI; no terminal or CLI step.</t>
+          <t>Add a Reset admin page to the vendor tool (#106), run on an owner computer (Hamid's or Saber's own computer, where the reset key lives): upload the .pemsrstreq, verify its signature, find the matching licence in the ledger (#341) by licence id, Install ID and fingerprint hash, show the customer and let the owner confirm or pick the customer (a mismatch is a warning that blocks issuing), enter the reason and the identity check performed, choose the validity in whole days (default 1, range 1 to 7, no unlimited option), then download the .pemsreset built with #344 and signed with the reset key (#349). Revoked or expired licences cannot be answered. Write an audit entry (who, when, customer, licence, request nonce, expiry, reason). Works fully offline. All in the UI; no terminal or CLI step.</t>
         </is>
       </c>
       <c r="J346" s="8" t="inlineStr">
@@ -42643,7 +42644,7 @@
       </c>
       <c r="I350" s="8" t="inlineStr">
         <is>
-          <t>1) Generate a separate reset key pair offline (Ed25519 recommended) and record its key id; the public key is embedded in the product with the key id, the private key lives on the owner's offline or local machine, never in the repository or on a shared server. 2) Decide in the ADR (#343) whether the assistant's computer may hold it. 3) Write docs/process/RESET_KEY_MANAGEMENT.md without secrets: holders, encrypted backups, rotation, how a revoked key id is delivered to installations through an update (#117), and the compromise plan. 4) Perform the ceremony and record who attended.</t>
+          <t>1) Generate a separate reset key pair offline (Ed25519 recommended) and record its key id; the public key is embedded in the product with the key id, the private key lives only on the owner computers (Hamid's and Saber's own), never in the repository, on a shared or CI server or in the assistant's environment. 2) Custody is decided: the key is created and used only on the owner computers; the ADR (#343) records the details (offline storage between uses, backup holders). 3) Write docs/process/RESET_KEY_MANAGEMENT.md without secrets: holders, encrypted backups, rotation, how a revoked key id is delivered to installations through an update (#117), and the compromise plan. 4) Perform the ceremony and record who attended (Hamid and Saber).</t>
         </is>
       </c>
       <c r="J350" s="8" t="inlineStr">

</xml_diff>

<commit_message>
SCRUM-367 docs(guidelines): development guideline for developers and AI agents
Add docs/guidelines (lifecycle, engineering standards, UI/components, libraries and research,
platform direction, environment, knowledge maintenance, learnings log) and AGENTS.md as entry point.
Enforcement: CLAUDE.md, PR template checkboxes, plan-sync Step 0 line. Two levels of done
(In Review = PR opened, Done = merged). .claude/CLAUDE.md is now a pointer (old directive moved to
docs/cmms), graphify hook path is portable. Plan row #350 added and backlog.csv regenerated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -11355,7 +11355,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -11774,7 +11773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U350"/>
+  <dimension ref="A1:U351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -42687,6 +42686,87 @@
       </c>
       <c r="T350" s="10" t="n"/>
       <c r="U350" s="10" t="n"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="10" t="n">
+        <v>350</v>
+      </c>
+      <c r="B351" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C351" s="8" t="inlineStr">
+        <is>
+          <t>Support, Operations &amp; Documentation</t>
+        </is>
+      </c>
+      <c r="D351" s="8" t="inlineStr">
+        <is>
+          <t>Development guideline for developers and AI agents (docs/guidelines, AGENTS.md) and enforcement layers</t>
+        </is>
+      </c>
+      <c r="E351" s="10" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="F351" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G351" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H351" s="8" t="inlineStr">
+        <is>
+          <t>Rules, preferences and conventions were spread over the Instructions sheet, README, .claude/CLAUDE.md and per-person agent memory, so other developers' AI agents could not see them.</t>
+        </is>
+      </c>
+      <c r="I351" s="8" t="inlineStr">
+        <is>
+          <t>Create docs/guidelines (task lifecycle, engineering standards, UI and components, libraries and research, platform direction, environment, knowledge maintenance, learnings log) with AGENTS.md as the entry point; add enforcement through CLAUDE.md, the pull request template and the tracker description line; bulk-update existing issues; two levels of done (In Review, Done).</t>
+        </is>
+      </c>
+      <c r="J351" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the guideline files exist in English and are merged; AGENTS.md and CLAUDE.md point to them; the PR template and plan-sync carry the checks; every existing issue carries the Step 0 line.</t>
+        </is>
+      </c>
+      <c r="K351" s="8" t="n"/>
+      <c r="L351" s="10" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="M351" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N351" s="10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O351" s="10" t="n"/>
+      <c r="P351" s="10" t="n"/>
+      <c r="Q351" s="10" t="n"/>
+      <c r="R351" s="8" t="inlineStr">
+        <is>
+          <t>Process &amp; documentation</t>
+        </is>
+      </c>
+      <c r="S351" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T351" s="10" t="n"/>
+      <c r="U351" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-368 ci: pipelines only on demo and staging, staging environment, deployment README
Reusable deploy-site.yml with thin demo/staging callers, build.yml manual only, env/staging files,
docs/deployment/DEPLOYMENT_README.md, plan rows #351-#353 (SCRUM-368..370).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -11773,7 +11773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U351"/>
+  <dimension ref="A1:U354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -42767,6 +42767,261 @@
       </c>
       <c r="T351" s="10" t="n"/>
       <c r="U351" s="10" t="n"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="10" t="n">
+        <v>351</v>
+      </c>
+      <c r="B352" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C352" s="8" t="inlineStr">
+        <is>
+          <t>DevOps, Source Control &amp; Release Management</t>
+        </is>
+      </c>
+      <c r="D352" s="8" t="inlineStr">
+        <is>
+          <t>CI and branch policy: pipelines run only on pushes to demo and staging (none on main or working branches), staging environment and subdomain, deployment README, dev branch retired</t>
+        </is>
+      </c>
+      <c r="E352" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F352" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G352" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H352" s="8" t="inlineStr">
+        <is>
+          <t>build.yml ran on every push and pull request to main/develop; there was no staging pipeline or environment; deployment steps (subdomains, databases, secrets, Actions, manual deploy and reset) were not written down in one place.</t>
+        </is>
+      </c>
+      <c r="I352" s="8" t="inlineStr">
+        <is>
+          <t>1) Make build.yml manual only; no workflow triggers on main or working branches. 2) Turn the demo pipeline into one reusable deploy workflow used by deploy-demo.yml (push to demo) and deploy-staging.yml (push to staging), secrets named DEMO_* and STAGING_*. 3) Add env/staging.env and its secrets example, keep every env file key-identical. 4) Create the staging branch from main, dev and demo. 5) Write docs/deployment/DEPLOYMENT_README.md (subdomains, databases, secrets, Actions, manual deploy and manual reset). 6) Merge dev into main and remove dev.</t>
+        </is>
+      </c>
+      <c r="J352" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a push to main or to a working branch starts no workflow; a push to demo deploys the demo subdomain and a push to staging deploys the staging subdomain; the README lets a new person set up both environments; the staging branch contains main, dev and demo; dev no longer exists.</t>
+        </is>
+      </c>
+      <c r="K352" s="8" t="n"/>
+      <c r="L352" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M352" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N352" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O352" s="10" t="inlineStr">
+        <is>
+          <t>#295</t>
+        </is>
+      </c>
+      <c r="P352" s="10" t="n"/>
+      <c r="Q352" s="10" t="n"/>
+      <c r="R352" s="8" t="inlineStr">
+        <is>
+          <t>DevOps &amp; release</t>
+        </is>
+      </c>
+      <c r="S352" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T352" s="10" t="n"/>
+      <c r="U352" s="10" t="n"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="10" t="n">
+        <v>352</v>
+      </c>
+      <c r="B353" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C353" s="8" t="inlineStr">
+        <is>
+          <t>Online Demo</t>
+        </is>
+      </c>
+      <c r="D353" s="8" t="inlineStr">
+        <is>
+          <t>Environment data package: export the current database as a versioned, hashed, importable package and import it from the admin UI (with the existing Excel importers alongside), role-protected</t>
+        </is>
+      </c>
+      <c r="E353" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F353" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G353" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H353" s="8" t="inlineStr">
+        <is>
+          <t>The application has no database export or import of its own data (only the Import Center for Excel files and the Database Update page for schema). Demo and staging need a repeatable way to capture and restore their data.</t>
+        </is>
+      </c>
+      <c r="I353" s="8" t="inlineStr">
+        <is>
+          <t>Design first (ADR): logical export of every user table to a package (.pemsdata, zip) with a manifest: format version, product version, last applied migration, schema fingerprint, per-table row counts and SHA-256, package hash; import = precheck (hash, format, schema compatibility) then replace. Admin UI page for the proper role/permission only; the same page links to the Import Center for Excel imports. Disabled by setting outside demo/staging unless the owner enables it. Audit every export and import.</t>
+        </is>
+      </c>
+      <c r="J353" s="8" t="inlineStr">
+        <is>
+          <t>Done when: an authorised administrator exports a package from the UI and re-imports it into an empty or existing database of the same version; a tampered or incompatible package is rejected with the reason; every action is audited; tests cover precheck, hash, round trip and the permission.</t>
+        </is>
+      </c>
+      <c r="K353" s="8" t="n"/>
+      <c r="L353" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M353" s="10" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="N353" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O353" s="10" t="inlineStr">
+        <is>
+          <t>#310 #245</t>
+        </is>
+      </c>
+      <c r="P353" s="10" t="n"/>
+      <c r="Q353" s="10" t="n"/>
+      <c r="R353" s="8" t="inlineStr">
+        <is>
+          <t>Online demo</t>
+        </is>
+      </c>
+      <c r="S353" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T353" s="10" t="n"/>
+      <c r="U353" s="10" t="n"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="10" t="n">
+        <v>353</v>
+      </c>
+      <c r="B354" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C354" s="8" t="inlineStr">
+        <is>
+          <t>Online Demo</t>
+        </is>
+      </c>
+      <c r="D354" s="8" t="inlineStr">
+        <is>
+          <t>Reset on deploy for demo and staging: a baseline data package shipped with the branch is applied after a version-compatibility precheck, from the UI or automatically when a new baseline arrives</t>
+        </is>
+      </c>
+      <c r="E354" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F354" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G354" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H354" s="8" t="inlineStr">
+        <is>
+          <t>Row #141 asks for a nightly and an admin reset but nothing exists; a push to demo or staging updates code and schema only, data is never reset.</t>
+        </is>
+      </c>
+      <c r="I354" s="8" t="inlineStr">
+        <is>
+          <t>Use the package from #352. A baseline package committed to the demo/staging overlay is uploaded by the pipeline; on first start after deploy the app compares the baseline hash with the one recorded in the database, runs the precheck and, if it passes and the environment setting allows it, resets the database to the baseline; otherwise it reports why in the admin UI. Admin UI offers the same reset by upload. Owners and developers only.</t>
+        </is>
+      </c>
+      <c r="J354" s="8" t="inlineStr">
+        <is>
+          <t>Done when: pushing a new baseline to demo (and to staging) resets that environment once; an incompatible baseline leaves data untouched and shows the reason; a manual reset by upload works in the UI; tests cover both paths.</t>
+        </is>
+      </c>
+      <c r="K354" s="8" t="n"/>
+      <c r="L354" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M354" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N354" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O354" s="10" t="inlineStr">
+        <is>
+          <t>#352 #141</t>
+        </is>
+      </c>
+      <c r="P354" s="10" t="n"/>
+      <c r="Q354" s="10" t="n"/>
+      <c r="R354" s="8" t="inlineStr">
+        <is>
+          <t>Online demo</t>
+        </is>
+      </c>
+      <c r="S354" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T354" s="10" t="n"/>
+      <c r="U354" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-371 plan: add row #354 (migrations assembly)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -11773,7 +11773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U354"/>
+  <dimension ref="A1:U355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -43022,6 +43022,91 @@
       </c>
       <c r="T354" s="10" t="n"/>
       <c r="U354" s="10" t="n"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="10" t="n">
+        <v>354</v>
+      </c>
+      <c r="B355" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C355" s="8" t="inlineStr">
+        <is>
+          <t>DevOps, Source Control &amp; Release Management</t>
+        </is>
+      </c>
+      <c r="D355" s="8" t="inlineStr">
+        <is>
+          <t>Move the EF Core migrations into their own assembly (PEMS.Migrations) so PEMS.Persistence.dll changes, and is deployed, only when its own code changes</t>
+        </is>
+      </c>
+      <c r="E355" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F355" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G355" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H355" s="8" t="inlineStr">
+        <is>
+          <t>PEMS.Persistence.dll is 29 MB, mostly ~120 migrations with their designers and the model snapshot, so every change to a data-layer service re-uploads all of it to demo and staging (difference upload).</t>
+        </is>
+      </c>
+      <c r="I355" s="8" t="inlineStr">
+        <is>
+          <t>Follow the EF Core guidance for a separate migrations project: new project PEMS.Migrations (references PEMS.Persistence) holds the migration files, the snapshot and the design-time factory; the context defaults its MigrationsAssembly to it so hosts, tests and tools find the migrations; Web and Tests reference the project; update the CI drift gate, deploy script, Dockerfile, solution and every documented dotnet ef command.</t>
+        </is>
+      </c>
+      <c r="J355" s="8" t="inlineStr">
+        <is>
+          <t>Done when: dotnet build and the migration/deployment tests pass; the drift gate runs with --project PEMS.Migrations; PEMS.Persistence.dll no longer contains migrations and a change in a Persistence service leaves PEMS.Migrations.dll byte-identical; docs and guideline use the new command.</t>
+        </is>
+      </c>
+      <c r="K355" s="8" t="n"/>
+      <c r="L355" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M355" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N355" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O355" s="10" t="inlineStr">
+        <is>
+          <t>#351</t>
+        </is>
+      </c>
+      <c r="P355" s="10" t="n"/>
+      <c r="Q355" s="10" t="n"/>
+      <c r="R355" s="8" t="inlineStr">
+        <is>
+          <t>DevOps &amp; release</t>
+        </is>
+      </c>
+      <c r="S355" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T355" s="10" t="n"/>
+      <c r="U355" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-371 refactor: EF migrations in their own assembly (PEMS.Migrations)
PEMS.Persistence.dll 29 -> 6 MB; PEMS.Migrations.dll stays byte-identical when only data-layer code changes.
Context defaults MigrationsAssembly; Web/Tests reference the project; drift gate, deploy script, Dockerfile, docs updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1576,7 +1576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3092,6 +3092,53 @@
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Export and check verified on the workbook; the issue tracker side not set up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>SM-33</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Schema migrations deployed separately from the data layer</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>PEMS.Migrations / PEMS.Persistence</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Migrations, snapshot and design-time factory live in PEMS.Migrations; a data-layer-only change leaves PEMS.Migrations.dll byte-identical (build with DebugType=none), so the difference upload skips it</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H37" s="10" t="inlineStr">
+        <is>
+          <t>#354 #351</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>Add a migration with the --project PEMS.Migrations option. Verified 2026-10-25: Persistence 29 MB -&gt; 6 MB, Migrations 23 MB.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SCRUM-372 plan: add field validation tasks #355-#365 (SCRUM-372..382)
Catalog, server engine, client shaping and accessibility, file validation, static-module audit, import/bulk, parity tests,
statistics hints, RFC 9457 error contract, canonicalisation and limits, standards-based and local validators.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -11820,7 +11820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U355"/>
+  <dimension ref="A1:U366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -43154,6 +43154,969 @@
       </c>
       <c r="T355" s="10" t="n"/>
       <c r="U355" s="10" t="n"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="10" t="n">
+        <v>355</v>
+      </c>
+      <c r="B356" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C356" s="8" t="inlineStr">
+        <is>
+          <t>Metadata Core &amp; Dynamic Platform</t>
+        </is>
+      </c>
+      <c r="D356" s="8" t="inlineStr">
+        <is>
+          <t>Field validation catalog: for every field type the constraints (required, range, length, decimals, size, count, pattern, date window, membership, uniqueness), their defaults, hard versus advisory, and the stored validation object</t>
+        </is>
+      </c>
+      <c r="E356" s="10" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="F356" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G356" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H356" s="8" t="inlineStr">
+        <is>
+          <t>Validation in PEMS today is thin and scattered: 260 entities but only 26 [Required] and 45 [MaxLength] attributes in 28 files, no [Range], [StringLength] or regular-expression rule anywhere, no validation library, ModelState.IsValid is checked in 8 controllers, and 64 of 65 plain text inputs in the views have no maxlength. Dynamic forms need one declarative description of the rules per field type before any engine or UI is built. Rule-builder row #46 covers user-defined rules; this row defines the built-in constraints every type carries.</t>
+        </is>
+      </c>
+      <c r="I356" s="8" t="inlineStr">
+        <is>
+          <t>1) For every type in #11 list its constraints. Text: required, min/max length, pattern (named presets: code, e-mail, phone, national id), allowed characters, allow digits. Number/decimal/money: min, max, strict range, step, integer only, allow negative, allow zero, scale and precision. Date/date-time: min/max date, relative window (not in the past, not in the future, within N days), Jalali-aware, time zone. Boolean: must be true. Select/multi-select: membership, min/max selected. Lookup/user: existence, active only, scope. File/image: max size per file and in total, count, extensions, MIME, dimensions. Rich text: max length of the text after sanitisation. JSON: schema. Computed/auto-number: read-only. 2) For each constraint: default, hard (blocks the save) or advisory (hint only), message key (fa/en) and parameters. 3) Define the versioned validation object stored in the metadata registry and which constraints the physical column must also enforce (length, precision, scale) so metadata and storage cannot disagree. 4) Cross-field and semantic rules (end after start, total equals sum) use the rule builder of #46 and the expression engine of #15. 5) Persian/Arabic digit normalisation and decimal separator rules (see #364). 6) Write docs/architecture/FIELD_VALIDATION_CATALOG.md and an ADR. Best-practice sources to apply: OWASP Input Validation Cheat Sheet (allowlist, syntactic and semantic checks, server-side authority, canonicalisation, limits before parsing, safe regular expressions); Microsoft Learn ASP.NET Core model validation; WCAG 2.2 success criteria 3.3.1 and 3.3.3; RFC 9457 problem details.</t>
+        </is>
+      </c>
+      <c r="J356" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the catalog lists every field type of #11 with its constraints, defaults, hard or advisory flag and message keys; the rule that derives column size and precision from the constraints is decided; the PM reviewed it; rows #356-#365 reference it.</t>
+        </is>
+      </c>
+      <c r="K356" s="8" t="n"/>
+      <c r="L356" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M356" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N356" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O356" s="10" t="inlineStr">
+        <is>
+          <t>#11 #338 #46</t>
+        </is>
+      </c>
+      <c r="P356" s="10" t="inlineStr">
+        <is>
+          <t>#10 #11 #12</t>
+        </is>
+      </c>
+      <c r="Q356" s="10" t="n"/>
+      <c r="R356" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic data core</t>
+        </is>
+      </c>
+      <c r="S356" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T356" s="10" t="n"/>
+      <c r="U356" s="10" t="n"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="10" t="n">
+        <v>356</v>
+      </c>
+      <c r="B357" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C357" s="8" t="inlineStr">
+        <is>
+          <t>Metadata Core &amp; Dynamic Platform</t>
+        </is>
+      </c>
+      <c r="D357" s="8" t="inlineStr">
+        <is>
+          <t>Server-side validation engine: one type-dispatched validator used by every write path (forms, API, import, bulk, static modules), full list of field errors, create versus partial-update modes, localised messages</t>
+        </is>
+      </c>
+      <c r="E357" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F357" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G357" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H357" s="8" t="inlineStr">
+        <is>
+          <t>A direct API call, an import or a bulk write bypasses whatever the page checks, and PEMS has no single validator to call. Validation must be authoritative on the server; the client only improves feedback.</t>
+        </is>
+      </c>
+      <c r="I357" s="8" t="inlineStr">
+        <is>
+          <t>1) Check libraries first (FluentValidation, JSON-schema validators) and record the licence in row L_OSS; custom code only with a stated reason. 2) Implement a validator in the engine layer with a dispatch table by field type (a new constraint is a new case, never a second parallel function): input = field descriptors + record + mode; create requires every required field, update checks only the keys present so an omitted key never means 'clear it'. Whitespace-only text counts as empty for required. 3) Return all violations (field, constraint code, message key, parameters), not only the first, capped by a setting (ASP.NET Core defaults to 200 errors and depth 32; set explicit limits). 4) Call it from one place in the generic CRUD pipeline and from static modules through an adapter (DataAnnotations and IValidatableObject keep working). 5) Messages resolved through the localisation resources (fa/en). 6) Validation never replaces authorisation, parameterised queries, output encoding or HTML sanitisation (OWASP). 7) Unit tests per type and constraint. Best-practice sources to apply: OWASP Input Validation Cheat Sheet (allowlist, syntactic and semantic checks, server-side authority, canonicalisation, limits before parsing, safe regular expressions); Microsoft Learn ASP.NET Core model validation; WCAG 2.2 success criteria 3.3.1 and 3.3.3; RFC 9457 problem details.</t>
+        </is>
+      </c>
+      <c r="J357" s="8" t="inlineStr">
+        <is>
+          <t>Done when: every write path of the generic engine calls the validator; a request that bypasses the UI is rejected with the full error list; partial updates never clear omitted fields; messages come in the user's language; the error and depth limits are settings; tests cover each type.</t>
+        </is>
+      </c>
+      <c r="K357" s="8" t="n"/>
+      <c r="L357" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M357" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N357" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O357" s="10" t="inlineStr">
+        <is>
+          <t>#355 #15</t>
+        </is>
+      </c>
+      <c r="P357" s="10" t="inlineStr">
+        <is>
+          <t>#10 #11 #12</t>
+        </is>
+      </c>
+      <c r="Q357" s="10" t="n"/>
+      <c r="R357" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic data core</t>
+        </is>
+      </c>
+      <c r="S357" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T357" s="10" t="n"/>
+      <c r="U357" s="10" t="n"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="10" t="n">
+        <v>357</v>
+      </c>
+      <c r="B358" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C358" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D358" s="8" t="inlineStr">
+        <is>
+          <t>Client input shaping and accessible inline validation from the same constraint descriptor: maxlength/min/max/step/pattern attributes, keystroke sanitising (Persian digits, decimals, thousands separators, RTL), counters, error text with suggestion, focus first error, advisory hints</t>
+        </is>
+      </c>
+      <c r="E358" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F358" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G358" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H358" s="8" t="inlineStr">
+        <is>
+          <t>Text and number inputs are hand-written per page (2,587 hand-written inputs in the audit) and carry no constraints. The component library needs one way to turn the constraint descriptor into HTML attributes, typing behaviour and accessible error messages.</t>
+        </is>
+      </c>
+      <c r="I358" s="8" t="inlineStr">
+        <is>
+          <t>1) The field components of #322 render the descriptor into HTML attributes (maxlength, min, max, step, pattern, accept, inputmode). 2) A small shared script shapes typing only (not a replacement for validation): normalise Persian/Arabic digits to ASCII, keep one decimal separator, cut decimals to the scale, show thousands separators without breaking RTL caret movement, strip disallowed characters. 3) Errors follow WCAG 2.2: text that identifies the field and says how to fix it (3.3.1, 3.3.3), not colour alone, aria-invalid on the field, message linked with aria-describedby, a summary with role alert, focus moved to the first invalid field. 4) Character counter and non-blocking hints. 5) No per-page script. 6) One shared JSON fixture file is run through the server validator and the script so both agree (parity test, see #361). Best-practice sources to apply: OWASP Input Validation Cheat Sheet (allowlist, syntactic and semantic checks, server-side authority, canonicalisation, limits before parsing, safe regular expressions); Microsoft Learn ASP.NET Core model validation; WCAG 2.2 success criteria 3.3.1 and 3.3.3; RFC 9457 problem details.</t>
+        </is>
+      </c>
+      <c r="J358" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a field built from metadata shows the right attributes and shapes typing for every type in the catalog; error text, aria attributes and focus pass an automated accessibility check (axe) and a screen-reader spot check; the parity fixtures pass on server and script; works in RTL and LTR.</t>
+        </is>
+      </c>
+      <c r="K358" s="8" t="n"/>
+      <c r="L358" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M358" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N358" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O358" s="10" t="inlineStr">
+        <is>
+          <t>#322 #356</t>
+        </is>
+      </c>
+      <c r="P358" s="10" t="inlineStr">
+        <is>
+          <t>#10 #11</t>
+        </is>
+      </c>
+      <c r="Q358" s="10" t="n"/>
+      <c r="R358" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S358" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T358" s="10" t="n"/>
+      <c r="U358" s="10" t="n"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="10" t="n">
+        <v>358</v>
+      </c>
+      <c r="B359" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C359" s="8" t="inlineStr">
+        <is>
+          <t>Access, RLS, Sessions &amp; Security</t>
+        </is>
+      </c>
+      <c r="D359" s="8" t="inlineStr">
+        <is>
+          <t>File and media field validation: per-field limits for size, total size, count, extensions, MIME with content check and image dimensions, aligned with the host request limit</t>
+        </is>
+      </c>
+      <c r="E359" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F359" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G359" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H359" s="8" t="inlineStr">
+        <is>
+          <t>Request-size limits exist in 7 files without one source of truth, so the page, the application and the web host can disagree about the allowed size and the user sees a server error instead of a message. OWASP: treat file names and content types as untrusted; an allowed extension does not prove safe content.</t>
+        </is>
+      </c>
+      <c r="I359" s="8" t="inlineStr">
+        <is>
+          <t>1) Per-field settings: max size per file, max total size, max count, extension allowlist, MIME allowlist, image min/max width and height. 2) Server check on the upload pipeline of #183: size while streaming, extension, MIME and magic bytes (never trust the browser MIME), image dimensions, safe stored file name. 3) Derive the Kestrel/IIS request limit from the largest configured field limit (one setting in env/*.env) and show the same limit in the UI before upload. 4) Clear localised messages. 5) Per-entity or per-user quota hook.</t>
+        </is>
+      </c>
+      <c r="J359" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a file over the limit, with a wrong extension or a mismatching content type is rejected with a clear message at the UI and at the server; the host limit follows the setting; tests cover size boundary, wrong extension and a renamed file.</t>
+        </is>
+      </c>
+      <c r="K359" s="8" t="n"/>
+      <c r="L359" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M359" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N359" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O359" s="10" t="inlineStr">
+        <is>
+          <t>#183 #355</t>
+        </is>
+      </c>
+      <c r="P359" s="10" t="n"/>
+      <c r="Q359" s="10" t="n"/>
+      <c r="R359" s="8" t="inlineStr">
+        <is>
+          <t>Security &amp; access</t>
+        </is>
+      </c>
+      <c r="S359" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T359" s="10" t="n"/>
+      <c r="U359" s="10" t="n"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="10" t="n">
+        <v>359</v>
+      </c>
+      <c r="B360" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C360" s="8" t="inlineStr">
+        <is>
+          <t>Quality, Testing &amp; Performance</t>
+        </is>
+      </c>
+      <c r="D360" s="8" t="inlineStr">
+        <is>
+          <t>Audit and harden validation of the existing static modules: string lengths, decimal precision and scale, numeric ranges, controllers without model validation, inputs without constraints, with a CI ratchet</t>
+        </is>
+      </c>
+      <c r="E360" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F360" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G360" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H360" s="8" t="inlineStr">
+        <is>
+          <t>Validation in PEMS today is thin and scattered: 260 entities but only 26 [Required] and 45 [MaxLength] attributes in 28 files, no [Range], [StringLength] or regular-expression rule anywhere, no validation library, ModelState.IsValid is checked in 8 controllers, and 64 of 65 plain text inputs in the views have no maxlength. 136 decimal properties exist but only 110 precision mappings, and the application logs 'No store type was specified for the decimal property' at start (for example SparePart.QuantityOnHand, ReorderPoint, WorkOrder.DowntimeHours), which silently truncates values.</t>
+        </is>
+      </c>
+      <c r="I360" s="8" t="inlineStr">
+        <is>
+          <t>1) Write an audit script (extend tools/UiAudit or a test) listing: string properties without a maximum length or with nvarchar(max) that should be bounded; decimal properties without explicit precision and scale; numeric and date properties that need a range (quantities, percentages, years); controllers that write without ModelState or a validator; inputs in views without maxlength/min/max/step/inputmode. 2) Fix the highest-risk 30 first (money, quantities, identifiers, document numbers) with a migration where the column changes. 3) Add a test that fails when a new string property has no maximum length (unless marked unbounded) or a new decimal has no precision. 4) Report counts before and after in docs/audits.</t>
+        </is>
+      </c>
+      <c r="J360" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the audit report exists with counts; every decimal has explicit precision and the start-up warnings are gone; the 30 highest-risk fields are fixed; the ratchet test is in CI.</t>
+        </is>
+      </c>
+      <c r="K360" s="8" t="n"/>
+      <c r="L360" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M360" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N360" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O360" s="10" t="inlineStr">
+        <is>
+          <t>#355</t>
+        </is>
+      </c>
+      <c r="P360" s="10" t="inlineStr">
+        <is>
+          <t>#11</t>
+        </is>
+      </c>
+      <c r="Q360" s="10" t="n"/>
+      <c r="R360" s="8" t="inlineStr">
+        <is>
+          <t>Quality &amp; testing</t>
+        </is>
+      </c>
+      <c r="S360" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T360" s="10" t="n"/>
+      <c r="U360" s="10" t="n"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="10" t="n">
+        <v>360</v>
+      </c>
+      <c r="B361" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C361" s="8" t="inlineStr">
+        <is>
+          <t>Metadata Core &amp; Dynamic Platform</t>
+        </is>
+      </c>
+      <c r="D361" s="8" t="inlineStr">
+        <is>
+          <t>Import and bulk paths use the same validation: row-level error report, partial-update semantics, defaults never NULL, malformed identifiers rejected as validation errors, size and row limits</t>
+        </is>
+      </c>
+      <c r="E361" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F361" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G361" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H361" s="8" t="inlineStr">
+        <is>
+          <t>Import Center has 11 imports with their own checks. A blank cell in an update row must leave the value alone, a malformed identifier must never reach the database as a server error, and a default value must never be saved as NULL by a bulk path.</t>
+        </is>
+      </c>
+      <c r="I361" s="8" t="inlineStr">
+        <is>
+          <t>1) The import designer (#25) and the Import Center call the validator of #356 per row. 2) Row-level error report (row, column, message, value) and a preview before commit. 3) Update mode: a blank cell leaves the stored value unchanged and 'required' applies only to columns present in the file. 4) Omitted columns with a default get the default (links to #26). 5) Reject malformed GUIDs and numeric keys as validation errors. 6) Limits for file size, rows and columns as settings (OWASP: cap sizes before parsing). 7) Persian digits and Jalali dates normalised (#364). 8) Test with 50,000 rows and mixed errors.</t>
+        </is>
+      </c>
+      <c r="J361" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a 50,000-row file with errors produces a complete row-level report and commits nothing, or only the valid rows if the user chooses; partial updates never clear data; a malformed identifier gives a message, not a server error.</t>
+        </is>
+      </c>
+      <c r="K361" s="8" t="n"/>
+      <c r="L361" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M361" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N361" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O361" s="10" t="inlineStr">
+        <is>
+          <t>#356 #25</t>
+        </is>
+      </c>
+      <c r="P361" s="10" t="inlineStr">
+        <is>
+          <t>#13 #14 #243</t>
+        </is>
+      </c>
+      <c r="Q361" s="10" t="n"/>
+      <c r="R361" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic data core</t>
+        </is>
+      </c>
+      <c r="S361" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T361" s="10" t="n"/>
+      <c r="U361" s="10" t="n"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="10" t="n">
+        <v>361</v>
+      </c>
+      <c r="B362" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C362" s="8" t="inlineStr">
+        <is>
+          <t>Quality, Testing &amp; Performance</t>
+        </is>
+      </c>
+      <c r="D362" s="8" t="inlineStr">
+        <is>
+          <t>Validation test matrix and client/server parity suite: type by constraint by boundary, run on the server and in the browser script from the same fixtures</t>
+        </is>
+      </c>
+      <c r="E362" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F362" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G362" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H362" s="8" t="inlineStr">
+        <is>
+          <t>A rule that the page and the server interpret differently is worse than no rule. No automated check exists today that proves they agree.</t>
+        </is>
+      </c>
+      <c r="I362" s="8" t="inlineStr">
+        <is>
+          <t>1) Data-driven fixtures: for each type and constraint the values min-1, min, max, max+1, zero, negative zero, very large numbers, scale+1, empty versus null versus whitespace, Persian and Arabic digits, mixed scripts, RTL marks and zero-width characters, characters outside the BMP counted by length. 2) Server test runs every fixture through the validator. 3) A browser-script test runs the same file through the client interpreter. 4) API-level tests prove a request that skips the UI is rejected. 5) CI runs both.</t>
+        </is>
+      </c>
+      <c r="J362" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the fixture file is the single source of truth, server and script give identical results for every case, and a deliberately broken rule fails the build.</t>
+        </is>
+      </c>
+      <c r="K362" s="8" t="n"/>
+      <c r="L362" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M362" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N362" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O362" s="10" t="inlineStr">
+        <is>
+          <t>#356 #357</t>
+        </is>
+      </c>
+      <c r="P362" s="10" t="inlineStr">
+        <is>
+          <t>#20 #117</t>
+        </is>
+      </c>
+      <c r="Q362" s="10" t="n"/>
+      <c r="R362" s="8" t="inlineStr">
+        <is>
+          <t>Quality &amp; testing</t>
+        </is>
+      </c>
+      <c r="S362" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T362" s="10" t="n"/>
+      <c r="U362" s="10" t="n"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="10" t="n">
+        <v>362</v>
+      </c>
+      <c r="B363" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C363" s="8" t="inlineStr">
+        <is>
+          <t>Metadata Core &amp; Dynamic Platform</t>
+        </is>
+      </c>
+      <c r="D363" s="8" t="inlineStr">
+        <is>
+          <t>Field statistics endpoint and non-blocking hints: count, min, max, average, standard deviation and empty rate of a numeric field to suggest ranges in the designer and to flag unusual values on forms</t>
+        </is>
+      </c>
+      <c r="E363" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F363" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G363" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H363" s="8" t="inlineStr">
+        <is>
+          <t>Choosing sensible min and max values blind is error-prone; the real data of the field is the best suggestion. Advisory hints must never block a save.</t>
+        </is>
+      </c>
+      <c r="I363" s="8" t="inlineStr">
+        <is>
+          <t>1) Endpoint returning count, min, max, average, standard deviation and empty rate for one numeric field, filtered by the central row-level security (#178) and cached. 2) Form designer shows the figures next to the range inputs and offers 'use observed range'. 3) The form shows a non-blocking 'unusual value' hint when a value is far from the average in units of the standard deviation. 4) Setting to turn hints off per field.</t>
+        </is>
+      </c>
+      <c r="J363" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the designer shows live statistics and can fill the range; an unusual value shows a hint but saves; a user cannot see statistics of records they cannot access.</t>
+        </is>
+      </c>
+      <c r="K363" s="8" t="n"/>
+      <c r="L363" s="10" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="M363" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N363" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O363" s="10" t="inlineStr">
+        <is>
+          <t>#356</t>
+        </is>
+      </c>
+      <c r="P363" s="10" t="inlineStr">
+        <is>
+          <t>#10</t>
+        </is>
+      </c>
+      <c r="Q363" s="10" t="n"/>
+      <c r="R363" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic data core</t>
+        </is>
+      </c>
+      <c r="S363" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T363" s="10" t="n"/>
+      <c r="U363" s="10" t="n"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="10" t="n">
+        <v>363</v>
+      </c>
+      <c r="B364" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C364" s="8" t="inlineStr">
+        <is>
+          <t>Metadata Core &amp; Dynamic Platform</t>
+        </is>
+      </c>
+      <c r="D364" s="8" t="inlineStr">
+        <is>
+          <t>Validation error contract: RFC 9457 problem details with a list of field errors (pointer, constraint code, message key, parameters), the same shape for API, forms and import, with stable codes and error limits</t>
+        </is>
+      </c>
+      <c r="E364" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F364" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G364" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H364" s="8" t="inlineStr">
+        <is>
+          <t>Each module reports errors in its own way (a page summary, a thrown message, a flash text), so clients and the form components cannot render or test them uniformly. RFC 9457 defines application/problem+json and leaves the validation list to an extension member; ASP.NET Core can produce problem details natively.</t>
+        </is>
+      </c>
+      <c r="I364" s="8" t="inlineStr">
+        <is>
+          <t>1) Define the response: status 400 or 422, type, title, detail and an 'errors' array where each item has field (JSON pointer), constraint code (for example min, max, maxLength, pattern, required, notUnique), message key, parameters and the localised text. 2) Implement it once (AddProblemDetails and an exception/validation filter) and use it for the generic engine, the API and import. 3) Stable constraint codes documented in the catalog (#355) so UI and tests depend on codes, not on text. 4) Settings for the maximum number of errors and the maximum nesting depth. 5) The form components of #357 and the import report of #360 render this one shape. 6) Never leak internal details, stack traces or SQL in the response.</t>
+        </is>
+      </c>
+      <c r="J364" s="8" t="inlineStr">
+        <is>
+          <t>Done when: an invalid API call, form post and import row all return the same structured errors in the user's language; codes are stable and listed; a test fails if a module returns a different shape.</t>
+        </is>
+      </c>
+      <c r="K364" s="8" t="n"/>
+      <c r="L364" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M364" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N364" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O364" s="10" t="inlineStr">
+        <is>
+          <t>#356</t>
+        </is>
+      </c>
+      <c r="P364" s="10" t="n"/>
+      <c r="Q364" s="10" t="n"/>
+      <c r="R364" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic data core</t>
+        </is>
+      </c>
+      <c r="S364" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T364" s="10" t="n"/>
+      <c r="U364" s="10" t="n"/>
+    </row>
+    <row r="365">
+      <c r="A365" s="10" t="n">
+        <v>364</v>
+      </c>
+      <c r="B365" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C365" s="8" t="inlineStr">
+        <is>
+          <t>Metadata Core &amp; Dynamic Platform</t>
+        </is>
+      </c>
+      <c r="D365" s="8" t="inlineStr">
+        <is>
+          <t>Input canonicalisation and safe limits: one Unicode and Persian normalisation policy (digits, Arabic versus Persian letters, zero-width and bidi characters, trimming), whole-value regular expressions with timeout, and size/depth/count limits before parsing</t>
+        </is>
+      </c>
+      <c r="E365" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F365" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G365" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H365" s="8" t="inlineStr">
+        <is>
+          <t>Persian text arrives with Arabic Yeh/Kaf instead of the Persian letters, Persian or Arabic digits, zero-width non-joiners and invisible bidi marks; without one policy the same name or code is stored in several forms, breaks uniqueness and search, and length checks count characters differently. OWASP: validate the canonical form, apply one normalisation policy before validation, storage and comparison, cap sizes before parsing, avoid regular expressions prone to catastrophic backtracking, treat a timeout as a failure.</t>
+        </is>
+      </c>
+      <c r="I365" s="8" t="inlineStr">
+        <is>
+          <t>1) Write the policy in the catalog (#355): Unicode NFC, Arabic Yeh/Kaf to Persian Yeh/Kaf, digits to ASCII for numbers and codes (keep the display digits as a presentation setting), trim and collapse spaces, remove or reject zero-width and bidi control characters except the zero-width non-joiner inside Persian words, per-field switch for exceptions. 2) Implement one normaliser used by the validator (#356), the import (#360) and the search; store the normalised form for unique keys and keep the original for display where needed. 3) Regular expressions: whole-value match, bounded input length, match timeout (the .NET regex timeout parameter or a non-backtracking engine), a failed timeout is a rejection. 4) Limits as settings: request body size, JSON nesting depth, array length, string length before any parsing. 5) Tests with Persian samples, look-alike characters and a catastrophic-backtracking pattern.</t>
+        </is>
+      </c>
+      <c r="J365" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the same Persian text typed with Arabic or Persian letters and digits is stored and compared as one value; a pattern that would backtrack catastrophically is stopped by the timeout; oversized or too deeply nested input is rejected before parsing; tests prove each case.</t>
+        </is>
+      </c>
+      <c r="K365" s="8" t="n"/>
+      <c r="L365" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M365" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N365" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O365" s="10" t="inlineStr">
+        <is>
+          <t>#355</t>
+        </is>
+      </c>
+      <c r="P365" s="10" t="n"/>
+      <c r="Q365" s="10" t="n"/>
+      <c r="R365" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic data core</t>
+        </is>
+      </c>
+      <c r="S365" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T365" s="10" t="n"/>
+      <c r="U365" s="10" t="n"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="10" t="n">
+        <v>365</v>
+      </c>
+      <c r="B366" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C366" s="8" t="inlineStr">
+        <is>
+          <t>Metadata Core &amp; Dynamic Platform</t>
+        </is>
+      </c>
+      <c r="D366" s="8" t="inlineStr">
+        <is>
+          <t>Standards-based and local validators as a validator pack: e-mail and phone through maintained libraries, URL, Iranian national code, mobile number, postal code and IBAN (Sheba) checksum, valid Jalali dates, rial and toman scale</t>
+        </is>
+      </c>
+      <c r="E366" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F366" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G366" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H366" s="8" t="inlineStr">
+        <is>
+          <t>Hand-written patterns for e-mail, phone and identifiers are the usual source of false rejections and of values that look valid but are not. OWASP: use a maintained library for e-mail and verify mailbox ownership separately; the local market also needs checksum rules (national code, IBAN mod 97) and Jalali calendar validity.</t>
+        </is>
+      </c>
+      <c r="I366" s="8" t="inlineStr">
+        <is>
+          <t>1) Check libraries first and record their licences (e-mail: the framework mail address parser; phone: a maintained E.164 library; IBAN: ISO 13616 mod-97). 2) Implement the Iranian rules as validators: ten-digit national code with its check digit, mobile number with accepted prefixes and normalisation to one stored form, postal code, economic code, legal-entity id. 3) Jalali date validity including leap years and conversion to the stored Gregorian date. 4) Currency fields: rial and toman scale, no floating point, decimal(18,2) style precision from #355. 5) Package them as a validator pack loaded through the extension SDK (#94) so other locales can add theirs. 6) Message keys in fa/en. 7) Tests with real valid and invalid samples.</t>
+        </is>
+      </c>
+      <c r="J366" s="8" t="inlineStr">
+        <is>
+          <t>Done when: each validator accepts documented valid samples and rejects documented invalid ones, including checksum failures and non-existent Jalali dates; the pack loads through the extension point; e-mail and phone use a maintained library.</t>
+        </is>
+      </c>
+      <c r="K366" s="8" t="n"/>
+      <c r="L366" s="10" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="M366" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N366" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O366" s="10" t="inlineStr">
+        <is>
+          <t>#356 #94</t>
+        </is>
+      </c>
+      <c r="P366" s="10" t="n"/>
+      <c r="Q366" s="10" t="n"/>
+      <c r="R366" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic data core</t>
+        </is>
+      </c>
+      <c r="S366" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T366" s="10" t="n"/>
+      <c r="U366" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-383 plan: add field format tasks #366-#373 (SCRUM-383..390)
Format catalog (canonical/display/input, hierarchy, pipeline with validation), number and date engines, masked inputs,
label and text presentation, export parity, round-trip test matrix, format settings UI.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -11820,7 +11820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U366"/>
+  <dimension ref="A1:U374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -44117,6 +44117,714 @@
       </c>
       <c r="T366" s="10" t="n"/>
       <c r="U366" s="10" t="n"/>
+    </row>
+    <row r="367">
+      <c r="A367" s="10" t="n">
+        <v>366</v>
+      </c>
+      <c r="B367" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C367" s="8" t="inlineStr">
+        <is>
+          <t>Metadata Core &amp; Dynamic Platform</t>
+        </is>
+      </c>
+      <c r="D367" s="8" t="inlineStr">
+        <is>
+          <t>Field format catalog: canonical storage form, display format, input format and parse rules per field type, presets, the settings hierarchy (system, app, model, field, user), label, help, placeholder, unit and empty-value formats, and the pipeline order with validation</t>
+        </is>
+      </c>
+      <c r="E367" s="10" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="F367" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G367" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H367" s="8" t="inlineStr">
+        <is>
+          <t>Formatting in PEMS is done page by page: 377 hand-written date and time format strings in 138 views using 12 different patterns, 217 number format strings, 103 native date, 8 datetime-local and 137 number inputs whose look follows the browser locale, and Jalali support in only 6 files. Existing rows #24, #205, #206, #208 and #209 ask for translated labels, Persian digits, the Jalali calendar and fixed reports, but nothing defines where a field's format lives or how it relates to validation. A comparable implementation shows the risks: one hard-coded locale in its date component, date strings built without zero padding, an invalid-date defect in downloaded reports and a deprecated date library for the Jalali picker.</t>
+        </is>
+      </c>
+      <c r="I367" s="8" t="inlineStr">
+        <is>
+          <t>1) For each type in #11 define three things: the canonical value that is stored and exchanged (ISO 8601 date-only for dates, UTC instant for date-times, decimal with fixed scale for numbers and money, normalised text), the display format, and the input and parse format. 2) Presets with examples (date: Jalali long/short, Gregorian ISO; number: grouping, decimal separator, digit shapes Latin or Persian; currency: rial, toman, symbol position, negative style; percent; units; boolean: yes/no, tick; empty value: dash). 3) Where a format lives: a settings hierarchy system -&gt; app -&gt; model -&gt; field -&gt; user preference with a defined fallback (a model or field setting wins for content, the user's setting for chrome), stored in the metadata registry as a versioned format object next to the validation object. 4) Label-related formats: label, help, placeholder, error and option text as translatable strings (#24), unit and prefix/suffix, direction. 5) State the pipeline order and the rule that validation always runs on the canonical value. 6) Write docs/architecture/FIELD_FORMAT_CATALOG.md and an ADR. Design rule (decided here, applies to #355-#365): formats and validations are designed together in one field descriptor and one test suite, but kept as separate layers of one pipeline: raw input -&gt; parse by input format -&gt; canonical value -&gt; normalise (#364) -&gt; validate the canonical value (#355/#356) -&gt; store canonical -&gt; format for display. Validation never runs on a display string, and a display format never changes what is stored. Best-practice sources: W3C Internationalization (date and number formats follow the language context, avoid ambiguous numeric dates, support non-Gregorian calendars, keep localisation separate from translation); MDN notes on input type=number (locale separators and non-ASCII digits are sanitised, no pattern support, so formatted or Persian input needs type=text with inputmode); ISO 8601 for stored dates; Unicode CLDR through Intl (browser) and ICU/CultureInfo (server); OWASP: validate the canonical form, one normalisation policy.</t>
+        </is>
+      </c>
+      <c r="J367" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the catalog lists canonical, display and input format for every type of #11 with presets and examples; the hierarchy and fallback are decided; the pipeline order and the validate-canonical rule are written down and referenced by #355; the PM reviewed it; rows #367-#373 reference it.</t>
+        </is>
+      </c>
+      <c r="K367" s="8" t="n"/>
+      <c r="L367" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M367" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N367" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O367" s="10" t="inlineStr">
+        <is>
+          <t>#11 #355 #24 #205</t>
+        </is>
+      </c>
+      <c r="P367" s="10" t="inlineStr">
+        <is>
+          <t>#190 #179 #230</t>
+        </is>
+      </c>
+      <c r="Q367" s="10" t="n"/>
+      <c r="R367" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic data core</t>
+        </is>
+      </c>
+      <c r="S367" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T367" s="10" t="n"/>
+      <c r="U367" s="10" t="n"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="10" t="n">
+        <v>367</v>
+      </c>
+      <c r="B368" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C368" s="8" t="inlineStr">
+        <is>
+          <t>Persian Localization, RTL &amp; Jalali Calendar</t>
+        </is>
+      </c>
+      <c r="D368" s="8" t="inlineStr">
+        <is>
+          <t>Number, money, percent and unit formatting engine used by server and client: grouping, decimal separator, Persian or Latin digits, rial/toman scale, negative style, fixed rounding rule, tolerant parsing, no type=number for formatted values</t>
+        </is>
+      </c>
+      <c r="E368" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F368" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G368" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H368" s="8" t="inlineStr">
+        <is>
+          <t>Formatting in PEMS is done page by page: 377 hand-written date and time format strings in 138 views using 12 different patterns, 217 number format strings, 103 native date, 8 datetime-local and 137 number inputs whose look follows the browser locale, and Jalali support in only 6 files. Existing rows #24, #205, #206, #208 and #209 ask for translated labels, Persian digits, the Jalali calendar and fixed reports, but nothing defines where a field's format lives or how it relates to validation. Money and quantities are formatted with 217 scattered format strings; type=number inputs show locale-dependent separators and reject non-Latin digits (the browser empties the value), so Persian digit entry silently fails.</t>
+        </is>
+      </c>
+      <c r="I368" s="8" t="inlineStr">
+        <is>
+          <t>1) One formatting service on the server (CultureInfo/ICU through one wrapper) and one on the client (Intl.NumberFormat), both driven by the format object of #366, so the same value looks the same in views, grids, reports and exports. 2) Digit shapes (Persian or Latin) and separators as settings, with the display digits a presentation choice only. 3) Money: decimal arithmetic, scale from the field, one documented rounding rule (half away from zero unless a field says otherwise), rial and toman conversion by scale and never by floating point. 4) Tolerant parser used for typing, paste and import: accepts Persian and Arabic digits, both separator styles, grouping marks, a leading minus or parentheses, and returns the canonical decimal or a parse error. 5) Formatted inputs use type=text with inputmode and keep the raw value; type=number is not used for money or formatted values (MDN caveats). 6) Replace the page-level ToString format strings through the audit of #359 and a ratchet. Best-practice sources: W3C Internationalization (date and number formats follow the language context, avoid ambiguous numeric dates, support non-Gregorian calendars, keep localisation separate from translation); MDN notes on input type=number (locale separators and non-ASCII digits are sanitised, no pattern support, so formatted or Persian input needs type=text with inputmode); ISO 8601 for stored dates; Unicode CLDR through Intl (browser) and ICU/CultureInfo (server); OWASP: validate the canonical form, one normalisation policy.</t>
+        </is>
+      </c>
+      <c r="J368" s="8" t="inlineStr">
+        <is>
+          <t>Done when: one service formats and parses numbers on server and client with identical results for the shared fixtures; Persian digit entry works in every numeric field; rial and toman amounts are exact; views no longer carry their own number format strings (ratchet in CI).</t>
+        </is>
+      </c>
+      <c r="K368" s="8" t="n"/>
+      <c r="L368" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M368" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N368" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O368" s="10" t="inlineStr">
+        <is>
+          <t>#366 #208</t>
+        </is>
+      </c>
+      <c r="P368" s="10" t="inlineStr">
+        <is>
+          <t>#60</t>
+        </is>
+      </c>
+      <c r="Q368" s="10" t="n"/>
+      <c r="R368" s="8" t="inlineStr">
+        <is>
+          <t>Persian &amp; localisation</t>
+        </is>
+      </c>
+      <c r="S368" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T368" s="10" t="n"/>
+      <c r="U368" s="10" t="n"/>
+    </row>
+    <row r="369">
+      <c r="A369" s="10" t="n">
+        <v>368</v>
+      </c>
+      <c r="B369" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C369" s="8" t="inlineStr">
+        <is>
+          <t>Persian Localization, RTL &amp; Jalali Calendar</t>
+        </is>
+      </c>
+      <c r="D369" s="8" t="inlineStr">
+        <is>
+          <t>Date, time and calendar formatting engine used by server and client: ISO 8601 canonical storage, date-only versus instant, user time zone, Jalali and Gregorian display and input, Persian digits, week start, maintained library instead of ad-hoc code</t>
+        </is>
+      </c>
+      <c r="E369" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F369" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G369" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H369" s="8" t="inlineStr">
+        <is>
+          <t>Formatting in PEMS is done page by page: 377 hand-written date and time format strings in 138 views using 12 different patterns, 217 number format strings, 103 native date, 8 datetime-local and 137 number inputs whose look follows the browser locale, and Jalali support in only 6 files. Existing rows #24, #205, #206, #208 and #209 ask for translated labels, Persian digits, the Jalali calendar and fixed reports, but nothing defines where a field's format lives or how it relates to validation. Dates are stored and shown inconsistently; native date inputs ignore the Jalali calendar, 12 different display patterns exist, and a native date control cannot be switched to Jalali.</t>
+        </is>
+      </c>
+      <c r="I369" s="8" t="inlineStr">
+        <is>
+          <t>1) Canonical forms: a date without time is stored as a date-only value (ISO 8601, no time zone, so a due date never shifts a day), an instant as UTC; the user's time zone is applied only for display and input of instants, daylight saving included. 2) Choose a maintained library for calendars and conversion (evaluate the .NET PersianCalendar and the browser Intl calendar support first; for the picker evaluate maintained Jalali date libraries; avoid unmaintained or deprecated packages; works offline; record licences in L_OSS). 3) Display presets from #366 (Jalali long and short, Gregorian ISO, weekday names, Saturday as week start), Persian digits optional. 4) Input: a date picker component in PEMS.UI showing Jalali or Gregorian per setting, with typed entry parsed tolerantly (separators, Persian digits, two-digit years rejected or expanded by a documented rule) and invalid dates such as 1403/12/30 in a non-leap year rejected with a suggestion. 5) Server and client use the same conversion tests. 6) Ranges and relative windows from #355 evaluate in the same calendar-independent canonical form. Best-practice sources: W3C Internationalization (date and number formats follow the language context, avoid ambiguous numeric dates, support non-Gregorian calendars, keep localisation separate from translation); MDN notes on input type=number (locale separators and non-ASCII digits are sanitised, no pattern support, so formatted or Persian input needs type=text with inputmode); ISO 8601 for stored dates; Unicode CLDR through Intl (browser) and ICU/CultureInfo (server); OWASP: validate the canonical form, one normalisation policy.</t>
+        </is>
+      </c>
+      <c r="J369" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a date picked as Jalali is stored as the correct Gregorian date-only value and shown back identically on every page; date-times display in the user's time zone across a daylight-saving change; invalid Jalali dates are rejected with a hint; the picker works in RTL and LTR and offline; views no longer carry their own date format strings (ratchet).</t>
+        </is>
+      </c>
+      <c r="K369" s="8" t="n"/>
+      <c r="L369" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M369" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N369" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O369" s="10" t="inlineStr">
+        <is>
+          <t>#366 #206</t>
+        </is>
+      </c>
+      <c r="P369" s="10" t="inlineStr">
+        <is>
+          <t>#154 #179</t>
+        </is>
+      </c>
+      <c r="Q369" s="10" t="n"/>
+      <c r="R369" s="8" t="inlineStr">
+        <is>
+          <t>Persian &amp; localisation</t>
+        </is>
+      </c>
+      <c r="S369" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T369" s="10" t="n"/>
+      <c r="U369" s="10" t="n"/>
+    </row>
+    <row r="370">
+      <c r="A370" s="10" t="n">
+        <v>369</v>
+      </c>
+      <c r="B370" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C370" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D370" s="8" t="inlineStr">
+        <is>
+          <t>Formatted and masked text inputs: phone, national code, IBAN and code patterns shown grouped while the raw value is kept, paste and caret handling in RTL, type=text with inputmode, accessible hints</t>
+        </is>
+      </c>
+      <c r="E370" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F370" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G370" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H370" s="8" t="inlineStr">
+        <is>
+          <t>Identifiers and codes are typed and shown inconsistently (with and without spaces, dashes, Persian digits); a number-typed input cannot hold leading zeros or grouped digits, and MDN advises type=text with inputmode and a pattern for such values.</t>
+        </is>
+      </c>
+      <c r="I370" s="8" t="inlineStr">
+        <is>
+          <t>1) Mask and display presets from the format catalog (#366): grouping pattern, separator, case, example. 2) The PEMS.UI field renders type=text with inputmode and the pattern attribute, shows the grouped form while typing and keeps the raw canonical value in a hidden or data attribute that is submitted. 3) Paste handling: strip separators and spaces, normalise digits (#364), re-group; caret stays correct in RTL and with Persian digits. 4) Screen readers read the example format and the error, not the mask characters. 5) Server accepts only the raw form and re-validates it. 6) Component docs with examples in the catalog. Best-practice sources: W3C Internationalization (date and number formats follow the language context, avoid ambiguous numeric dates, support non-Gregorian calendars, keep localisation separate from translation); MDN notes on input type=number (locale separators and non-ASCII digits are sanitised, no pattern support, so formatted or Persian input needs type=text with inputmode); ISO 8601 for stored dates; Unicode CLDR through Intl (browser) and ICU/CultureInfo (server); OWASP: validate the canonical form, one normalisation policy.</t>
+        </is>
+      </c>
+      <c r="J370" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a phone number, national code, IBAN and a pattern code are shown grouped, pasted in any common form and submitted raw; leading zeros are kept; caret and selection work in RTL; screen-reader and keyboard checks pass.</t>
+        </is>
+      </c>
+      <c r="K370" s="8" t="n"/>
+      <c r="L370" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M370" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N370" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O370" s="10" t="inlineStr">
+        <is>
+          <t>#357 #366</t>
+        </is>
+      </c>
+      <c r="P370" s="10" t="n"/>
+      <c r="Q370" s="10" t="n"/>
+      <c r="R370" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S370" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T370" s="10" t="n"/>
+      <c r="U370" s="10" t="n"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="10" t="n">
+        <v>370</v>
+      </c>
+      <c r="B371" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C371" s="8" t="inlineStr">
+        <is>
+          <t>Persian Localization, RTL &amp; Jalali Calendar</t>
+        </is>
+      </c>
+      <c r="D371" s="8" t="inlineStr">
+        <is>
+          <t>Label and text presentation rules: resolve translated label, help, placeholder, error and option text through the field, model, app and user hierarchy, direction isolation of LTR tokens in RTL text, text transforms, empty/boolean/option display, missing-translation report</t>
+        </is>
+      </c>
+      <c r="E371" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F371" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G371" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H371" s="8" t="inlineStr">
+        <is>
+          <t>Row #24 stores translatable strings in metadata; nothing defines how they are resolved in a context or how mixed-direction text (codes, e-mail, URLs, numbers inside Persian sentences) is displayed. W3C: keep localisation separate from translation.</t>
+        </is>
+      </c>
+      <c r="I371" s="8" t="inlineStr">
+        <is>
+          <t>1) Resolution order for every visible string: field setting -&gt; model language -&gt; app -&gt; user preference -&gt; system default, with a documented fallback to the default language and a visible marker in the designer when a translation is missing. 2) Direction: set dir per field and per value type; wrap LTR tokens (codes, e-mail, URLs, Latin words, numbers with units) in directional isolates so punctuation and order stay correct inside RTL text, and keep the zero-width non-joiner rules of #364. 3) Display rules for empty values, booleans, option labels (translated, with the stored code unchanged), long text (truncate with tooltip, never cut mid-grapheme) and optional transforms (upper case for codes). 4) Report of missing and untranslated strings per language, usable in CI. 5) Tests with mixed-direction samples. Best-practice sources: W3C Internationalization (date and number formats follow the language context, avoid ambiguous numeric dates, support non-Gregorian calendars, keep localisation separate from translation); MDN notes on input type=number (locale separators and non-ASCII digits are sanitised, no pattern support, so formatted or Persian input needs type=text with inputmode); ISO 8601 for stored dates; Unicode CLDR through Intl (browser) and ICU/CultureInfo (server); OWASP: validate the canonical form, one normalisation policy.</t>
+        </is>
+      </c>
+      <c r="J371" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the same label shows in the right language for field, model, app and user contexts with a defined fallback; mixed-direction samples render correctly; a CI report lists missing translations; option labels change without touching stored values.</t>
+        </is>
+      </c>
+      <c r="K371" s="8" t="n"/>
+      <c r="L371" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M371" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N371" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O371" s="10" t="inlineStr">
+        <is>
+          <t>#24 #366</t>
+        </is>
+      </c>
+      <c r="P371" s="10" t="inlineStr">
+        <is>
+          <t>#190 #230 #42</t>
+        </is>
+      </c>
+      <c r="Q371" s="10" t="n"/>
+      <c r="R371" s="8" t="inlineStr">
+        <is>
+          <t>Persian &amp; localisation</t>
+        </is>
+      </c>
+      <c r="S371" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T371" s="10" t="n"/>
+      <c r="U371" s="10" t="n"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="10" t="n">
+        <v>371</v>
+      </c>
+      <c r="B372" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C372" s="8" t="inlineStr">
+        <is>
+          <t>Reporting, Dashboards &amp; Export</t>
+        </is>
+      </c>
+      <c r="D372" s="8" t="inlineStr">
+        <is>
+          <t>Export, print and report formatting parity: Excel cells typed as real numbers and dates with number-format codes, CSV canonical option, PDF and print use the same formatters and direction as the screen</t>
+        </is>
+      </c>
+      <c r="E372" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F372" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G372" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H372" s="8" t="inlineStr">
+        <is>
+          <t>Exports are a second place where formats drift: strings instead of typed cells cannot be sorted or summed, and a comparable platform shipped an invalid-date defect in downloaded reports and layout overflow in PDF exports.</t>
+        </is>
+      </c>
+      <c r="I372" s="8" t="inlineStr">
+        <is>
+          <t>1) The export service of #210 asks the formatting engine for display text where text is wanted, and writes typed cells (number, date, boolean) with matching Excel number-format codes where the user will calculate; Jalali display is a cell format or an extra column, the stored date stays a real date. 2) CSV: canonical values by default (ISO dates, dot decimals) with an option for display format. 3) PDF and print use the same formatters, the user's language and direction, and wrap LTR tokens correctly. 4) Header labels use the translated field labels. 5) Tests that open a generated file and check cell types, values and an invalid-date regression. Best-practice sources: W3C Internationalization (date and number formats follow the language context, avoid ambiguous numeric dates, support non-Gregorian calendars, keep localisation separate from translation); MDN notes on input type=number (locale separators and non-ASCII digits are sanitised, no pattern support, so formatted or Persian input needs type=text with inputmode); ISO 8601 for stored dates; Unicode CLDR through Intl (browser) and ICU/CultureInfo (server); OWASP: validate the canonical form, one normalisation policy.</t>
+        </is>
+      </c>
+      <c r="J372" s="8" t="inlineStr">
+        <is>
+          <t>Done when: an Excel export sorts and sums numbers and dates correctly and shows Jalali dates as configured; CSV defaults to canonical values; PDF text, direction and dates match the screen; the invalid-date regression test passes.</t>
+        </is>
+      </c>
+      <c r="K372" s="8" t="n"/>
+      <c r="L372" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M372" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N372" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O372" s="10" t="inlineStr">
+        <is>
+          <t>#366 #367 #368 #210 #209</t>
+        </is>
+      </c>
+      <c r="P372" s="10" t="inlineStr">
+        <is>
+          <t>#56 #60 #154 #62</t>
+        </is>
+      </c>
+      <c r="Q372" s="10" t="n"/>
+      <c r="R372" s="8" t="inlineStr">
+        <is>
+          <t>Reporting &amp; export</t>
+        </is>
+      </c>
+      <c r="S372" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T372" s="10" t="n"/>
+      <c r="U372" s="10" t="n"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="10" t="n">
+        <v>372</v>
+      </c>
+      <c r="B373" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C373" s="8" t="inlineStr">
+        <is>
+          <t>Quality, Testing &amp; Performance</t>
+        </is>
+      </c>
+      <c r="D373" s="8" t="inlineStr">
+        <is>
+          <t>Format and parse round-trip test matrix together with validation: format(parse(x)) and parse(format(v)) identity across locales, calendars, digit shapes, time zones and rounding, then validation of the parsed canonical value</t>
+        </is>
+      </c>
+      <c r="E373" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F373" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G373" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H373" s="8" t="inlineStr">
+        <is>
+          <t>A format that cannot be parsed back, or a parse result that validation rejects although the user typed what was displayed, is a classic defect; the same fixtures must cover format, parse and validation together (design rule of #366).</t>
+        </is>
+      </c>
+      <c r="I373" s="8" t="inlineStr">
+        <is>
+          <t>1) Extend the fixture file of #361 with format cases: for each type, locale (fa, en), calendar (Jalali, Gregorian), digit shape, time zone (including a daylight-saving change) and rounding mode, the value, its display text and the accepted input spellings. 2) Properties: parse(format(v)) = v, format(parse(s)) = canonical display of s, validation outcome equals the expected one for the parsed canonical value. 3) Edge cases: Jalali leap years and 30 Esfand, 31 Shahrivar, month and year boundaries, very large and very small numbers, rounding ties, negative zero, mixed digit scripts, ambiguous numeric dates rejected. 4) Run on server and client from the same file; CI fails on any difference. Best-practice sources: W3C Internationalization (date and number formats follow the language context, avoid ambiguous numeric dates, support non-Gregorian calendars, keep localisation separate from translation); MDN notes on input type=number (locale separators and non-ASCII digits are sanitised, no pattern support, so formatted or Persian input needs type=text with inputmode); ISO 8601 for stored dates; Unicode CLDR through Intl (browser) and ICU/CultureInfo (server); OWASP: validate the canonical form, one normalisation policy.</t>
+        </is>
+      </c>
+      <c r="J373" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the shared fixture file covers format, parse and validation for every type; server and client agree on every case; a broken formatter, parser or rule fails the build.</t>
+        </is>
+      </c>
+      <c r="K373" s="8" t="n"/>
+      <c r="L373" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M373" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N373" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O373" s="10" t="inlineStr">
+        <is>
+          <t>#361 #367 #368</t>
+        </is>
+      </c>
+      <c r="P373" s="10" t="inlineStr">
+        <is>
+          <t>#154 #20</t>
+        </is>
+      </c>
+      <c r="Q373" s="10" t="n"/>
+      <c r="R373" s="8" t="inlineStr">
+        <is>
+          <t>Quality &amp; testing</t>
+        </is>
+      </c>
+      <c r="S373" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T373" s="10" t="n"/>
+      <c r="U373" s="10" t="n"/>
+    </row>
+    <row r="374">
+      <c r="A374" s="10" t="n">
+        <v>373</v>
+      </c>
+      <c r="B374" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C374" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic Form Builder</t>
+        </is>
+      </c>
+      <c r="D374" s="8" t="inlineStr">
+        <is>
+          <t>Format and locale settings UI: system defaults, per app, model and field overrides in the designer with live examples, and per-user preferences for calendar, digits, number style, time zone and week start, permission-protected and audited</t>
+        </is>
+      </c>
+      <c r="E374" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F374" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G374" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H374" s="8" t="inlineStr">
+        <is>
+          <t>Without a settings surface the format hierarchy of #366 stays code-only; users in an Iranian company expect to switch calendar and digit style themselves, and designers need to see the effect of a format before saving.</t>
+        </is>
+      </c>
+      <c r="I374" s="8" t="inlineStr">
+        <is>
+          <t>1) Admin page for system defaults and per-app/per-model settings; the field properties panel of the form designer (#44) gets Format next to Validation, with presets, a custom pattern where allowed, and a live preview that shows sample values formatted and an input that is parsed and validated against both. 2) User profile page: calendar (Jalali/Gregorian), digit shape, number style, time zone, week start, language (links to #207). 3) Permission to change system and model settings, audit of every change, versioned with the metadata package (#23). 4) Settings cached with invalidation (#28). 5) Accessible and RTL-correct controls built from PEMS.UI components. Best-practice sources: W3C Internationalization (date and number formats follow the language context, avoid ambiguous numeric dates, support non-Gregorian calendars, keep localisation separate from translation); MDN notes on input type=number (locale separators and non-ASCII digits are sanitised, no pattern support, so formatted or Persian input needs type=text with inputmode); ISO 8601 for stored dates; Unicode CLDR through Intl (browser) and ICU/CultureInfo (server); OWASP: validate the canonical form, one normalisation policy.</t>
+        </is>
+      </c>
+      <c r="J374" s="8" t="inlineStr">
+        <is>
+          <t>Done when: an administrator changes a model's date and number format and sees it in lists, forms and exports without a deploy; a user switches calendar and digits for themselves; every change is audited; the designer preview shows formatted, parsed and validated values.</t>
+        </is>
+      </c>
+      <c r="K374" s="8" t="n"/>
+      <c r="L374" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M374" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N374" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O374" s="10" t="inlineStr">
+        <is>
+          <t>#366 #44</t>
+        </is>
+      </c>
+      <c r="P374" s="10" t="inlineStr">
+        <is>
+          <t>#176 #190</t>
+        </is>
+      </c>
+      <c r="Q374" s="10" t="n"/>
+      <c r="R374" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic form builder</t>
+        </is>
+      </c>
+      <c r="S374" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T374" s="10" t="n"/>
+      <c r="U374" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-368 docs: close-out of staging environment and migrations assembly (plan Report, Supportability Matrix, changelog)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1576,7 +1576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3139,6 +3139,100 @@
       <c r="I37" s="8" t="inlineStr">
         <is>
           <t>Add a migration with the --project PEMS.Migrations option. Verified 2026-10-25: Persistence 29 MB -&gt; 6 MB, Migrations 23 MB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>SM-34</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Pre-production staging environment</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Core / deploy pipeline</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>staging branch -&gt; staging subdomain, own database, env/staging.env, STAGING_* secrets; same reusable pipeline as demo</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G38" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H38" s="10" t="inlineStr">
+        <is>
+          <t>#351</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>Verified 2026-10-25 (run 40208748572).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>SM-35</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Deployments upload only changed files and skip repeated tests</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Deploy pipeline</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>FTP difference upload (sync state file); tag gate-pass/&lt;source tree hash&gt; skips build, drift gate and tests for an identical tree; first full upload ~245 MB, later ~34 MB</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G39" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H39" s="10" t="inlineStr">
+        <is>
+          <t>#351 #354</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>Package slimmed 285 -&gt; 245 MB.</t>
         </is>
       </c>
     </row>
@@ -42841,7 +42935,7 @@
       </c>
       <c r="F352" s="10" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G352" s="10" t="inlineStr">
@@ -42864,7 +42958,11 @@
           <t>Done when: a push to main or to a working branch starts no workflow; a push to demo deploys the demo subdomain and a push to staging deploys the staging subdomain; the README lets a new person set up both environments; the staging branch contains main, dev and demo; dev no longer exists.</t>
         </is>
       </c>
-      <c r="K352" s="8" t="n"/>
+      <c r="K352" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-25: no workflow runs on main or working branches (build.yml manual); reusable deploy-site.yml called by deploy-demo.yml and deploy-staging.yml; env/staging files; staging branch created from main+dev+demo; dev merged into main and deleted; docs/deployment/DEPLOYMENT_README.md. Staging run 40208748572 green: HTTP 200, database up to date, upload of changed files only (33.8 MB). Fixes found on the way: stale migration-chain test, FTP protocol default, FTP precheck, health check with server logs.</t>
+        </is>
+      </c>
       <c r="L352" s="10" t="inlineStr">
         <is>
           <t>M2</t>
@@ -43096,7 +43194,7 @@
       </c>
       <c r="F355" s="10" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G355" s="10" t="inlineStr">
@@ -43119,7 +43217,11 @@
           <t>Done when: dotnet build and the migration/deployment tests pass; the drift gate runs with --project PEMS.Migrations; PEMS.Persistence.dll no longer contains migrations and a change in a Persistence service leaves PEMS.Migrations.dll byte-identical; docs and guideline use the new command.</t>
         </is>
       </c>
-      <c r="K355" s="8" t="n"/>
+      <c r="K355" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-25: migrations moved to PEMS.Migrations (239 files git-mv'd); PEMS.Persistence.dll 29 MB -&gt; 6 MB, PEMS.Migrations.dll 23 MB stays byte-identical when only data-layer code changes (verified with DebugType=none); drift gate, deploy.ps1, Dockerfile, docs updated; migration tests 10/10 on a real SQL Server and 65/65 database-free tests pass.</t>
+        </is>
+      </c>
       <c r="L355" s="10" t="inlineStr">
         <is>
           <t>M2</t>

</xml_diff>

<commit_message>
SCRUM-17 docs(security): rotation runbook, exposure report, follow-up tasks, Jira reporting rule
- docs/deployment/CREDENTIAL_ROTATION_RUNBOOK.md and scripts/security/Report-DefaultCredentialExposure.sql (read-only) for plan row #317
- LoadTestSeed reads LoadTest__Password from env/local.secrets.env (key added to the example) or PEMS_LOADTEST_PASSWORD
- plan rows #374 (held), #375 (held), #376, #377, #378 added; plan/backlog.csv regenerated; Instructions rule 27 (keep the Jira report current)
- guideline chapters 00 and 06 updated; audit report updated with the owner's decisions of 2026-10-26

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -11474,7 +11474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11900,6 +11900,21 @@
       <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Owner decision 2026-10-23 (docs/design/COMPONENT_LIBRARY_PLAN.md): once PEMS.UI exists, new pages are built from its components and templates; raw form-control/table/modal/badge markup, inline styles, inline scripts and CDN references are not added (CI ratchet). A missing component is added to the library first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Keep the Jira report current</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Owner decision 2026-10-26: every task keeps its Jira issue report up to date while the work runs and when it ends, not only at the end. (1) At start: comment 'Started by &lt;agent or person&gt;' with the plan. (2) During the work: a short comment at every milestone, decision, blocker or change of scope (what is done, what is next, what blocks), and a comment before any hand-over or stop. (3) At the end: a closing comment with what changed, files, tests run and not run, PR link, evidence for each 'Done when' item and open items for the owner. The same text goes in the PR description. An issue without a current report is not moved to In Review or Done. Never put a secret value in a report (mask to two characters at most).</t>
         </is>
       </c>
     </row>
@@ -11914,7 +11929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U374"/>
+  <dimension ref="A1:U379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -44927,6 +44942,439 @@
       </c>
       <c r="T374" s="10" t="n"/>
       <c r="U374" s="10" t="n"/>
+    </row>
+    <row r="375">
+      <c r="A375" s="10" t="n">
+        <v>374</v>
+      </c>
+      <c r="B375" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C375" s="8" t="inlineStr">
+        <is>
+          <t>Foundation, Architecture Decisions &amp; Baseline</t>
+        </is>
+      </c>
+      <c r="D375" s="8" t="inlineStr">
+        <is>
+          <t>Purge the old built-in credentials and the runtime user files from the git history (all branches), after rotation</t>
+        </is>
+      </c>
+      <c r="E375" s="10" t="inlineStr">
+        <is>
+          <t>Ops Process</t>
+        </is>
+      </c>
+      <c r="F375" s="10" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="G375" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H375" s="8" t="inlineStr">
+        <is>
+          <t>The SCRUM-17 audit (docs/audits/SECRETS_AUDIT_2026-10.md) found five built-in or shared passwords and 13 runtime user files (PEMS.Web/filestore) that remain readable in the history of every branch. PM 2026-10-26: not important for now; add the task and hold it.</t>
+        </is>
+      </c>
+      <c r="I375" s="8" t="inlineStr">
+        <is>
+          <t>1) Finish the rotation of #317 first (docs/deployment/CREDENTIAL_ROTATION_RUNBOOK.md). 2) Decide the scope: only the filestore folder and the old credential literals, or a full rewrite. 3) Rewrite with git filter-repo on a fresh mirror clone, verify with the audit scans, force-push all branches and tags in one agreed window, re-clone every working copy and runner. 4) Remove the files from the index (git rm --cached PEMS.Web/filestore) if still tracked. 5) Re-run the secrets scan and update the audit report.</t>
+        </is>
+      </c>
+      <c r="J375" s="8" t="inlineStr">
+        <is>
+          <t>Done when: no branch or tag contains the old built-in passwords or PEMS.Web/filestore files (scan output attached); every developer and CI runner has a fresh clone; the audit report states the date of the rewrite.</t>
+        </is>
+      </c>
+      <c r="K375" s="8" t="inlineStr">
+        <is>
+          <t>ON HOLD per PM 2026-10-26 (history items are not important for now; rotation in #317 comes first).</t>
+        </is>
+      </c>
+      <c r="L375" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M375" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N375" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O375" s="10" t="inlineStr">
+        <is>
+          <t>#9 #317</t>
+        </is>
+      </c>
+      <c r="P375" s="10" t="n"/>
+      <c r="Q375" s="10" t="n"/>
+      <c r="R375" s="8" t="inlineStr">
+        <is>
+          <t>Foundation &amp; decisions</t>
+        </is>
+      </c>
+      <c r="S375" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T375" s="10" t="n"/>
+      <c r="U375" s="10" t="n"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="10" t="n">
+        <v>375</v>
+      </c>
+      <c r="B376" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C376" s="8" t="inlineStr">
+        <is>
+          <t>Main Host: Landing &amp; Demo Deployment</t>
+        </is>
+      </c>
+      <c r="D376" s="8" t="inlineStr">
+        <is>
+          <t>Verify the server certificate on the FTPS upload in the deploy workflow (remove curl --insecure)</t>
+        </is>
+      </c>
+      <c r="E376" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F376" s="10" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="G376" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H376" s="8" t="inlineStr">
+        <is>
+          <t>SCRUM-17 audit S-2: .github/workflows/deploy-site.yml uploads over FTPS with curl --insecure at four places, so the FTP password is sent over a TLS channel whose certificate is not verified. PM 2026-10-26: accepted for now, conditionally; add the task and hold it.</t>
+        </is>
+      </c>
+      <c r="I376" s="8" t="inlineStr">
+        <is>
+          <t>1) Get the certificate or CA of the demo/staging FTP host (Plesk). 2) Store it as a GitHub secret or repository file and pass --cacert (or pin the public key with --pinnedpubkey) in all four curl calls and the upload action settings. 3) Remove --insecure from FTP calls; keep it only for the HTTP health probe if the site certificate is not yet valid, with a comment. 4) Test a deploy to staging, then demo.</t>
+        </is>
+      </c>
+      <c r="J376" s="8" t="inlineStr">
+        <is>
+          <t>Done when: no FTP call in deploy-site.yml uses --insecure; a deploy to staging and demo succeeds; a wrong certificate makes the run fail.</t>
+        </is>
+      </c>
+      <c r="K376" s="8" t="inlineStr">
+        <is>
+          <t>ON HOLD per PM 2026-10-26 (risk accepted conditionally: shared host, demo and staging only; revisit before customer data goes to demo).</t>
+        </is>
+      </c>
+      <c r="L376" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M376" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N376" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O376" s="10" t="inlineStr">
+        <is>
+          <t>#9 #295</t>
+        </is>
+      </c>
+      <c r="P376" s="10" t="n"/>
+      <c r="Q376" s="10" t="n"/>
+      <c r="R376" s="8" t="inlineStr">
+        <is>
+          <t>Main host: landing &amp; demo deployment</t>
+        </is>
+      </c>
+      <c r="S376" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T376" s="10" t="n"/>
+      <c r="U376" s="10" t="n"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="10" t="n">
+        <v>376</v>
+      </c>
+      <c r="B377" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C377" s="8" t="inlineStr">
+        <is>
+          <t>Quality, Testing &amp; Performance</t>
+        </is>
+      </c>
+      <c r="D377" s="8" t="inlineStr">
+        <is>
+          <t>Review and optimise the automated tests: split database-free and SQL tests, remove duplicate, skipped and flaky tests, speed up the run</t>
+        </is>
+      </c>
+      <c r="E377" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F377" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G377" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H377" s="8" t="inlineStr">
+        <is>
+          <t>About 1,400 Fact/Theory tests exist (#249) and many need SQL Server; the SCRUM-17 session could not run any of them. A suite that is slow, environment-bound or partly red is not run after every task.</t>
+        </is>
+      </c>
+      <c r="I377" s="8" t="inlineStr">
+        <is>
+          <t>1) Use the baseline report of #1 (counts, durations, failures). 2) Classify every test class: database-free, in-memory, SQL Server, browser. 3) Add traits/categories so a task can run only the affected group plus the fast database-free group. 4) Fix, quarantine with a Jira key, or delete tests that are red, skipped or flaky (never skip silently). 5) Remove duplicates and slow set-up; target a database-free run under a few minutes. 6) Document the commands in docs/guidelines/05-environment-and-commands.md.</t>
+        </is>
+      </c>
+      <c r="J377" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the suite has categories; a database-free run and a SQL run each have a documented command and duration; no test is skipped without a Jira key; the before/after numbers are in the Jira report.</t>
+        </is>
+      </c>
+      <c r="K377" s="8" t="n"/>
+      <c r="L377" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M377" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N377" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O377" s="10" t="inlineStr">
+        <is>
+          <t>#1 #249</t>
+        </is>
+      </c>
+      <c r="P377" s="10" t="n"/>
+      <c r="Q377" s="10" t="n"/>
+      <c r="R377" s="8" t="inlineStr">
+        <is>
+          <t>Quality &amp; testing</t>
+        </is>
+      </c>
+      <c r="S377" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T377" s="10" t="n"/>
+      <c r="U377" s="10" t="n"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="10" t="n">
+        <v>377</v>
+      </c>
+      <c r="B378" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C378" s="8" t="inlineStr">
+        <is>
+          <t>Quality, Testing &amp; Performance</t>
+        </is>
+      </c>
+      <c r="D378" s="8" t="inlineStr">
+        <is>
+          <t>Define and introduce the test-maintenance procedure that runs after every finished task</t>
+        </is>
+      </c>
+      <c r="E378" s="10" t="inlineStr">
+        <is>
+          <t>Ops Process</t>
+        </is>
+      </c>
+      <c r="F378" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G378" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H378" s="8" t="inlineStr">
+        <is>
+          <t>Tests drift: the baseline of #1 already lists tests that fail on a clean main. Nothing today forces the author of a task to re-run, update or retire the tests it affects, or to keep the Test Plan sheet current (rule 14).</t>
+        </is>
+      </c>
+      <c r="I378" s="8" t="inlineStr">
+        <is>
+          <t>1) Write the procedure as a chapter or section of docs/guidelines (after each task: run the fast group and the affected groups, fix or update stale tests in the same PR, add a regression test per bug, update the Test Plan sheet status, record counts in the Jira report). 2) Add the check to the PR template and to the closing steps in chapter 00. 3) Add a periodic (weekly) full-suite run and a stale/skipped test report. 4) Propose the Instructions-sheet rule to the owner.</t>
+        </is>
+      </c>
+      <c r="J378" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the procedure is in the guideline, the PR template and chapter 00; one finished task has been closed with it; the owner has confirmed whether it becomes an Instructions rule.</t>
+        </is>
+      </c>
+      <c r="K378" s="8" t="n"/>
+      <c r="L378" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M378" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N378" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O378" s="10" t="inlineStr">
+        <is>
+          <t>#1 #376</t>
+        </is>
+      </c>
+      <c r="P378" s="10" t="n"/>
+      <c r="Q378" s="10" t="n"/>
+      <c r="R378" s="8" t="inlineStr">
+        <is>
+          <t>Quality &amp; testing</t>
+        </is>
+      </c>
+      <c r="S378" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T378" s="10" t="n"/>
+      <c r="U378" s="10" t="n"/>
+    </row>
+    <row r="379">
+      <c r="A379" s="10" t="n">
+        <v>378</v>
+      </c>
+      <c r="B379" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C379" s="8" t="inlineStr">
+        <is>
+          <t>Foundation, Architecture Decisions &amp; Baseline</t>
+        </is>
+      </c>
+      <c r="D379" s="8" t="inlineStr">
+        <is>
+          <t>Review and optimise the roles and setup of Claude: .claude/Role directives, AGENTS.md, CLAUDE.md, .claude/settings.json, skills and the session prompts</t>
+        </is>
+      </c>
+      <c r="E379" s="10" t="inlineStr">
+        <is>
+          <t>Ops Process</t>
+        </is>
+      </c>
+      <c r="F379" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G379" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H379" s="8" t="inlineStr">
+        <is>
+          <t>Claude works from several overlapping sources: AGENTS.md, CLAUDE.md files, two identical copies of the Role documents (#8), skills and per-session prompts. Cloud sessions run in parallel with limited credits and need clear scope and stop rules.</t>
+        </is>
+      </c>
+      <c r="I379" s="8" t="inlineStr">
+        <is>
+          <t>1) Inventory what Claude reads at session start and what each source says (roles, rules, tools). 2) Remove duplicates and contradictions; give the Role documents one home (with #8); keep AGENTS.md short and the guideline the single source of rules. 3) Define the roles (for example implementer, auditor, reviewer, planner) with scope, allowed actions, outputs and when to stop and ask. 4) Define the standard session brief for parallel cloud sessions (branch, forbidden files, Jira steps, report format). 5) Measure with two sample tasks before and after.</t>
+        </is>
+      </c>
+      <c r="J379" s="8" t="inlineStr">
+        <is>
+          <t>Done when: one documented set of Claude roles and one session-brief template exist; no duplicated Role document remains; two sample tasks run with the new setup follow the guideline without reminders.</t>
+        </is>
+      </c>
+      <c r="K379" s="8" t="n"/>
+      <c r="L379" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M379" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N379" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O379" s="10" t="inlineStr">
+        <is>
+          <t>#8</t>
+        </is>
+      </c>
+      <c r="P379" s="10" t="n"/>
+      <c r="Q379" s="10" t="n"/>
+      <c r="R379" s="8" t="inlineStr">
+        <is>
+          <t>Foundation &amp; decisions</t>
+        </is>
+      </c>
+      <c r="S379" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T379" s="10" t="n"/>
+      <c r="U379" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-17 docs(plan): add task #379 (file-store and upload paths as env settings)
Found by the secrets audit (rule R24). Plan row #379 = SCRUM-396; plan/backlog.csv regenerated (plan_sync check: 0 findings); audit report references the task.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -11929,7 +11929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U379"/>
+  <dimension ref="A1:U380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -45375,6 +45375,91 @@
       </c>
       <c r="T379" s="10" t="n"/>
       <c r="U379" s="10" t="n"/>
+    </row>
+    <row r="380">
+      <c r="A380" s="10" t="n">
+        <v>379</v>
+      </c>
+      <c r="B380" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C380" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D380" s="8" t="inlineStr">
+        <is>
+          <t>Move the file-store and upload folder paths into env settings (no hard-coded paths in Program.cs and controllers)</t>
+        </is>
+      </c>
+      <c r="E380" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F380" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G380" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H380" s="8" t="inlineStr">
+        <is>
+          <t>Found by the SCRUM-17 audit (rule R24): the file-store root is built from the working directory in PEMS.Web/Program.cs:686, and three controllers build upload folders the same way (LetterController.cs:690, MyProfileController.cs:65 and :111). The location cannot be set per environment.</t>
+        </is>
+      </c>
+      <c r="I380" s="8" t="inlineStr">
+        <is>
+          <t>1) Add required settings to every env/*.env file (for example FileStorage__RootPath, Uploads__RootPath; relative defaults keep today's behaviour) and read them with the Required* helpers; keep the key-parity test green. 2) Use them in Program.cs and the three controllers, through the existing file-storage service where possible. 3) Map them to the volumes of docker-compose.yml and deploy/docker/compose.pems-web.yml and to the exclusions in deploy/Build-Package.ps1. 4) Unit test for the path resolution, the existing Linux deployment artifact tests, upload and download of one file per area. 5) Document in env/README.md.</t>
+        </is>
+      </c>
+      <c r="J380" s="8" t="inlineStr">
+        <is>
+          <t>Done when: no Path.Combine(Directory.GetCurrentDirectory(), ...) remains for the file store or upload folders; every env file defines the settings; a changed value moves the storage in a local run; deployment artifact tests pass.</t>
+        </is>
+      </c>
+      <c r="K380" s="8" t="n"/>
+      <c r="L380" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M380" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N380" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O380" s="10" t="inlineStr">
+        <is>
+          <t>#315 #183</t>
+        </is>
+      </c>
+      <c r="P380" s="10" t="n"/>
+      <c r="Q380" s="10" t="n"/>
+      <c r="R380" s="8" t="inlineStr">
+        <is>
+          <t>Install &amp; update</t>
+        </is>
+      </c>
+      <c r="S380" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T380" s="10" t="n"/>
+      <c r="U380" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-17 docs: close the six artefacts, extend #317 #318 #119 for audit S-5/S-6, rule 28
- CHANGELOG, learnings-log, Supportability Matrix SM-36, plan row #9 Report
- #317 (rotation runbook, AllowedHosts), #318 (password-policy default), #119 (delivery scan for internal addresses) modified instead of adding tasks
- Instructions rule 28 and chapter 00 step 5b: study existing tasks before adding one
- chapter 05: database-free test command for the new tests

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1576,7 +1576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3233,6 +3233,53 @@
       <c r="I39" s="8" t="inlineStr">
         <is>
           <t>Package slimmed 285 -&gt; 245 MB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>SM-36</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>No built-in credentials in source, container or tool files</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Core / compose / tools</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>No default or hard-coded password: the first administrator comes only from Seed__Admin__Password; users created from an employee get a random one-time password; docker-compose publishes ports on 127.0.0.1 only and requires SQL_SA_PASSWORD</t>
+        </is>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G40" s="10" t="inlineStr">
+        <is>
+          <t>Supported (unverified)</t>
+        </is>
+      </c>
+      <c r="H40" s="10" t="inlineStr">
+        <is>
+          <t>#9 #317</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>Implemented 2026-10-26 (SCRUM-17); status becomes Done when the build and EnvironmentFilesTests and TemporaryPasswordGeneratorTests have run green. Environments created before 2026-10-23 need rotation (#317); the old values stay in git history (#374, on hold).</t>
         </is>
       </c>
     </row>
@@ -11474,7 +11521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11915,6 +11962,21 @@
       <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Owner decision 2026-10-26: every task keeps its Jira issue report up to date while the work runs and when it ends, not only at the end. (1) At start: comment 'Started by &lt;agent or person&gt;' with the plan. (2) During the work: a short comment at every milestone, decision, blocker or change of scope (what is done, what is next, what blocks), and a comment before any hand-over or stop. (3) At the end: a closing comment with what changed, files, tests run and not run, PR link, evidence for each 'Done when' item and open items for the owner. The same text goes in the PR description. An issue without a current report is not moved to In Review or Done. Never put a secret value in a report (mask to two characters at most).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Study existing tasks before adding one</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Owner decision 2026-10-26: before adding a task (backlog row and Jira issue) read the existing ones - search the backlog and Jira by area, files, goal and keywords, including Done and Hold rows. If an existing task covers the work or can absorb it, modify that task (extend What to do / Done when, update the workbook row, the Jira issue and a comment saying what changed and why) instead of adding a new one. Add a new row only when no task fits, and name the tasks that were checked in its Evidence. A new row keeps the next free Plan ID; held (Hold) tasks count as not open.</t>
         </is>
       </c>
     </row>
@@ -12839,7 +12901,11 @@
           <t>Done when: the report exists; HEAD is clean; every historical finding has a decision and an owner.</t>
         </is>
       </c>
-      <c r="K10" s="8" t="n"/>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>Merged 2026-10-26 (PR atapems-tech/PEMS#6, merge bc717dc): HEAD and full history (202 commits, all refs) scanned; no tokens, keys or real connection strings; five built-in passwords found and removed from HEAD (default administrator, employee-created users, compose SQL sa fallback, load-test accounts, weak example); rotation list and runbook handed to #317; held follow-ups #374 and #375; open items in docs/audits/SECRETS_AUDIT_2026-10.md. Tests NOT run (no .NET SDK): the row is Done only after the build and the new tests pass.</t>
+        </is>
+      </c>
       <c r="L10" s="10" t="inlineStr">
         <is>
           <t>M0</t>
@@ -22721,12 +22787,12 @@
       </c>
       <c r="I120" s="8" t="inlineStr">
         <is>
-          <t>A package content control script.</t>
+          <t>A package content control script. Extend the scan to everything handed to a customer or auditor (package, docs, sources): internal IP addresses, host names and SSH or service account names (audit finding S-6: 192.168.1.x addresses and an SSH account in deploy/caddy/Caddyfile, docs/audits/* and docs/deployment/*), and run a secrets scan (gitleaks, MIT licence) over the delivery.</t>
         </is>
       </c>
       <c r="J120" s="8" t="inlineStr">
         <is>
-          <t>A release with a disallowed file fails.</t>
+          <t>A release with a disallowed file fails. A delivery that contains an internal address, account name or secret fails the scan.</t>
         </is>
       </c>
       <c r="K120" s="8" t="n"/>
@@ -40031,12 +40097,12 @@
       </c>
       <c r="I318" s="8" t="inlineStr">
         <is>
-          <t>Rotate the demo FTP and demo database passwords; add DEMO_FTP_*, DEMO_SQL_CONNECTION_STRING, DEMO_ADMIN_PASSWORD and DEMO_SITE_URL as GitHub secrets; set the Kangan domain and name in env/production-kangan.env; create env/production-kangan.secrets.env (mode 600) on the server; change the default admin password on every existing database.</t>
+          <t>Rotate the demo FTP and demo database passwords; add DEMO_FTP_*, DEMO_SQL_CONNECTION_STRING, DEMO_ADMIN_PASSWORD and DEMO_SITE_URL as GitHub secrets; set the Kangan domain and name in env/production-kangan.env; create env/production-kangan.secrets.env (mode 600) on the server; change the default admin password on every existing database. 6) Rotate the exposed built-in credentials found by the SCRUM-17 audit with docs/deployment/CREDENTIAL_ROTATION_RUNBOOK.md and scripts/security/Report-DefaultCredentialExposure.sql on every environment (administrator account, employee-created users, SQL sa of containers from the old compose file, loadtest accounts, developer secrets files). 7) Set AllowedHosts in every non-local env file (production-kangan, demo, staging, uat) to the real host names instead of * (audit finding S-5).</t>
         </is>
       </c>
       <c r="J318" s="8" t="inlineStr">
         <is>
-          <t>No still-valid secret remains in the repository, its history or chat; the demo pipeline runs with GitHub secrets only.</t>
+          <t>No still-valid secret remains in the repository, its history or chat; the demo pipeline runs with GitHub secrets only. The exposure report shows only recognised accounts with changed passwords; AllowedHosts is not * in any non-local env file.</t>
         </is>
       </c>
       <c r="K318" s="8" t="n"/>
@@ -40057,7 +40123,7 @@
       </c>
       <c r="O318" s="10" t="inlineStr">
         <is>
-          <t>#315 #295</t>
+          <t>#315 #295 #9</t>
         </is>
       </c>
       <c r="P318" s="10" t="n"/>
@@ -40116,12 +40182,12 @@
       </c>
       <c r="I319" s="8" t="inlineStr">
         <is>
-          <t>Search Program.cs and the services for numeric/string literals, decide per item, move the settings into every env file with Required* and a test, and record the policy constants in a short document.</t>
+          <t>Search Program.cs and the services for numeric/string literals, decide per item, move the settings into every env file with Required* and a test, and record the policy constants in a short document. Include the production default password policy (audit finding S-5: every env file has length 8 and no upper-case or symbol requirement today): decide the product default and the per-customer override, set it in env/production-kangan.env and record it in the document. The file-store and upload folder paths are handled by #379 and are excluded here.</t>
         </is>
       </c>
       <c r="J319" s="8" t="inlineStr">
         <is>
-          <t>A list of each remaining literal with its classification; settings moved; tests keep the key sets identical.</t>
+          <t>A list of each remaining literal with its classification; settings moved; tests keep the key sets identical. The production password-policy default is decided, recorded and set in the production env file.</t>
         </is>
       </c>
       <c r="K319" s="8" t="n"/>

</xml_diff>

<commit_message>
SCRUM-335 feat(config): second pass over in-code constants, production password policy
- docs/design/CONFIGURATION_CONSTANTS.md: setting / policy constant / domain rule / tuning classification of the remaining literals
- new settings in all six env files (values equal today's behaviour): Hosting__HstsMaxAgeDays, Authentication__Cookie__SlidingExpiration, Database__MigrationCommandTimeoutMinutes; read with Required* in Program.cs
- DatabaseUpdateService takes the migration command timeout as an optional constructor parameter; the host passes the setting
- env/production-kangan.env: password minimum length 12 (decision S-5); EnvironmentFilesTests gains a policy test
- plan row #318 Report, Supportability Matrix SM-37, CHANGELOG, learnings-log

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1576,7 +1576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3280,6 +3280,53 @@
       <c r="I40" s="8" t="inlineStr">
         <is>
           <t>Implemented 2026-10-26 (SCRUM-17); status becomes Done when the build and EnvironmentFilesTests and TemporaryPasswordGeneratorTests have run green. Environments created before 2026-10-23 need rotation (#317); the old values stay in git history (#374, on hold).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>SM-37</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Production password policy</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Core / env files</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Production installations: minimum length 12, digit required, no upper-case/symbol rule, lockout 5 attempts / 10 minutes; other environments keep length 8</t>
+        </is>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G41" s="10" t="inlineStr">
+        <is>
+          <t>Supported (unverified)</t>
+        </is>
+      </c>
+      <c r="H41" s="10" t="inlineStr">
+        <is>
+          <t>#318 #9</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>Decision 2026-10-26 (NIST SP 800-63B, OWASP ASVS V2). HSTS age, cookie sliding expiry and the migration command timeout are settings. Unverified until EnvironmentFilesTests have run.</t>
         </is>
       </c>
     </row>
@@ -40190,7 +40237,11 @@
           <t>A list of each remaining literal with its classification; settings moved; tests keep the key sets identical. The production password-policy default is decided, recorded and set in the production env file.</t>
         </is>
       </c>
-      <c r="K319" s="8" t="n"/>
+      <c r="K319" s="8" t="inlineStr">
+        <is>
+          <t>Second pass done 2026-10-26: every option literal in Program.cs, controllers and services classified in docs/design/CONFIGURATION_CONSTANTS.md (setting / policy constant / domain rule / tuning with trigger). Moved to all six env files: Hosting__HstsMaxAgeDays, Authentication__Cookie__SlidingExpiration, Database__MigrationCommandTimeoutMinutes (values equal to today's behaviour). Production password policy decided: length 12, no composition rules (env/production-kangan.env). Tests: EnvironmentFilesTests (key parity + new policy test) NOT run - no .NET SDK; run before Done.</t>
+        </is>
+      </c>
       <c r="L319" s="10" t="inlineStr">
         <is>
           <t>M3</t>

</xml_diff>

<commit_message>
SCRUM-14 docs(plan): point backlog rows #2, #4, #5, #96, #97, #300, #309, #315 at their ADRs
Report column updated in the workbook; plan/backlog.csv regenerated with plan_sync export (check: 0 findings).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$350</definedName>
@@ -12501,7 +12501,11 @@
           <t>Done when: plan/adr contains the template and six ADRs approved by Member A; every backlog row marked decided points to its ADR.</t>
         </is>
       </c>
-      <c r="K3" s="8" t="n"/>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Added plan/adr: TEMPLATE.md, README index and ADR-0001..0006 (hybrid storage, Razor + PEMS.UI, code-first database, env/secrets files, licensing threat model + VM policy, demo/staging branch policy), each linked from its explaining doc. Merged in atapems-tech/PEMS#4. No Supportability Matrix change.</t>
+        </is>
+      </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
           <t>M0</t>
@@ -12689,7 +12693,8 @@
       </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>Decided 2026-10-18: hybrid - real SQL tables for fully user-built entities, one JSON column for custom fields on existing entities. Prototype validation happens in D_DDL/D_SCHEMA; ADR to be written under F_ADR.</t>
+          <t>Decided 2026-10-18: hybrid - real SQL tables for fully user-built entities, one JSON column for custom fields on existing entities. Prototype validation happens in D_DDL/D_SCHEMA; ADR to be written under F_ADR.
+ADR: plan/adr/0001-hybrid-storage-for-user-built-entities.md</t>
         </is>
       </c>
       <c r="L5" s="10" t="inlineStr">
@@ -12778,7 +12783,8 @@
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>Decided 2026-10-18: keep Razor and build a reusable component library, with the form/workflow designers as embedded JavaScript components. ADR to be written under F_ADR. 2026-10-23: refined in docs/design/COMPONENT_LIBRARY_PLAN.md - separate Razor Class Library PEMS.UI (decided); canonical technology recommended as descriptor-driven static Razor components with an MVC Tag Helper facade, gated by spike #319 (the vertical-slice comparison this row asked for was never run).</t>
+          <t>Decided 2026-10-18: keep Razor and build a reusable component library, with the form/workflow designers as embedded JavaScript components. ADR to be written under F_ADR. 2026-10-23: refined in docs/design/COMPONENT_LIBRARY_PLAN.md - separate Razor Class Library PEMS.UI (decided); canonical technology recommended as descriptor-driven static Razor components with an MVC Tag Helper facade, gated by spike #319 (the vertical-slice comparison this row asked for was never run).
+ADR: plan/adr/0002-razor-with-separate-pems-ui-library.md (component technology D3 still open, spike #319)</t>
         </is>
       </c>
       <c r="L6" s="10" t="inlineStr">
@@ -20925,7 +20931,8 @@
       </c>
       <c r="K97" s="8" t="inlineStr">
         <is>
-          <t>Decided 2026-10-18: casual-copy defense plus contract - machine fingerprint, install seal, signed licence, restore-detection counter, code obfuscation and strong EULA. No hardware token. ADR to be written under F_ADR.</t>
+          <t>Decided 2026-10-18: casual-copy defense plus contract - machine fingerprint, install seal, signed licence, restore-detection counter, code obfuscation and strong EULA. No hardware token. ADR to be written under F_ADR.
+ADR: plan/adr/0005-licensing-threat-model-and-vm-policy.md</t>
         </is>
       </c>
       <c r="L97" s="10" t="inlineStr">
@@ -21018,7 +21025,8 @@
       </c>
       <c r="K98" s="8" t="inlineStr">
         <is>
-          <t>Decided 2026-10-18: VMs and Docker are allowed with extra protection (virtual TPM/hypervisor ID where available, restore-detection counter, no-cloning EULA clause).</t>
+          <t>Decided 2026-10-18: VMs and Docker are allowed with extra protection (virtual TPM/hypervisor ID where available, restore-detection counter, no-cloning EULA clause).
+ADR: plan/adr/0005-licensing-threat-model-and-vm-policy.md</t>
         </is>
       </c>
       <c r="L98" s="10" t="inlineStr">
@@ -38875,7 +38883,11 @@
           <t>The demo branch differs from main only by the overlay directory; a sync from main runs automatically and reports conflicts; a check fails any change on demo outside the overlay; no commit from demo is ever merged into main.</t>
         </is>
       </c>
-      <c r="K301" s="8" t="n"/>
+      <c r="K301" s="8" t="inlineStr">
+        <is>
+          <t>ADR: plan/adr/0006-demo-and-staging-branch-policy.md (overlay and automatic sync still planned)</t>
+        </is>
+      </c>
       <c r="L301" s="10" t="inlineStr">
         <is>
           <t>M0</t>
@@ -39642,7 +39654,8 @@
       </c>
       <c r="K310" s="8" t="inlineStr">
         <is>
-          <t>Local commits on branch temp/code-first-database: 'feat(database): fully code-first startup ...' and the follow-up 'feat(database): install-vs-update migrator, Admin Database Update page, legacy SQL retired, demo pipeline wired'. Not versioned (no system version yet - F_CI). Not pushed (no write grant).</t>
+          <t>Local commits on branch temp/code-first-database: 'feat(database): fully code-first startup ...' and the follow-up 'feat(database): install-vs-update migrator, Admin Database Update page, legacy SQL retired, demo pipeline wired'. Not versioned (no system version yet - F_CI). Not pushed (no write grant).
+ADR: plan/adr/0003-code-first-database.md</t>
         </is>
       </c>
       <c r="L310" s="10" t="inlineStr">
@@ -40168,7 +40181,8 @@
       </c>
       <c r="K316" s="8" t="inlineStr">
         <is>
-          <t>Local commits on branch temp/code-first-database ('feat(config): environment settings and secrets files ...'). Not pushed.</t>
+          <t>Local commits on branch temp/code-first-database ('feat(config): environment settings and secrets files ...'). Not pushed.
+ADR: plan/adr/0004-environment-and-secrets-files.md</t>
         </is>
       </c>
       <c r="L316" s="10" t="inlineStr">

</xml_diff>

<commit_message>
SCRUM-410: plan rows #380 and #381, changelog
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12226,7 +12226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U380"/>
+  <dimension ref="A1:U382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -45779,6 +45779,176 @@
       </c>
       <c r="T380" s="10" t="n"/>
       <c r="U380" s="10" t="n"/>
+    </row>
+    <row r="381">
+      <c r="A381" s="10" t="n">
+        <v>380</v>
+      </c>
+      <c r="B381" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C381" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D381" s="8" t="inlineStr">
+        <is>
+          <t>Guarantee that no deploy, update or migration resets or changes an existing administrator password (staging, demo, client servers): tests, guideline, runbooks</t>
+        </is>
+      </c>
+      <c r="E381" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F381" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G381" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H381" s="8" t="inlineStr">
+        <is>
+          <t>Owner requirement 2026-10-27. Code check: IdentitySeeder seeds only on an empty user table; DevAdminPasswordReset needs Development plus PEMS_DEV_RESET_ADMIN_PASSWORD=true; deploy-site.yml only writes the secrets file; the client update kit only swaps the container and runs the migration script. Nothing proved or documented it.</t>
+        </is>
+      </c>
+      <c r="I381" s="8" t="inlineStr">
+        <is>
+          <t>1) Regression tests (AdminPasswordSurvivesUpdateTests). 2) Rule in guideline chapter 01 security and in DEPLOYMENT_README section 9 and LINUX_VM_DEPLOYMENT. 3) Manual check M-14. 4) Extend #353, #169, #170 with the later part.</t>
+        </is>
+      </c>
+      <c r="J381" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the tests pass and fail if a seeder or deploy step starts changing an existing account; the guideline and both runbooks state the rule; the manual check exists; #353, #169 and #170 carry the extended Done-when.</t>
+        </is>
+      </c>
+      <c r="K381" s="8" t="n"/>
+      <c r="L381" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M381" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N381" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O381" s="10" t="inlineStr">
+        <is>
+          <t>#315</t>
+        </is>
+      </c>
+      <c r="P381" s="10" t="n"/>
+      <c r="Q381" s="10" t="n"/>
+      <c r="R381" s="8" t="inlineStr">
+        <is>
+          <t>Install &amp; update</t>
+        </is>
+      </c>
+      <c r="S381" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T381" s="10" t="n"/>
+      <c r="U381" s="10" t="n"/>
+    </row>
+    <row r="382">
+      <c r="A382" s="10" t="n">
+        <v>381</v>
+      </c>
+      <c r="B382" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C382" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D382" s="8" t="inlineStr">
+        <is>
+          <t>First-install administrator password: random one-time password the administrator can read once in the UI (fresh install, database reset, local dev, client server)</t>
+        </is>
+      </c>
+      <c r="E382" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F382" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G382" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H382" s="8" t="inlineStr">
+        <is>
+          <t>Owner question 2026-10-27: how does the administrator get the first random password in the UI? Today the administrator comes from Seed__Admin__Password in the secrets file; nothing shows a generated password, and after a database reset the first-install flow must restart.</t>
+        </is>
+      </c>
+      <c r="I382" s="8" t="inlineStr">
+        <is>
+          <t>Design to confirm: 1) empty user table and no Seed__Admin__Password: the seeder generates a random password and stores it Data-Protection encrypted in a one-time record (migration). 2) Pre-login page /first-install shows it once and deletes it; only from the server itself or the management networks, only while the administrator never signed in, rate limited, 404 otherwise (as break-glass, SCRUM-356). 3) Same flow after a database reset; 404 after an update. 4) Local run prints only a pointer to the page. 5) Reads go to Security Events.</t>
+        </is>
+      </c>
+      <c r="J382" s="8" t="inlineStr">
+        <is>
+          <t>Done when: fresh install, database reset and local first run each show the generated password once and force a change; a second view, a view after first sign-in, from another network and after an update answer 404; tests, README manual check, guideline and runbooks updated.</t>
+        </is>
+      </c>
+      <c r="K382" s="8" t="n"/>
+      <c r="L382" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M382" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N382" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O382" s="10" t="inlineStr">
+        <is>
+          <t>#380 #169</t>
+        </is>
+      </c>
+      <c r="P382" s="10" t="n"/>
+      <c r="Q382" s="10" t="n"/>
+      <c r="R382" s="8" t="inlineStr">
+        <is>
+          <t>Install &amp; update</t>
+        </is>
+      </c>
+      <c r="S382" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T382" s="10" t="n"/>
+      <c r="U382" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-412: plan row #382 password history
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12226,7 +12226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U382"/>
+  <dimension ref="A1:U383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -45949,6 +45949,91 @@
       </c>
       <c r="T382" s="10" t="n"/>
       <c r="U382" s="10" t="n"/>
+    </row>
+    <row r="383">
+      <c r="A383" s="10" t="n">
+        <v>382</v>
+      </c>
+      <c r="B383" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C383" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D383" s="8" t="inlineStr">
+        <is>
+          <t>Password history: a new password (forced first change, voluntary change, every reset) must differ from the current and the previous passwords</t>
+        </is>
+      </c>
+      <c r="E383" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F383" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G383" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H383" s="8" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-27: the password chosen at the first (forced) change and at any later change must not equal the previous one. ASP.NET Identity accepts the same password again, so the forced change of a one-time or temporary password can be answered with the same value.</t>
+        </is>
+      </c>
+      <c r="I383" s="8" t="inlineStr">
+        <is>
+          <t>1) Study the change-password, forced-change, admin reset, recovery-code and break-glass paths and the validators in use. 2) One IPasswordValidator shared by all paths: reject the current hash and the last N hashes (Authentication__Password__HistoryCount, default 5, in every env file; key-parity test green); the one-time or temporary password counts as current. 3) Store previous hashes (new table, migration; hashes only, trimmed to N). 4) Localized message fa/en. 5) Tests per path and for inside/outside N. 6) Document in env/README.md, guideline security rule, README manual check.</t>
+        </is>
+      </c>
+      <c r="J383" s="8" t="inlineStr">
+        <is>
+          <t>Done when: every path that sets a password refuses the current and the last N passwords with a clear message; the setting is in every env file; tests pass; manual check and docs exist.</t>
+        </is>
+      </c>
+      <c r="K383" s="8" t="n"/>
+      <c r="L383" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M383" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N383" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O383" s="10" t="inlineStr">
+        <is>
+          <t>#315</t>
+        </is>
+      </c>
+      <c r="P383" s="10" t="n"/>
+      <c r="Q383" s="10" t="n"/>
+      <c r="R383" s="8" t="inlineStr">
+        <is>
+          <t>Install &amp; update</t>
+        </is>
+      </c>
+      <c r="S383" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T383" s="10" t="n"/>
+      <c r="U383" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-413: migration chain gate on a real SQL Server and account-safety test (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12226,7 +12226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U383"/>
+  <dimension ref="A1:U384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -46034,6 +46034,91 @@
       </c>
       <c r="T383" s="10" t="n"/>
       <c r="U383" s="10" t="n"/>
+    </row>
+    <row r="384">
+      <c r="A384" s="10" t="n">
+        <v>383</v>
+      </c>
+      <c r="B384" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C384" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D384" s="8" t="inlineStr">
+        <is>
+          <t>Migration chain gate: every task that changes the model ships its migration, and the chain is applied and verified on a real SQL Server before any staging or demo upload; migrations and pipelines never touch accounts</t>
+        </is>
+      </c>
+      <c r="E384" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F384" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G384" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H384" s="8" t="inlineStr">
+        <is>
+          <t>Owner requirement 2026-10-27: after each task the proper migrations must run through the proper migrator, otherwise the database can break (also an updater requirement). The pipeline only runs the model-drift gate (no database); a migration that compiles but fails on SQL Server shows up only as a failed start / 503 on the site. build.yml is manual only.</t>
+        </is>
+      </c>
+      <c r="I384" s="8" t="inlineStr">
+        <is>
+          <t>1) scripts/ci/test-migration-chain.sh: install the chain on an empty SQL Server, upgrade from the last migration of the base ref, model agrees, failing migration named. 2) Workflow migration-chain.yml (manual + reusable, throw-away SQL Server container, no secrets). 3) Prove it on GitHub (green on head, red on a broken migration), then make deploy-site.yml depend on it. 4) AccountSafetyOfMigrationsAndPipelinesTests. 5) Guideline ch.01, CODE_FIRST_DATABASE.md, DEPLOYMENT_README.md, README M-15. 6) Extend #262 (Saber, SCRUM-280) after confirmation.</t>
+        </is>
+      </c>
+      <c r="J384" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the workflow passes on GitHub for head and fails with the migration name on a broken one; staging and demo deploys depend on it; the account-safety test passes; guideline and docs updated; #262 extended.</t>
+        </is>
+      </c>
+      <c r="K384" s="8" t="n"/>
+      <c r="L384" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M384" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N384" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O384" s="10" t="inlineStr">
+        <is>
+          <t>#309 #380</t>
+        </is>
+      </c>
+      <c r="P384" s="10" t="n"/>
+      <c r="Q384" s="10" t="n"/>
+      <c r="R384" s="8" t="inlineStr">
+        <is>
+          <t>Install &amp; update</t>
+        </is>
+      </c>
+      <c r="S384" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T384" s="10" t="n"/>
+      <c r="U384" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-14: record Member A approval of ADR-0001..0006 and update plan rows #2, #5, #319 (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12503,7 +12503,7 @@
       </c>
       <c r="K3" s="8" t="inlineStr">
         <is>
-          <t>Added plan/adr: TEMPLATE.md, README index and ADR-0001..0006 (hybrid storage, Razor + PEMS.UI, code-first database, env/secrets files, licensing threat model + VM policy, demo/staging branch policy), each linked from its explaining doc. Merged in atapems-tech/PEMS#4. No Supportability Matrix change.</t>
+          <t>Added plan/adr: TEMPLATE.md, README index and ADR-0001..0006 (hybrid storage, Razor + PEMS.UI, code-first database, env/secrets files, licensing threat model + VM policy, demo/staging branch policy), each linked from its explaining doc. Merged in atapems-tech/PEMS#4. Approved by Member A (Hamid Maleki) 2026-10-27. No Supportability Matrix change.</t>
         </is>
       </c>
       <c r="L3" s="10" t="inlineStr">
@@ -12784,7 +12784,8 @@
       <c r="K6" s="8" t="inlineStr">
         <is>
           <t>Decided 2026-10-18: keep Razor and build a reusable component library, with the form/workflow designers as embedded JavaScript components. ADR to be written under F_ADR. 2026-10-23: refined in docs/design/COMPONENT_LIBRARY_PLAN.md - separate Razor Class Library PEMS.UI (decided); canonical technology recommended as descriptor-driven static Razor components with an MVC Tag Helper facade, gated by spike #319 (the vertical-slice comparison this row asked for was never run).
-ADR: plan/adr/0002-razor-with-separate-pems-ui-library.md (component technology D3 still open, spike #319)</t>
+ADR: plan/adr/0002-razor-with-separate-pems-ui-library.md (component technology D3 still open, spike #319)
+ADR-0001..0006 approved by Member A 2026-10-27. Component technology (D3): spike #319 run 2026-10-27, see ADR-0007 (proposed, static Razor components + Tag Helper facade).</t>
         </is>
       </c>
       <c r="L6" s="10" t="inlineStr">
@@ -40528,7 +40529,11 @@
           <t>Done when: the ADR exists with the measured table and a clear decision; the contract classes compile; the decision is recorded in #5 and #320 can start. If static Razor components fail a criterion, the ADR names the fallback per component class.</t>
         </is>
       </c>
-      <c r="K320" s="8" t="n"/>
+      <c r="K320" s="8" t="inlineStr">
+        <is>
+          <t>Spike run 2026-10-27 (SCRUM-23, PR atapems-tech/PEMS#26): standalone PEMS.UI.Abstractions / PEMS.UI / PEMS.UI.Tests, 14 tests; ADR-0007 proposed: static Razor components + Tag Helper facade, measured vs View Components (rows in one component equal speed, per-cell 5-8x slower). Awaiting Member A approval of ADR-0007 before #320/#321 start.</t>
+        </is>
+      </c>
       <c r="L320" s="10" t="inlineStr">
         <is>
           <t>M0</t>

</xml_diff>

<commit_message>
SCRUM-414, SCRUM-415: plan rows #384 migration data-safety guard and #385 post-deploy proof and safe failure (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12226,7 +12226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U384"/>
+  <dimension ref="A1:U386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -46124,6 +46124,176 @@
       </c>
       <c r="T384" s="10" t="n"/>
       <c r="U384" s="10" t="n"/>
+    </row>
+    <row r="385">
+      <c r="A385" s="10" t="n">
+        <v>384</v>
+      </c>
+      <c r="B385" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C385" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D385" s="8" t="inlineStr">
+        <is>
+          <t>Migration data-safety guard: no standard migration may lose or change existing data (destructive-operation check, data-preservation upgrade test, pre-update backup)</t>
+        </is>
+      </c>
+      <c r="E385" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F385" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G385" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H385" s="8" t="inlineStr">
+        <is>
+          <t>Owner requirement 2026-10-27: all data, not only accounts and passwords, must be guarded against standard migrations. #383 proves the chain applies and does not touch accounts; it does not prove existing rows survive. A migration that drops or narrows a column, deletes reference data or truncates a table passes every current gate.</t>
+        </is>
+      </c>
+      <c r="I385" s="8" t="inlineStr">
+        <is>
+          <t>1) Static test: new migrations with DropTable, DropColumn, narrowing AlterColumn, NOT NULL without default, DeleteData, or Sql DELETE/TRUNCATE/DROP/UPDATE-without-WHERE need a marker comment data-loss-approved: SCRUM-xxx. 2) Chain gate: fill the base schema with representative rows, upgrade to head, compare row counts and checksums per table; name table and migration on loss. 3) Pre-update backup (Database__PreUpdateBackupFolder, recorded in DatabaseUpdateRuns; with #171). 4) Guideline ch.01, CODE_FIRST_DATABASE.md, README check.</t>
+        </is>
+      </c>
+      <c r="J385" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a scratch migration that drops a populated column or deletes rows fails the static guard and the gate with the table name; an approved destructive migration passes with its marker; a normal additive migration passes; the backup is taken or the update refuses; docs updated.</t>
+        </is>
+      </c>
+      <c r="K385" s="8" t="n"/>
+      <c r="L385" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M385" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N385" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O385" s="10" t="inlineStr">
+        <is>
+          <t>#383 #171</t>
+        </is>
+      </c>
+      <c r="P385" s="10" t="n"/>
+      <c r="Q385" s="10" t="n"/>
+      <c r="R385" s="8" t="inlineStr">
+        <is>
+          <t>Install &amp; update</t>
+        </is>
+      </c>
+      <c r="S385" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T385" s="10" t="n"/>
+      <c r="U385" s="10" t="n"/>
+    </row>
+    <row r="386">
+      <c r="A386" s="10" t="n">
+        <v>385</v>
+      </c>
+      <c r="B386" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C386" s="8" t="inlineStr">
+        <is>
+          <t>Installation, Deployment &amp; Updates</t>
+        </is>
+      </c>
+      <c r="D386" s="8" t="inlineStr">
+        <is>
+          <t>After a merge into staging or demo the migration must be proven applied, and a failed start-up migration must not crash or corrupt the site (post-deploy verification, safe failure mode, rollback path)</t>
+        </is>
+      </c>
+      <c r="E386" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F386" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G386" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H386" s="8" t="inlineStr">
+        <is>
+          <t>Owner requirement 2026-10-27: after a merge into staging or demo the migration must really run, otherwise the application crashes. The deploy polls /health/database for UpToDate, and #383 stops a chain that fails on SQL Server before upload, but UpToDate does not prove the newest migration of this commit is applied, a failed start-up migration stops the app, and no tested way back exists.</t>
+        </is>
+      </c>
+      <c r="I386" s="8" t="inlineStr">
+        <is>
+          <t>1) Post-deploy proof: the pipeline compares the newest applied migration id with the newest migration of the deployed commit and fails with both ids. 2) Safe failure mode: a failed or newer-than-build database leaves the app up in a maintenance state (static page, /health/database 503 with state name, failed attempt in DatabaseUpdateRuns); check every migration runs in a transaction and list the exceptions. 3) Rollback path documented and exercised (backup, previous build, restore). 4) Tests, README check.</t>
+        </is>
+      </c>
+      <c r="J386" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a deploy whose database ends on an older migration than the commit fails the run with both ids; a deliberately failing start-up migration on staging leaves the maintenance page and a 503 health state, not a crash loop, visible in Admin &gt; Database Update; rollback steps exercised once; docs updated.</t>
+        </is>
+      </c>
+      <c r="K386" s="8" t="n"/>
+      <c r="L386" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M386" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N386" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O386" s="10" t="inlineStr">
+        <is>
+          <t>#383 #309</t>
+        </is>
+      </c>
+      <c r="P386" s="10" t="n"/>
+      <c r="Q386" s="10" t="n"/>
+      <c r="R386" s="8" t="inlineStr">
+        <is>
+          <t>Install &amp; update</t>
+        </is>
+      </c>
+      <c r="S386" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T386" s="10" t="n"/>
+      <c r="U386" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-280 docs(plan): report for plan row #262
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -35668,7 +35668,11 @@
           <t>An automated job upgrades a database from every supported release to the candidate and verifies schema and data.</t>
         </is>
       </c>
-      <c r="K263" s="8" t="n"/>
+      <c r="K263" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27 SCRUM-280 (branch feature/SCRUM-280-db-upgrade-pipeline): deploy/db/supported-releases.json lists the releases to upgrade from (2026-10-22 self-installing build, 2026-10-25 demo) as exact migration sets; DatabaseUpgradePathSqlTests rebuilds each, fills 320+ tables with a representative row, upgrades with the real migrator and compares with a fresh install (schema) and row counts; a NOT NULL column without default is caught (fresh install passes, upgrade fails). Runs in the Migration Chain Gate workflow (SCRUM-413). Released migrations frozen by checksum (MigrationCompatibilityRulesTests); expand/contract rules in CODE_FIRST_DATABASE.md. Rollback = automatic COPY_ONLY pre-update backup (Database__BackupBeforeUpdate, on in production/uat) + documented restore, proven by a SQL test. SM-42.</t>
+        </is>
+      </c>
       <c r="L263" s="10" t="inlineStr">
         <is>
           <t>M2</t>

</xml_diff>

<commit_message>
SCRUM-29 SCRUM-23: PEMS.Web consumes PEMS.UI, move _KpiCard and loading overlay, accept ADR-0007 (hamid)
PEMS.Web references PEMS.UI (registry and renderer registered, tag helper available, pems-ui.css published but not linked). _KpiCard with KpiCardViewModel (namespace kept) and _PemsLoadingOverlay move into PEMS.UI; golden-output tests recorded on the unchanged code prove byte-identical output. ADR-0007 accepted by Member A. Registry, guideline, learnings, CHANGELOG and plan rows #319/#320 updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -40531,7 +40531,7 @@
       </c>
       <c r="K320" s="8" t="inlineStr">
         <is>
-          <t>Spike run 2026-10-27 (SCRUM-23, PR atapems-tech/PEMS#26): standalone PEMS.UI.Abstractions / PEMS.UI / PEMS.UI.Tests, 14 tests; ADR-0007 proposed: static Razor components + Tag Helper facade, measured vs View Components (rows in one component equal speed, per-cell 5-8x slower). Awaiting Member A approval of ADR-0007 before #320/#321 start.</t>
+          <t>Spike run 2026-10-27 (SCRUM-23, PR atapems-tech/PEMS#26): standalone PEMS.UI.Abstractions / PEMS.UI / PEMS.UI.Tests, 14 tests; ADR-0007 proposed: static Razor components + Tag Helper facade, measured vs View Components (rows in one component equal speed, per-cell 5-8x slower). ADR-0007 accepted by Member A 2026-10-27; #320 started.</t>
         </is>
       </c>
       <c r="L320" s="10" t="inlineStr">
@@ -40626,7 +40626,11 @@
           <t>Done when: the solution builds and the tests pass; the HTTP smoke tests still pass; PEMS.Web renders the same pages with its assets served from PEMS.UI.</t>
         </is>
       </c>
-      <c r="K321" s="8" t="n"/>
+      <c r="K321" s="8" t="inlineStr">
+        <is>
+          <t>Step 1 (SCRUM-29): PEMS.Web references PEMS.UI; component registry/renderer registered; pems-ui.css published (not linked); _KpiCard (+KpiCardViewModel) and _PemsLoadingOverlay moved with byte-identical output (golden tests PEMS.Tests/Ui). Open: PEMS.UI localisation, then _PageHeader and _Pagination (need PEMS.Web SharedResource), token file after #30. HTTP smoke tests need SQL Server and were not run in the cloud session.</t>
+        </is>
+      </c>
       <c r="L321" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-414, SCRUM-415: narrow plan rows #384 and #385 after SCRUM-280 merged (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$350</definedName>
@@ -1604,7 +1604,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -46193,7 +46192,7 @@
       </c>
       <c r="D385" s="8" t="inlineStr">
         <is>
-          <t>Migration data-safety guard: no standard migration may lose or change existing data (destructive-operation check, data-preservation upgrade test, pre-update backup)</t>
+          <t>Migration data-safety guard: destructive-operation check with an approval marker, and a value-level preservation check on top of the #262 upgrade tests</t>
         </is>
       </c>
       <c r="E385" s="10" t="inlineStr">
@@ -46213,17 +46212,17 @@
       </c>
       <c r="H385" s="8" t="inlineStr">
         <is>
-          <t>Owner requirement 2026-10-27: all data, not only accounts and passwords, must be guarded against standard migrations. #383 proves the chain applies and does not touch accounts; it does not prove existing rows survive. A migration that drops or narrows a column, deletes reference data or truncates a table passes every current gate.</t>
+          <t>Owner requirement 2026-10-27: all data, not only accounts and passwords, must be guarded against standard migrations. #383 proves the chain applies and does not touch accounts; it does not prove existing rows survive. A migration that drops or narrows a column, deletes reference data or truncates a table passes every current gate. 2026-10-27 after #262 (SCRUM-280, merged): the per-release upgrade test already fills tables, checks that no table lost rows, that the schema equals a fresh install and that nothing is pending, and a pre-update backup exists (Database__BackupBeforeUpdate). Not covered: a migration that rewrites or nulls values keeps the row count, and a destructive operation is not flagged for approval before it is merged.</t>
         </is>
       </c>
       <c r="I385" s="8" t="inlineStr">
         <is>
-          <t>1) Static test: new migrations with DropTable, DropColumn, narrowing AlterColumn, NOT NULL without default, DeleteData, or Sql DELETE/TRUNCATE/DROP/UPDATE-without-WHERE need a marker comment data-loss-approved: SCRUM-xxx. 2) Chain gate: fill the base schema with representative rows, upgrade to head, compare row counts and checksums per table; name table and migration on loss. 3) Pre-update backup (Database__PreUpdateBackupFolder, recorded in DatabaseUpdateRuns; with #171). 4) Guideline ch.01, CODE_FIRST_DATABASE.md, README check.</t>
+          <t>1) Static test: new migrations (not in deploy/db/released-migrations.sha256) with DropTable, DropColumn, narrowing AlterColumn, NOT NULL without default, DeleteData, or Sql DELETE/TRUNCATE/DROP/UPDATE-without-WHERE need a marker comment data-loss-approved: SCRUM-xxx; the guideline says who approves. 2) Extend DatabaseUpgradePathSqlTests: compare a per-table checksum of the unchanged columns before and after the upgrade (rows are kept but values must not change); name table and migration. 3) Guideline ch.01, CODE_FIRST_DATABASE.md, README check. Backup and rollback are done by #262 and are not repeated.</t>
         </is>
       </c>
       <c r="J385" s="8" t="inlineStr">
         <is>
-          <t>Done when: a scratch migration that drops a populated column or deletes rows fails the static guard and the gate with the table name; an approved destructive migration passes with its marker; a normal additive migration passes; the backup is taken or the update refuses; docs updated.</t>
+          <t>Done when: a scratch migration that nulls or rewrites a populated column fails the checksum check with the table name; one that drops a populated column or deletes rows fails the static guard; an approved destructive migration passes with its marker; a normal additive migration passes; docs updated.</t>
         </is>
       </c>
       <c r="K385" s="8" t="n"/>
@@ -46234,7 +46233,7 @@
       </c>
       <c r="M385" s="10" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="N385" s="10" t="inlineStr">
@@ -46244,7 +46243,7 @@
       </c>
       <c r="O385" s="10" t="inlineStr">
         <is>
-          <t>#383 #171</t>
+          <t>#383 #262</t>
         </is>
       </c>
       <c r="P385" s="10" t="n"/>
@@ -46278,7 +46277,7 @@
       </c>
       <c r="D386" s="8" t="inlineStr">
         <is>
-          <t>After a merge into staging or demo the migration must be proven applied, and a failed start-up migration must not crash or corrupt the site (post-deploy verification, safe failure mode, rollback path)</t>
+          <t>After a merge into staging or demo the migration must be proven applied, and a failed start-up migration must not crash the site (post-deploy proof, safe failure mode)</t>
         </is>
       </c>
       <c r="E386" s="10" t="inlineStr">
@@ -46298,17 +46297,17 @@
       </c>
       <c r="H386" s="8" t="inlineStr">
         <is>
-          <t>Owner requirement 2026-10-27: after a merge into staging or demo the migration must really run, otherwise the application crashes. The deploy polls /health/database for UpToDate, and #383 stops a chain that fails on SQL Server before upload, but UpToDate does not prove the newest migration of this commit is applied, a failed start-up migration stops the app, and no tested way back exists.</t>
+          <t>Owner requirement 2026-10-27: after a merge into staging or demo the migration must really run, otherwise the application crashes. The deploy polls /health/database for UpToDate, and #383 stops a chain that fails on SQL Server before upload, but UpToDate does not prove the newest migration of this commit is applied, a failed start-up migration stops the app, and no tested way back exists. 2026-10-27 after #262 (SCRUM-280, merged): the rollback procedure with the automatic pre-update backup and a restore test now exist (CODE_FIRST_DATABASE.md "Rollback"), so only the proof and the failure mode remain here.</t>
         </is>
       </c>
       <c r="I386" s="8" t="inlineStr">
         <is>
-          <t>1) Post-deploy proof: the pipeline compares the newest applied migration id with the newest migration of the deployed commit and fails with both ids. 2) Safe failure mode: a failed or newer-than-build database leaves the app up in a maintenance state (static page, /health/database 503 with state name, failed attempt in DatabaseUpdateRuns); check every migration runs in a transaction and list the exceptions. 3) Rollback path documented and exercised (backup, previous build, restore). 4) Tests, README check.</t>
+          <t>1) Post-deploy proof: the pipeline compares the newest applied migration id with the newest migration of the deployed commit and fails with both ids. 2) Safe failure mode: a failed or newer-than-build database leaves the app up in a maintenance state (static page, /health/database 503 with state name, failed attempt in DatabaseUpdateRuns); check every migration runs in a transaction and list the exceptions. 3) The pipeline run summary prints the previous good commit and links the #262 rollback steps. 4) Tests, README check.</t>
         </is>
       </c>
       <c r="J386" s="8" t="inlineStr">
         <is>
-          <t>Done when: a deploy whose database ends on an older migration than the commit fails the run with both ids; a deliberately failing start-up migration on staging leaves the maintenance page and a 503 health state, not a crash loop, visible in Admin &gt; Database Update; rollback steps exercised once; docs updated.</t>
+          <t>Done when: a deploy whose database ends on an older migration than the commit fails the run with both ids; a deliberately failing start-up migration on staging leaves the maintenance page and a 503 health state, not a crash loop, visible in Admin &gt; Database Update; docs updated.</t>
         </is>
       </c>
       <c r="K386" s="8" t="n"/>
@@ -46329,7 +46328,7 @@
       </c>
       <c r="O386" s="10" t="inlineStr">
         <is>
-          <t>#383 #309</t>
+          <t>#383 #309 #262</t>
         </is>
       </c>
       <c r="P386" s="10" t="n"/>

</xml_diff>

<commit_message>
SCRUM-413: plan row #383 reflects the confirmed SCRUM-280 slice and the proof runs (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -46132,12 +46132,12 @@
       </c>
       <c r="I384" s="8" t="inlineStr">
         <is>
-          <t>1) scripts/ci/test-migration-chain.sh: install the chain on an empty SQL Server, upgrade from the last migration of the base ref, model agrees, failing migration named. 2) Workflow migration-chain.yml (manual + reusable, throw-away SQL Server container, no secrets). 3) Prove it on GitHub (green on head, red on a broken migration), then make deploy-site.yml depend on it. 4) AccountSafetyOfMigrationsAndPipelinesTests. 5) Guideline ch.01, CODE_FIRST_DATABASE.md, DEPLOYMENT_README.md, README M-15. 6) Extend #262 (Saber, SCRUM-280) after confirmation.</t>
+          <t>1) scripts/ci/test-migration-chain.sh: install the chain on an empty SQL Server, upgrade from the last migration of the base ref, model agrees, failing migration named. 2) Workflow migration-chain.yml (manual + reusable, throw-away SQL Server container, no secrets). 3) Prove it on GitHub (green on head, red on a broken migration), then make deploy-site.yml depend on it. 4) AccountSafetyOfMigrationsAndPipelinesTests. 5) Guideline ch.01, CODE_FIRST_DATABASE.md, DEPLOYMENT_README.md, README M-15. 6) #262 (SCRUM-280, Saber) confirmed this as its near-term slice and extended the same workflow with the data upgrade tests, the pre-update backup and the rollback (merged 2026-10-27); follow-ups narrowed to #384 and #385.</t>
         </is>
       </c>
       <c r="J384" s="8" t="inlineStr">
         <is>
-          <t>Done when: the workflow passes on GitHub for head and fails with the migration name on a broken one; staging and demo deploys depend on it; the account-safety test passes; guideline and docs updated; #262 extended.</t>
+          <t>Done when: the workflow passes on GitHub for head and fails with the migration name on a broken one; staging and demo deploys depend on it; the account-safety test passes; guideline and docs updated. Evidence: green run 40483241640, red run 40484730111; the first real staging/demo deploy through the wired job is still to be seen (QA).</t>
         </is>
       </c>
       <c r="K384" s="8" t="n"/>

</xml_diff>

<commit_message>
SCRUM-29: plan rows #319 and #320 Report after step 1 (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -40582,7 +40582,7 @@
       </c>
       <c r="K320" s="8" t="inlineStr">
         <is>
-          <t>Spike run 2026-10-27 (SCRUM-23, PR atapems-tech/PEMS#26): standalone PEMS.UI.Abstractions / PEMS.UI / PEMS.UI.Tests, 14 tests; ADR-0007 proposed: static Razor components + Tag Helper facade, measured vs View Components (rows in one component equal speed, per-cell 5-8x slower). Awaiting Member A approval of ADR-0007 before #320/#321 start.</t>
+          <t>Spike run 2026-10-27 (SCRUM-23, PR atapems-tech/PEMS#26): standalone PEMS.UI.Abstractions / PEMS.UI / PEMS.UI.Tests, 14 tests; ADR-0007 proposed: static Razor components + Tag Helper facade, measured vs View Components (rows in one component equal speed, per-cell 5-8x slower). ADR-0007 accepted by Member A 2026-10-27; #320 started.</t>
         </is>
       </c>
       <c r="L320" s="10" t="inlineStr">
@@ -40677,7 +40677,11 @@
           <t>Done when: the solution builds and the tests pass; the HTTP smoke tests still pass; PEMS.Web renders the same pages with its assets served from PEMS.UI.</t>
         </is>
       </c>
-      <c r="K321" s="8" t="n"/>
+      <c r="K321" s="8" t="inlineStr">
+        <is>
+          <t>Step 1 (SCRUM-29, PR atapems-tech/PEMS#30): PEMS.Web references PEMS.UI; component registry/renderer registered; pems-ui.css published (not linked); _KpiCard (+KpiCardViewModel) and _PemsLoadingOverlay moved with byte-identical output (golden tests PEMS.Tests/Ui). Open: PEMS.UI localisation, then _PageHeader and _Pagination (need PEMS.Web SharedResource), token file after #30. HTTP smoke tests need SQL Server and were not run in the cloud session.</t>
+        </is>
+      </c>
       <c r="L321" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-416: plan rows #386-#389 for translatable component texts and scope notes on #321, #322, #327 (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12273,7 +12273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U386"/>
+  <dimension ref="A1:U390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -40766,7 +40766,7 @@
       </c>
       <c r="I322" s="8" t="inlineStr">
         <is>
-          <t>Define the descriptors and a renderer that maps a descriptor to a component by type; keep them free of Razor/MVC types.</t>
+          <t>Define the descriptors and a renderer that maps a descriptor to a component by type; keep them free of Razor/MVC types. Scope note 2026-10-27 (ADR-0008): label, help, placeholder, option and error texts in the descriptors are TranslatableText, not strings (see #386).</t>
         </is>
       </c>
       <c r="J322" s="8" t="inlineStr">
@@ -40851,7 +40851,7 @@
       </c>
       <c r="I323" s="8" t="inlineStr">
         <is>
-          <t>Implement each field as a component with MVC model binding and unobtrusive validation parity, localization keys and accessibility per the Definition of Done.</t>
+          <t>Implement each field as a component with MVC model binding and unobtrusive validation parity, localization keys and accessibility per the Definition of Done. Scope note 2026-10-27 (ADR-0008): no literal text in the field components; all texts are TranslatableText inputs and values are formatted by culture (see #386); replaces 'localization keys'.</t>
         </is>
       </c>
       <c r="J323" s="8" t="inlineStr">
@@ -41276,7 +41276,7 @@
       </c>
       <c r="I328" s="8" t="inlineStr">
         <is>
-          <t>Add the tests and a baseline file; fail CI when a count rises or a CDN reference appears; lower the baseline after each wave.</t>
+          <t>Add the tests and a baseline file; fail CI when a count rises or a CDN reference appears; lower the baseline after each wave. Scope note 2026-10-27 (ADR-0008): the gates include 'no literal user-visible text in a PEMS.UI component' (first version in #386).</t>
         </is>
       </c>
       <c r="J328" s="8" t="inlineStr">
@@ -46349,6 +46349,354 @@
       </c>
       <c r="T386" s="10" t="n"/>
       <c r="U386" s="10" t="n"/>
+    </row>
+    <row r="387">
+      <c r="A387" s="10" t="n">
+        <v>386</v>
+      </c>
+      <c r="B387" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C387" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D387" s="8" t="inlineStr">
+        <is>
+          <t>Translatable text and locale contract for PEMS.UI: every user-visible text is a component input (TranslatableText, JSON map of language slug to text); components hold no literal text; values are formatted by culture, not translated</t>
+        </is>
+      </c>
+      <c r="E387" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F387" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G387" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H387" s="8" t="inlineStr">
+        <is>
+          <t>Owner requirement 2026-10-27: the texts a component shows (labels, placeholders, help, notes, errors, empty and loading texts) are inputs of the component and later come from the database form tables, one row per form, as JSON that maps a language slug to the text. User-entered data is never translated, only formatted (dates, numbers). Today _PageHeader and _Pagination read PEMS.Web SharedResource, so the library cannot own text.</t>
+        </is>
+      </c>
+      <c r="I387" s="8" t="inlineStr">
+        <is>
+          <t>1) TranslatableText in PEMS.UI.Abstractions: immutable, JSON {"fa":"..","en":".."}, fallback chain (culture, neutral language, default language, language-neutral, first). 2) IPemsLocale: text resolution plus value formatting by culture (Jalali dates for fa, numbers). 3) Descriptors and every PEMS.UI component take TranslatableText inputs and hold no literal text; a test fails when one is added. 4) JSON round trip of FormDefinition and ViewDescriptor. 5) ADR-0008 and the guideline rule. SCRUM-416.</t>
+        </is>
+      </c>
+      <c r="J387" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a FormDefinition loaded from JSON renders in fa and en with no text in the component code; a test fails when a literal text is added to a PEMS.UI component; dates and numbers follow the culture; ADR-0008 is accepted.</t>
+        </is>
+      </c>
+      <c r="K387" s="8" t="n"/>
+      <c r="L387" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M387" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N387" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O387" s="10" t="inlineStr">
+        <is>
+          <t>#320 #321</t>
+        </is>
+      </c>
+      <c r="P387" s="10" t="n"/>
+      <c r="Q387" s="10" t="n"/>
+      <c r="R387" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S387" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T387" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="U387" s="10" t="inlineStr">
+        <is>
+          <t>Member A</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="10" t="n">
+        <v>387</v>
+      </c>
+      <c r="B388" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C388" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D388" s="8" t="inlineStr">
+        <is>
+          <t>Hydrate the UI descriptors from the database: form table with JSON TranslatableText columns, loader, cache and invalidation, to and from the descriptor contract</t>
+        </is>
+      </c>
+      <c r="E388" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F388" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G388" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H388" s="8" t="inlineStr">
+        <is>
+          <t>ADR-0008: component texts are inputs. In the dynamic BPMS the form definition and its translations live in the database (one form row, texts as JSON per language slug) and must fill and be written back from the components without component changes.</t>
+        </is>
+      </c>
+      <c r="I388" s="8" t="inlineStr">
+        <is>
+          <t>Design the form, field, option and view tables with the registry (#10); JSON columns typed as TranslatableText; a loader to FormDefinition and ViewDescriptor; cache with invalidation on designer save; a migration (never edit an applied one); central row-level filter. SCRUM-417.</t>
+        </is>
+      </c>
+      <c r="J388" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a form created in the database renders through PEMS.UI in fa and en with no deploy; a saved translation shows on the next request; tests prove the round trip and the fallback.</t>
+        </is>
+      </c>
+      <c r="K388" s="8" t="n"/>
+      <c r="L388" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M388" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N388" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O388" s="10" t="inlineStr">
+        <is>
+          <t>#386 #10 #334</t>
+        </is>
+      </c>
+      <c r="P388" s="10" t="n"/>
+      <c r="Q388" s="10" t="n"/>
+      <c r="R388" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S388" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T388" s="10" t="n"/>
+      <c r="U388" s="10" t="n"/>
+    </row>
+    <row r="389">
+      <c r="A389" s="10" t="n">
+        <v>388</v>
+      </c>
+      <c r="B389" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C389" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D389" s="8" t="inlineStr">
+        <is>
+          <t>Move _PageHeader and _Pagination into PEMS.UI with their texts as inputs; PEMS.Web supplies the texts (adapter over SharedResource) until the form tables exist</t>
+        </is>
+      </c>
+      <c r="E389" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F389" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G389" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H389" s="8" t="inlineStr">
+        <is>
+          <t>Step 1 of #320 could not move these partials: they read PEMS.Web SharedResource and PaginationViewModel; _Pagination is used by 54 pages. ADR-0008: the library never looks texts up, the host passes them in.</t>
+        </is>
+      </c>
+      <c r="I389" s="8" t="inlineStr">
+        <is>
+          <t>Neutral view models and TranslatableText inputs in PEMS.UI; a thin PEMS.Web adapter fills the texts from SharedResource (English text is the key, as today); golden-output tests recorded on the unchanged partials in fa and en; database-free view tests before and after; HTTP smoke tests where SQL Server exists. SCRUM-418.</t>
+        </is>
+      </c>
+      <c r="J389" s="8" t="inlineStr">
+        <is>
+          <t>Done when: both partials live in PEMS.UI, the 54 pagination pages and every page header render byte-identically in fa and en, and PEMS.Web has no copy.</t>
+        </is>
+      </c>
+      <c r="K389" s="8" t="n"/>
+      <c r="L389" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M389" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N389" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O389" s="10" t="inlineStr">
+        <is>
+          <t>#386 #320</t>
+        </is>
+      </c>
+      <c r="P389" s="10" t="n"/>
+      <c r="Q389" s="10" t="n"/>
+      <c r="R389" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S389" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T389" s="10" t="n"/>
+      <c r="U389" s="10" t="n"/>
+    </row>
+    <row r="390">
+      <c r="A390" s="10" t="n">
+        <v>389</v>
+      </c>
+      <c r="B390" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C390" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D390" s="8" t="inlineStr">
+        <is>
+          <t>Translation completeness and preview in the designers: missing-language report per form, fallback preview, RTL and LTR preview</t>
+        </is>
+      </c>
+      <c r="E390" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F390" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G390" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H390" s="8" t="inlineStr">
+        <is>
+          <t>With texts stored per language in the database, a designer must see what is missing and what a user sees when a translation is absent.</t>
+        </is>
+      </c>
+      <c r="I390" s="8" t="inlineStr">
+        <is>
+          <t>Report of missing languages per form and field (TranslatableText.MissingLanguages), fallback preview per language, RTL/LTR preview with the request-free renderer. SCRUM-419.</t>
+        </is>
+      </c>
+      <c r="J390" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a designer sees every missing translation of a form and the preview in fa and en matches the page.</t>
+        </is>
+      </c>
+      <c r="K390" s="8" t="n"/>
+      <c r="L390" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M390" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N390" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O390" s="10" t="inlineStr">
+        <is>
+          <t>#387 #334</t>
+        </is>
+      </c>
+      <c r="P390" s="10" t="n"/>
+      <c r="Q390" s="10" t="n"/>
+      <c r="R390" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S390" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T390" s="10" t="n"/>
+      <c r="U390" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-20: offline PDF viewers (vendored pdf.js 4.0.379) and an external-URL check (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -16203,7 +16203,11 @@
           <t>Done when: no .cshtml references an external host; the PDF preview works offline in both viewers; the audit check runs in CI (#327 will reuse it).</t>
         </is>
       </c>
-      <c r="K43" s="8" t="n"/>
+      <c r="K43" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27 (SCRUM-20, Claude for Hamid): pdf.js 4.0.379 vendored under PEMS.Web/wwwroot/lib/pdfjs (npm pdfjs-dist, Apache-2.0, hashes in README-PEMS.txt); 4.x is ES-module only, so both viewers load it through wwwroot/js/pdfjs-loader.js. cdnjs references removed from Engineering Documents and VDR Details. OfflineAssetsTests (4) scan views, areas, PEMS.UI, wwwroot js/css for external hosts (allow-list: www.w3.org, learn.microsoft.com, www.iso.org placeholder); tools/UiAudit/pattern-audit.py exits 1 on a CDN reference. Tests: OfflineAssetsTests 4/4 and mutation (a cdnjs reference in a view fails it); audit script exit 1/0; Chromium with all external requests blocked rendered a PDF through the loader (0 external requests, 0 page errors); inline scripts parse as strict-mode modules. Not run: the two real pages in the running app (needs SQL Server and a login) - README M-17.</t>
+        </is>
+      </c>
       <c r="L43" s="10" t="inlineStr">
         <is>
           <t>M0</t>
@@ -23262,7 +23266,7 @@
       </c>
       <c r="K122" s="8" t="inlineStr">
         <is>
-          <t>PM 2026-10-18: simplified to a manual list plus lawyer check; automation moved to L_SBOMAUTO (Hold).</t>
+          <t>PM 2026-10-18: simplified to a manual list plus lawyer check; automation moved to L_SBOMAUTO (Hold). 2026-10-27: pdf.js 4.0.379 (pdfjs-dist, Apache-2.0, Mozilla) added to the front-end list - see PEMS.Web/wwwroot/lib/pdfjs/README-PEMS.txt.</t>
         </is>
       </c>
       <c r="L122" s="10" t="inlineStr">
@@ -41276,7 +41280,7 @@
       </c>
       <c r="I328" s="8" t="inlineStr">
         <is>
-          <t>Add the tests and a baseline file; fail CI when a count rises or a CDN reference appears; lower the baseline after each wave. Scope note 2026-10-27 (ADR-0008): the gates include 'no literal user-visible text in a PEMS.UI component' (first version in #386).</t>
+          <t>Add the tests and a baseline file; fail CI when a count rises or a CDN reference appears; lower the baseline after each wave. Scope note 2026-10-27 (ADR-0008): the gates include 'no literal user-visible text in a PEMS.UI component' (first version in #386). Reuse OfflineAssetsTests and the failing exit of tools/UiAudit/pattern-audit.py from #42 for the CDN gate.</t>
         </is>
       </c>
       <c r="J328" s="8" t="inlineStr">
@@ -41781,12 +41785,12 @@
       </c>
       <c r="H334" s="8" t="inlineStr">
         <is>
-          <t>Audit 2026-10-23. The CDN references break the offline rule and block a strict CSP.</t>
+          <t>Audit 2026-10-23. The CDN references break the offline rule and block a strict CSP. 2026-10-27: the pdf.js CDN references were removed by #42 (SCRUM-20); this row keeps the inline styles/scripts/style blocks and the CSP.</t>
         </is>
       </c>
       <c r="I334" s="8" t="inlineStr">
         <is>
-          <t>Vendor pdf.js under wwwroot/lib, move scripts into modules, enable CSP in report-only first.</t>
+          <t>pdf.js is vendored by #42 (SCRUM-20); move the other scripts into modules, enable CSP in report-only first.</t>
         </is>
       </c>
       <c r="J334" s="8" t="inlineStr">

</xml_diff>

<commit_message>
SCRUM-420 SCRUM-421: plan rows #390 (time zone, lowest priority) and #391 (Persian data-entry bug) (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12273,7 +12273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U390"/>
+  <dimension ref="A1:U392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -46701,6 +46701,176 @@
       </c>
       <c r="T390" s="10" t="n"/>
       <c r="U390" s="10" t="n"/>
+    </row>
+    <row r="391">
+      <c r="A391" s="10" t="n">
+        <v>390</v>
+      </c>
+      <c r="B391" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C391" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D391" s="8" t="inlineStr">
+        <is>
+          <t>Time-zone policy for displayed date-times: convert stored UTC values to the user's time zone in PEMS.UI</t>
+        </is>
+      </c>
+      <c r="E391" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F391" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G391" s="10" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H391" s="8" t="inlineStr">
+        <is>
+          <t>ADR-0008: IPemsLocale.Format shows date-times as given and does not convert time zones; stored values are UTC (Instructions rule 5). Owner decision 2026-10-27: not important now, backlog with the lowest priority.</t>
+        </is>
+      </c>
+      <c r="I391" s="8" t="inlineStr">
+        <is>
+          <t>Decide the policy (per-user or per-organisation time zone, server default, what a DateTimeOffset shows), add it to IPemsLocale or a companion, test daylight-saving transitions and the Persian and ISO formats; record it in an ADR. SCRUM-420.</t>
+        </is>
+      </c>
+      <c r="J391" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a UTC date-time stored in the database is shown in the configured time zone in tables and read-only fields, in fa and en, and the policy is recorded in an ADR.</t>
+        </is>
+      </c>
+      <c r="K391" s="8" t="n"/>
+      <c r="L391" s="10" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="M391" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N391" s="10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O391" s="10" t="inlineStr">
+        <is>
+          <t>#386</t>
+        </is>
+      </c>
+      <c r="P391" s="10" t="n"/>
+      <c r="Q391" s="10" t="n"/>
+      <c r="R391" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S391" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T391" s="10" t="n"/>
+      <c r="U391" s="10" t="n"/>
+    </row>
+    <row r="392">
+      <c r="A392" s="10" t="n">
+        <v>391</v>
+      </c>
+      <c r="B392" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C392" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D392" s="8" t="inlineStr">
+        <is>
+          <t>Persian pages reject decimal numbers from number inputs (12.5) and typed Persian digits; the fa culture expects the separator U+066B and Latin digits</t>
+        </is>
+      </c>
+      <c r="E392" s="10" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="F392" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G392" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H392" s="8" t="inlineStr">
+        <is>
+          <t>Found 2026-10-27 by the data-entry check of SCRUM-416 (PEMS.UI.Tests DataEntryUnaffectedTests): a number input posts 12.5, the fa culture decimal separator is U+066B, so the binder rejects 12.5 while 12 binds; typed Persian digits are rejected. Dates are safe because PEMS.Web keeps the Gregorian calendar on fa (Program.cs).</t>
+        </is>
+      </c>
+      <c r="I392" s="8" t="inlineStr">
+        <is>
+          <t>One rule for numeric and date input binding: type=number and type=date bind with the invariant culture, and Persian or Arabic-Indic digits and U+066B are normalised to Latin digits and a dot before parsing; implement where the field components live (#322) and apply it to PEMS.Web through one binder. SCRUM-421.</t>
+        </is>
+      </c>
+      <c r="J392" s="8" t="inlineStr">
+        <is>
+          <t>Done when: on a Persian page 12.5 (and 12٫5) and a date typed with Persian digits are accepted and stored as 12.5 and 2026-10-27; English pages are unchanged; the known-issue tests become regression tests.</t>
+        </is>
+      </c>
+      <c r="K392" s="8" t="n"/>
+      <c r="L392" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M392" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N392" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O392" s="10" t="inlineStr">
+        <is>
+          <t>#322</t>
+        </is>
+      </c>
+      <c r="P392" s="10" t="n"/>
+      <c r="Q392" s="10" t="n"/>
+      <c r="R392" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S392" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T392" s="10" t="n"/>
+      <c r="U392" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-412: password history - a new password must differ from the current and the last N (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -46063,7 +46063,11 @@
           <t>Done when: every path that sets a password refuses the current and the last N passwords with a clear message; the setting is in every env file; tests pass; manual check and docs exist.</t>
         </is>
       </c>
-      <c r="K383" s="8" t="n"/>
+      <c r="K383" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27 (SCRUM-412, Claude for Hamid): one mechanism for every password path. PasswordHistoryValidator (Identity IPasswordValidator, PEMS.Web.Security) refuses a password equal to the current hash or one of the last N stored hashes (Authentication__Password__HistoryCount, default 5, 0 = off, in all six env files); PemsUserManager overrides ChangePasswordAsync/ResetPasswordAsync and stores the replaced hash in the new table PasswordHistory (migration PasswordHistory, hashes only, trimmed to N). Message in fa and en (Password_Reused). DevAdminPasswordReset uses an explicit PasswordHistoryBypass. Tests: PasswordHistoryTests 9/9 (forced first change, voluntary change, inside/outside N, trimming, token reset, hashes only, count 0, bypass, no code assigns PasswordHash); mutation (validator off) turns 6 of 9 red. Not run: SQL Server migration gate result, the real screens in fa/en (README M-18).</t>
+        </is>
+      </c>
       <c r="L383" s="10" t="inlineStr">
         <is>
           <t>M2</t>

</xml_diff>

<commit_message>
SCRUM-337 feat(ui): list page tag helpers, pages, tests and docs (completes the previous commit, which only carried the file moves)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1576,7 +1576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3610,6 +3610,53 @@
       <c r="I47" s="8" t="inlineStr">
         <is>
           <t>Stage names in a contract cannot be renamed (labels can). Running instances are not migrated to a new version (SCRUM-90). Document, MOC and TQ status still come from stage names; switching them to BusinessStatus would free those names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>SM-44</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>List page component (frame, toolbar, filters, KPIs on demand, chips, grid)</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>PEMS.UI (pems-list-* tag helpers, pems-list.css/js)</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>One component for record list pages: full-window table with sticky header and bottom pager, one icon toolbar (search over the title with the shared autocomplete, filters dropdown with count badge, KPI row on demand remembered per browser, Excel, reset columns, New), removable filter chips, empty state with clear-all. Each page keeps its own columns, filters, actions and permissions. In use: Engineering Documents, VDR (wave 0).</t>
+        </is>
+      </c>
+      <c r="F48" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G48" s="10" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H48" s="10" t="inlineStr">
+        <is>
+          <t>SCRUM-337</t>
+        </is>
+      </c>
+      <c r="I48" s="8" t="inlineStr">
+        <is>
+          <t>Waves W1-W4 (document control, CMMS, warehouse/procurement, admin) still to move. Saved views, column picker, pinning and virtualization are SCRUM-54.</t>
         </is>
       </c>
     </row>
@@ -41000,7 +41047,11 @@
           <t>A list page is built from DataTable + FilterBar + StatusBadge + EmptyState + Skeleton only; 1,000 rows render within the budget set in #319.</t>
         </is>
       </c>
-      <c r="K324" s="8" t="n"/>
+      <c r="K324" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27 SCRUM-337 wave 0: list-page component in PEMS.UI (pems-list-* tag helpers, texts as inputs, pems-list.css/js moved from PEMS.Web); Engineering Documents and VDR built from it with no visible change. Waves W1-W4 move the other list pages (docs/design/LIST_PAGE_COMPONENT.md). InfoGrid, KpiTile, Chart and the skeleton family remain open. SM-44.</t>
+        </is>
+      </c>
       <c r="L324" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-411: first-run administrator setup - the administrator chooses the password as the last install step (plan rows #381 and #169, guideline) (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$350</definedName>
@@ -1604,7 +1604,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -27479,7 +27478,7 @@
       </c>
       <c r="H170" s="8" t="inlineStr">
         <is>
-          <t>A per-machine TLS certificate generated at first run, with no shipped private key (fail-closed), is a proven approach.</t>
+          <t>A per-machine TLS certificate generated at first run, with no shipped private key (fail-closed), is a proven approach. 2026-10-27: the administrator step is #381 (the administrator chooses the password as the last install step, guarded by a one-time setup code); this row keeps the wizard frame, licence, TLS and MFA steps.</t>
         </is>
       </c>
       <c r="I170" s="8" t="inlineStr">
@@ -45997,7 +45996,7 @@
       </c>
       <c r="D382" s="8" t="inlineStr">
         <is>
-          <t>First-install administrator password: random one-time password the administrator can read once in the UI (fresh install, database reset, local dev, client server)</t>
+          <t>First-run administrator setup: the administrator chooses the password in the UI as the last install step (fresh install, database reset, local dev, client server); the install is complete only after it</t>
         </is>
       </c>
       <c r="E382" s="10" t="inlineStr">
@@ -46017,17 +46016,17 @@
       </c>
       <c r="H382" s="8" t="inlineStr">
         <is>
-          <t>Owner question 2026-10-27: how does the administrator get the first random password in the UI? Today the administrator comes from Seed__Admin__Password in the secrets file; nothing shows a generated password, and after a database reset the first-install flow must restart.</t>
+          <t>Owner question 2026-10-27: how does the administrator get the first random password in the UI? Today the administrator comes from Seed__Admin__Password in the secrets file; nothing shows a generated password, and after a database reset the first-install flow must restart. 2026-10-27 owner decision: instead of generating, storing and revealing a random one-time password, the administrator sets the password in the UI as the last install step (no secret to generate or store, replaces the forced first change, uses the policy and the history rule of #382). This is the administrator step of the first-run wizard #169.</t>
         </is>
       </c>
       <c r="I382" s="8" t="inlineStr">
         <is>
-          <t>Design to confirm: 1) empty user table and no Seed__Admin__Password: the seeder generates a random password and stores it Data-Protection encrypted in a one-time record (migration). 2) Pre-login page /first-install shows it once and deletes it; only from the server itself or the management networks, only while the administrator never signed in, rate limited, 404 otherwise (as break-glass, SCRUM-356). 3) Same flow after a database reset; 404 after an update. 4) Local run prints only a pointer to the page. 5) Reads go to Security Events.</t>
+          <t>1) Condition: user table empty and no Seed__Admin__Password. Every request goes to /setup (static page) until done; staging and demo keep Seed__Admin__Password and skip it; an update never reaches it. 2) Guard against first-comer takeover: a one-time setup code written to a file next to the application and logged as a pointer only; /setup asks for it (optionally also server/management network only); rate limited; code and file deleted when the administrator exists; /setup is 404 afterwards. 3) Step: user name, e-mail, password (policy and history apply), confirm, sign in; MustChangePassword=false; the install is complete; licence/TLS/MFA steps of #169 attach to the same frame later. 4) After a database reset the page appears again with a new code. 5) Attempts go to Security Events (no password, no code).</t>
         </is>
       </c>
       <c r="J382" s="8" t="inlineStr">
         <is>
-          <t>Done when: fresh install, database reset and local first run each show the generated password once and force a change; a second view, a view after first sign-in, from another network and after an update answer 404; tests, README manual check, guideline and runbooks updated.</t>
+          <t>Done when: fresh install, database reset and local first run show /setup and nothing else until the administrator exists; the setup code is required and removed afterwards; the chosen password follows the policy; /setup is 404 once an administrator exists and after an update; staging/demo with Seed__Admin__Password skip it; tests, README check, guideline and runbooks updated.</t>
         </is>
       </c>
       <c r="K382" s="8" t="n"/>
@@ -46048,7 +46047,7 @@
       </c>
       <c r="O382" s="10" t="inlineStr">
         <is>
-          <t>#380 #169</t>
+          <t>#380 #382 #169</t>
         </is>
       </c>
       <c r="P382" s="10" t="n"/>

</xml_diff>

<commit_message>
SCRUM-411: two modes - setup in the UI when no env password, forced change when it comes from an env file (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016JvDrGNEsrzfB2BHfyESJM
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -46021,12 +46021,12 @@
       </c>
       <c r="I382" s="8" t="inlineStr">
         <is>
-          <t>1) Condition: user table empty and no Seed__Admin__Password. Every request goes to /setup (static page) until done; staging and demo keep Seed__Admin__Password and skip it; an update never reaches it. 2) Guard against first-comer takeover: a one-time setup code written to a file next to the application and logged as a pointer only; /setup asks for it (optionally also server/management network only); rate limited; code and file deleted when the administrator exists; /setup is 404 afterwards. 3) Step: user name, e-mail, password (policy and history apply), confirm, sign in; MustChangePassword=false; the install is complete; licence/TLS/MFA steps of #169 attach to the same frame later. 4) After a database reset the page appears again with a new code. 5) Attempts go to Security Events (no password, no code).</t>
+          <t>1) Condition: user table empty and no Seed__Admin__Password. Every request goes to /setup (static page) until done; staging and demo keep Seed__Admin__Password and skip it; an update never reaches it. 2) Guard against first-comer takeover: a one-time setup code written to a file next to the application and logged as a pointer only; /setup asks for it (optionally also server/management network only); rate limited; code and file deleted when the administrator exists; /setup is 404 afterwards. 3) Step: user name, e-mail, password (policy and history apply), confirm, sign in; MustChangePassword=false; the install is complete; licence/TLS/MFA steps of #169 attach to the same frame later. 4) After a database reset the page appears again with a new code. 5) Attempts go to Security Events (no password, no code). Two modes, decided only by whether Seed__Admin__Password is set: not set -&gt; the administrator chooses the password on /setup, install complete, no forced change; set from an env/secrets file (staging, demo) -&gt; the administrator is created from it and the first sign-in forces a change (MustChangePassword=true, history rule applies). An administrator password is never part of a client build.</t>
         </is>
       </c>
       <c r="J382" s="8" t="inlineStr">
         <is>
-          <t>Done when: fresh install, database reset and local first run show /setup and nothing else until the administrator exists; the setup code is required and removed afterwards; the chosen password follows the policy; /setup is 404 once an administrator exists and after an update; staging/demo with Seed__Admin__Password skip it; tests, README check, guideline and runbooks updated.</t>
+          <t>Done when: fresh install, database reset and local first run show /setup and nothing else until the administrator exists; the setup code is required and removed afterwards; the chosen password follows the policy; /setup is 404 once an administrator exists and after an update; staging/demo with Seed__Admin__Password skip it; tests, README check, guideline and runbooks updated. Setup mode leaves MustChangePassword=false; seeded mode sets it true and the first change cannot keep the seed password.</t>
         </is>
       </c>
       <c r="K382" s="8" t="n"/>

</xml_diff>

<commit_message>
SCRUM-422: plan row #392 for the CRLF bug of the literal-text gate (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12320,7 +12320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U392"/>
+  <dimension ref="A1:U393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -46926,6 +46926,103 @@
       </c>
       <c r="T392" s="10" t="n"/>
       <c r="U392" s="10" t="n"/>
+    </row>
+    <row r="393">
+      <c r="A393" s="10" t="n">
+        <v>392</v>
+      </c>
+      <c r="B393" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C393" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D393" s="8" t="inlineStr">
+        <is>
+          <t>The PEMS.UI literal-text gate fails on Windows (CRLF) checkouts: switch labels are read as UI text</t>
+        </is>
+      </c>
+      <c r="E393" s="10" t="inlineStr">
+        <is>
+          <t>Bug Fix</t>
+        </is>
+      </c>
+      <c r="F393" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G393" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H393" s="8" t="inlineStr">
+        <is>
+          <t>Reported by Saber during SCRUM-337 (2026-10-27): LiteralTextGateTests failed on PemsField.razor on a Windows checkout. In .NET RegexOptions.Multiline, $ matches before \n but not before \r, so case/break lines of an @switch were read as UI text; the gate had only been run on LF.</t>
+        </is>
+      </c>
+      <c r="I393" s="8" t="inlineStr">
+        <is>
+          <t>Normalise line endings in the scanner before the line-anchored pattern and test both endings. SCRUM-422.</t>
+        </is>
+      </c>
+      <c r="J393" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the gate passes on LF and on CRLF files and a test covers both endings.</t>
+        </is>
+      </c>
+      <c r="K393" s="8" t="inlineStr">
+        <is>
+          <t>Fixed in PR atapems-tech/PEMS#44 (merged): scanner normalises CRLF; Theory with LF and CRLF; verified on CRLF-converted library files; PEMS.UI.Tests 70/70. Recorded retroactively as its own issue; QA pending (SQL Server tests, HTTP smoke tests and a Windows run not done in the cloud container).</t>
+        </is>
+      </c>
+      <c r="L393" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M393" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N393" s="10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O393" s="10" t="inlineStr">
+        <is>
+          <t>#386</t>
+        </is>
+      </c>
+      <c r="P393" s="10" t="n"/>
+      <c r="Q393" s="10" t="n"/>
+      <c r="R393" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S393" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T393" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="U393" s="10" t="inlineStr">
+        <is>
+          <t>Member A</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-421: plan row #391 Report after the fix (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -46868,7 +46868,7 @@
       </c>
       <c r="F392" s="10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G392" s="10" t="inlineStr">
@@ -46891,7 +46891,11 @@
           <t>Done when: on a Persian page 12.5 (and 12٫5) and a date typed with Persian digits are accepted and stored as 12.5 and 2026-10-27; English pages are unchanged; the known-issue tests become regression tests.</t>
         </is>
       </c>
-      <c r="K392" s="8" t="n"/>
+      <c r="K392" s="8" t="inlineStr">
+        <is>
+          <t>Fixed in PR atapems-tech/PEMS#48 (merged): one model binder (PEMS.UI.Binding, registered once in PEMS.Web) parses numbers with the invariant culture, dates as ISO first, and normalises Persian and Arabic-Indic digits and the Persian decimal mark; empty values, nullable types and MVC error messages unchanged. PEMS.UI.Tests 85/85 (6 failed before the fix); database-free PEMS.Tests set 513 pass, 1 known SQL Server failure. QA pending: SQL Server tests, HTTP smoke tests and manual check M-19 not run in the cloud container.</t>
+        </is>
+      </c>
       <c r="L392" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-418: plan row #388 report (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -46613,7 +46613,7 @@
       </c>
       <c r="F389" s="10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G389" s="10" t="inlineStr">
@@ -46636,7 +46636,11 @@
           <t>Done when: both partials live in PEMS.UI, the 54 pagination pages and every page header render byte-identically in fa and en, and PEMS.Web has no copy.</t>
         </is>
       </c>
-      <c r="K389" s="8" t="n"/>
+      <c r="K389" s="8" t="inlineStr">
+        <is>
+          <t>Pagination moved in PR atapems-tech/PEMS#51 (merged): footer is the PEMS.UI component _PemsPagination (PaginationModel + PaginationTexts as TranslatableText inputs); _Pagination in PEMS.Web is a thin adapter over SharedResource; the 54 callers are unchanged. 8 golden cases (en/fa) recorded on the unchanged partial are byte-identical; mutation check fails 3. PEMS.UI.Tests 92/92; PEMS.Tests Ui set 30 pass. _PageHeader not moved: no callers, owner decides. QA pending (SQL Server tests, HTTP smoke tests, browser check not done in the cloud container).</t>
+        </is>
+      </c>
       <c r="L389" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-418: plan row #388 report (hamid) (#52)
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -46613,7 +46613,7 @@
       </c>
       <c r="F389" s="10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G389" s="10" t="inlineStr">
@@ -46636,7 +46636,11 @@
           <t>Done when: both partials live in PEMS.UI, the 54 pagination pages and every page header render byte-identically in fa and en, and PEMS.Web has no copy.</t>
         </is>
       </c>
-      <c r="K389" s="8" t="n"/>
+      <c r="K389" s="8" t="inlineStr">
+        <is>
+          <t>Pagination moved in PR atapems-tech/PEMS#51 (merged): footer is the PEMS.UI component _PemsPagination (PaginationModel + PaginationTexts as TranslatableText inputs); _Pagination in PEMS.Web is a thin adapter over SharedResource; the 54 callers are unchanged. 8 golden cases (en/fa) recorded on the unchanged partial are byte-identical; mutation check fails 3. PEMS.UI.Tests 92/92; PEMS.Tests Ui set 30 pass. _PageHeader not moved: no callers, owner decides. QA pending (SQL Server tests, HTTP smoke tests, browser check not done in the cloud container).</t>
+        </is>
+      </c>
       <c r="L389" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-423: procurement & supply chain section in the sidebar (saber)
Purchasing (MR, package, tender, PO), contracts, vendors and the warehouse
now sit under one sidebar section, like CMMS, in both the data-driven menu
and the classic sidebar used by demo, UAT and production. Each link keeps
its former gate plus its former section module, so no role sees more or
less. Old menu keys are retired by the startup sync; no migration.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$350</definedName>
@@ -12320,7 +12320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U393"/>
+  <dimension ref="A1:U394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -47027,6 +47027,103 @@
         </is>
       </c>
       <c r="U393" s="10" t="inlineStr">
+        <is>
+          <t>Member A</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="10" t="n">
+        <v>393</v>
+      </c>
+      <c r="B394" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C394" s="8" t="inlineStr">
+        <is>
+          <t>Domain: HR, Projects, Finance &amp; Procurement</t>
+        </is>
+      </c>
+      <c r="D394" s="8" t="inlineStr">
+        <is>
+          <t>Procurement &amp; supply chain section in the sidebar: purchasing, contracts, vendors and warehouse under one menu (like CMMS)</t>
+        </is>
+      </c>
+      <c r="E394" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F394" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G394" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H394" s="8" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-27: procurement pages were spread over Engineering Management (package, tender, MR), Contract Management (contracts, vendors, PO) and Warehouse. Owner decision: the warehouse goes in too. SCRUM-423.</t>
+        </is>
+      </c>
+      <c r="I394" s="8" t="inlineStr">
+        <is>
+          <t>One section "Procurement &amp; Supply Chain" with sub-headings Purchasing, Contracts and Warehouse (vendors as a direct link) in both sidebars: NavigationMenuDefaults (new keys, old keys retired by the sync, no migration) and the classic _SidebarMenu.cshtml. Each link keeps its former gate plus its former section module, so no role sees more or less.</t>
+        </is>
+      </c>
+      <c r="J394" s="8" t="inlineStr">
+        <is>
+          <t>Done when: both sidebars show the section in fa and en with the right item active; per-role visibility unchanged (tests); old menu rows deactivated, not deleted; QA in the browser.</t>
+        </is>
+      </c>
+      <c r="K394" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27 SCRUM-423: built on feature/SCRUM-423-procurement-menu-saber; DynamicSidebarTests 57/57 (new: former gates kept, retired rows, classic sidebar source); browser check on PEMSDB_QA407, both sidebars, fa and en.</t>
+        </is>
+      </c>
+      <c r="L394" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M394" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N394" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O394" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P394" s="10" t="n"/>
+      <c r="Q394" s="10" t="n"/>
+      <c r="R394" s="8" t="inlineStr">
+        <is>
+          <t>Domain modules</t>
+        </is>
+      </c>
+      <c r="S394" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T394" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="U394" s="10" t="inlineStr">
         <is>
           <t>Member A</t>
         </is>

</xml_diff>

<commit_message>
SCRUM-424: unified loading, empty and error states; component inputs as named-property objects (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$350</definedName>
@@ -12320,7 +12320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U394"/>
+  <dimension ref="A1:U397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -47128,6 +47128,249 @@
           <t>Member A</t>
         </is>
       </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="10" t="n">
+        <v>424</v>
+      </c>
+      <c r="B395" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C395" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D395" s="8" t="inlineStr">
+        <is>
+          <t>Unified loading, empty and error states: PemsEmptyState, PemsErrorState and PemsLoadingState in PEMS.UI, one look and one accessibility contract, texts as inputs</t>
+        </is>
+      </c>
+      <c r="E395" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F395" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G395" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H395" s="8" t="inlineStr">
+        <is>
+          <t>Today only 8 of 303 pages have an empty state and 3 a loading state (see #323). #323 (Saber, In Progress) is not touched; this carves out only the three state components.</t>
+        </is>
+      </c>
+      <c r="I395" s="8" t="n"/>
+      <c r="J395" s="8" t="inlineStr">
+        <is>
+          <t>Three components, a partial facade, golden tests en/fa, registry and guideline; no page changes.</t>
+        </is>
+      </c>
+      <c r="K395" s="8" t="n"/>
+      <c r="L395" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M395" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N395" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O395" s="10" t="inlineStr">
+        <is>
+          <t>#386 #320</t>
+        </is>
+      </c>
+      <c r="P395" s="10" t="n"/>
+      <c r="Q395" s="10" t="n"/>
+      <c r="R395" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S395" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T395" s="10" t="n"/>
+      <c r="U395" s="10" t="n"/>
+    </row>
+    <row r="396">
+      <c r="A396" s="10" t="n">
+        <v>425</v>
+      </c>
+      <c r="B396" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C396" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D396" s="8" t="inlineStr">
+        <is>
+          <t>Page header component: give _PageHeader its first callers, then move it into PEMS.UI with its texts as inputs</t>
+        </is>
+      </c>
+      <c r="E396" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F396" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G396" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H396" s="8" t="inlineStr">
+        <is>
+          <t>Found in #388: _PageHeader has no callers, so it could not be moved with a golden proof. Owner decision 2026-10-27: give it callers, then componentize.</t>
+        </is>
+      </c>
+      <c r="I396" s="8" t="n"/>
+      <c r="J396" s="8" t="inlineStr">
+        <is>
+          <t>PemsPageHeader in PEMS.UI, an approved first wave of pages calls it, goldens identical before and after.</t>
+        </is>
+      </c>
+      <c r="K396" s="8" t="n"/>
+      <c r="L396" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M396" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N396" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O396" s="10" t="inlineStr">
+        <is>
+          <t>#388 #424</t>
+        </is>
+      </c>
+      <c r="P396" s="10" t="n"/>
+      <c r="Q396" s="10" t="n"/>
+      <c r="R396" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S396" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T396" s="10" t="n"/>
+      <c r="U396" s="10" t="n"/>
+    </row>
+    <row r="397">
+      <c r="A397" s="10" t="n">
+        <v>426</v>
+      </c>
+      <c r="B397" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C397" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D397" s="8" t="inlineStr">
+        <is>
+          <t>Persian digits in pagination counts: range text and page numbers use the locale digits in Persian, Latin in English</t>
+        </is>
+      </c>
+      <c r="E397" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F397" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G397" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H397" s="8" t="inlineStr">
+        <is>
+          <t>The pagination move (#388) kept Latin digits to stay byte-identical; owner asked for Persian digits as a separate task (2026-10-27, ADR-0008).</t>
+        </is>
+      </c>
+      <c r="I397" s="8" t="n"/>
+      <c r="J397" s="8" t="inlineStr">
+        <is>
+          <t>Persian pages show Persian digits in the footer text and numbers; English byte-identical; links and page parameters unchanged.</t>
+        </is>
+      </c>
+      <c r="K397" s="8" t="n"/>
+      <c r="L397" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M397" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N397" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O397" s="10" t="inlineStr">
+        <is>
+          <t>#388 #386</t>
+        </is>
+      </c>
+      <c r="P397" s="10" t="n"/>
+      <c r="Q397" s="10" t="n"/>
+      <c r="R397" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S397" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T397" s="10" t="n"/>
+      <c r="U397" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-424: unified loading, empty and error states; component inputs as named-property objects (hamid) (#56)
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$350</definedName>
@@ -12320,7 +12320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U394"/>
+  <dimension ref="A1:U397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -47128,6 +47128,249 @@
           <t>Member A</t>
         </is>
       </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="10" t="n">
+        <v>424</v>
+      </c>
+      <c r="B395" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C395" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D395" s="8" t="inlineStr">
+        <is>
+          <t>Unified loading, empty and error states: PemsEmptyState, PemsErrorState and PemsLoadingState in PEMS.UI, one look and one accessibility contract, texts as inputs</t>
+        </is>
+      </c>
+      <c r="E395" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F395" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G395" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H395" s="8" t="inlineStr">
+        <is>
+          <t>Today only 8 of 303 pages have an empty state and 3 a loading state (see #323). #323 (Saber, In Progress) is not touched; this carves out only the three state components.</t>
+        </is>
+      </c>
+      <c r="I395" s="8" t="n"/>
+      <c r="J395" s="8" t="inlineStr">
+        <is>
+          <t>Three components, a partial facade, golden tests en/fa, registry and guideline; no page changes.</t>
+        </is>
+      </c>
+      <c r="K395" s="8" t="n"/>
+      <c r="L395" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M395" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N395" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O395" s="10" t="inlineStr">
+        <is>
+          <t>#386 #320</t>
+        </is>
+      </c>
+      <c r="P395" s="10" t="n"/>
+      <c r="Q395" s="10" t="n"/>
+      <c r="R395" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S395" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T395" s="10" t="n"/>
+      <c r="U395" s="10" t="n"/>
+    </row>
+    <row r="396">
+      <c r="A396" s="10" t="n">
+        <v>425</v>
+      </c>
+      <c r="B396" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C396" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D396" s="8" t="inlineStr">
+        <is>
+          <t>Page header component: give _PageHeader its first callers, then move it into PEMS.UI with its texts as inputs</t>
+        </is>
+      </c>
+      <c r="E396" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F396" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G396" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H396" s="8" t="inlineStr">
+        <is>
+          <t>Found in #388: _PageHeader has no callers, so it could not be moved with a golden proof. Owner decision 2026-10-27: give it callers, then componentize.</t>
+        </is>
+      </c>
+      <c r="I396" s="8" t="n"/>
+      <c r="J396" s="8" t="inlineStr">
+        <is>
+          <t>PemsPageHeader in PEMS.UI, an approved first wave of pages calls it, goldens identical before and after.</t>
+        </is>
+      </c>
+      <c r="K396" s="8" t="n"/>
+      <c r="L396" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M396" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N396" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O396" s="10" t="inlineStr">
+        <is>
+          <t>#388 #424</t>
+        </is>
+      </c>
+      <c r="P396" s="10" t="n"/>
+      <c r="Q396" s="10" t="n"/>
+      <c r="R396" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S396" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T396" s="10" t="n"/>
+      <c r="U396" s="10" t="n"/>
+    </row>
+    <row r="397">
+      <c r="A397" s="10" t="n">
+        <v>426</v>
+      </c>
+      <c r="B397" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C397" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D397" s="8" t="inlineStr">
+        <is>
+          <t>Persian digits in pagination counts: range text and page numbers use the locale digits in Persian, Latin in English</t>
+        </is>
+      </c>
+      <c r="E397" s="10" t="inlineStr">
+        <is>
+          <t>Tech Debt</t>
+        </is>
+      </c>
+      <c r="F397" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G397" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H397" s="8" t="inlineStr">
+        <is>
+          <t>The pagination move (#388) kept Latin digits to stay byte-identical; owner asked for Persian digits as a separate task (2026-10-27, ADR-0008).</t>
+        </is>
+      </c>
+      <c r="I397" s="8" t="n"/>
+      <c r="J397" s="8" t="inlineStr">
+        <is>
+          <t>Persian pages show Persian digits in the footer text and numbers; English byte-identical; links and page parameters unchanged.</t>
+        </is>
+      </c>
+      <c r="K397" s="8" t="n"/>
+      <c r="L397" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M397" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N397" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O397" s="10" t="inlineStr">
+        <is>
+          <t>#388 #386</t>
+        </is>
+      </c>
+      <c r="P397" s="10" t="n"/>
+      <c r="Q397" s="10" t="n"/>
+      <c r="R397" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S397" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T397" s="10" t="n"/>
+      <c r="U397" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-424: plan row #424 report (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -47174,7 +47174,11 @@
           <t>Three components, a partial facade, golden tests en/fa, registry and guideline; no page changes.</t>
         </is>
       </c>
-      <c r="K395" s="8" t="n"/>
+      <c r="K395" s="8" t="inlineStr">
+        <is>
+          <t>Built in PR atapems-tech/PEMS#56 (merged): PemsEmptyState, PemsErrorState, PemsLoadingState + _PemsState partial, CSS, registry keys; texts are TranslatableText inputs; no page changed. Owner request in the same PR: component inputs are named-property objects (not positional), shared property-name table in guideline chapter 02. PEMS.UI.Tests 98/98, 6 new golden cases en/fa, all 17 SharedPartialsGoldenTests identical. QA pending (SQL Server tests, HTTP smoke tests, browser check; Titan name list from owner).</t>
+        </is>
+      </c>
       <c r="L395" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-424: plan row #424 report (hamid) (#57)
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -47174,7 +47174,11 @@
           <t>Three components, a partial facade, golden tests en/fa, registry and guideline; no page changes.</t>
         </is>
       </c>
-      <c r="K395" s="8" t="n"/>
+      <c r="K395" s="8" t="inlineStr">
+        <is>
+          <t>Built in PR atapems-tech/PEMS#56 (merged): PemsEmptyState, PemsErrorState, PemsLoadingState + _PemsState partial, CSS, registry keys; texts are TranslatableText inputs; no page changed. Owner request in the same PR: component inputs are named-property objects (not positional), shared property-name table in guideline chapter 02. PEMS.UI.Tests 98/98, 6 new golden cases en/fa, all 17 SharedPartialsGoldenTests identical. QA pending (SQL Server tests, HTTP smoke tests, browser check; Titan name list from owner).</t>
+        </is>
+      </c>
       <c r="L395" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-427: procurement standards gap analysis (saber)
PEMS procurement mapped against the CIPS cycle, PMI procurement management,
EPC/oil & gas practice, ISO 20400 and internal-control principles: 32 stages
and controls (5 present, 14 partial, 13 missing), evidence per row, indent =
Store Requisition (exists), and 11 follow-up proposals ordered by value.
No code.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12320,7 +12320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U394"/>
+  <dimension ref="A1:U395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -47124,6 +47124,103 @@
         </is>
       </c>
       <c r="U394" s="10" t="inlineStr">
+        <is>
+          <t>Member A</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="10" t="n">
+        <v>394</v>
+      </c>
+      <c r="B395" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C395" s="8" t="inlineStr">
+        <is>
+          <t>Domain: HR, Projects, Finance &amp; Procurement</t>
+        </is>
+      </c>
+      <c r="D395" s="8" t="inlineStr">
+        <is>
+          <t>Procurement gap analysis: PEMS against international procurement practice (EPC/oil &amp; gas, CIPS, PMI, ISO 20400) with proposed tickets</t>
+        </is>
+      </c>
+      <c r="E395" s="10" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="F395" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G395" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H395" s="8" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-27 (compare PEMS procurement with world standards; check indent). SCRUM-427; first of the approved batch SCRUM-427, SCRUM-40, SCRUM-57, SCRUM-428, SCRUM-429.</t>
+        </is>
+      </c>
+      <c r="I395" s="8" t="inlineStr">
+        <is>
+          <t>Inventory of PEMS procurement (entities, workflows, SoD, numbering), reference lifecycle and controls, gap matrix present/partial/missing with evidence, proposed tickets by value. No code.</t>
+        </is>
+      </c>
+      <c r="J395" s="8" t="inlineStr">
+        <is>
+          <t>Done when: docs/procurement/PROCUREMENT_STANDARDS_GAP_ANALYSIS.md is merged and the owner reviewed the proposed tickets.</t>
+        </is>
+      </c>
+      <c r="K395" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27 SCRUM-427: gap analysis written (32 stages/controls: 5 present, 14 partial, 13 missing); indent = Store Requisition (exists), missing link shortage -&gt; MR; 11 follow-up proposals, PO lines + approval first.</t>
+        </is>
+      </c>
+      <c r="L395" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M395" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N395" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O395" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P395" s="10" t="n"/>
+      <c r="Q395" s="10" t="n"/>
+      <c r="R395" s="8" t="inlineStr">
+        <is>
+          <t>Domain modules</t>
+        </is>
+      </c>
+      <c r="S395" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T395" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="U395" s="10" t="inlineStr">
         <is>
           <t>Member A</t>
         </is>

</xml_diff>

<commit_message>
SCRUM-40: automatic numbering of procurement documents from admin-defined patterns (saber)
Admin > Numbering: pattern per document type (MR, package, tender, bid, PO,
contract) with {YYYY}/{YY} (Jalali or Gregorian), {PROJECT}, {DISC}, {SEQ},
counter digits, yearly or no reset, active and manual-entry flags, live
preview, version per change. New table NumberingSchemes (migration) and an
idempotent seeder with active Jalali defaults. NumberingService allocates
atomically per pattern scope and skips numbers that already exist; create
services resolve the number (typed only when the scheme allows it; no active
scheme = typed as before). Forms use the DocumentNumberField view component.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -13900,7 +13900,7 @@
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -13923,7 +13923,11 @@
           <t>A 50-parallel-request test yields no duplicate numbers; the pattern is editable and versioned.</t>
         </is>
       </c>
-      <c r="K17" s="8" t="n"/>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-28 SCRUM-40: patterns per document type (NumberingSchemes, Admin &gt; Numbering: tokens YYYY/YY Jalali or Gregorian, PROJECT, DISC, SEQ; yearly or no reset; manual entry flag; version + audit) applied to all procurement documents (MR, package, tender, bid, PO, contract); atomic counter per scope, existing numbers skipped, 50-parallel SQL test without duplicates. Other modules (work order, IRN, ...) still use the built-in formats.</t>
+        </is>
+      </c>
       <c r="L17" s="10" t="inlineStr">
         <is>
           <t>M4</t>

</xml_diff>

<commit_message>
SCRUM-425, SCRUM-426: plan row reports (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$350</definedName>
@@ -47295,7 +47295,7 @@
       </c>
       <c r="F396" s="10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G396" s="10" t="inlineStr">
@@ -47314,7 +47314,11 @@
           <t>PemsPageHeader in PEMS.UI, an approved first wave of pages calls it, goldens identical before and after.</t>
         </is>
       </c>
-      <c r="K396" s="8" t="n"/>
+      <c r="K396" s="8" t="inlineStr">
+        <is>
+          <t>Part 1 in PR atapems-tech/PEMS#60 (merged): title row moved to PEMS.UI _PemsPageHeader (PageHeaderModel Title/Section as TranslatableText); _PageHeader stays as adapter (localizes, honours HidePageTitle); 7 golden cases en/fa byte-identical, mutation check fails 1; design doc corrected. Finding: the layout stopped rendering the header on owner request (guard test GlobalPageHeaderTests) and almost no page hand-writes a page title, so any caller ADDS a visible row. Callers wait for the owner's choice of pages (task stays In Progress). QA pending (SQL Server tests, HTTP smoke tests, browser check).</t>
+        </is>
+      </c>
       <c r="L396" s="10" t="inlineStr">
         <is>
           <t>M1</t>
@@ -47376,7 +47380,7 @@
       </c>
       <c r="F397" s="10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G397" s="10" t="inlineStr">
@@ -47395,7 +47399,11 @@
           <t>Persian pages show Persian digits in the footer text and numbers; English byte-identical; links and page parameters unchanged.</t>
         </is>
       </c>
-      <c r="K397" s="8" t="n"/>
+      <c r="K397" s="8" t="inlineStr">
+        <is>
+          <t>Done in PR atapems-tech/PEMS#61 (merged): new IPemsLocale.Digits (digit swap, no reformatting; Format not used because it adds thousands separators); _PemsPagination shows Persian digits in the range text, page numbers and page-size buttons; hrefs and aria-labels stay Latin; English goldens byte-identical, 3 Persian goldens re-recorded and diffed (digits only). PEMS.UI.Tests 99/99, PEMS.Tests.Ui 25/25, mutation check fails 4. QA pending (SQL Server tests, HTTP smoke tests incl. clicking a Persian page link, browser check).</t>
+        </is>
+      </c>
       <c r="L397" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-425, SCRUM-426: plan row reports (hamid) (#62)
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$350</definedName>
@@ -47295,7 +47295,7 @@
       </c>
       <c r="F396" s="10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G396" s="10" t="inlineStr">
@@ -47314,7 +47314,11 @@
           <t>PemsPageHeader in PEMS.UI, an approved first wave of pages calls it, goldens identical before and after.</t>
         </is>
       </c>
-      <c r="K396" s="8" t="n"/>
+      <c r="K396" s="8" t="inlineStr">
+        <is>
+          <t>Part 1 in PR atapems-tech/PEMS#60 (merged): title row moved to PEMS.UI _PemsPageHeader (PageHeaderModel Title/Section as TranslatableText); _PageHeader stays as adapter (localizes, honours HidePageTitle); 7 golden cases en/fa byte-identical, mutation check fails 1; design doc corrected. Finding: the layout stopped rendering the header on owner request (guard test GlobalPageHeaderTests) and almost no page hand-writes a page title, so any caller ADDS a visible row. Callers wait for the owner's choice of pages (task stays In Progress). QA pending (SQL Server tests, HTTP smoke tests, browser check).</t>
+        </is>
+      </c>
       <c r="L396" s="10" t="inlineStr">
         <is>
           <t>M1</t>
@@ -47376,7 +47380,7 @@
       </c>
       <c r="F397" s="10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G397" s="10" t="inlineStr">
@@ -47395,7 +47399,11 @@
           <t>Persian pages show Persian digits in the footer text and numbers; English byte-identical; links and page parameters unchanged.</t>
         </is>
       </c>
-      <c r="K397" s="8" t="n"/>
+      <c r="K397" s="8" t="inlineStr">
+        <is>
+          <t>Done in PR atapems-tech/PEMS#61 (merged): new IPemsLocale.Digits (digit swap, no reformatting; Format not used because it adds thousands separators); _PemsPagination shows Persian digits in the range text, page numbers and page-size buttons; hrefs and aria-labels stay Latin; English goldens byte-identical, 3 Persian goldens re-recorded and diffed (digits only). PEMS.UI.Tests 99/99, PEMS.Tests.Ui 25/25, mutation check fails 4. QA pending (SQL Server tests, HTTP smoke tests incl. clicking a Persian page link, browser check).</t>
+        </is>
+      </c>
       <c r="L397" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-57: searchable dropdowns on every form (saber)
PEMS.UI pems-select.js/.css on the vendored Tom Select, loaded once by the
layout: single selects with 8+ options become searchable, large lists can
search the permission-aware /SearchApi (data-pems-select-source), opt-out
with data-pems-select="off". Opens in place inside modals and dropdown
panels, re-reads replaced options, keeps an empty choice only where the page
has one, RTL and dark theme, fa/en texts from the layout. User pages no
longer load Tom Select twice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -15643,7 +15643,7 @@
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="G36" s="10" t="inlineStr">
@@ -15666,7 +15666,11 @@
           <t>Selecting from 200k equipment records is smooth.</t>
         </is>
       </c>
-      <c r="K36" s="8" t="n"/>
+      <c r="K36" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-28 SCRUM-57: searchable select on every form (PEMS.UI pems-select.js on vendored Tom Select, loaded by the layout; &gt;=8 options automatic, data-pems-select-source for permission-aware server search via /SearchApi, opt-out, inline in modals/dropdowns, cascading refresh, RTL/dark, fa/en). TreeSelect (unit/PBS) and paging beyond the first 20 server results are still open.</t>
+        </is>
+      </c>
       <c r="L36" s="10" t="inlineStr">
         <is>
           <t>M4</t>

</xml_diff>

<commit_message>
docs: plan audit for a dynamic, REST-based PEMS; rows #430-#441; dependency fixes (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12367,7 +12367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U398"/>
+  <dimension ref="A1:U410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>The root contains WebApplication1, 'New Text Document.txt' and two identical copies of the Role documents under .claude and .github.</t>
+          <t>The root contains WebApplication1, 'New Text Document.txt' and two identical copies of the Role documents under .claude and .github. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
@@ -13206,7 +13206,7 @@
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="10" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="M9" s="10" t="inlineStr">
@@ -13555,12 +13555,12 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>Build one /api/d/{entity} endpoint with a single query contract (page/sort/filter/search/columns) used by every list and relation list.</t>
+          <t>Build one /api/d/{entity} endpoint with a single query contract (page/sort/filter/search/columns) used by every list and relation list. Route shape, paging style and error format come from the REST ADR (#431), not from this row; the first version must pass the API quality gates (#436).</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>Test: 500k records, filter+sort under 500 ms; a record outside the user's access never appears in results or counts.</t>
+          <t>Test: 500k records, filter+sort under 500 ms; a record outside the user's access never appears in results or counts. The route and contract follow the REST API standard (#431): resource-oriented URLs instead of verbs, ETag/If-Match, RFC 9457 errors, OpenAPI.</t>
         </is>
       </c>
       <c r="K13" s="8" t="n"/>
@@ -13581,7 +13581,7 @@
       </c>
       <c r="O13" s="10" t="inlineStr">
         <is>
-          <t>#10 #11 #178</t>
+          <t>#10 #11 #178 #431 #435</t>
         </is>
       </c>
       <c r="P13" s="10" t="inlineStr">
@@ -14270,7 +14270,7 @@
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>The current menu in _SidebarMenu.cshtml is static.</t>
+          <t>The current menu in _SidebarMenu.cshtml is static. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
@@ -14305,7 +14305,7 @@
       </c>
       <c r="O21" s="10" t="inlineStr">
         <is>
-          <t>#10</t>
+          <t>#10 #434</t>
         </is>
       </c>
       <c r="P21" s="10" t="inlineStr"/>
@@ -15742,7 +15742,7 @@
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>PEMS has static _PemsStageDiagram and _WorkOrderStagesDiagram.</t>
+          <t>PEMS has static _PemsStageDiagram and _WorkOrderStagesDiagram. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I37" s="8" t="inlineStr">
@@ -15773,7 +15773,7 @@
       </c>
       <c r="O37" s="10" t="inlineStr">
         <is>
-          <t>#31 #80</t>
+          <t>#31</t>
         </is>
       </c>
       <c r="P37" s="10" t="inlineStr"/>
@@ -15920,7 +15920,7 @@
       </c>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t>Often required in enterprise and government contracts.</t>
+          <t>Often required in enterprise and government contracts. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I39" s="8" t="inlineStr">
@@ -15936,7 +15936,7 @@
       <c r="K39" s="8" t="n"/>
       <c r="L39" s="10" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="M39" s="10" t="inlineStr">
@@ -16478,7 +16478,7 @@
       </c>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t>PEMS forms are fixed Razor; the audit found no general form builder. This is the line between software and a platform.</t>
+          <t>PEMS forms are fixed Razor; the audit found no general form builder. This is the line between software and a platform. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
         </is>
       </c>
       <c r="I45" s="8" t="inlineStr">
@@ -16509,7 +16509,7 @@
       </c>
       <c r="O45" s="10" t="inlineStr">
         <is>
-          <t>#10 #34</t>
+          <t>#10 #34 #434</t>
         </is>
       </c>
       <c r="P45" s="10" t="inlineStr">
@@ -16660,7 +16660,7 @@
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>All rules should live in one validation object with one interpreter.</t>
+          <t>All rules should live in one validation object with one interpreter. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I47" s="8" t="inlineStr">
@@ -16691,7 +16691,7 @@
       </c>
       <c r="O47" s="10" t="inlineStr">
         <is>
-          <t>#15 #45</t>
+          <t>#15 #45 #355</t>
         </is>
       </c>
       <c r="P47" s="10" t="inlineStr">
@@ -17554,7 +17554,7 @@
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>Without a guided scaffold the 'module builder' is only a table builder.</t>
+          <t>Without a guided scaffold the 'module builder' is only a table builder. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
         </is>
       </c>
       <c r="I57" s="8" t="inlineStr">
@@ -17585,7 +17585,7 @@
       </c>
       <c r="O57" s="10" t="inlineStr">
         <is>
-          <t>#10 #44 #20</t>
+          <t>#10 #44 #20 #434</t>
         </is>
       </c>
       <c r="P57" s="10" t="inlineStr">
@@ -17643,7 +17643,7 @@
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>List sizes must be structured metadata, not ad-hoc.</t>
+          <t>List sizes must be structured metadata, not ad-hoc. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
         </is>
       </c>
       <c r="I58" s="8" t="inlineStr">
@@ -17674,7 +17674,7 @@
       </c>
       <c r="O58" s="10" t="inlineStr">
         <is>
-          <t>#32</t>
+          <t>#32 #434</t>
         </is>
       </c>
       <c r="P58" s="10" t="inlineStr">
@@ -20124,7 +20124,7 @@
       </c>
       <c r="I86" s="8" t="inlineStr">
         <is>
-          <t>A module table with risk, data volume, dependencies and migration wave.</t>
+          <t>A module table with risk, data volume, dependencies and migration wave. Also classify the ~303 pages and the 147 controllers: definable from a Page definition (#438), convertible form/list/detail, or code-only; reuse the REST inventory (#432).</t>
         </is>
       </c>
       <c r="J86" s="8" t="inlineStr">
@@ -20150,7 +20150,7 @@
       </c>
       <c r="O86" s="10" t="inlineStr">
         <is>
-          <t>#29</t>
+          <t>#29 #432</t>
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr"/>
@@ -29877,7 +29877,7 @@
       </c>
       <c r="J196" s="8" t="inlineStr">
         <is>
-          <t>A customer can read/write dynamic records and receive webhooks using the documentation.</t>
+          <t>A customer can read/write dynamic records and receive webhooks using the documentation. Scope: external governance (keys/tokens, rate limit, signing, documentation, monitoring) on top of the internal standard (#431) and skeleton (#435); it does not redefine the API style.</t>
         </is>
       </c>
       <c r="K196" s="8" t="n"/>
@@ -29898,7 +29898,7 @@
       </c>
       <c r="O196" s="10" t="inlineStr">
         <is>
-          <t>#12</t>
+          <t>#12 #431 #435</t>
         </is>
       </c>
       <c r="P196" s="10" t="inlineStr"/>
@@ -31044,7 +31044,7 @@
       </c>
       <c r="H209" s="8" t="inlineStr">
         <is>
-          <t>Audit E22: number/currency/ZWNJ standards are not defined.</t>
+          <t>Audit E22: number/currency/ZWNJ standards are not defined. 2026-10-28 audit: overlaps #367 (formatting engine); merge when #367 starts. Digit swap exists (IPemsLocale.Digits, SCRUM-426). 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I209" s="8" t="inlineStr">
@@ -31060,7 +31060,7 @@
       <c r="K209" s="8" t="n"/>
       <c r="L209" s="10" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="M209" s="10" t="inlineStr">
@@ -32379,7 +32379,7 @@
       </c>
       <c r="H224" s="8" t="inlineStr">
         <is>
-          <t>A basic PWA exists (manifest + service worker). A working mobile view for every screen type and on-site time/material tracking are known needs.</t>
+          <t>A basic PWA exists (manifest + service worker). A working mobile view for every screen type and on-site time/material tracking are known needs. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I224" s="8" t="inlineStr">
@@ -32395,7 +32395,7 @@
       <c r="K224" s="8" t="n"/>
       <c r="L224" s="10" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="M224" s="10" t="inlineStr">
@@ -32472,7 +32472,7 @@
       </c>
       <c r="H225" s="8" t="inlineStr">
         <is>
-          <t>Audit E16: permits, LOTO and gas tests are desktop only.</t>
+          <t>Audit E16: permits, LOTO and gas tests are desktop only. 2026-10-28 plan audit: follows #223 to M5.</t>
         </is>
       </c>
       <c r="I225" s="8" t="inlineStr">
@@ -32488,7 +32488,7 @@
       <c r="K225" s="8" t="n"/>
       <c r="L225" s="10" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="M225" s="10" t="inlineStr">
@@ -39887,7 +39887,7 @@
       </c>
       <c r="H311" s="8" t="inlineStr">
         <is>
-          <t>IDatabaseUpdateService (PEMS.Application) + DatabaseUpdateService (PEMS.Persistence) with the pure DatabaseSetupClassifier: FirstRun, UpdateAvailable, UpToDate, UnmanagedSchema, DatabaseNewerThanApplication, Unreachable. Entity DatabaseUpdateRun + migration DatabaseUpdateRuns (audit of every attempt). Admin &gt; System Monitoring &gt; Database Update (/Admin/DatabaseUpdate, SystemAdmin, backup confirmation, antiforgery). GET /health/database (anonymous, state only). Verified 2026-10-22: 9 tests (classifier + real SQL Server install/update/unmanaged on throw-away LocalDB databases); page compiled and anonymous access redirects to login. Driven in a browser as the seeded dev admin on 2026-10-23: state card, pending list, backup confirmation refused/accepted, update applied, run recorded as Admin/Update.</t>
+          <t>IDatabaseUpdateService (PEMS.Application) + DatabaseUpdateService (PEMS.Persistence) with the pure DatabaseSetupClassifier: FirstRun, UpdateAvailable, UpToDate, UnmanagedSchema, DatabaseNewerThanApplication, Unreachable. Entity DatabaseUpdateRun + migration DatabaseUpdateRuns (audit of every attempt). Admin &gt; System Monitoring &gt; Database Update (/Admin/DatabaseUpdate, SystemAdmin, backup confirmation, antiforgery). GET /health/database (anonymous, state only). Verified 2026-10-22: 9 tests (classifier + real SQL Server install/update/unmanaged on throw-away LocalDB databases); page compiled and anonymous access redirects to login. Driven in a browser as the seeded dev admin on 2026-10-23: state card, pending list, backup confirmation refused/accepted, update applied, run recorded as Admin/Update. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I311" s="8" t="inlineStr">
@@ -39920,11 +39920,7 @@
           <t>Sales blocker</t>
         </is>
       </c>
-      <c r="O311" s="10" t="inlineStr">
-        <is>
-          <t>#309</t>
-        </is>
-      </c>
+      <c r="O311" s="10" t="n"/>
       <c r="P311" s="10" t="n"/>
       <c r="Q311" s="10" t="n"/>
       <c r="R311" s="8" t="inlineStr">
@@ -39976,7 +39972,7 @@
       </c>
       <c r="H312" s="8" t="inlineStr">
         <is>
-          <t>Moved with git mv to legacy-trash/manual-sql/ (same relative paths, README maps each to its replacement): PEMS.Persistence/Scripts/EnableFullTextSearch.sql (now migration FullTextSearch), docs/procurement/*.migration.sql and P4_P5_delta/PREFLIGHT, docs/task manager/TaskManagerCore_migration.sql, plus the root InitialCreate.sql (full-schema script). References in docs and code comments updated. Operator tools that are not schema setup (scripts/cmms, scripts/rcm data repairs and read-only reports, docs/sql checks, deploy/ reviewed-script flow) were deliberately left in place; see #313.</t>
+          <t>Moved with git mv to legacy-trash/manual-sql/ (same relative paths, README maps each to its replacement): PEMS.Persistence/Scripts/EnableFullTextSearch.sql (now migration FullTextSearch), docs/procurement/*.migration.sql and P4_P5_delta/PREFLIGHT, docs/task manager/TaskManagerCore_migration.sql, plus the root InitialCreate.sql (full-schema script). References in docs and code comments updated. Operator tools that are not schema setup (scripts/cmms, scripts/rcm data repairs and read-only reports, docs/sql checks, deploy/ reviewed-script flow) were deliberately left in place; see #313. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I312" s="8" t="inlineStr">
@@ -40009,11 +40005,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="O312" s="10" t="inlineStr">
-        <is>
-          <t>#309</t>
-        </is>
-      </c>
+      <c r="O312" s="10" t="n"/>
       <c r="P312" s="10" t="n"/>
       <c r="Q312" s="10" t="n"/>
       <c r="R312" s="8" t="inlineStr">
@@ -40065,7 +40057,7 @@
       </c>
       <c r="H313" s="8" t="inlineStr">
         <is>
-          <t>deploy-demo.yml: model-drift gate (dotnet ef migrations has-pending-model-changes), jq injects the demo connection string and Database={CreateIfMissing:false,MigrateOnStartup:true}, sed raises the IIS startupTimeLimit to 900 s (the first run installs the whole schema before serving), FTP upload, then polls DEMO_SITE_URL/health/database until UpToDate (fails the run after 30 minutes). YAML validated; web.config patch checked on a real publish. Not yet executed on GitHub. 2026-10-24 first runs on the demo branch: build, drift gate, database-free tests, publish and the FTP upload from the GitHub runner PASS; the post-deploy health check failed - the demo site has no valid TLS certificate and the application does not answer on first start (details and steps: docs/deployment/DEMO_DEPLOYMENT.md, row #340).</t>
+          <t>deploy-demo.yml: model-drift gate (dotnet ef migrations has-pending-model-changes), jq injects the demo connection string and Database={CreateIfMissing:false,MigrateOnStartup:true}, sed raises the IIS startupTimeLimit to 900 s (the first run installs the whole schema before serving), FTP upload, then polls DEMO_SITE_URL/health/database until UpToDate (fails the run after 30 minutes). YAML validated; web.config patch checked on a real publish. Not yet executed on GitHub. 2026-10-24 first runs on the demo branch: build, drift gate, database-free tests, publish and the FTP upload from the GitHub runner PASS; the post-deploy health check failed - the demo site has no valid TLS certificate and the application does not answer on first start (details and steps: docs/deployment/DEMO_DEPLOYMENT.md, row #340). 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I313" s="8" t="inlineStr">
@@ -40100,7 +40092,7 @@
       </c>
       <c r="O313" s="10" t="inlineStr">
         <is>
-          <t>#295 #309 #310</t>
+          <t>#295 #310</t>
         </is>
       </c>
       <c r="P313" s="10" t="n"/>
@@ -42320,12 +42312,12 @@
       </c>
       <c r="H339" s="8" t="inlineStr">
         <is>
-          <t>Row #10 (the registry) is an XL implementation task and #12-#17 all depend on it. Nothing can be built safely until the data model, versioning and publishing rules are written down and agreed. Decided inputs: hybrid storage (#4): real tables for user-built entities, a JSON column for custom fields on existing entities.</t>
+          <t>Row #10 (the registry) is an XL implementation task and #12-#17 all depend on it. Nothing can be built safely until the data model, versioning and publishing rules are written down and agreed. Decided inputs: hybrid storage (#4): real tables for user-built entities, a JSON column for custom fields on existing entities. 2026-10-28 audit: the registry must cover UI definitions, not only data entities (row #430).</t>
         </is>
       </c>
       <c r="I339" s="8" t="inlineStr">
         <is>
-          <t>1) List the registry objects and their relations (App, Module, Entity, Field, Relation, View, Form, Workflow reference, Version). 2) Define draft/published versions, rollback and what a publish changes. 3) Define how static (existing) entities appear in the registry (#14 JSON extension column). 4) Define the cache and invalidation contract (#28). 5) Sketch the EF entity classes (compile-only, in a branch, not merged). 6) List open questions. Output: docs/architecture/METADATA_REGISTRY_DESIGN.md and an ADR under plan/adr.</t>
+          <t>1) List the registry objects and their relations (App, Module, Entity, Field, Relation, View, Form, Workflow reference, Version). 2) Define draft/published versions, rollback and what a publish changes. 3) Define how static (existing) entities appear in the registry (#14 JSON extension column). 4) Define the cache and invalidation contract (#28). 5) Sketch the EF entity classes (compile-only, in a branch, not merged). 6) List open questions. Output: docs/architecture/METADATA_REGISTRY_DESIGN.md and an ADR under plan/adr. 6) Put UI definitions (page, layout, component instance, data source, action, menu, theme) in the same envelope and versioning rules; see the ADR row #430.</t>
         </is>
       </c>
       <c r="J339" s="8" t="inlineStr">
@@ -42773,7 +42765,7 @@
       </c>
       <c r="H344" s="8" t="inlineStr">
         <is>
-          <t>A customer whose production server is offline must be able to recover a lost administrator password with the vendor's help, without a back door in the product and without any remote access. The licence flow already proves that file exchange works offline; the reset reuses its shape with its own key. Gate: this row can start only after #342 (licence flow end to end) is Done. Independent of the separate administrator-recovery work done by Saber (second-admin reset, one-time recovery codes, server-side break-glass, shared audit/notification/session revocation): that work does not wait for the licence flow and this row does not block it; this flow plugs into it as the optional vendor-assisted recovery path, which must stay off until the customer enables it.</t>
+          <t>A customer whose production server is offline must be able to recover a lost administrator password with the vendor's help, without a back door in the product and without any remote access. The licence flow already proves that file exchange works offline; the reset reuses its shape with its own key. Gate: this row can start only after #342 (licence flow end to end) is Done. Independent of the separate administrator-recovery work done by Saber (second-admin reset, one-time recovery codes, server-side break-glass, shared audit/notification/session revocation): that work does not wait for the licence flow and this row does not block it; this flow plugs into it as the optional vendor-assisted recovery path, which must stay off until the customer enables it. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I344" s="8" t="inlineStr">
@@ -42804,7 +42796,7 @@
       </c>
       <c r="O344" s="10" t="inlineStr">
         <is>
-          <t>#96 #107 #178 #182 #184 #339 #342</t>
+          <t>#96 #107 #178 #182 #339 #342</t>
         </is>
       </c>
       <c r="P344" s="10" t="n"/>
@@ -43797,7 +43789,7 @@
       </c>
       <c r="H356" s="8" t="inlineStr">
         <is>
-          <t>Validation in PEMS today is thin and scattered: 260 entities but only 26 [Required] and 45 [MaxLength] attributes in 28 files, no [Range], [StringLength] or regular-expression rule anywhere, no validation library, ModelState.IsValid is checked in 8 controllers, and 64 of 65 plain text inputs in the views have no maxlength. Dynamic forms need one declarative description of the rules per field type before any engine or UI is built. Rule-builder row #46 covers user-defined rules; this row defines the built-in constraints every type carries.</t>
+          <t>Validation in PEMS today is thin and scattered: 260 entities but only 26 [Required] and 45 [MaxLength] attributes in 28 files, no [Range], [StringLength] or regular-expression rule anywhere, no validation library, ModelState.IsValid is checked in 8 controllers, and 64 of 65 plain text inputs in the views have no maxlength. Dynamic forms need one declarative description of the rules per field type before any engine or UI is built. Rule-builder row #46 covers user-defined rules; this row defines the built-in constraints every type carries. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I356" s="8" t="inlineStr">
@@ -43828,7 +43820,7 @@
       </c>
       <c r="O356" s="10" t="inlineStr">
         <is>
-          <t>#11 #338 #46</t>
+          <t>#11 #338</t>
         </is>
       </c>
       <c r="P356" s="10" t="inlineStr">
@@ -44238,7 +44230,7 @@
       </c>
       <c r="H361" s="8" t="inlineStr">
         <is>
-          <t>Import Center has 11 imports with their own checks. A blank cell in an update row must leave the value alone, a malformed identifier must never reach the database as a server error, and a default value must never be saved as NULL by a bulk path.</t>
+          <t>Import Center has 11 imports with their own checks. A blank cell in an update row must leave the value alone, a malformed identifier must never reach the database as a server error, and a default value must never be saved as NULL by a bulk path. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I361" s="8" t="inlineStr">
@@ -44254,7 +44246,7 @@
       <c r="K361" s="8" t="n"/>
       <c r="L361" s="10" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="M361" s="10" t="inlineStr">
@@ -44760,7 +44752,7 @@
       </c>
       <c r="H367" s="8" t="inlineStr">
         <is>
-          <t>Formatting in PEMS is done page by page: 377 hand-written date and time format strings in 138 views using 12 different patterns, 217 number format strings, 103 native date, 8 datetime-local and 137 number inputs whose look follows the browser locale, and Jalali support in only 6 files. Existing rows #24, #205, #206, #208 and #209 ask for translated labels, Persian digits, the Jalali calendar and fixed reports, but nothing defines where a field's format lives or how it relates to validation. A comparable implementation shows the risks: one hard-coded locale in its date component, date strings built without zero padding, an invalid-date defect in downloaded reports and a deprecated date library for the Jalali picker.</t>
+          <t>Formatting in PEMS is done page by page: 377 hand-written date and time format strings in 138 views using 12 different patterns, 217 number format strings, 103 native date, 8 datetime-local and 137 number inputs whose look follows the browser locale, and Jalali support in only 6 files. Existing rows #24, #205, #206, #208 and #209 ask for translated labels, Persian digits, the Jalali calendar and fixed reports, but nothing defines where a field's format lives or how it relates to validation. A comparable implementation shows the risks: one hard-coded locale in its date component, date strings built without zero padding, an invalid-date defect in downloaded reports and a deprecated date library for the Jalali picker. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I367" s="8" t="inlineStr">
@@ -44791,7 +44783,7 @@
       </c>
       <c r="O367" s="10" t="inlineStr">
         <is>
-          <t>#11 #355 #24 #205</t>
+          <t>#11 #355 #205 #386</t>
         </is>
       </c>
       <c r="P367" s="10" t="inlineStr">
@@ -45112,7 +45104,7 @@
       </c>
       <c r="H371" s="8" t="inlineStr">
         <is>
-          <t>Row #24 stores translatable strings in metadata; nothing defines how they are resolved in a context or how mixed-direction text (codes, e-mail, URLs, numbers inside Persian sentences) is displayed. W3C: keep localisation separate from translation.</t>
+          <t>Row #24 stores translatable strings in metadata; nothing defines how they are resolved in a context or how mixed-direction text (codes, e-mail, URLs, numbers inside Persian sentences) is displayed. W3C: keep localisation separate from translation. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I371" s="8" t="inlineStr">
@@ -45143,7 +45135,7 @@
       </c>
       <c r="O371" s="10" t="inlineStr">
         <is>
-          <t>#24 #366</t>
+          <t>#366 #386</t>
         </is>
       </c>
       <c r="P371" s="10" t="inlineStr">
@@ -45201,7 +45193,7 @@
       </c>
       <c r="H372" s="8" t="inlineStr">
         <is>
-          <t>Exports are a second place where formats drift: strings instead of typed cells cannot be sorted or summed, and a comparable platform shipped an invalid-date defect in downloaded reports and layout overflow in PDF exports.</t>
+          <t>Exports are a second place where formats drift: strings instead of typed cells cannot be sorted or summed, and a comparable platform shipped an invalid-date defect in downloaded reports and layout overflow in PDF exports. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I372" s="8" t="inlineStr">
@@ -45217,7 +45209,7 @@
       <c r="K372" s="8" t="n"/>
       <c r="L372" s="10" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="M372" s="10" t="inlineStr">
@@ -46603,7 +46595,7 @@
       </c>
       <c r="J388" s="8" t="inlineStr">
         <is>
-          <t>Done when: a form created in the database renders through PEMS.UI in fa and en with no deploy; a saved translation shows on the next request; tests prove the round trip and the fallback.</t>
+          <t>Done when: a form created in the database renders through PEMS.UI in fa and en with no deploy; a saved translation shows on the next request; tests prove the round trip and the fallback. Reads and writes go through the definition store API (#434) in the shared definition envelope (#430).</t>
         </is>
       </c>
       <c r="K388" s="8" t="n"/>
@@ -46624,7 +46616,7 @@
       </c>
       <c r="O388" s="10" t="inlineStr">
         <is>
-          <t>#386 #10 #334</t>
+          <t>#386 #10 #334 #430 #434</t>
         </is>
       </c>
       <c r="P388" s="10" t="n"/>
@@ -47535,6 +47527,1026 @@
           <t>Member A</t>
         </is>
       </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="10" t="n">
+        <v>430</v>
+      </c>
+      <c r="B399" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C399" s="8" t="inlineStr">
+        <is>
+          <t>Foundation, Architecture Decisions &amp; Baseline</t>
+        </is>
+      </c>
+      <c r="D399" s="8" t="inlineStr">
+        <is>
+          <t>ADR: UI definition model - everything is a definition. One versioned envelope (key, version, status draft/published/archived, owner app, ETag, translations as TranslatableText JSON) for pages, layouts, component instances, forms, views, dashboards, reports, menus, themes, data sources and actions, stored in the database and edited from the UI</t>
+        </is>
+      </c>
+      <c r="E399" s="10" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="F399" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G399" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H399" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. The backlog designs forms (#44), views (#57), dashboards (#58), reports (#59), menus (#20) and workflows (#67) one by one, each with its own storage idea, and nothing defines a page or a component instance. 'All pages, components and forms creatable and editable from the UI' needs one shared definition model first.</t>
+        </is>
+      </c>
+      <c r="I399" s="8" t="inlineStr">
+        <is>
+          <t>1) List the definition kinds and their relations (Page, Layout, Region, ComponentInstance, DataSource, Action, Form, View, Dashboard, Report, Menu, Theme). 2) One envelope and one version/publish/rollback rule for all of them, reusing the registry (#338). 3) Component instance = component key + options JSON that validates against the component manifest (#433). 4) Static-to-dynamic coexistence: a database definition may override or extend a code default; rollback = delete the override. 5) Cache, invalidation, size limits, security (who can publish). 6) Write plan/adr/NNNN and update the registry design.</t>
+        </is>
+      </c>
+      <c r="J399" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the ADR is accepted (storage, envelope, draft/publish/rollback, how a static page and a database page coexist, cache and invalidation, size and security limits); rows #338, #387, #44, #57 and #20 reference it; open questions have an owner.</t>
+        </is>
+      </c>
+      <c r="K399" s="8" t="n"/>
+      <c r="L399" s="10" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="M399" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N399" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O399" s="10" t="inlineStr">
+        <is>
+          <t>#338</t>
+        </is>
+      </c>
+      <c r="P399" s="10" t="n"/>
+      <c r="Q399" s="10" t="n"/>
+      <c r="R399" s="8" t="inlineStr">
+        <is>
+          <t>Foundation &amp; decisions</t>
+        </is>
+      </c>
+      <c r="S399" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T399" s="10" t="n"/>
+      <c r="U399" s="10" t="n"/>
+    </row>
+    <row r="400">
+      <c r="A400" s="10" t="n">
+        <v>431</v>
+      </c>
+      <c r="B400" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C400" s="8" t="inlineStr">
+        <is>
+          <t>Foundation, Architecture Decisions &amp; Baseline</t>
+        </is>
+      </c>
+      <c r="D400" s="8" t="inlineStr">
+        <is>
+          <t>ADR: REST API standard - resource-oriented routes (nouns, no verbs), HTTP semantics and status codes, paging/filter/sort, ETag and If-Match, Idempotency-Key, PATCH semantics, bulk and long-running operations, RFC 9457 errors, versioning, Accept-Language and TranslatableText, dates and time zones, allowed-actions links; OpenAPI 3.1 as the contract; plus a guideline chapter</t>
+        </is>
+      </c>
+      <c r="E400" s="10" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="F400" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G400" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H400" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Today there is no REST surface: 147 controllers, none marked [ApiController], 163 GET and 668 POST actions, no PUT/PATCH/DELETE, no OpenAPI, no ProblemDetails, no API versioning; 22 controller files return ad hoc JSON. Row #12 plans /api/d/{entity} without a standard to follow.</t>
+        </is>
+      </c>
+      <c r="I400" s="8" t="inlineStr">
+        <is>
+          <t>1) Resource naming and URL rules (plural nouns, nested only for ownership, actions as POST sub-resources, e.g. POST /work-orders/{id}/actions/approve). 2) Verbs and status codes (200/201+Location/204/202, 400/401/403/404/409/412/422/428/429). 3) Query contract for paging, sorting, filtering, search, field selection (offset vs cursor decision). 4) Concurrency (ETag/If-Match, 412/428) and idempotency (Idempotency-Key). 5) Errors: RFC 9457 with the field-error list of #363. 6) Versioning and deprecation. 7) i18n: Accept-Language, TranslatableText JSON shape, UTC/ISO dates. 8) Allowed-actions and permission hints for dynamic UIs. 9) Browser auth (cookie plus antiforgery) vs integration auth (token). 10) Write the ADR and the guideline chapter.</t>
+        </is>
+      </c>
+      <c r="J400" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the ADR is accepted and a short guideline chapter (docs/guidelines) lists the rules with one good and one bad example each; rows #12, #195, #363, #18, #28 and #387 reference it; the open questions have an owner.</t>
+        </is>
+      </c>
+      <c r="K400" s="8" t="n"/>
+      <c r="L400" s="10" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="M400" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N400" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O400" s="10" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+      <c r="P400" s="10" t="n"/>
+      <c r="Q400" s="10" t="n"/>
+      <c r="R400" s="8" t="inlineStr">
+        <is>
+          <t>Foundation &amp; decisions</t>
+        </is>
+      </c>
+      <c r="S400" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T400" s="10" t="n"/>
+      <c r="U400" s="10" t="n"/>
+    </row>
+    <row r="401">
+      <c r="A401" s="10" t="n">
+        <v>432</v>
+      </c>
+      <c r="B401" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C401" s="8" t="inlineStr">
+        <is>
+          <t>Foundation, Architecture Decisions &amp; Baseline</t>
+        </is>
+      </c>
+      <c r="D401" s="8" t="inlineStr">
+        <is>
+          <t>REST inventory of the existing 147 controllers and ~830 actions: classify each as view-only MVC (stays), form post (becomes a resource call later), JSON endpoint (normalise), or API candidate; produce the target resource map and a conformance score per controller</t>
+        </is>
+      </c>
+      <c r="E401" s="10" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="F401" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G401" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H401" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Needed to plan the strangler for the API the same way #85 plans it for modules; without it the API work cannot be sized.</t>
+        </is>
+      </c>
+      <c r="I401" s="8" t="inlineStr">
+        <is>
+          <t>Script the inventory (routes, verbs, return types, [Authorize] policies, antiforgery) with Roslyn or reflection; classify by hand the heaviest 30 controllers; list verbs-in-URL, state-changing GETs and missing authorization; propose the target resource names per #431.</t>
+        </is>
+      </c>
+      <c r="J401" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a table (controller, actions, kind, target resource, wave, owner) is committed under docs/audits; the 22 JSON-returning controllers each have a target shape; rows #85 and #12 reference it.</t>
+        </is>
+      </c>
+      <c r="K401" s="8" t="n"/>
+      <c r="L401" s="10" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="M401" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N401" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O401" s="10" t="inlineStr">
+        <is>
+          <t>#431</t>
+        </is>
+      </c>
+      <c r="P401" s="10" t="n"/>
+      <c r="Q401" s="10" t="n"/>
+      <c r="R401" s="8" t="inlineStr">
+        <is>
+          <t>Foundation &amp; decisions</t>
+        </is>
+      </c>
+      <c r="S401" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T401" s="10" t="n"/>
+      <c r="U401" s="10" t="n"/>
+    </row>
+    <row r="402">
+      <c r="A402" s="10" t="n">
+        <v>433</v>
+      </c>
+      <c r="B402" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C402" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D402" s="8" t="inlineStr">
+        <is>
+          <t>Component manifest: every PEMS.UI component publishes a machine-readable description (key, options JSON Schema generated from the options records, slots, events, accessibility notes, sample) that drives the designers' property panels, validates stored JSON and feeds the component catalog</t>
+        </is>
+      </c>
+      <c r="E402" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F402" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G402" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H402" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Options are now named-property records with required/optional members (SCRUM-424), so a schema can be generated rather than written. A designer cannot offer 'add a component to a page' without knowing each component's inputs.</t>
+        </is>
+      </c>
+      <c r="I402" s="8" t="inlineStr">
+        <is>
+          <t>Generate JSON Schema (System.Text.Json schema exporter or NJsonSchema, licence recorded) from the options types; add [PemsComponent] metadata (category, icon key, TranslatableText name/description); expose through the definition store (#434) and the catalog (#326); add the completeness test.</t>
+        </is>
+      </c>
+      <c r="J402" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a generator produces one JSON manifest per component from the code (no hand-written schema); a stored options JSON that violates the schema is rejected with a field error list; the manifest of Button, Badge, Field, Table, Form, Empty/Error/Loading state exists and a test fails when a component has no manifest.</t>
+        </is>
+      </c>
+      <c r="K402" s="8" t="n"/>
+      <c r="L402" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M402" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N402" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O402" s="10" t="inlineStr">
+        <is>
+          <t>#321 #430</t>
+        </is>
+      </c>
+      <c r="P402" s="10" t="n"/>
+      <c r="Q402" s="10" t="n"/>
+      <c r="R402" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S402" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T402" s="10" t="n"/>
+      <c r="U402" s="10" t="n"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="10" t="n">
+        <v>434</v>
+      </c>
+      <c r="B403" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C403" s="8" t="inlineStr">
+        <is>
+          <t>Metadata Core &amp; Dynamic Platform</t>
+        </is>
+      </c>
+      <c r="D403" s="8" t="inlineStr">
+        <is>
+          <t>Definition store REST API: create, read, update (If-Match), list, publish, unpublish, roll back, export and import of definitions under /api/v1/definitions, with ETag, RFC 9457 errors, OpenAPI, draft/published versions and audit; the designers are ordinary clients of it</t>
+        </is>
+      </c>
+      <c r="E403" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F403" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G403" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H403" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. The designers (#44, #57, #20, #56) otherwise each invent their own save path. One REST surface also proves the REST standard (#431) on real data and is the first step to a separable front end.</t>
+        </is>
+      </c>
+      <c r="I403" s="8" t="inlineStr">
+        <is>
+          <t>Tables and EF entities per #430; controller(s) per #431; optimistic concurrency with row version as ETag; publish creates an immutable version; rollback = republish an older version; import/export uses the signed package of #23; reuse #387 hydration for the read path; new migration (never edit an applied one).</t>
+        </is>
+      </c>
+      <c r="J403" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a form definition can be created as a draft, edited with If-Match, published and rolled back through the API only; two concurrent edits give 412 for the second; every call is authorized and audited; the OpenAPI document lists the operations; tests cover all of it.</t>
+        </is>
+      </c>
+      <c r="K403" s="8" t="n"/>
+      <c r="L403" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M403" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N403" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O403" s="10" t="inlineStr">
+        <is>
+          <t>#430 #431 #338</t>
+        </is>
+      </c>
+      <c r="P403" s="10" t="n"/>
+      <c r="Q403" s="10" t="n"/>
+      <c r="R403" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic data core</t>
+        </is>
+      </c>
+      <c r="S403" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T403" s="10" t="n"/>
+      <c r="U403" s="10" t="n"/>
+    </row>
+    <row r="404">
+      <c r="A404" s="10" t="n">
+        <v>435</v>
+      </c>
+      <c r="B404" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C404" s="8" t="inlineStr">
+        <is>
+          <t>Integration, Events &amp; API</t>
+        </is>
+      </c>
+      <c r="D404" s="8" t="inlineStr">
+        <is>
+          <t>API walking skeleton inside the current application: /api/v1 area with OpenAPI 3.1 generation, versioning, RFC 9457 ProblemDetails, authorization on every endpoint, RLS applied, antiforgery for browser calls and token auth for integrations, ETag support and one pilot resource</t>
+        </is>
+      </c>
+      <c r="E404" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F404" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G404" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H404" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Proves the standard end to end before 147 controllers are touched and gives the front/back separation spike (#441) something real to measure.</t>
+        </is>
+      </c>
+      <c r="I404" s="8" t="inlineStr">
+        <is>
+          <t>Use the built-in Microsoft.AspNetCore.OpenApi (no CDN, offline docs UI only if packaged locally); ProblemDetails middleware; API versioning package (licence recorded) or route-based; filter that requires an authorization policy; pilot = a base-data entity from migration wave 1 (#87) or the definition store (#434); keep MVC and API in one deployable.</t>
+        </is>
+      </c>
+      <c r="J404" s="8" t="inlineStr">
+        <is>
+          <t>Done when: GET/POST/PUT/PATCH/DELETE on the pilot resource follow #431 and are covered by tests; the OpenAPI document is served offline and lints clean; an endpoint without authorization fails a test; the browser and an integration token can both call it.</t>
+        </is>
+      </c>
+      <c r="K404" s="8" t="n"/>
+      <c r="L404" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M404" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N404" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O404" s="10" t="inlineStr">
+        <is>
+          <t>#431</t>
+        </is>
+      </c>
+      <c r="P404" s="10" t="n"/>
+      <c r="Q404" s="10" t="n"/>
+      <c r="R404" s="8" t="inlineStr">
+        <is>
+          <t>Integration &amp; API</t>
+        </is>
+      </c>
+      <c r="S404" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T404" s="10" t="n"/>
+      <c r="U404" s="10" t="n"/>
+    </row>
+    <row r="405">
+      <c r="A405" s="10" t="n">
+        <v>436</v>
+      </c>
+      <c r="B405" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C405" s="8" t="inlineStr">
+        <is>
+          <t>Integration, Events &amp; API</t>
+        </is>
+      </c>
+      <c r="D405" s="8" t="inlineStr">
+        <is>
+          <t>API quality gates in CI: OpenAPI lint (Spectral rules for naming, status codes, errors, pagination), REST conformance tests (no verbs in URLs, correct status codes, ETag/If-Match, authorization on every endpoint, ProblemDetails shape), contract/snapshot test of the published OpenAPI, and an API performance baseline with the k6 suite</t>
+        </is>
+      </c>
+      <c r="E405" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F405" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G405" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H405" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Without gates a REST standard decays within weeks (see the literal-text and component gates already used for PEMS.UI).</t>
+        </is>
+      </c>
+      <c r="I405" s="8" t="inlineStr">
+        <is>
+          <t>Spectral ruleset in the repo (offline); xUnit conformance suite using WebApplicationFactory; OpenAPI snapshot approval file; extend #202 with API scenarios; document how to update the snapshot.</t>
+        </is>
+      </c>
+      <c r="J405" s="8" t="inlineStr">
+        <is>
+          <t>Done when: CI fails on a new endpoint that breaks a rule or changes the OpenAPI document without an approved snapshot update; the k6 API baseline (p95 latency, error rate) is stored; the rules are listed in the guideline chapter.</t>
+        </is>
+      </c>
+      <c r="K405" s="8" t="n"/>
+      <c r="L405" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M405" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N405" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O405" s="10" t="inlineStr">
+        <is>
+          <t>#435</t>
+        </is>
+      </c>
+      <c r="P405" s="10" t="n"/>
+      <c r="Q405" s="10" t="n"/>
+      <c r="R405" s="8" t="inlineStr">
+        <is>
+          <t>Integration &amp; API</t>
+        </is>
+      </c>
+      <c r="S405" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T405" s="10" t="n"/>
+      <c r="U405" s="10" t="n"/>
+    </row>
+    <row r="406">
+      <c r="A406" s="10" t="n">
+        <v>437</v>
+      </c>
+      <c r="B406" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C406" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic Module Builder</t>
+        </is>
+      </c>
+      <c r="D406" s="8" t="inlineStr">
+        <is>
+          <t>Declarative data-source and action bindings: a component instance binds to an entity query, saved view, REST endpoint or static value, and its actions (navigate, call endpoint, run workflow action, open dialog, refresh) are data, not code; with parameters, permissions and error/empty/loading states from the unified states</t>
+        </is>
+      </c>
+      <c r="E406" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F406" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G406" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H406" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. A page made of components is useless until the components can be wired to data and behaviour without code.</t>
+        </is>
+      </c>
+      <c r="I406" s="8" t="inlineStr">
+        <is>
+          <t>Define DataSource (kind, entity/view/endpoint, parameters, paging, filters) and Action (kind, target, confirmation, permission) definitions per #430; resolve them on the server through the REST API (#431/#12) with RLS; component options reference them by key; use the PemsEmptyState/ErrorState/LoadingState for the three result states.</t>
+        </is>
+      </c>
+      <c r="J406" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a list component and a button on a database page load data and trigger a workflow action using only stored definitions; a user without permission sees neither the data nor the action; the binding model is validated against the manifests (#433).</t>
+        </is>
+      </c>
+      <c r="K406" s="8" t="n"/>
+      <c r="L406" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M406" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N406" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O406" s="10" t="inlineStr">
+        <is>
+          <t>#430 #434 #12</t>
+        </is>
+      </c>
+      <c r="P406" s="10" t="n"/>
+      <c r="Q406" s="10" t="n"/>
+      <c r="R406" s="8" t="inlineStr">
+        <is>
+          <t>Module builder</t>
+        </is>
+      </c>
+      <c r="S406" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T406" s="10" t="n"/>
+      <c r="U406" s="10" t="n"/>
+    </row>
+    <row r="407">
+      <c r="A407" s="10" t="n">
+        <v>438</v>
+      </c>
+      <c r="B407" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C407" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic Module Builder</t>
+        </is>
+      </c>
+      <c r="D407" s="8" t="inlineStr">
+        <is>
+          <t>Page definition and PageHost runtime: a page is a stored layout of regions and component instances; one generic host renders any published page from the database in Persian and English, with caching and invalidation, permission and visibility rules, and a fallback to the static page</t>
+        </is>
+      </c>
+      <c r="E407" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F407" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G407" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H407" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Today 303 pages are hand-written views; this is the runtime that makes a page data.</t>
+        </is>
+      </c>
+      <c r="I407" s="8" t="inlineStr">
+        <is>
+          <t>PageHost controller/view that loads the definition, resolves layout and regions, renders each instance through the component renderer (PEMS.UI) with its manifest-validated options; cache per definition version with invalidation on publish; routing for database pages; visibility rules from the expression engine (#15).</t>
+        </is>
+      </c>
+      <c r="J407" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a page created only in the database renders at its route in fa and en with no deploy; a published change shows on the next request; an unauthorized user gets 403 and a missing page 404; a static page keeps working when its override is removed; render time is within the budget set in #319.</t>
+        </is>
+      </c>
+      <c r="K407" s="8" t="n"/>
+      <c r="L407" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M407" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N407" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O407" s="10" t="inlineStr">
+        <is>
+          <t>#430 #433 #434 #437 #325</t>
+        </is>
+      </c>
+      <c r="P407" s="10" t="n"/>
+      <c r="Q407" s="10" t="n"/>
+      <c r="R407" s="8" t="inlineStr">
+        <is>
+          <t>Module builder</t>
+        </is>
+      </c>
+      <c r="S407" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T407" s="10" t="n"/>
+      <c r="U407" s="10" t="n"/>
+    </row>
+    <row r="408">
+      <c r="A408" s="10" t="n">
+        <v>439</v>
+      </c>
+      <c r="B408" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C408" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic Module Builder</t>
+        </is>
+      </c>
+      <c r="D408" s="8" t="inlineStr">
+        <is>
+          <t>Page designer: visual editor to create and edit a page from the UI (choose layout, drag component instances into regions, edit options through generated property panels, bind data sources and actions, set visibility, preview in fa/en and RTL/LTR, save draft, publish, roll back)</t>
+        </is>
+      </c>
+      <c r="E408" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F408" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G408" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H408" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. This is the user-facing half of 'all pages and components editable by the UI'.</t>
+        </is>
+      </c>
+      <c r="I408" s="8" t="inlineStr">
+        <is>
+          <t>Embedded JavaScript component per ADR-0002 (library choice recorded, offline); property panels generated from the component manifests; undo/redo; autosave to draft; uses the definition store API only (no direct DB); share the preview with the PageHost renderer.</t>
+        </is>
+      </c>
+      <c r="J408" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a non-developer builds a list-plus-detail page and a form page with the designer, previews it in both directions, publishes it and rolls it back; every save goes through the definition store API (#434); the designer is keyboard accessible.</t>
+        </is>
+      </c>
+      <c r="K408" s="8" t="n"/>
+      <c r="L408" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M408" s="10" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="N408" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O408" s="10" t="inlineStr">
+        <is>
+          <t>#438 #433</t>
+        </is>
+      </c>
+      <c r="P408" s="10" t="n"/>
+      <c r="Q408" s="10" t="n"/>
+      <c r="R408" s="8" t="inlineStr">
+        <is>
+          <t>Module builder</t>
+        </is>
+      </c>
+      <c r="S408" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T408" s="10" t="n"/>
+      <c r="U408" s="10" t="n"/>
+    </row>
+    <row r="409">
+      <c r="A409" s="10" t="n">
+        <v>440</v>
+      </c>
+      <c r="B409" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C409" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic Module Builder</t>
+        </is>
+      </c>
+      <c r="D409" s="8" t="inlineStr">
+        <is>
+          <t>Design-time governance: who may create, edit, publish or roll back each kind of definition (design roles), field-level audit of definition changes, protection and one-click reset of system pages and forms, change comments, and approval for published changes on critical pages</t>
+        </is>
+      </c>
+      <c r="E409" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F409" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G409" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H409" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Editable-by-UI without governance means any admin can break a production page; the audit and rollback must exist before the designers ship.</t>
+        </is>
+      </c>
+      <c r="I409" s="8" t="inlineStr">
+        <is>
+          <t>Design permissions in the access matrix (#60/#178); reuse the generic audit (#17) for definition tables; 'system' flag on shipped definitions with reset; optional two-person publish rule through the workflow platform.</t>
+        </is>
+      </c>
+      <c r="J409" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a user without the design role cannot change or publish a definition (API and UI); every definition change is in the audit trail with who/what/when and a diff; resetting a system page returns the shipped default; a publish on a protected page needs a second approver.</t>
+        </is>
+      </c>
+      <c r="K409" s="8" t="n"/>
+      <c r="L409" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M409" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N409" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O409" s="10" t="inlineStr">
+        <is>
+          <t>#434 #17 #178</t>
+        </is>
+      </c>
+      <c r="P409" s="10" t="n"/>
+      <c r="Q409" s="10" t="n"/>
+      <c r="R409" s="8" t="inlineStr">
+        <is>
+          <t>Module builder</t>
+        </is>
+      </c>
+      <c r="S409" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T409" s="10" t="n"/>
+      <c r="U409" s="10" t="n"/>
+    </row>
+    <row r="410">
+      <c r="A410" s="10" t="n">
+        <v>441</v>
+      </c>
+      <c r="B410" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C410" s="8" t="inlineStr">
+        <is>
+          <t>Foundation, Architecture Decisions &amp; Baseline</t>
+        </is>
+      </c>
+      <c r="D410" s="8" t="inlineStr">
+        <is>
+          <t>Frontend and backend separation: an evidence-based spike and ADR comparing (A) server-rendered Razor with PEMS.UI and JS islands, (B) the same plus a public REST API, (C) a separate single-page front end on the REST API, and (D) a BFF, scored on performance, offline installation, licence protection, Persian RTL/i18n, security (cookies, CSRF, tokens), delivery speed and team skills</t>
+        </is>
+      </c>
+      <c r="E410" s="10" t="inlineStr">
+        <is>
+          <t>Decision Needed</t>
+        </is>
+      </c>
+      <c r="F410" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G410" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H410" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. The owner wants to separate backend and frontend if there is no performance issue. The product installs on customer servers, works offline and ships no readable source of record, so the decision needs measurements, not preference. Recommendation until then: API-first (#431, #435), no front-end split yet.</t>
+        </is>
+      </c>
+      <c r="I410" s="8" t="inlineStr">
+        <is>
+          <t>Build the same list and form twice (Razor/PEMS.UI vs a small SPA on the walking-skeleton API); measure with the k6/Playwright setups (#202, #41); record bundle size, TTFB/TTI, memory, build and install impact, licence-protection impact (#96), RTL/i18n effort; write plan/adr/NNNN with the decision and what would change it.</t>
+        </is>
+      </c>
+      <c r="J410" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the spike measures time to first byte, time to interactive, payload size and server cost for one real list and one form in options A and C on the same data; the ADR records the scores, the decision and the revisit trigger; if C is chosen a migration path from the API of #435 is listed.</t>
+        </is>
+      </c>
+      <c r="K410" s="8" t="n"/>
+      <c r="L410" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M410" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N410" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O410" s="10" t="inlineStr">
+        <is>
+          <t>#435 #319 #202</t>
+        </is>
+      </c>
+      <c r="P410" s="10" t="n"/>
+      <c r="Q410" s="10" t="n"/>
+      <c r="R410" s="8" t="inlineStr">
+        <is>
+          <t>Foundation &amp; decisions</t>
+        </is>
+      </c>
+      <c r="S410" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T410" s="10" t="n"/>
+      <c r="U410" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
docs: plan audit for a dynamic, REST-based PEMS; rows #430-#441; dependency fixes (hamid) (#64)
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12367,7 +12367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U398"/>
+  <dimension ref="A1:U410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -13190,7 +13190,7 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>The root contains WebApplication1, 'New Text Document.txt' and two identical copies of the Role documents under .claude and .github.</t>
+          <t>The root contains WebApplication1, 'New Text Document.txt' and two identical copies of the Role documents under .claude and .github. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
@@ -13206,7 +13206,7 @@
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="10" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="M9" s="10" t="inlineStr">
@@ -13555,12 +13555,12 @@
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>Build one /api/d/{entity} endpoint with a single query contract (page/sort/filter/search/columns) used by every list and relation list.</t>
+          <t>Build one /api/d/{entity} endpoint with a single query contract (page/sort/filter/search/columns) used by every list and relation list. Route shape, paging style and error format come from the REST ADR (#431), not from this row; the first version must pass the API quality gates (#436).</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>Test: 500k records, filter+sort under 500 ms; a record outside the user's access never appears in results or counts.</t>
+          <t>Test: 500k records, filter+sort under 500 ms; a record outside the user's access never appears in results or counts. The route and contract follow the REST API standard (#431): resource-oriented URLs instead of verbs, ETag/If-Match, RFC 9457 errors, OpenAPI.</t>
         </is>
       </c>
       <c r="K13" s="8" t="n"/>
@@ -13581,7 +13581,7 @@
       </c>
       <c r="O13" s="10" t="inlineStr">
         <is>
-          <t>#10 #11 #178</t>
+          <t>#10 #11 #178 #431 #435</t>
         </is>
       </c>
       <c r="P13" s="10" t="inlineStr">
@@ -14270,7 +14270,7 @@
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>The current menu in _SidebarMenu.cshtml is static.</t>
+          <t>The current menu in _SidebarMenu.cshtml is static. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
@@ -14305,7 +14305,7 @@
       </c>
       <c r="O21" s="10" t="inlineStr">
         <is>
-          <t>#10</t>
+          <t>#10 #434</t>
         </is>
       </c>
       <c r="P21" s="10" t="inlineStr"/>
@@ -15742,7 +15742,7 @@
       </c>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>PEMS has static _PemsStageDiagram and _WorkOrderStagesDiagram.</t>
+          <t>PEMS has static _PemsStageDiagram and _WorkOrderStagesDiagram. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I37" s="8" t="inlineStr">
@@ -15773,7 +15773,7 @@
       </c>
       <c r="O37" s="10" t="inlineStr">
         <is>
-          <t>#31 #80</t>
+          <t>#31</t>
         </is>
       </c>
       <c r="P37" s="10" t="inlineStr"/>
@@ -15920,7 +15920,7 @@
       </c>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t>Often required in enterprise and government contracts.</t>
+          <t>Often required in enterprise and government contracts. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I39" s="8" t="inlineStr">
@@ -15936,7 +15936,7 @@
       <c r="K39" s="8" t="n"/>
       <c r="L39" s="10" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="M39" s="10" t="inlineStr">
@@ -16478,7 +16478,7 @@
       </c>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t>PEMS forms are fixed Razor; the audit found no general form builder. This is the line between software and a platform.</t>
+          <t>PEMS forms are fixed Razor; the audit found no general form builder. This is the line between software and a platform. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
         </is>
       </c>
       <c r="I45" s="8" t="inlineStr">
@@ -16509,7 +16509,7 @@
       </c>
       <c r="O45" s="10" t="inlineStr">
         <is>
-          <t>#10 #34</t>
+          <t>#10 #34 #434</t>
         </is>
       </c>
       <c r="P45" s="10" t="inlineStr">
@@ -16660,7 +16660,7 @@
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>All rules should live in one validation object with one interpreter.</t>
+          <t>All rules should live in one validation object with one interpreter. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I47" s="8" t="inlineStr">
@@ -16691,7 +16691,7 @@
       </c>
       <c r="O47" s="10" t="inlineStr">
         <is>
-          <t>#15 #45</t>
+          <t>#15 #45 #355</t>
         </is>
       </c>
       <c r="P47" s="10" t="inlineStr">
@@ -17554,7 +17554,7 @@
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>Without a guided scaffold the 'module builder' is only a table builder.</t>
+          <t>Without a guided scaffold the 'module builder' is only a table builder. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
         </is>
       </c>
       <c r="I57" s="8" t="inlineStr">
@@ -17585,7 +17585,7 @@
       </c>
       <c r="O57" s="10" t="inlineStr">
         <is>
-          <t>#10 #44 #20</t>
+          <t>#10 #44 #20 #434</t>
         </is>
       </c>
       <c r="P57" s="10" t="inlineStr">
@@ -17643,7 +17643,7 @@
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>List sizes must be structured metadata, not ad-hoc.</t>
+          <t>List sizes must be structured metadata, not ad-hoc. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
         </is>
       </c>
       <c r="I58" s="8" t="inlineStr">
@@ -17674,7 +17674,7 @@
       </c>
       <c r="O58" s="10" t="inlineStr">
         <is>
-          <t>#32</t>
+          <t>#32 #434</t>
         </is>
       </c>
       <c r="P58" s="10" t="inlineStr">
@@ -20124,7 +20124,7 @@
       </c>
       <c r="I86" s="8" t="inlineStr">
         <is>
-          <t>A module table with risk, data volume, dependencies and migration wave.</t>
+          <t>A module table with risk, data volume, dependencies and migration wave. Also classify the ~303 pages and the 147 controllers: definable from a Page definition (#438), convertible form/list/detail, or code-only; reuse the REST inventory (#432).</t>
         </is>
       </c>
       <c r="J86" s="8" t="inlineStr">
@@ -20150,7 +20150,7 @@
       </c>
       <c r="O86" s="10" t="inlineStr">
         <is>
-          <t>#29</t>
+          <t>#29 #432</t>
         </is>
       </c>
       <c r="P86" s="10" t="inlineStr"/>
@@ -29877,7 +29877,7 @@
       </c>
       <c r="J196" s="8" t="inlineStr">
         <is>
-          <t>A customer can read/write dynamic records and receive webhooks using the documentation.</t>
+          <t>A customer can read/write dynamic records and receive webhooks using the documentation. Scope: external governance (keys/tokens, rate limit, signing, documentation, monitoring) on top of the internal standard (#431) and skeleton (#435); it does not redefine the API style.</t>
         </is>
       </c>
       <c r="K196" s="8" t="n"/>
@@ -29898,7 +29898,7 @@
       </c>
       <c r="O196" s="10" t="inlineStr">
         <is>
-          <t>#12</t>
+          <t>#12 #431 #435</t>
         </is>
       </c>
       <c r="P196" s="10" t="inlineStr"/>
@@ -31044,7 +31044,7 @@
       </c>
       <c r="H209" s="8" t="inlineStr">
         <is>
-          <t>Audit E22: number/currency/ZWNJ standards are not defined.</t>
+          <t>Audit E22: number/currency/ZWNJ standards are not defined. 2026-10-28 audit: overlaps #367 (formatting engine); merge when #367 starts. Digit swap exists (IPemsLocale.Digits, SCRUM-426). 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I209" s="8" t="inlineStr">
@@ -31060,7 +31060,7 @@
       <c r="K209" s="8" t="n"/>
       <c r="L209" s="10" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="M209" s="10" t="inlineStr">
@@ -32379,7 +32379,7 @@
       </c>
       <c r="H224" s="8" t="inlineStr">
         <is>
-          <t>A basic PWA exists (manifest + service worker). A working mobile view for every screen type and on-site time/material tracking are known needs.</t>
+          <t>A basic PWA exists (manifest + service worker). A working mobile view for every screen type and on-site time/material tracking are known needs. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I224" s="8" t="inlineStr">
@@ -32395,7 +32395,7 @@
       <c r="K224" s="8" t="n"/>
       <c r="L224" s="10" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="M224" s="10" t="inlineStr">
@@ -32472,7 +32472,7 @@
       </c>
       <c r="H225" s="8" t="inlineStr">
         <is>
-          <t>Audit E16: permits, LOTO and gas tests are desktop only.</t>
+          <t>Audit E16: permits, LOTO and gas tests are desktop only. 2026-10-28 plan audit: follows #223 to M5.</t>
         </is>
       </c>
       <c r="I225" s="8" t="inlineStr">
@@ -32488,7 +32488,7 @@
       <c r="K225" s="8" t="n"/>
       <c r="L225" s="10" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="M225" s="10" t="inlineStr">
@@ -39887,7 +39887,7 @@
       </c>
       <c r="H311" s="8" t="inlineStr">
         <is>
-          <t>IDatabaseUpdateService (PEMS.Application) + DatabaseUpdateService (PEMS.Persistence) with the pure DatabaseSetupClassifier: FirstRun, UpdateAvailable, UpToDate, UnmanagedSchema, DatabaseNewerThanApplication, Unreachable. Entity DatabaseUpdateRun + migration DatabaseUpdateRuns (audit of every attempt). Admin &gt; System Monitoring &gt; Database Update (/Admin/DatabaseUpdate, SystemAdmin, backup confirmation, antiforgery). GET /health/database (anonymous, state only). Verified 2026-10-22: 9 tests (classifier + real SQL Server install/update/unmanaged on throw-away LocalDB databases); page compiled and anonymous access redirects to login. Driven in a browser as the seeded dev admin on 2026-10-23: state card, pending list, backup confirmation refused/accepted, update applied, run recorded as Admin/Update.</t>
+          <t>IDatabaseUpdateService (PEMS.Application) + DatabaseUpdateService (PEMS.Persistence) with the pure DatabaseSetupClassifier: FirstRun, UpdateAvailable, UpToDate, UnmanagedSchema, DatabaseNewerThanApplication, Unreachable. Entity DatabaseUpdateRun + migration DatabaseUpdateRuns (audit of every attempt). Admin &gt; System Monitoring &gt; Database Update (/Admin/DatabaseUpdate, SystemAdmin, backup confirmation, antiforgery). GET /health/database (anonymous, state only). Verified 2026-10-22: 9 tests (classifier + real SQL Server install/update/unmanaged on throw-away LocalDB databases); page compiled and anonymous access redirects to login. Driven in a browser as the seeded dev admin on 2026-10-23: state card, pending list, backup confirmation refused/accepted, update applied, run recorded as Admin/Update. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I311" s="8" t="inlineStr">
@@ -39920,11 +39920,7 @@
           <t>Sales blocker</t>
         </is>
       </c>
-      <c r="O311" s="10" t="inlineStr">
-        <is>
-          <t>#309</t>
-        </is>
-      </c>
+      <c r="O311" s="10" t="n"/>
       <c r="P311" s="10" t="n"/>
       <c r="Q311" s="10" t="n"/>
       <c r="R311" s="8" t="inlineStr">
@@ -39976,7 +39972,7 @@
       </c>
       <c r="H312" s="8" t="inlineStr">
         <is>
-          <t>Moved with git mv to legacy-trash/manual-sql/ (same relative paths, README maps each to its replacement): PEMS.Persistence/Scripts/EnableFullTextSearch.sql (now migration FullTextSearch), docs/procurement/*.migration.sql and P4_P5_delta/PREFLIGHT, docs/task manager/TaskManagerCore_migration.sql, plus the root InitialCreate.sql (full-schema script). References in docs and code comments updated. Operator tools that are not schema setup (scripts/cmms, scripts/rcm data repairs and read-only reports, docs/sql checks, deploy/ reviewed-script flow) were deliberately left in place; see #313.</t>
+          <t>Moved with git mv to legacy-trash/manual-sql/ (same relative paths, README maps each to its replacement): PEMS.Persistence/Scripts/EnableFullTextSearch.sql (now migration FullTextSearch), docs/procurement/*.migration.sql and P4_P5_delta/PREFLIGHT, docs/task manager/TaskManagerCore_migration.sql, plus the root InitialCreate.sql (full-schema script). References in docs and code comments updated. Operator tools that are not schema setup (scripts/cmms, scripts/rcm data repairs and read-only reports, docs/sql checks, deploy/ reviewed-script flow) were deliberately left in place; see #313. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I312" s="8" t="inlineStr">
@@ -40009,11 +40005,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="O312" s="10" t="inlineStr">
-        <is>
-          <t>#309</t>
-        </is>
-      </c>
+      <c r="O312" s="10" t="n"/>
       <c r="P312" s="10" t="n"/>
       <c r="Q312" s="10" t="n"/>
       <c r="R312" s="8" t="inlineStr">
@@ -40065,7 +40057,7 @@
       </c>
       <c r="H313" s="8" t="inlineStr">
         <is>
-          <t>deploy-demo.yml: model-drift gate (dotnet ef migrations has-pending-model-changes), jq injects the demo connection string and Database={CreateIfMissing:false,MigrateOnStartup:true}, sed raises the IIS startupTimeLimit to 900 s (the first run installs the whole schema before serving), FTP upload, then polls DEMO_SITE_URL/health/database until UpToDate (fails the run after 30 minutes). YAML validated; web.config patch checked on a real publish. Not yet executed on GitHub. 2026-10-24 first runs on the demo branch: build, drift gate, database-free tests, publish and the FTP upload from the GitHub runner PASS; the post-deploy health check failed - the demo site has no valid TLS certificate and the application does not answer on first start (details and steps: docs/deployment/DEMO_DEPLOYMENT.md, row #340).</t>
+          <t>deploy-demo.yml: model-drift gate (dotnet ef migrations has-pending-model-changes), jq injects the demo connection string and Database={CreateIfMissing:false,MigrateOnStartup:true}, sed raises the IIS startupTimeLimit to 900 s (the first run installs the whole schema before serving), FTP upload, then polls DEMO_SITE_URL/health/database until UpToDate (fails the run after 30 minutes). YAML validated; web.config patch checked on a real publish. Not yet executed on GitHub. 2026-10-24 first runs on the demo branch: build, drift gate, database-free tests, publish and the FTP upload from the GitHub runner PASS; the post-deploy health check failed - the demo site has no valid TLS certificate and the application does not answer on first start (details and steps: docs/deployment/DEMO_DEPLOYMENT.md, row #340). 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I313" s="8" t="inlineStr">
@@ -40100,7 +40092,7 @@
       </c>
       <c r="O313" s="10" t="inlineStr">
         <is>
-          <t>#295 #309 #310</t>
+          <t>#295 #310</t>
         </is>
       </c>
       <c r="P313" s="10" t="n"/>
@@ -42320,12 +42312,12 @@
       </c>
       <c r="H339" s="8" t="inlineStr">
         <is>
-          <t>Row #10 (the registry) is an XL implementation task and #12-#17 all depend on it. Nothing can be built safely until the data model, versioning and publishing rules are written down and agreed. Decided inputs: hybrid storage (#4): real tables for user-built entities, a JSON column for custom fields on existing entities.</t>
+          <t>Row #10 (the registry) is an XL implementation task and #12-#17 all depend on it. Nothing can be built safely until the data model, versioning and publishing rules are written down and agreed. Decided inputs: hybrid storage (#4): real tables for user-built entities, a JSON column for custom fields on existing entities. 2026-10-28 audit: the registry must cover UI definitions, not only data entities (row #430).</t>
         </is>
       </c>
       <c r="I339" s="8" t="inlineStr">
         <is>
-          <t>1) List the registry objects and their relations (App, Module, Entity, Field, Relation, View, Form, Workflow reference, Version). 2) Define draft/published versions, rollback and what a publish changes. 3) Define how static (existing) entities appear in the registry (#14 JSON extension column). 4) Define the cache and invalidation contract (#28). 5) Sketch the EF entity classes (compile-only, in a branch, not merged). 6) List open questions. Output: docs/architecture/METADATA_REGISTRY_DESIGN.md and an ADR under plan/adr.</t>
+          <t>1) List the registry objects and their relations (App, Module, Entity, Field, Relation, View, Form, Workflow reference, Version). 2) Define draft/published versions, rollback and what a publish changes. 3) Define how static (existing) entities appear in the registry (#14 JSON extension column). 4) Define the cache and invalidation contract (#28). 5) Sketch the EF entity classes (compile-only, in a branch, not merged). 6) List open questions. Output: docs/architecture/METADATA_REGISTRY_DESIGN.md and an ADR under plan/adr. 6) Put UI definitions (page, layout, component instance, data source, action, menu, theme) in the same envelope and versioning rules; see the ADR row #430.</t>
         </is>
       </c>
       <c r="J339" s="8" t="inlineStr">
@@ -42773,7 +42765,7 @@
       </c>
       <c r="H344" s="8" t="inlineStr">
         <is>
-          <t>A customer whose production server is offline must be able to recover a lost administrator password with the vendor's help, without a back door in the product and without any remote access. The licence flow already proves that file exchange works offline; the reset reuses its shape with its own key. Gate: this row can start only after #342 (licence flow end to end) is Done. Independent of the separate administrator-recovery work done by Saber (second-admin reset, one-time recovery codes, server-side break-glass, shared audit/notification/session revocation): that work does not wait for the licence flow and this row does not block it; this flow plugs into it as the optional vendor-assisted recovery path, which must stay off until the customer enables it.</t>
+          <t>A customer whose production server is offline must be able to recover a lost administrator password with the vendor's help, without a back door in the product and without any remote access. The licence flow already proves that file exchange works offline; the reset reuses its shape with its own key. Gate: this row can start only after #342 (licence flow end to end) is Done. Independent of the separate administrator-recovery work done by Saber (second-admin reset, one-time recovery codes, server-side break-glass, shared audit/notification/session revocation): that work does not wait for the licence flow and this row does not block it; this flow plugs into it as the optional vendor-assisted recovery path, which must stay off until the customer enables it. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I344" s="8" t="inlineStr">
@@ -42804,7 +42796,7 @@
       </c>
       <c r="O344" s="10" t="inlineStr">
         <is>
-          <t>#96 #107 #178 #182 #184 #339 #342</t>
+          <t>#96 #107 #178 #182 #339 #342</t>
         </is>
       </c>
       <c r="P344" s="10" t="n"/>
@@ -43797,7 +43789,7 @@
       </c>
       <c r="H356" s="8" t="inlineStr">
         <is>
-          <t>Validation in PEMS today is thin and scattered: 260 entities but only 26 [Required] and 45 [MaxLength] attributes in 28 files, no [Range], [StringLength] or regular-expression rule anywhere, no validation library, ModelState.IsValid is checked in 8 controllers, and 64 of 65 plain text inputs in the views have no maxlength. Dynamic forms need one declarative description of the rules per field type before any engine or UI is built. Rule-builder row #46 covers user-defined rules; this row defines the built-in constraints every type carries.</t>
+          <t>Validation in PEMS today is thin and scattered: 260 entities but only 26 [Required] and 45 [MaxLength] attributes in 28 files, no [Range], [StringLength] or regular-expression rule anywhere, no validation library, ModelState.IsValid is checked in 8 controllers, and 64 of 65 plain text inputs in the views have no maxlength. Dynamic forms need one declarative description of the rules per field type before any engine or UI is built. Rule-builder row #46 covers user-defined rules; this row defines the built-in constraints every type carries. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I356" s="8" t="inlineStr">
@@ -43828,7 +43820,7 @@
       </c>
       <c r="O356" s="10" t="inlineStr">
         <is>
-          <t>#11 #338 #46</t>
+          <t>#11 #338</t>
         </is>
       </c>
       <c r="P356" s="10" t="inlineStr">
@@ -44238,7 +44230,7 @@
       </c>
       <c r="H361" s="8" t="inlineStr">
         <is>
-          <t>Import Center has 11 imports with their own checks. A blank cell in an update row must leave the value alone, a malformed identifier must never reach the database as a server error, and a default value must never be saved as NULL by a bulk path.</t>
+          <t>Import Center has 11 imports with their own checks. A blank cell in an update row must leave the value alone, a malformed identifier must never reach the database as a server error, and a default value must never be saved as NULL by a bulk path. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I361" s="8" t="inlineStr">
@@ -44254,7 +44246,7 @@
       <c r="K361" s="8" t="n"/>
       <c r="L361" s="10" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="M361" s="10" t="inlineStr">
@@ -44760,7 +44752,7 @@
       </c>
       <c r="H367" s="8" t="inlineStr">
         <is>
-          <t>Formatting in PEMS is done page by page: 377 hand-written date and time format strings in 138 views using 12 different patterns, 217 number format strings, 103 native date, 8 datetime-local and 137 number inputs whose look follows the browser locale, and Jalali support in only 6 files. Existing rows #24, #205, #206, #208 and #209 ask for translated labels, Persian digits, the Jalali calendar and fixed reports, but nothing defines where a field's format lives or how it relates to validation. A comparable implementation shows the risks: one hard-coded locale in its date component, date strings built without zero padding, an invalid-date defect in downloaded reports and a deprecated date library for the Jalali picker.</t>
+          <t>Formatting in PEMS is done page by page: 377 hand-written date and time format strings in 138 views using 12 different patterns, 217 number format strings, 103 native date, 8 datetime-local and 137 number inputs whose look follows the browser locale, and Jalali support in only 6 files. Existing rows #24, #205, #206, #208 and #209 ask for translated labels, Persian digits, the Jalali calendar and fixed reports, but nothing defines where a field's format lives or how it relates to validation. A comparable implementation shows the risks: one hard-coded locale in its date component, date strings built without zero padding, an invalid-date defect in downloaded reports and a deprecated date library for the Jalali picker. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I367" s="8" t="inlineStr">
@@ -44791,7 +44783,7 @@
       </c>
       <c r="O367" s="10" t="inlineStr">
         <is>
-          <t>#11 #355 #24 #205</t>
+          <t>#11 #355 #205 #386</t>
         </is>
       </c>
       <c r="P367" s="10" t="inlineStr">
@@ -45112,7 +45104,7 @@
       </c>
       <c r="H371" s="8" t="inlineStr">
         <is>
-          <t>Row #24 stores translatable strings in metadata; nothing defines how they are resolved in a context or how mixed-direction text (codes, e-mail, URLs, numbers inside Persian sentences) is displayed. W3C: keep localisation separate from translation.</t>
+          <t>Row #24 stores translatable strings in metadata; nothing defines how they are resolved in a context or how mixed-direction text (codes, e-mail, URLs, numbers inside Persian sentences) is displayed. W3C: keep localisation separate from translation. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I371" s="8" t="inlineStr">
@@ -45143,7 +45135,7 @@
       </c>
       <c r="O371" s="10" t="inlineStr">
         <is>
-          <t>#24 #366</t>
+          <t>#366 #386</t>
         </is>
       </c>
       <c r="P371" s="10" t="inlineStr">
@@ -45201,7 +45193,7 @@
       </c>
       <c r="H372" s="8" t="inlineStr">
         <is>
-          <t>Exports are a second place where formats drift: strings instead of typed cells cannot be sorted or summed, and a comparable platform shipped an invalid-date defect in downloaded reports and layout overflow in PDF exports.</t>
+          <t>Exports are a second place where formats drift: strings instead of typed cells cannot be sorted or summed, and a comparable platform shipped an invalid-date defect in downloaded reports and layout overflow in PDF exports. 2026-10-28 plan audit: dependency/milestone corrected (see docs/audits/2026-10-28-dynamic-restful-audit.md).</t>
         </is>
       </c>
       <c r="I372" s="8" t="inlineStr">
@@ -45217,7 +45209,7 @@
       <c r="K372" s="8" t="n"/>
       <c r="L372" s="10" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="M372" s="10" t="inlineStr">
@@ -46603,7 +46595,7 @@
       </c>
       <c r="J388" s="8" t="inlineStr">
         <is>
-          <t>Done when: a form created in the database renders through PEMS.UI in fa and en with no deploy; a saved translation shows on the next request; tests prove the round trip and the fallback.</t>
+          <t>Done when: a form created in the database renders through PEMS.UI in fa and en with no deploy; a saved translation shows on the next request; tests prove the round trip and the fallback. Reads and writes go through the definition store API (#434) in the shared definition envelope (#430).</t>
         </is>
       </c>
       <c r="K388" s="8" t="n"/>
@@ -46624,7 +46616,7 @@
       </c>
       <c r="O388" s="10" t="inlineStr">
         <is>
-          <t>#386 #10 #334</t>
+          <t>#386 #10 #334 #430 #434</t>
         </is>
       </c>
       <c r="P388" s="10" t="n"/>
@@ -47535,6 +47527,1026 @@
           <t>Member A</t>
         </is>
       </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="10" t="n">
+        <v>430</v>
+      </c>
+      <c r="B399" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C399" s="8" t="inlineStr">
+        <is>
+          <t>Foundation, Architecture Decisions &amp; Baseline</t>
+        </is>
+      </c>
+      <c r="D399" s="8" t="inlineStr">
+        <is>
+          <t>ADR: UI definition model - everything is a definition. One versioned envelope (key, version, status draft/published/archived, owner app, ETag, translations as TranslatableText JSON) for pages, layouts, component instances, forms, views, dashboards, reports, menus, themes, data sources and actions, stored in the database and edited from the UI</t>
+        </is>
+      </c>
+      <c r="E399" s="10" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="F399" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G399" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H399" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. The backlog designs forms (#44), views (#57), dashboards (#58), reports (#59), menus (#20) and workflows (#67) one by one, each with its own storage idea, and nothing defines a page or a component instance. 'All pages, components and forms creatable and editable from the UI' needs one shared definition model first.</t>
+        </is>
+      </c>
+      <c r="I399" s="8" t="inlineStr">
+        <is>
+          <t>1) List the definition kinds and their relations (Page, Layout, Region, ComponentInstance, DataSource, Action, Form, View, Dashboard, Report, Menu, Theme). 2) One envelope and one version/publish/rollback rule for all of them, reusing the registry (#338). 3) Component instance = component key + options JSON that validates against the component manifest (#433). 4) Static-to-dynamic coexistence: a database definition may override or extend a code default; rollback = delete the override. 5) Cache, invalidation, size limits, security (who can publish). 6) Write plan/adr/NNNN and update the registry design.</t>
+        </is>
+      </c>
+      <c r="J399" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the ADR is accepted (storage, envelope, draft/publish/rollback, how a static page and a database page coexist, cache and invalidation, size and security limits); rows #338, #387, #44, #57 and #20 reference it; open questions have an owner.</t>
+        </is>
+      </c>
+      <c r="K399" s="8" t="n"/>
+      <c r="L399" s="10" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="M399" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N399" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O399" s="10" t="inlineStr">
+        <is>
+          <t>#338</t>
+        </is>
+      </c>
+      <c r="P399" s="10" t="n"/>
+      <c r="Q399" s="10" t="n"/>
+      <c r="R399" s="8" t="inlineStr">
+        <is>
+          <t>Foundation &amp; decisions</t>
+        </is>
+      </c>
+      <c r="S399" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T399" s="10" t="n"/>
+      <c r="U399" s="10" t="n"/>
+    </row>
+    <row r="400">
+      <c r="A400" s="10" t="n">
+        <v>431</v>
+      </c>
+      <c r="B400" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C400" s="8" t="inlineStr">
+        <is>
+          <t>Foundation, Architecture Decisions &amp; Baseline</t>
+        </is>
+      </c>
+      <c r="D400" s="8" t="inlineStr">
+        <is>
+          <t>ADR: REST API standard - resource-oriented routes (nouns, no verbs), HTTP semantics and status codes, paging/filter/sort, ETag and If-Match, Idempotency-Key, PATCH semantics, bulk and long-running operations, RFC 9457 errors, versioning, Accept-Language and TranslatableText, dates and time zones, allowed-actions links; OpenAPI 3.1 as the contract; plus a guideline chapter</t>
+        </is>
+      </c>
+      <c r="E400" s="10" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="F400" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G400" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H400" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Today there is no REST surface: 147 controllers, none marked [ApiController], 163 GET and 668 POST actions, no PUT/PATCH/DELETE, no OpenAPI, no ProblemDetails, no API versioning; 22 controller files return ad hoc JSON. Row #12 plans /api/d/{entity} without a standard to follow.</t>
+        </is>
+      </c>
+      <c r="I400" s="8" t="inlineStr">
+        <is>
+          <t>1) Resource naming and URL rules (plural nouns, nested only for ownership, actions as POST sub-resources, e.g. POST /work-orders/{id}/actions/approve). 2) Verbs and status codes (200/201+Location/204/202, 400/401/403/404/409/412/422/428/429). 3) Query contract for paging, sorting, filtering, search, field selection (offset vs cursor decision). 4) Concurrency (ETag/If-Match, 412/428) and idempotency (Idempotency-Key). 5) Errors: RFC 9457 with the field-error list of #363. 6) Versioning and deprecation. 7) i18n: Accept-Language, TranslatableText JSON shape, UTC/ISO dates. 8) Allowed-actions and permission hints for dynamic UIs. 9) Browser auth (cookie plus antiforgery) vs integration auth (token). 10) Write the ADR and the guideline chapter.</t>
+        </is>
+      </c>
+      <c r="J400" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the ADR is accepted and a short guideline chapter (docs/guidelines) lists the rules with one good and one bad example each; rows #12, #195, #363, #18, #28 and #387 reference it; the open questions have an owner.</t>
+        </is>
+      </c>
+      <c r="K400" s="8" t="n"/>
+      <c r="L400" s="10" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="M400" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N400" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O400" s="10" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+      <c r="P400" s="10" t="n"/>
+      <c r="Q400" s="10" t="n"/>
+      <c r="R400" s="8" t="inlineStr">
+        <is>
+          <t>Foundation &amp; decisions</t>
+        </is>
+      </c>
+      <c r="S400" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T400" s="10" t="n"/>
+      <c r="U400" s="10" t="n"/>
+    </row>
+    <row r="401">
+      <c r="A401" s="10" t="n">
+        <v>432</v>
+      </c>
+      <c r="B401" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C401" s="8" t="inlineStr">
+        <is>
+          <t>Foundation, Architecture Decisions &amp; Baseline</t>
+        </is>
+      </c>
+      <c r="D401" s="8" t="inlineStr">
+        <is>
+          <t>REST inventory of the existing 147 controllers and ~830 actions: classify each as view-only MVC (stays), form post (becomes a resource call later), JSON endpoint (normalise), or API candidate; produce the target resource map and a conformance score per controller</t>
+        </is>
+      </c>
+      <c r="E401" s="10" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="F401" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G401" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H401" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Needed to plan the strangler for the API the same way #85 plans it for modules; without it the API work cannot be sized.</t>
+        </is>
+      </c>
+      <c r="I401" s="8" t="inlineStr">
+        <is>
+          <t>Script the inventory (routes, verbs, return types, [Authorize] policies, antiforgery) with Roslyn or reflection; classify by hand the heaviest 30 controllers; list verbs-in-URL, state-changing GETs and missing authorization; propose the target resource names per #431.</t>
+        </is>
+      </c>
+      <c r="J401" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a table (controller, actions, kind, target resource, wave, owner) is committed under docs/audits; the 22 JSON-returning controllers each have a target shape; rows #85 and #12 reference it.</t>
+        </is>
+      </c>
+      <c r="K401" s="8" t="n"/>
+      <c r="L401" s="10" t="inlineStr">
+        <is>
+          <t>M0</t>
+        </is>
+      </c>
+      <c r="M401" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N401" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O401" s="10" t="inlineStr">
+        <is>
+          <t>#431</t>
+        </is>
+      </c>
+      <c r="P401" s="10" t="n"/>
+      <c r="Q401" s="10" t="n"/>
+      <c r="R401" s="8" t="inlineStr">
+        <is>
+          <t>Foundation &amp; decisions</t>
+        </is>
+      </c>
+      <c r="S401" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T401" s="10" t="n"/>
+      <c r="U401" s="10" t="n"/>
+    </row>
+    <row r="402">
+      <c r="A402" s="10" t="n">
+        <v>433</v>
+      </c>
+      <c r="B402" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C402" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D402" s="8" t="inlineStr">
+        <is>
+          <t>Component manifest: every PEMS.UI component publishes a machine-readable description (key, options JSON Schema generated from the options records, slots, events, accessibility notes, sample) that drives the designers' property panels, validates stored JSON and feeds the component catalog</t>
+        </is>
+      </c>
+      <c r="E402" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F402" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G402" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H402" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Options are now named-property records with required/optional members (SCRUM-424), so a schema can be generated rather than written. A designer cannot offer 'add a component to a page' without knowing each component's inputs.</t>
+        </is>
+      </c>
+      <c r="I402" s="8" t="inlineStr">
+        <is>
+          <t>Generate JSON Schema (System.Text.Json schema exporter or NJsonSchema, licence recorded) from the options types; add [PemsComponent] metadata (category, icon key, TranslatableText name/description); expose through the definition store (#434) and the catalog (#326); add the completeness test.</t>
+        </is>
+      </c>
+      <c r="J402" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a generator produces one JSON manifest per component from the code (no hand-written schema); a stored options JSON that violates the schema is rejected with a field error list; the manifest of Button, Badge, Field, Table, Form, Empty/Error/Loading state exists and a test fails when a component has no manifest.</t>
+        </is>
+      </c>
+      <c r="K402" s="8" t="n"/>
+      <c r="L402" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M402" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N402" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O402" s="10" t="inlineStr">
+        <is>
+          <t>#321 #430</t>
+        </is>
+      </c>
+      <c r="P402" s="10" t="n"/>
+      <c r="Q402" s="10" t="n"/>
+      <c r="R402" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S402" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T402" s="10" t="n"/>
+      <c r="U402" s="10" t="n"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="10" t="n">
+        <v>434</v>
+      </c>
+      <c r="B403" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C403" s="8" t="inlineStr">
+        <is>
+          <t>Metadata Core &amp; Dynamic Platform</t>
+        </is>
+      </c>
+      <c r="D403" s="8" t="inlineStr">
+        <is>
+          <t>Definition store REST API: create, read, update (If-Match), list, publish, unpublish, roll back, export and import of definitions under /api/v1/definitions, with ETag, RFC 9457 errors, OpenAPI, draft/published versions and audit; the designers are ordinary clients of it</t>
+        </is>
+      </c>
+      <c r="E403" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F403" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G403" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H403" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. The designers (#44, #57, #20, #56) otherwise each invent their own save path. One REST surface also proves the REST standard (#431) on real data and is the first step to a separable front end.</t>
+        </is>
+      </c>
+      <c r="I403" s="8" t="inlineStr">
+        <is>
+          <t>Tables and EF entities per #430; controller(s) per #431; optimistic concurrency with row version as ETag; publish creates an immutable version; rollback = republish an older version; import/export uses the signed package of #23; reuse #387 hydration for the read path; new migration (never edit an applied one).</t>
+        </is>
+      </c>
+      <c r="J403" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a form definition can be created as a draft, edited with If-Match, published and rolled back through the API only; two concurrent edits give 412 for the second; every call is authorized and audited; the OpenAPI document lists the operations; tests cover all of it.</t>
+        </is>
+      </c>
+      <c r="K403" s="8" t="n"/>
+      <c r="L403" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M403" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N403" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O403" s="10" t="inlineStr">
+        <is>
+          <t>#430 #431 #338</t>
+        </is>
+      </c>
+      <c r="P403" s="10" t="n"/>
+      <c r="Q403" s="10" t="n"/>
+      <c r="R403" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic data core</t>
+        </is>
+      </c>
+      <c r="S403" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T403" s="10" t="n"/>
+      <c r="U403" s="10" t="n"/>
+    </row>
+    <row r="404">
+      <c r="A404" s="10" t="n">
+        <v>435</v>
+      </c>
+      <c r="B404" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C404" s="8" t="inlineStr">
+        <is>
+          <t>Integration, Events &amp; API</t>
+        </is>
+      </c>
+      <c r="D404" s="8" t="inlineStr">
+        <is>
+          <t>API walking skeleton inside the current application: /api/v1 area with OpenAPI 3.1 generation, versioning, RFC 9457 ProblemDetails, authorization on every endpoint, RLS applied, antiforgery for browser calls and token auth for integrations, ETag support and one pilot resource</t>
+        </is>
+      </c>
+      <c r="E404" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F404" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G404" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H404" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Proves the standard end to end before 147 controllers are touched and gives the front/back separation spike (#441) something real to measure.</t>
+        </is>
+      </c>
+      <c r="I404" s="8" t="inlineStr">
+        <is>
+          <t>Use the built-in Microsoft.AspNetCore.OpenApi (no CDN, offline docs UI only if packaged locally); ProblemDetails middleware; API versioning package (licence recorded) or route-based; filter that requires an authorization policy; pilot = a base-data entity from migration wave 1 (#87) or the definition store (#434); keep MVC and API in one deployable.</t>
+        </is>
+      </c>
+      <c r="J404" s="8" t="inlineStr">
+        <is>
+          <t>Done when: GET/POST/PUT/PATCH/DELETE on the pilot resource follow #431 and are covered by tests; the OpenAPI document is served offline and lints clean; an endpoint without authorization fails a test; the browser and an integration token can both call it.</t>
+        </is>
+      </c>
+      <c r="K404" s="8" t="n"/>
+      <c r="L404" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M404" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N404" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O404" s="10" t="inlineStr">
+        <is>
+          <t>#431</t>
+        </is>
+      </c>
+      <c r="P404" s="10" t="n"/>
+      <c r="Q404" s="10" t="n"/>
+      <c r="R404" s="8" t="inlineStr">
+        <is>
+          <t>Integration &amp; API</t>
+        </is>
+      </c>
+      <c r="S404" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T404" s="10" t="n"/>
+      <c r="U404" s="10" t="n"/>
+    </row>
+    <row r="405">
+      <c r="A405" s="10" t="n">
+        <v>436</v>
+      </c>
+      <c r="B405" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C405" s="8" t="inlineStr">
+        <is>
+          <t>Integration, Events &amp; API</t>
+        </is>
+      </c>
+      <c r="D405" s="8" t="inlineStr">
+        <is>
+          <t>API quality gates in CI: OpenAPI lint (Spectral rules for naming, status codes, errors, pagination), REST conformance tests (no verbs in URLs, correct status codes, ETag/If-Match, authorization on every endpoint, ProblemDetails shape), contract/snapshot test of the published OpenAPI, and an API performance baseline with the k6 suite</t>
+        </is>
+      </c>
+      <c r="E405" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F405" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G405" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H405" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Without gates a REST standard decays within weeks (see the literal-text and component gates already used for PEMS.UI).</t>
+        </is>
+      </c>
+      <c r="I405" s="8" t="inlineStr">
+        <is>
+          <t>Spectral ruleset in the repo (offline); xUnit conformance suite using WebApplicationFactory; OpenAPI snapshot approval file; extend #202 with API scenarios; document how to update the snapshot.</t>
+        </is>
+      </c>
+      <c r="J405" s="8" t="inlineStr">
+        <is>
+          <t>Done when: CI fails on a new endpoint that breaks a rule or changes the OpenAPI document without an approved snapshot update; the k6 API baseline (p95 latency, error rate) is stored; the rules are listed in the guideline chapter.</t>
+        </is>
+      </c>
+      <c r="K405" s="8" t="n"/>
+      <c r="L405" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M405" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N405" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O405" s="10" t="inlineStr">
+        <is>
+          <t>#435</t>
+        </is>
+      </c>
+      <c r="P405" s="10" t="n"/>
+      <c r="Q405" s="10" t="n"/>
+      <c r="R405" s="8" t="inlineStr">
+        <is>
+          <t>Integration &amp; API</t>
+        </is>
+      </c>
+      <c r="S405" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T405" s="10" t="n"/>
+      <c r="U405" s="10" t="n"/>
+    </row>
+    <row r="406">
+      <c r="A406" s="10" t="n">
+        <v>437</v>
+      </c>
+      <c r="B406" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C406" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic Module Builder</t>
+        </is>
+      </c>
+      <c r="D406" s="8" t="inlineStr">
+        <is>
+          <t>Declarative data-source and action bindings: a component instance binds to an entity query, saved view, REST endpoint or static value, and its actions (navigate, call endpoint, run workflow action, open dialog, refresh) are data, not code; with parameters, permissions and error/empty/loading states from the unified states</t>
+        </is>
+      </c>
+      <c r="E406" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F406" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G406" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H406" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. A page made of components is useless until the components can be wired to data and behaviour without code.</t>
+        </is>
+      </c>
+      <c r="I406" s="8" t="inlineStr">
+        <is>
+          <t>Define DataSource (kind, entity/view/endpoint, parameters, paging, filters) and Action (kind, target, confirmation, permission) definitions per #430; resolve them on the server through the REST API (#431/#12) with RLS; component options reference them by key; use the PemsEmptyState/ErrorState/LoadingState for the three result states.</t>
+        </is>
+      </c>
+      <c r="J406" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a list component and a button on a database page load data and trigger a workflow action using only stored definitions; a user without permission sees neither the data nor the action; the binding model is validated against the manifests (#433).</t>
+        </is>
+      </c>
+      <c r="K406" s="8" t="n"/>
+      <c r="L406" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M406" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N406" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O406" s="10" t="inlineStr">
+        <is>
+          <t>#430 #434 #12</t>
+        </is>
+      </c>
+      <c r="P406" s="10" t="n"/>
+      <c r="Q406" s="10" t="n"/>
+      <c r="R406" s="8" t="inlineStr">
+        <is>
+          <t>Module builder</t>
+        </is>
+      </c>
+      <c r="S406" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T406" s="10" t="n"/>
+      <c r="U406" s="10" t="n"/>
+    </row>
+    <row r="407">
+      <c r="A407" s="10" t="n">
+        <v>438</v>
+      </c>
+      <c r="B407" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C407" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic Module Builder</t>
+        </is>
+      </c>
+      <c r="D407" s="8" t="inlineStr">
+        <is>
+          <t>Page definition and PageHost runtime: a page is a stored layout of regions and component instances; one generic host renders any published page from the database in Persian and English, with caching and invalidation, permission and visibility rules, and a fallback to the static page</t>
+        </is>
+      </c>
+      <c r="E407" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F407" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G407" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H407" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Today 303 pages are hand-written views; this is the runtime that makes a page data.</t>
+        </is>
+      </c>
+      <c r="I407" s="8" t="inlineStr">
+        <is>
+          <t>PageHost controller/view that loads the definition, resolves layout and regions, renders each instance through the component renderer (PEMS.UI) with its manifest-validated options; cache per definition version with invalidation on publish; routing for database pages; visibility rules from the expression engine (#15).</t>
+        </is>
+      </c>
+      <c r="J407" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a page created only in the database renders at its route in fa and en with no deploy; a published change shows on the next request; an unauthorized user gets 403 and a missing page 404; a static page keeps working when its override is removed; render time is within the budget set in #319.</t>
+        </is>
+      </c>
+      <c r="K407" s="8" t="n"/>
+      <c r="L407" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M407" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N407" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O407" s="10" t="inlineStr">
+        <is>
+          <t>#430 #433 #434 #437 #325</t>
+        </is>
+      </c>
+      <c r="P407" s="10" t="n"/>
+      <c r="Q407" s="10" t="n"/>
+      <c r="R407" s="8" t="inlineStr">
+        <is>
+          <t>Module builder</t>
+        </is>
+      </c>
+      <c r="S407" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T407" s="10" t="n"/>
+      <c r="U407" s="10" t="n"/>
+    </row>
+    <row r="408">
+      <c r="A408" s="10" t="n">
+        <v>439</v>
+      </c>
+      <c r="B408" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C408" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic Module Builder</t>
+        </is>
+      </c>
+      <c r="D408" s="8" t="inlineStr">
+        <is>
+          <t>Page designer: visual editor to create and edit a page from the UI (choose layout, drag component instances into regions, edit options through generated property panels, bind data sources and actions, set visibility, preview in fa/en and RTL/LTR, save draft, publish, roll back)</t>
+        </is>
+      </c>
+      <c r="E408" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F408" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G408" s="10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H408" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. This is the user-facing half of 'all pages and components editable by the UI'.</t>
+        </is>
+      </c>
+      <c r="I408" s="8" t="inlineStr">
+        <is>
+          <t>Embedded JavaScript component per ADR-0002 (library choice recorded, offline); property panels generated from the component manifests; undo/redo; autosave to draft; uses the definition store API only (no direct DB); share the preview with the PageHost renderer.</t>
+        </is>
+      </c>
+      <c r="J408" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a non-developer builds a list-plus-detail page and a form page with the designer, previews it in both directions, publishes it and rolls it back; every save goes through the definition store API (#434); the designer is keyboard accessible.</t>
+        </is>
+      </c>
+      <c r="K408" s="8" t="n"/>
+      <c r="L408" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M408" s="10" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="N408" s="10" t="inlineStr">
+        <is>
+          <t>Sales blocker</t>
+        </is>
+      </c>
+      <c r="O408" s="10" t="inlineStr">
+        <is>
+          <t>#438 #433</t>
+        </is>
+      </c>
+      <c r="P408" s="10" t="n"/>
+      <c r="Q408" s="10" t="n"/>
+      <c r="R408" s="8" t="inlineStr">
+        <is>
+          <t>Module builder</t>
+        </is>
+      </c>
+      <c r="S408" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T408" s="10" t="n"/>
+      <c r="U408" s="10" t="n"/>
+    </row>
+    <row r="409">
+      <c r="A409" s="10" t="n">
+        <v>440</v>
+      </c>
+      <c r="B409" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C409" s="8" t="inlineStr">
+        <is>
+          <t>Dynamic Module Builder</t>
+        </is>
+      </c>
+      <c r="D409" s="8" t="inlineStr">
+        <is>
+          <t>Design-time governance: who may create, edit, publish or roll back each kind of definition (design roles), field-level audit of definition changes, protection and one-click reset of system pages and forms, change comments, and approval for published changes on critical pages</t>
+        </is>
+      </c>
+      <c r="E409" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F409" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G409" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H409" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. Editable-by-UI without governance means any admin can break a production page; the audit and rollback must exist before the designers ship.</t>
+        </is>
+      </c>
+      <c r="I409" s="8" t="inlineStr">
+        <is>
+          <t>Design permissions in the access matrix (#60/#178); reuse the generic audit (#17) for definition tables; 'system' flag on shipped definitions with reset; optional two-person publish rule through the workflow platform.</t>
+        </is>
+      </c>
+      <c r="J409" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a user without the design role cannot change or publish a definition (API and UI); every definition change is in the audit trail with who/what/when and a diff; resetting a system page returns the shipped default; a publish on a protected page needs a second approver.</t>
+        </is>
+      </c>
+      <c r="K409" s="8" t="n"/>
+      <c r="L409" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M409" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N409" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O409" s="10" t="inlineStr">
+        <is>
+          <t>#434 #17 #178</t>
+        </is>
+      </c>
+      <c r="P409" s="10" t="n"/>
+      <c r="Q409" s="10" t="n"/>
+      <c r="R409" s="8" t="inlineStr">
+        <is>
+          <t>Module builder</t>
+        </is>
+      </c>
+      <c r="S409" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T409" s="10" t="n"/>
+      <c r="U409" s="10" t="n"/>
+    </row>
+    <row r="410">
+      <c r="A410" s="10" t="n">
+        <v>441</v>
+      </c>
+      <c r="B410" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C410" s="8" t="inlineStr">
+        <is>
+          <t>Foundation, Architecture Decisions &amp; Baseline</t>
+        </is>
+      </c>
+      <c r="D410" s="8" t="inlineStr">
+        <is>
+          <t>Frontend and backend separation: an evidence-based spike and ADR comparing (A) server-rendered Razor with PEMS.UI and JS islands, (B) the same plus a public REST API, (C) a separate single-page front end on the REST API, and (D) a BFF, scored on performance, offline installation, licence protection, Persian RTL/i18n, security (cookies, CSRF, tokens), delivery speed and team skills</t>
+        </is>
+      </c>
+      <c r="E410" s="10" t="inlineStr">
+        <is>
+          <t>Decision Needed</t>
+        </is>
+      </c>
+      <c r="F410" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G410" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H410" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit 2026-10-28: docs/audits/2026-10-28-dynamic-restful-audit.md. The owner wants to separate backend and frontend if there is no performance issue. The product installs on customer servers, works offline and ships no readable source of record, so the decision needs measurements, not preference. Recommendation until then: API-first (#431, #435), no front-end split yet.</t>
+        </is>
+      </c>
+      <c r="I410" s="8" t="inlineStr">
+        <is>
+          <t>Build the same list and form twice (Razor/PEMS.UI vs a small SPA on the walking-skeleton API); measure with the k6/Playwright setups (#202, #41); record bundle size, TTFB/TTI, memory, build and install impact, licence-protection impact (#96), RTL/i18n effort; write plan/adr/NNNN with the decision and what would change it.</t>
+        </is>
+      </c>
+      <c r="J410" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the spike measures time to first byte, time to interactive, payload size and server cost for one real list and one form in options A and C on the same data; the ADR records the scores, the decision and the revisit trigger; if C is chosen a migration path from the API of #435 is listed.</t>
+        </is>
+      </c>
+      <c r="K410" s="8" t="n"/>
+      <c r="L410" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M410" s="10" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="N410" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O410" s="10" t="inlineStr">
+        <is>
+          <t>#435 #319 #202</t>
+        </is>
+      </c>
+      <c r="P410" s="10" t="n"/>
+      <c r="Q410" s="10" t="n"/>
+      <c r="R410" s="8" t="inlineStr">
+        <is>
+          <t>Foundation &amp; decisions</t>
+        </is>
+      </c>
+      <c r="S410" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T410" s="10" t="n"/>
+      <c r="U410" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
docs: shorten the titles of plan rows #430-#441 (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -47544,7 +47544,7 @@
       </c>
       <c r="D399" s="8" t="inlineStr">
         <is>
-          <t>ADR: UI definition model - everything is a definition. One versioned envelope (key, version, status draft/published/archived, owner app, ETag, translations as TranslatableText JSON) for pages, layouts, component instances, forms, views, dashboards, reports, menus, themes, data sources and actions, stored in the database and edited from the UI</t>
+          <t>ADR: UI definition model - one versioned envelope for pages, layouts, component instances, forms, views, menus, themes, data sources and actions, stored in the database and edited from the UI</t>
         </is>
       </c>
       <c r="E399" s="10" t="inlineStr">
@@ -47629,7 +47629,7 @@
       </c>
       <c r="D400" s="8" t="inlineStr">
         <is>
-          <t>ADR: REST API standard - resource-oriented routes (nouns, no verbs), HTTP semantics and status codes, paging/filter/sort, ETag and If-Match, Idempotency-Key, PATCH semantics, bulk and long-running operations, RFC 9457 errors, versioning, Accept-Language and TranslatableText, dates and time zones, allowed-actions links; OpenAPI 3.1 as the contract; plus a guideline chapter</t>
+          <t>ADR: REST API standard - resource-oriented routes, HTTP semantics, ETag/If-Match, RFC 9457 errors, paging/filter/sort, versioning, OpenAPI 3.1 contract, plus a guideline chapter</t>
         </is>
       </c>
       <c r="E400" s="10" t="inlineStr">
@@ -47714,7 +47714,7 @@
       </c>
       <c r="D401" s="8" t="inlineStr">
         <is>
-          <t>REST inventory of the existing 147 controllers and ~830 actions: classify each as view-only MVC (stays), form post (becomes a resource call later), JSON endpoint (normalise), or API candidate; produce the target resource map and a conformance score per controller</t>
+          <t>REST inventory of the 147 controllers and ~830 actions: classify (view-only MVC, form post, JSON endpoint, API candidate) and map each to a target resource</t>
         </is>
       </c>
       <c r="E401" s="10" t="inlineStr">
@@ -47799,7 +47799,7 @@
       </c>
       <c r="D402" s="8" t="inlineStr">
         <is>
-          <t>Component manifest: every PEMS.UI component publishes a machine-readable description (key, options JSON Schema generated from the options records, slots, events, accessibility notes, sample) that drives the designers' property panels, validates stored JSON and feeds the component catalog</t>
+          <t>Component manifest: every PEMS.UI component publishes its key, options JSON Schema (generated from the options records), slots, events and samples to drive designers and validate stored JSON</t>
         </is>
       </c>
       <c r="E402" s="10" t="inlineStr">
@@ -47884,7 +47884,7 @@
       </c>
       <c r="D403" s="8" t="inlineStr">
         <is>
-          <t>Definition store REST API: create, read, update (If-Match), list, publish, unpublish, roll back, export and import of definitions under /api/v1/definitions, with ETag, RFC 9457 errors, OpenAPI, draft/published versions and audit; the designers are ordinary clients of it</t>
+          <t>Definition store REST API: create, edit (If-Match), publish, roll back, export and import of UI definitions under /api/v1/definitions; the designers are ordinary clients of it</t>
         </is>
       </c>
       <c r="E403" s="10" t="inlineStr">
@@ -47969,7 +47969,7 @@
       </c>
       <c r="D404" s="8" t="inlineStr">
         <is>
-          <t>API walking skeleton inside the current application: /api/v1 area with OpenAPI 3.1 generation, versioning, RFC 9457 ProblemDetails, authorization on every endpoint, RLS applied, antiforgery for browser calls and token auth for integrations, ETag support and one pilot resource</t>
+          <t>API walking skeleton in the current app: /api/v1 with OpenAPI 3.1, ProblemDetails, versioning, authorization on every endpoint, RLS, ETag and one pilot resource</t>
         </is>
       </c>
       <c r="E404" s="10" t="inlineStr">
@@ -48054,7 +48054,7 @@
       </c>
       <c r="D405" s="8" t="inlineStr">
         <is>
-          <t>API quality gates in CI: OpenAPI lint (Spectral rules for naming, status codes, errors, pagination), REST conformance tests (no verbs in URLs, correct status codes, ETag/If-Match, authorization on every endpoint, ProblemDetails shape), contract/snapshot test of the published OpenAPI, and an API performance baseline with the k6 suite</t>
+          <t>API quality gates in CI: OpenAPI lint, REST conformance tests, OpenAPI snapshot test and an API performance baseline</t>
         </is>
       </c>
       <c r="E405" s="10" t="inlineStr">
@@ -48139,7 +48139,7 @@
       </c>
       <c r="D406" s="8" t="inlineStr">
         <is>
-          <t>Declarative data-source and action bindings: a component instance binds to an entity query, saved view, REST endpoint or static value, and its actions (navigate, call endpoint, run workflow action, open dialog, refresh) are data, not code; with parameters, permissions and error/empty/loading states from the unified states</t>
+          <t>Declarative data-source and action bindings: components bind to queries, views and endpoints, and their actions are stored data, not code</t>
         </is>
       </c>
       <c r="E406" s="10" t="inlineStr">
@@ -48224,7 +48224,7 @@
       </c>
       <c r="D407" s="8" t="inlineStr">
         <is>
-          <t>Page definition and PageHost runtime: a page is a stored layout of regions and component instances; one generic host renders any published page from the database in Persian and English, with caching and invalidation, permission and visibility rules, and a fallback to the static page</t>
+          <t>Page definition and PageHost runtime: a page is a stored layout of component instances rendered by one generic host in fa and en, with cache, permissions and a static fallback</t>
         </is>
       </c>
       <c r="E407" s="10" t="inlineStr">
@@ -48309,7 +48309,7 @@
       </c>
       <c r="D408" s="8" t="inlineStr">
         <is>
-          <t>Page designer: visual editor to create and edit a page from the UI (choose layout, drag component instances into regions, edit options through generated property panels, bind data sources and actions, set visibility, preview in fa/en and RTL/LTR, save draft, publish, roll back)</t>
+          <t>Page designer: build, preview, publish and roll back a page from the UI (layouts, drag-and-drop component instances, generated property panels, bindings, visibility)</t>
         </is>
       </c>
       <c r="E408" s="10" t="inlineStr">
@@ -48394,7 +48394,7 @@
       </c>
       <c r="D409" s="8" t="inlineStr">
         <is>
-          <t>Design-time governance: who may create, edit, publish or roll back each kind of definition (design roles), field-level audit of definition changes, protection and one-click reset of system pages and forms, change comments, and approval for published changes on critical pages</t>
+          <t>Design-time governance: design roles, field-level audit of definition changes, system-page protection and reset, approval for critical pages</t>
         </is>
       </c>
       <c r="E409" s="10" t="inlineStr">
@@ -48479,7 +48479,7 @@
       </c>
       <c r="D410" s="8" t="inlineStr">
         <is>
-          <t>Frontend and backend separation: an evidence-based spike and ADR comparing (A) server-rendered Razor with PEMS.UI and JS islands, (B) the same plus a public REST API, (C) a separate single-page front end on the REST API, and (D) a BFF, scored on performance, offline installation, licence protection, Persian RTL/i18n, security (cookies, CSRF, tokens), delivery speed and team skills</t>
+          <t>Frontend and backend separation: measured spike and ADR comparing Razor + PEMS.UI, Razor + public REST API, a separate SPA and a BFF</t>
         </is>
       </c>
       <c r="E410" s="10" t="inlineStr">

</xml_diff>

<commit_message>
docs: shorten the titles of plan rows #430-#441 (hamid) (#65)
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -47544,7 +47544,7 @@
       </c>
       <c r="D399" s="8" t="inlineStr">
         <is>
-          <t>ADR: UI definition model - everything is a definition. One versioned envelope (key, version, status draft/published/archived, owner app, ETag, translations as TranslatableText JSON) for pages, layouts, component instances, forms, views, dashboards, reports, menus, themes, data sources and actions, stored in the database and edited from the UI</t>
+          <t>ADR: UI definition model - one versioned envelope for pages, layouts, component instances, forms, views, menus, themes, data sources and actions, stored in the database and edited from the UI</t>
         </is>
       </c>
       <c r="E399" s="10" t="inlineStr">
@@ -47629,7 +47629,7 @@
       </c>
       <c r="D400" s="8" t="inlineStr">
         <is>
-          <t>ADR: REST API standard - resource-oriented routes (nouns, no verbs), HTTP semantics and status codes, paging/filter/sort, ETag and If-Match, Idempotency-Key, PATCH semantics, bulk and long-running operations, RFC 9457 errors, versioning, Accept-Language and TranslatableText, dates and time zones, allowed-actions links; OpenAPI 3.1 as the contract; plus a guideline chapter</t>
+          <t>ADR: REST API standard - resource-oriented routes, HTTP semantics, ETag/If-Match, RFC 9457 errors, paging/filter/sort, versioning, OpenAPI 3.1 contract, plus a guideline chapter</t>
         </is>
       </c>
       <c r="E400" s="10" t="inlineStr">
@@ -47714,7 +47714,7 @@
       </c>
       <c r="D401" s="8" t="inlineStr">
         <is>
-          <t>REST inventory of the existing 147 controllers and ~830 actions: classify each as view-only MVC (stays), form post (becomes a resource call later), JSON endpoint (normalise), or API candidate; produce the target resource map and a conformance score per controller</t>
+          <t>REST inventory of the 147 controllers and ~830 actions: classify (view-only MVC, form post, JSON endpoint, API candidate) and map each to a target resource</t>
         </is>
       </c>
       <c r="E401" s="10" t="inlineStr">
@@ -47799,7 +47799,7 @@
       </c>
       <c r="D402" s="8" t="inlineStr">
         <is>
-          <t>Component manifest: every PEMS.UI component publishes a machine-readable description (key, options JSON Schema generated from the options records, slots, events, accessibility notes, sample) that drives the designers' property panels, validates stored JSON and feeds the component catalog</t>
+          <t>Component manifest: every PEMS.UI component publishes its key, options JSON Schema (generated from the options records), slots, events and samples to drive designers and validate stored JSON</t>
         </is>
       </c>
       <c r="E402" s="10" t="inlineStr">
@@ -47884,7 +47884,7 @@
       </c>
       <c r="D403" s="8" t="inlineStr">
         <is>
-          <t>Definition store REST API: create, read, update (If-Match), list, publish, unpublish, roll back, export and import of definitions under /api/v1/definitions, with ETag, RFC 9457 errors, OpenAPI, draft/published versions and audit; the designers are ordinary clients of it</t>
+          <t>Definition store REST API: create, edit (If-Match), publish, roll back, export and import of UI definitions under /api/v1/definitions; the designers are ordinary clients of it</t>
         </is>
       </c>
       <c r="E403" s="10" t="inlineStr">
@@ -47969,7 +47969,7 @@
       </c>
       <c r="D404" s="8" t="inlineStr">
         <is>
-          <t>API walking skeleton inside the current application: /api/v1 area with OpenAPI 3.1 generation, versioning, RFC 9457 ProblemDetails, authorization on every endpoint, RLS applied, antiforgery for browser calls and token auth for integrations, ETag support and one pilot resource</t>
+          <t>API walking skeleton in the current app: /api/v1 with OpenAPI 3.1, ProblemDetails, versioning, authorization on every endpoint, RLS, ETag and one pilot resource</t>
         </is>
       </c>
       <c r="E404" s="10" t="inlineStr">
@@ -48054,7 +48054,7 @@
       </c>
       <c r="D405" s="8" t="inlineStr">
         <is>
-          <t>API quality gates in CI: OpenAPI lint (Spectral rules for naming, status codes, errors, pagination), REST conformance tests (no verbs in URLs, correct status codes, ETag/If-Match, authorization on every endpoint, ProblemDetails shape), contract/snapshot test of the published OpenAPI, and an API performance baseline with the k6 suite</t>
+          <t>API quality gates in CI: OpenAPI lint, REST conformance tests, OpenAPI snapshot test and an API performance baseline</t>
         </is>
       </c>
       <c r="E405" s="10" t="inlineStr">
@@ -48139,7 +48139,7 @@
       </c>
       <c r="D406" s="8" t="inlineStr">
         <is>
-          <t>Declarative data-source and action bindings: a component instance binds to an entity query, saved view, REST endpoint or static value, and its actions (navigate, call endpoint, run workflow action, open dialog, refresh) are data, not code; with parameters, permissions and error/empty/loading states from the unified states</t>
+          <t>Declarative data-source and action bindings: components bind to queries, views and endpoints, and their actions are stored data, not code</t>
         </is>
       </c>
       <c r="E406" s="10" t="inlineStr">
@@ -48224,7 +48224,7 @@
       </c>
       <c r="D407" s="8" t="inlineStr">
         <is>
-          <t>Page definition and PageHost runtime: a page is a stored layout of regions and component instances; one generic host renders any published page from the database in Persian and English, with caching and invalidation, permission and visibility rules, and a fallback to the static page</t>
+          <t>Page definition and PageHost runtime: a page is a stored layout of component instances rendered by one generic host in fa and en, with cache, permissions and a static fallback</t>
         </is>
       </c>
       <c r="E407" s="10" t="inlineStr">
@@ -48309,7 +48309,7 @@
       </c>
       <c r="D408" s="8" t="inlineStr">
         <is>
-          <t>Page designer: visual editor to create and edit a page from the UI (choose layout, drag component instances into regions, edit options through generated property panels, bind data sources and actions, set visibility, preview in fa/en and RTL/LTR, save draft, publish, roll back)</t>
+          <t>Page designer: build, preview, publish and roll back a page from the UI (layouts, drag-and-drop component instances, generated property panels, bindings, visibility)</t>
         </is>
       </c>
       <c r="E408" s="10" t="inlineStr">
@@ -48394,7 +48394,7 @@
       </c>
       <c r="D409" s="8" t="inlineStr">
         <is>
-          <t>Design-time governance: who may create, edit, publish or roll back each kind of definition (design roles), field-level audit of definition changes, protection and one-click reset of system pages and forms, change comments, and approval for published changes on critical pages</t>
+          <t>Design-time governance: design roles, field-level audit of definition changes, system-page protection and reset, approval for critical pages</t>
         </is>
       </c>
       <c r="E409" s="10" t="inlineStr">
@@ -48479,7 +48479,7 @@
       </c>
       <c r="D410" s="8" t="inlineStr">
         <is>
-          <t>Frontend and backend separation: an evidence-based spike and ADR comparing (A) server-rendered Razor with PEMS.UI and JS islands, (B) the same plus a public REST API, (C) a separate single-page front end on the REST API, and (D) a BFF, scored on performance, offline installation, licence protection, Persian RTL/i18n, security (cookies, CSRF, tokens), delivery speed and team skills</t>
+          <t>Frontend and backend separation: measured spike and ADR comparing Razor + PEMS.UI, Razor + public REST API, a separate SPA and a BFF</t>
         </is>
       </c>
       <c r="E410" s="10" t="inlineStr">

</xml_diff>

<commit_message>
SCRUM-425: show the shared title row on five pages that had no heading (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$350</definedName>
@@ -47312,7 +47312,7 @@
       </c>
       <c r="K396" s="8" t="inlineStr">
         <is>
-          <t>Part 1 in PR atapems-tech/PEMS#60 (merged): title row moved to PEMS.UI _PemsPageHeader (PageHeaderModel Title/Section as TranslatableText); _PageHeader stays as adapter (localizes, honours HidePageTitle); 7 golden cases en/fa byte-identical, mutation check fails 1; design doc corrected. Finding: the layout stopped rendering the header on owner request (guard test GlobalPageHeaderTests) and almost no page hand-writes a page title, so any caller ADDS a visible row. Callers wait for the owner's choice of pages (task stays In Progress). QA pending (SQL Server tests, HTTP smoke tests, browser check).</t>
+          <t>Part 1 in PR atapems-tech/PEMS#60 (merged): title row moved to PEMS.UI _PemsPageHeader, _PageHeader stays as adapter, 7 golden cases byte-identical. Part 2 (owner delegated the choice to Claude, 2026-10-28): evaluated the 48 views that set a title; five show no heading at all and now call the row: Finding/Index, ImportCenter/Index, ShiftHandover/Create, CriticalityAssessment/Create, Barcode/Verify (render test + source guard, mutation check fails 2). Other pages unchanged. QA pending (SQL Server tests, HTTP smoke tests, browser check of the five pages in en/fa, desktop and 375 px).</t>
         </is>
       </c>
       <c r="L396" s="10" t="inlineStr">

</xml_diff>

<commit_message>
SCRUM-425: show the shared title row on five pages that had no heading (hamid) (#67)
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$350</definedName>
@@ -47312,7 +47312,7 @@
       </c>
       <c r="K396" s="8" t="inlineStr">
         <is>
-          <t>Part 1 in PR atapems-tech/PEMS#60 (merged): title row moved to PEMS.UI _PemsPageHeader (PageHeaderModel Title/Section as TranslatableText); _PageHeader stays as adapter (localizes, honours HidePageTitle); 7 golden cases en/fa byte-identical, mutation check fails 1; design doc corrected. Finding: the layout stopped rendering the header on owner request (guard test GlobalPageHeaderTests) and almost no page hand-writes a page title, so any caller ADDS a visible row. Callers wait for the owner's choice of pages (task stays In Progress). QA pending (SQL Server tests, HTTP smoke tests, browser check).</t>
+          <t>Part 1 in PR atapems-tech/PEMS#60 (merged): title row moved to PEMS.UI _PemsPageHeader, _PageHeader stays as adapter, 7 golden cases byte-identical. Part 2 (owner delegated the choice to Claude, 2026-10-28): evaluated the 48 views that set a title; five show no heading at all and now call the row: Finding/Index, ImportCenter/Index, ShiftHandover/Create, CriticalityAssessment/Create, Barcode/Verify (render test + source guard, mutation check fails 2). Other pages unchanged. QA pending (SQL Server tests, HTTP smoke tests, browser check of the five pages in en/fa, desktop and 375 px).</t>
         </is>
       </c>
       <c r="L396" s="10" t="inlineStr">

</xml_diff>

<commit_message>
docs: plan row #442 site-wide digits (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12367,7 +12367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U410"/>
+  <dimension ref="A1:U411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -48551,6 +48551,95 @@
       </c>
       <c r="T410" s="10" t="n"/>
       <c r="U410" s="10" t="n"/>
+    </row>
+    <row r="411">
+      <c r="A411" s="10" t="n">
+        <v>442</v>
+      </c>
+      <c r="B411" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C411" s="8" t="inlineStr">
+        <is>
+          <t>Persian Localization, RTL &amp; Jalali Calendar</t>
+        </is>
+      </c>
+      <c r="D411" s="8" t="inlineStr">
+        <is>
+          <t>Site-wide digits: Persian digits for numbers, counts and dates shown to Persian users on every page and in scripts, Latin in English; display only, never in links, ids, posted values or exports</t>
+        </is>
+      </c>
+      <c r="E411" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F411" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G411" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H411" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit follow-up, owner request 2026-10-28 (after SCRUM-426 did the pagination footer). Measured: 168 views call ToString(format) (243 ISO dates, 112 date-times, 92 N0, 35 N1, 32 N3, 14 0.###, 11 0.0), about 156 views print counts, quantities or amounts, 3 script files format numbers (toFixed, Intl.NumberFormat). .NET never swaps digits itself, so a Persian page prints Latin digits today. IPemsLocale.Digits and Format exist (SCRUM-426, ADR-0008). Calendar choice (Jalali for fa) is NOT part of this task; see #367, #208 and the dates decision in ADR-0008.</t>
+        </is>
+      </c>
+      <c r="I411" s="8" t="inlineStr">
+        <is>
+          <t>1) Design first (small PR): one view helper and one script helper over IPemsLocale (number, integer, percent, decimal, date, date-time, count) with explicit raw escape hatch for attributes and values; decide how pages opt in (HtmlHelper or Tag Helper) and how scripts get the locale (data attribute). 2) Codemod the repeated patterns (ToString N0/N1/N3/0.###/0.0, yyyy-MM-dd, yyyy-MM-dd HH:mm) in waves by area with golden or render proof per wave (en byte-identical, fa digits only). 3) Scripts: replace toFixed and Intl.NumberFormat without a locale by the shared helper. 4) Ratchet test like the component raw-markup ratchet (#327): count of raw ToString format calls in views may only go down. 5) Exports (Excel, CSV, PDF) are covered by #371, not here. 6) Document in guideline chapter 02 what is display and what is data.</t>
+        </is>
+      </c>
+      <c r="J411" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a Persian user sees Persian digits in every displayed number and date on the migrated pages and in the scripts that draw numbers, an English user sees Latin digits exactly as today; links, ids, form values, CSV/Excel exports and API output stay Latin; a ratchet test fails when a view formats a number or date for display without the shared helper; every wave has before/after golden or render proof.</t>
+        </is>
+      </c>
+      <c r="K411" s="8" t="inlineStr">
+        <is>
+          <t>Done in PR atapems-tech/PEMS#61 (merged): new IPemsLocale.Digits (digit swap, no reformatting; Format not used because it adds thousands separators); _PemsPagination shows Persian digits in the range text, page numbers and page-size buttons; hrefs and aria-labels stay Latin; English goldens byte-identical, 3 Persian goldens re-recorded and diffed (digits only). PEMS.UI.Tests 99/99, PEMS.Tests.Ui 25/25, mutation check fails 4. QA pending (SQL Server tests, HTTP smoke tests incl. clicking a Persian page link, browser check).</t>
+        </is>
+      </c>
+      <c r="L411" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M411" s="10" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="N411" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O411" s="10" t="inlineStr">
+        <is>
+          <t>#426 #367 #386</t>
+        </is>
+      </c>
+      <c r="P411" s="10" t="n"/>
+      <c r="Q411" s="10" t="n"/>
+      <c r="R411" s="8" t="inlineStr">
+        <is>
+          <t>Persian localization</t>
+        </is>
+      </c>
+      <c r="S411" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T411" s="10" t="n"/>
+      <c r="U411" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
docs: clear the report copied into plan row #442 (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -48601,11 +48601,7 @@
           <t>Done when: a Persian user sees Persian digits in every displayed number and date on the migrated pages and in the scripts that draw numbers, an English user sees Latin digits exactly as today; links, ids, form values, CSV/Excel exports and API output stay Latin; a ratchet test fails when a view formats a number or date for display without the shared helper; every wave has before/after golden or render proof.</t>
         </is>
       </c>
-      <c r="K411" s="8" t="inlineStr">
-        <is>
-          <t>Done in PR atapems-tech/PEMS#61 (merged): new IPemsLocale.Digits (digit swap, no reformatting; Format not used because it adds thousands separators); _PemsPagination shows Persian digits in the range text, page numbers and page-size buttons; hrefs and aria-labels stay Latin; English goldens byte-identical, 3 Persian goldens re-recorded and diffed (digits only). PEMS.UI.Tests 99/99, PEMS.Tests.Ui 25/25, mutation check fails 4. QA pending (SQL Server tests, HTTP smoke tests incl. clicking a Persian page link, browser check).</t>
-        </is>
-      </c>
+      <c r="K411" s="8" t="n"/>
       <c r="L411" s="10" t="inlineStr">
         <is>
           <t>M2</t>

</xml_diff>

<commit_message>
docs: plan row #442 site-wide digits (hamid) (#68)
* docs: plan row #442 site-wide digits (hamid)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

* docs: clear the report copied into plan row #442 (hamid)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12367,7 +12367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U410"/>
+  <dimension ref="A1:U411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -48551,6 +48551,91 @@
       </c>
       <c r="T410" s="10" t="n"/>
       <c r="U410" s="10" t="n"/>
+    </row>
+    <row r="411">
+      <c r="A411" s="10" t="n">
+        <v>442</v>
+      </c>
+      <c r="B411" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C411" s="8" t="inlineStr">
+        <is>
+          <t>Persian Localization, RTL &amp; Jalali Calendar</t>
+        </is>
+      </c>
+      <c r="D411" s="8" t="inlineStr">
+        <is>
+          <t>Site-wide digits: Persian digits for numbers, counts and dates shown to Persian users on every page and in scripts, Latin in English; display only, never in links, ids, posted values or exports</t>
+        </is>
+      </c>
+      <c r="E411" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F411" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G411" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H411" s="8" t="inlineStr">
+        <is>
+          <t>Plan audit follow-up, owner request 2026-10-28 (after SCRUM-426 did the pagination footer). Measured: 168 views call ToString(format) (243 ISO dates, 112 date-times, 92 N0, 35 N1, 32 N3, 14 0.###, 11 0.0), about 156 views print counts, quantities or amounts, 3 script files format numbers (toFixed, Intl.NumberFormat). .NET never swaps digits itself, so a Persian page prints Latin digits today. IPemsLocale.Digits and Format exist (SCRUM-426, ADR-0008). Calendar choice (Jalali for fa) is NOT part of this task; see #367, #208 and the dates decision in ADR-0008.</t>
+        </is>
+      </c>
+      <c r="I411" s="8" t="inlineStr">
+        <is>
+          <t>1) Design first (small PR): one view helper and one script helper over IPemsLocale (number, integer, percent, decimal, date, date-time, count) with explicit raw escape hatch for attributes and values; decide how pages opt in (HtmlHelper or Tag Helper) and how scripts get the locale (data attribute). 2) Codemod the repeated patterns (ToString N0/N1/N3/0.###/0.0, yyyy-MM-dd, yyyy-MM-dd HH:mm) in waves by area with golden or render proof per wave (en byte-identical, fa digits only). 3) Scripts: replace toFixed and Intl.NumberFormat without a locale by the shared helper. 4) Ratchet test like the component raw-markup ratchet (#327): count of raw ToString format calls in views may only go down. 5) Exports (Excel, CSV, PDF) are covered by #371, not here. 6) Document in guideline chapter 02 what is display and what is data.</t>
+        </is>
+      </c>
+      <c r="J411" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a Persian user sees Persian digits in every displayed number and date on the migrated pages and in the scripts that draw numbers, an English user sees Latin digits exactly as today; links, ids, form values, CSV/Excel exports and API output stay Latin; a ratchet test fails when a view formats a number or date for display without the shared helper; every wave has before/after golden or render proof.</t>
+        </is>
+      </c>
+      <c r="K411" s="8" t="n"/>
+      <c r="L411" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M411" s="10" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="N411" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O411" s="10" t="inlineStr">
+        <is>
+          <t>#426 #367 #386</t>
+        </is>
+      </c>
+      <c r="P411" s="10" t="n"/>
+      <c r="Q411" s="10" t="n"/>
+      <c r="R411" s="8" t="inlineStr">
+        <is>
+          <t>Persian localization</t>
+        </is>
+      </c>
+      <c r="S411" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T411" s="10" t="n"/>
+      <c r="U411" s="10" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-428: pick registered part numbers in material requisition items (saber)
MR items resolve their part number on the server against the registered
parts (completed part catalogue requests, then Material Master; exact and
normalised) and store the link (new nullable MaterialItemId and
PartCatalogueRequestId, migration MaterialRequisitionItemRegisteredPart). A
registered part fills an empty description and unit; a typed unregistered
part stays free text, shown "Not catalogued". New MR form: searchable
part lookup per item (reusing SearchExistingPartsAsync, now with the unit),
typed parts allowed, "request a new part" shortcut; MR details show the
catalogue state. pems-select gains data-pems-select-url and -create.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12367,7 +12367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U410"/>
+  <dimension ref="A1:U411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -48551,6 +48551,103 @@
       </c>
       <c r="T410" s="10" t="n"/>
       <c r="U410" s="10" t="n"/>
+    </row>
+    <row r="411">
+      <c r="A411" s="10" t="n">
+        <v>428</v>
+      </c>
+      <c r="B411" s="10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C411" s="8" t="inlineStr">
+        <is>
+          <t>Domain: HR, Projects, Finance &amp; Procurement</t>
+        </is>
+      </c>
+      <c r="D411" s="8" t="inlineStr">
+        <is>
+          <t>Pick registered part numbers from the part catalogue in material requisition items</t>
+        </is>
+      </c>
+      <c r="E411" s="10" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F411" s="10" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G411" s="10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H411" s="8" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-27: after the part catalogue registers a part number it must be selectable in procurement. SCRUM-428; batch 427 -&gt; 40 -&gt; 57 -&gt; 428 -&gt; 429.</t>
+        </is>
+      </c>
+      <c r="I411" s="8" t="inlineStr">
+        <is>
+          <t>Server-side resolution of each MR item part number against completed catalogue requests and Material Master (exact, normalised), nullable links on MaterialRequisitionItem (migration), lookup endpoint on the reused SearchExistingPartsAsync, pems-select url/create options, MR form and details.</t>
+        </is>
+      </c>
+      <c r="J411" s="8" t="inlineStr">
+        <is>
+          <t>Done when: a registered part is found in the MR item lookup, its description and unit fill in, the link is stored; a typed unregistered part stays free text, marked not catalogued.</t>
+        </is>
+      </c>
+      <c r="K411" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-28 SCRUM-428: built on feature/SCRUM-428-mr-registered-parts-saber; MrRegisteredPartTests + related 83/83; browser QA on PEMSDB_QA407 (lookup by MPN, fill, typed part, details badges). PO lines (gap analysis proposal 1) will carry the same link.</t>
+        </is>
+      </c>
+      <c r="L411" s="10" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="M411" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N411" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O411" s="10" t="inlineStr">
+        <is>
+          <t>#427</t>
+        </is>
+      </c>
+      <c r="P411" s="10" t="n"/>
+      <c r="Q411" s="10" t="n"/>
+      <c r="R411" s="8" t="inlineStr">
+        <is>
+          <t>Domain modules</t>
+        </is>
+      </c>
+      <c r="S411" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T411" s="10" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="U411" s="10" t="inlineStr">
+        <is>
+          <t>Member A</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
docs: plan rows #443 (reference naming) and #444 (page titles review) (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12367,7 +12367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U411"/>
+  <dimension ref="A1:U413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -48636,6 +48636,180 @@
       </c>
       <c r="T411" s="10" t="n"/>
       <c r="U411" s="10" t="n"/>
+    </row>
+    <row r="412">
+      <c r="A412" s="10" t="n">
+        <v>443</v>
+      </c>
+      <c r="B412" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C412" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D412" s="8" t="inlineStr">
+        <is>
+          <t>Component naming table vs the reference library's component names: owner supplies the list, then the shared property and key names in guideline chapter 02 are aligned or the differences are justified</t>
+        </is>
+      </c>
+      <c r="E412" s="10" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="F412" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G412" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H412" s="8" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-28. The naming table in guideline chapter 02 (Label, Title, Description, Detail, Icon, Action, Href, Tone, Size, Kind, Name/Key/Id; kebab-case registry keys) was written from common practice because the reference library's names are not in this repository. See the Reference column.</t>
+        </is>
+      </c>
+      <c r="I412" s="8" t="inlineStr">
+        <is>
+          <t>1) Owner supplies the reference list (names of components, their options, keys). 2) Compare with the table and the registry keys. 3) Rename in code where cheap (options records are named-property objects, registry keys are strings) and update goldens; otherwise record why. 4) Update guideline chapter 02.</t>
+        </is>
+      </c>
+      <c r="J412" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the reference component and property names are in the repository docs (owner supplies them); every difference from the table in guideline chapter 02 is either aligned in code or recorded with a reason; the table and the component registry keys agree.</t>
+        </is>
+      </c>
+      <c r="K412" s="8" t="n"/>
+      <c r="L412" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M412" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N412" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O412" s="10" t="n"/>
+      <c r="P412" s="10" t="inlineStr">
+        <is>
+          <t>Titan component names (owner list)</t>
+        </is>
+      </c>
+      <c r="Q412" s="10" t="n"/>
+      <c r="R412" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S412" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T412" s="10" t="n"/>
+      <c r="U412" s="10" t="inlineStr">
+        <is>
+          <t>Hamid</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="10" t="n">
+        <v>444</v>
+      </c>
+      <c r="B413" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C413" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D413" s="8" t="inlineStr">
+        <is>
+          <t>Page titles review: check every page title and module label (English and Persian), which pages should show the title row, and whether the default of no global header still serves users</t>
+        </is>
+      </c>
+      <c r="E413" s="10" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="F413" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G413" s="10" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H413" s="8" t="inlineStr">
+        <is>
+          <t>SCRUM-425 gave five pages the shared title row by code evaluation only; the owner asked for a later look at the real pages. Titles come from controllers as English literals and are localized in one place (_PageHeader); untranslated titles show English.</t>
+        </is>
+      </c>
+      <c r="I413" s="8" t="inlineStr">
+        <is>
+          <t>1) Walk the sidebar pages in en and fa on desktop and 375 px. 2) Note missing, duplicate, untranslated or misleading titles. 3) Decide per page: add the row, remove it, or translate the title (SharedResource.fa.resx). 4) Create follow-up tasks or small PRs.</t>
+        </is>
+      </c>
+      <c r="J413" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the owner has walked the main pages in English and Persian; a list names pages that need the title row (added through the _PageHeader call), pages whose title is missing or untranslated, and pages where the row should go; follow-up tasks exist for the findings.</t>
+        </is>
+      </c>
+      <c r="K413" s="8" t="n"/>
+      <c r="L413" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M413" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N413" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O413" s="10" t="n"/>
+      <c r="P413" s="10" t="n"/>
+      <c r="Q413" s="10" t="n"/>
+      <c r="R413" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S413" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T413" s="10" t="n"/>
+      <c r="U413" s="10" t="inlineStr">
+        <is>
+          <t>Hamid</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
docs: plan rows #443 (reference naming) and #444 (page titles review) (hamid) (#70)
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -12367,7 +12367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U411"/>
+  <dimension ref="A1:U413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -48636,6 +48636,180 @@
       </c>
       <c r="T411" s="10" t="n"/>
       <c r="U411" s="10" t="n"/>
+    </row>
+    <row r="412">
+      <c r="A412" s="10" t="n">
+        <v>443</v>
+      </c>
+      <c r="B412" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C412" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D412" s="8" t="inlineStr">
+        <is>
+          <t>Component naming table vs the reference library's component names: owner supplies the list, then the shared property and key names in guideline chapter 02 are aligned or the differences are justified</t>
+        </is>
+      </c>
+      <c r="E412" s="10" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="F412" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G412" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H412" s="8" t="inlineStr">
+        <is>
+          <t>Owner request 2026-10-28. The naming table in guideline chapter 02 (Label, Title, Description, Detail, Icon, Action, Href, Tone, Size, Kind, Name/Key/Id; kebab-case registry keys) was written from common practice because the reference library's names are not in this repository. See the Reference column.</t>
+        </is>
+      </c>
+      <c r="I412" s="8" t="inlineStr">
+        <is>
+          <t>1) Owner supplies the reference list (names of components, their options, keys). 2) Compare with the table and the registry keys. 3) Rename in code where cheap (options records are named-property objects, registry keys are strings) and update goldens; otherwise record why. 4) Update guideline chapter 02.</t>
+        </is>
+      </c>
+      <c r="J412" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the reference component and property names are in the repository docs (owner supplies them); every difference from the table in guideline chapter 02 is either aligned in code or recorded with a reason; the table and the component registry keys agree.</t>
+        </is>
+      </c>
+      <c r="K412" s="8" t="n"/>
+      <c r="L412" s="10" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="M412" s="10" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N412" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O412" s="10" t="n"/>
+      <c r="P412" s="10" t="inlineStr">
+        <is>
+          <t>Titan component names (owner list)</t>
+        </is>
+      </c>
+      <c r="Q412" s="10" t="n"/>
+      <c r="R412" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S412" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T412" s="10" t="n"/>
+      <c r="U412" s="10" t="inlineStr">
+        <is>
+          <t>Hamid</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="10" t="n">
+        <v>444</v>
+      </c>
+      <c r="B413" s="10" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C413" s="8" t="inlineStr">
+        <is>
+          <t>Component Library &amp; Design System</t>
+        </is>
+      </c>
+      <c r="D413" s="8" t="inlineStr">
+        <is>
+          <t>Page titles review: check every page title and module label (English and Persian), which pages should show the title row, and whether the default of no global header still serves users</t>
+        </is>
+      </c>
+      <c r="E413" s="10" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="F413" s="10" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G413" s="10" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H413" s="8" t="inlineStr">
+        <is>
+          <t>SCRUM-425 gave five pages the shared title row by code evaluation only; the owner asked for a later look at the real pages. Titles come from controllers as English literals and are localized in one place (_PageHeader); untranslated titles show English.</t>
+        </is>
+      </c>
+      <c r="I413" s="8" t="inlineStr">
+        <is>
+          <t>1) Walk the sidebar pages in en and fa on desktop and 375 px. 2) Note missing, duplicate, untranslated or misleading titles. 3) Decide per page: add the row, remove it, or translate the title (SharedResource.fa.resx). 4) Create follow-up tasks or small PRs.</t>
+        </is>
+      </c>
+      <c r="J413" s="8" t="inlineStr">
+        <is>
+          <t>Done when: the owner has walked the main pages in English and Persian; a list names pages that need the title row (added through the _PageHeader call), pages whose title is missing or untranslated, and pages where the row should go; follow-up tasks exist for the findings.</t>
+        </is>
+      </c>
+      <c r="K413" s="8" t="n"/>
+      <c r="L413" s="10" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="M413" s="10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="N413" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O413" s="10" t="n"/>
+      <c r="P413" s="10" t="n"/>
+      <c r="Q413" s="10" t="n"/>
+      <c r="R413" s="8" t="inlineStr">
+        <is>
+          <t>UI component library</t>
+        </is>
+      </c>
+      <c r="S413" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T413" s="10" t="n"/>
+      <c r="U413" s="10" t="inlineStr">
+        <is>
+          <t>Hamid</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:U350"/>

</xml_diff>

<commit_message>
SCRUM-431: REST API standard ADR-0009 and guideline chapter 08 (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -14092,7 +14092,7 @@
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>PEMS has SignalR hubs but no generic record lock. Real-time and locking is a new subsystem, not an extension.</t>
+          <t>PEMS has SignalR hubs but no generic record lock. Real-time and locking is a new subsystem, not an extension. 2026-10-28: follows the REST API standard ADR-0009 / guideline chapter 08 (#431).</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
@@ -14998,7 +14998,7 @@
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>A cached registry (TTL + write invalidation) with ETag/gzip cured slow database access on a comparable platform; a registry change must not need a rebuild.</t>
+          <t>A cached registry (TTL + write invalidation) with ETag/gzip cured slow database access on a comparable platform; a registry change must not need a rebuild. 2026-10-28: follows the REST API standard ADR-0009 / guideline chapter 08 (#431).</t>
         </is>
       </c>
       <c r="I29" s="8" t="inlineStr">
@@ -44501,7 +44501,7 @@
       </c>
       <c r="H364" s="8" t="inlineStr">
         <is>
-          <t>Each module reports errors in its own way (a page summary, a thrown message, a flash text), so clients and the form components cannot render or test them uniformly. RFC 9457 defines application/problem+json and leaves the validation list to an extension member; ASP.NET Core can produce problem details natively.</t>
+          <t>Each module reports errors in its own way (a page summary, a thrown message, a flash text), so clients and the form components cannot render or test them uniformly. RFC 9457 defines application/problem+json and leaves the validation list to an extension member; ASP.NET Core can produce problem details natively. 2026-10-28: follows the REST API standard ADR-0009 / guideline chapter 08 (#431).</t>
         </is>
       </c>
       <c r="I364" s="8" t="inlineStr">
@@ -47666,7 +47666,11 @@
           <t>Done when: the ADR is accepted and a short guideline chapter (docs/guidelines) lists the rules with one good and one bad example each; rows #12, #195, #363, #18, #28 and #387 reference it; the open questions have an owner.</t>
         </is>
       </c>
-      <c r="K400" s="8" t="n"/>
+      <c r="K400" s="8" t="inlineStr">
+        <is>
+          <t>Written in PR (this branch): ADR-0009 (status Proposed, owner review) and guideline chapter 08 with a good and a bad example per rule; paging decision recorded (offset for grids, cursor for exports and very large tables, one implementation); rows #12, #195, #387 already reference #431, #363, #18 and #28 now do. QA pending: owner acceptance of the ADR.</t>
+        </is>
+      </c>
       <c r="L400" s="10" t="inlineStr">
         <is>
           <t>M0</t>

</xml_diff>

<commit_message>
SCRUM-431: REST API standard ADR-0009 and guideline chapter 08 (hamid) (#71)
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -14092,7 +14092,7 @@
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>PEMS has SignalR hubs but no generic record lock. Real-time and locking is a new subsystem, not an extension.</t>
+          <t>PEMS has SignalR hubs but no generic record lock. Real-time and locking is a new subsystem, not an extension. 2026-10-28: follows the REST API standard ADR-0009 / guideline chapter 08 (#431).</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
@@ -14998,7 +14998,7 @@
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>A cached registry (TTL + write invalidation) with ETag/gzip cured slow database access on a comparable platform; a registry change must not need a rebuild.</t>
+          <t>A cached registry (TTL + write invalidation) with ETag/gzip cured slow database access on a comparable platform; a registry change must not need a rebuild. 2026-10-28: follows the REST API standard ADR-0009 / guideline chapter 08 (#431).</t>
         </is>
       </c>
       <c r="I29" s="8" t="inlineStr">
@@ -44501,7 +44501,7 @@
       </c>
       <c r="H364" s="8" t="inlineStr">
         <is>
-          <t>Each module reports errors in its own way (a page summary, a thrown message, a flash text), so clients and the form components cannot render or test them uniformly. RFC 9457 defines application/problem+json and leaves the validation list to an extension member; ASP.NET Core can produce problem details natively.</t>
+          <t>Each module reports errors in its own way (a page summary, a thrown message, a flash text), so clients and the form components cannot render or test them uniformly. RFC 9457 defines application/problem+json and leaves the validation list to an extension member; ASP.NET Core can produce problem details natively. 2026-10-28: follows the REST API standard ADR-0009 / guideline chapter 08 (#431).</t>
         </is>
       </c>
       <c r="I364" s="8" t="inlineStr">
@@ -47666,7 +47666,11 @@
           <t>Done when: the ADR is accepted and a short guideline chapter (docs/guidelines) lists the rules with one good and one bad example each; rows #12, #195, #363, #18, #28 and #387 reference it; the open questions have an owner.</t>
         </is>
       </c>
-      <c r="K400" s="8" t="n"/>
+      <c r="K400" s="8" t="inlineStr">
+        <is>
+          <t>Written in PR (this branch): ADR-0009 (status Proposed, owner review) and guideline chapter 08 with a good and a bad example per rule; paging decision recorded (offset for grids, cursor for exports and very large tables, one implementation); rows #12, #195, #387 already reference #431, #363, #18 and #28 now do. QA pending: owner acceptance of the ADR.</t>
+        </is>
+      </c>
       <c r="L400" s="10" t="inlineStr">
         <is>
           <t>M0</t>

</xml_diff>

<commit_message>
SCRUM-338, SCRUM-430: metadata registry design, ADR-0010 and ADR-0011 (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -13368,7 +13368,7 @@
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>PEMS has no general App/Entity/Field registry (audit E1/E2). The proven pattern is that everything is a database row, not code.</t>
+          <t>PEMS has no general App/Entity/Field registry (audit E1/E2). The proven pattern is that everything is a database row, not code. 2026-10-28: design in docs/architecture/METADATA_REGISTRY_DESIGN.md (ADR-0010); payload and lifecycle follow the definition envelope.</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>A single type definition from day one avoids the field-type vs column-type duplication seen in comparable platforms.</t>
+          <t>A single type definition from day one avoids the field-type vs column-type duplication seen in comparable platforms. 2026-10-28: design in docs/architecture/METADATA_REGISTRY_DESIGN.md (ADR-0010); payload and lifecycle follow the definition envelope.</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
@@ -13643,7 +13643,7 @@
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>Changing a field type on live data is the riskiest operation of any dynamic platform.</t>
+          <t>Changing a field type on live data is the riskiest operation of any dynamic platform. 2026-10-28: design in docs/architecture/METADATA_REGISTRY_DESIGN.md (ADR-0010); payload and lifecycle follow the definition envelope.</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
@@ -14270,7 +14270,7 @@
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>The current menu in _SidebarMenu.cshtml is static. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
+          <t>The current menu in _SidebarMenu.cshtml is static. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage. 2026-10-28: the stored shape follows ADR-0011 (UI definition model).</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
@@ -14998,7 +14998,7 @@
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>A cached registry (TTL + write invalidation) with ETag/gzip cured slow database access on a comparable platform; a registry change must not need a rebuild. 2026-10-28: follows the REST API standard ADR-0009 / guideline chapter 08 (#431).</t>
+          <t>A cached registry (TTL + write invalidation) with ETag/gzip cured slow database access on a comparable platform; a registry change must not need a rebuild. 2026-10-28: follows the REST API standard ADR-0009 / guideline chapter 08 (#431). 2026-10-28: design in docs/architecture/METADATA_REGISTRY_DESIGN.md (ADR-0010); payload and lifecycle follow the definition envelope.</t>
         </is>
       </c>
       <c r="I29" s="8" t="inlineStr">
@@ -16482,7 +16482,7 @@
       </c>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t>PEMS forms are fixed Razor; the audit found no general form builder. This is the line between software and a platform. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
+          <t>PEMS forms are fixed Razor; the audit found no general form builder. This is the line between software and a platform. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage. 2026-10-28: the stored shape follows ADR-0011 (UI definition model).</t>
         </is>
       </c>
       <c r="I45" s="8" t="inlineStr">
@@ -17647,7 +17647,7 @@
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>List sizes must be structured metadata, not ad-hoc. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
+          <t>List sizes must be structured metadata, not ad-hoc. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage. 2026-10-28: the stored shape follows ADR-0011 (UI definition model).</t>
         </is>
       </c>
       <c r="I58" s="8" t="inlineStr">
@@ -42329,7 +42329,11 @@
           <t>Done when: the design document and ADR exist; Member A and Member B have reviewed them; the sketched classes compile; open questions are listed with an owner; rows #10, #11, #13 and #28 reference the document.</t>
         </is>
       </c>
-      <c r="K339" s="8" t="n"/>
+      <c r="K339" s="8" t="inlineStr">
+        <is>
+          <t>Written in the PR of branch feature/SCRUM-338-430-definition-registry-hamid: docs/architecture/METADATA_REGISTRY_DESIGN.md and ADR-0010 (status Proposed); one envelope (Definitions, DefinitionVersions, DefinitionReferences, DefinitionStamps), lifecycle reused from the workflow platform, shipped vs customer rule reused from the dynamic sidebar, cache stamp contract, five open questions with owners; C# sketch compiles (warnings as errors). QA pending: owner review and acceptance.</t>
+        </is>
+      </c>
       <c r="L339" s="10" t="inlineStr">
         <is>
           <t>M0</t>
@@ -46589,7 +46593,7 @@
       </c>
       <c r="H388" s="8" t="inlineStr">
         <is>
-          <t>ADR-0008: component texts are inputs. In the dynamic BPMS the form definition and its translations live in the database (one form row, texts as JSON per language slug) and must fill and be written back from the components without component changes.</t>
+          <t>ADR-0008: component texts are inputs. In the dynamic BPMS the form definition and its translations live in the database (one form row, texts as JSON per language slug) and must fill and be written back from the components without component changes. 2026-10-28: the stored shape follows ADR-0011 (UI definition model).</t>
         </is>
       </c>
       <c r="I388" s="8" t="inlineStr">
@@ -47581,7 +47585,11 @@
           <t>Done when: the ADR is accepted (storage, envelope, draft/publish/rollback, how a static page and a database page coexist, cache and invalidation, size and security limits); rows #338, #387, #44, #57 and #20 reference it; open questions have an owner.</t>
         </is>
       </c>
-      <c r="K399" s="8" t="n"/>
+      <c r="K399" s="8" t="inlineStr">
+        <is>
+          <t>Written together with #338: ADR-0011 (status Proposed): page, layout, component instance, data source and action definitions in the same envelope, coexistence with static pages by override and reset, PageHost runtime and publish-time validation, installations identical by migration (owner decision 2026-10-28). Rows #338, #387, #44, #57 and #20 reference it. QA pending: owner acceptance.</t>
+        </is>
+      </c>
       <c r="L399" s="10" t="inlineStr">
         <is>
           <t>M0</t>

</xml_diff>

<commit_message>
SCRUM-338, SCRUM-430: metadata registry design, ADR-0010 and ADR-0011 (hamid) (#72)
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -13368,7 +13368,7 @@
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>PEMS has no general App/Entity/Field registry (audit E1/E2). The proven pattern is that everything is a database row, not code.</t>
+          <t>PEMS has no general App/Entity/Field registry (audit E1/E2). The proven pattern is that everything is a database row, not code. 2026-10-28: design in docs/architecture/METADATA_REGISTRY_DESIGN.md (ADR-0010); payload and lifecycle follow the definition envelope.</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>A single type definition from day one avoids the field-type vs column-type duplication seen in comparable platforms.</t>
+          <t>A single type definition from day one avoids the field-type vs column-type duplication seen in comparable platforms. 2026-10-28: design in docs/architecture/METADATA_REGISTRY_DESIGN.md (ADR-0010); payload and lifecycle follow the definition envelope.</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
@@ -13643,7 +13643,7 @@
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>Changing a field type on live data is the riskiest operation of any dynamic platform.</t>
+          <t>Changing a field type on live data is the riskiest operation of any dynamic platform. 2026-10-28: design in docs/architecture/METADATA_REGISTRY_DESIGN.md (ADR-0010); payload and lifecycle follow the definition envelope.</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
@@ -14270,7 +14270,7 @@
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>The current menu in _SidebarMenu.cshtml is static. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
+          <t>The current menu in _SidebarMenu.cshtml is static. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage. 2026-10-28: the stored shape follows ADR-0011 (UI definition model).</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
@@ -14998,7 +14998,7 @@
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>A cached registry (TTL + write invalidation) with ETag/gzip cured slow database access on a comparable platform; a registry change must not need a rebuild. 2026-10-28: follows the REST API standard ADR-0009 / guideline chapter 08 (#431).</t>
+          <t>A cached registry (TTL + write invalidation) with ETag/gzip cured slow database access on a comparable platform; a registry change must not need a rebuild. 2026-10-28: follows the REST API standard ADR-0009 / guideline chapter 08 (#431). 2026-10-28: design in docs/architecture/METADATA_REGISTRY_DESIGN.md (ADR-0010); payload and lifecycle follow the definition envelope.</t>
         </is>
       </c>
       <c r="I29" s="8" t="inlineStr">
@@ -16482,7 +16482,7 @@
       </c>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t>PEMS forms are fixed Razor; the audit found no general form builder. This is the line between software and a platform. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
+          <t>PEMS forms are fixed Razor; the audit found no general form builder. This is the line between software and a platform. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage. 2026-10-28: the stored shape follows ADR-0011 (UI definition model).</t>
         </is>
       </c>
       <c r="I45" s="8" t="inlineStr">
@@ -17647,7 +17647,7 @@
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>List sizes must be structured metadata, not ad-hoc. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage.</t>
+          <t>List sizes must be structured metadata, not ad-hoc. 2026-10-28 audit: the designer saves through the definition store API (#434), not its own storage. 2026-10-28: the stored shape follows ADR-0011 (UI definition model).</t>
         </is>
       </c>
       <c r="I58" s="8" t="inlineStr">
@@ -42329,7 +42329,11 @@
           <t>Done when: the design document and ADR exist; Member A and Member B have reviewed them; the sketched classes compile; open questions are listed with an owner; rows #10, #11, #13 and #28 reference the document.</t>
         </is>
       </c>
-      <c r="K339" s="8" t="n"/>
+      <c r="K339" s="8" t="inlineStr">
+        <is>
+          <t>Written in the PR of branch feature/SCRUM-338-430-definition-registry-hamid: docs/architecture/METADATA_REGISTRY_DESIGN.md and ADR-0010 (status Proposed); one envelope (Definitions, DefinitionVersions, DefinitionReferences, DefinitionStamps), lifecycle reused from the workflow platform, shipped vs customer rule reused from the dynamic sidebar, cache stamp contract, five open questions with owners; C# sketch compiles (warnings as errors). QA pending: owner review and acceptance.</t>
+        </is>
+      </c>
       <c r="L339" s="10" t="inlineStr">
         <is>
           <t>M0</t>
@@ -46589,7 +46593,7 @@
       </c>
       <c r="H388" s="8" t="inlineStr">
         <is>
-          <t>ADR-0008: component texts are inputs. In the dynamic BPMS the form definition and its translations live in the database (one form row, texts as JSON per language slug) and must fill and be written back from the components without component changes.</t>
+          <t>ADR-0008: component texts are inputs. In the dynamic BPMS the form definition and its translations live in the database (one form row, texts as JSON per language slug) and must fill and be written back from the components without component changes. 2026-10-28: the stored shape follows ADR-0011 (UI definition model).</t>
         </is>
       </c>
       <c r="I388" s="8" t="inlineStr">
@@ -47581,7 +47585,11 @@
           <t>Done when: the ADR is accepted (storage, envelope, draft/publish/rollback, how a static page and a database page coexist, cache and invalidation, size and security limits); rows #338, #387, #44, #57 and #20 reference it; open questions have an owner.</t>
         </is>
       </c>
-      <c r="K399" s="8" t="n"/>
+      <c r="K399" s="8" t="inlineStr">
+        <is>
+          <t>Written together with #338: ADR-0011 (status Proposed): page, layout, component instance, data source and action definitions in the same envelope, coexistence with static pages by override and reset, PageHost runtime and publish-time validation, installations identical by migration (owner decision 2026-10-28). Rows #338, #387, #44, #57 and #20 reference it. QA pending: owner acceptance.</t>
+        </is>
+      </c>
       <c r="L399" s="10" t="inlineStr">
         <is>
           <t>M0</t>

</xml_diff>

<commit_message>
SCRUM-432: REST inventory of the controllers (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -13550,7 +13550,7 @@
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>Server-side paging above ~1,000 rows regressed twice on a comparable platform; one query contract from the start is required.</t>
+          <t>Server-side paging above ~1,000 rows regressed twice on a comparable platform; one query contract from the start is required. 2026-10-28: REST inventory done, see docs/audits/REST_INVENTORY_2026-10-28.md and rest-inventory.csv (#432).</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
@@ -20123,7 +20123,7 @@
       </c>
       <c r="H86" s="8" t="inlineStr">
         <is>
-          <t>98 controllers and 91 view folders (Asset, Contract, Crew, Permit, WorkOrder, DocumentRegister, VDR, ...).</t>
+          <t>98 controllers and 91 view folders (Asset, Contract, Crew, Permit, WorkOrder, DocumentRegister, VDR, ...). 2026-10-28: REST inventory done, see docs/audits/REST_INVENTORY_2026-10-28.md and rest-inventory.csv (#432).</t>
         </is>
       </c>
       <c r="I86" s="8" t="inlineStr">
@@ -47730,7 +47730,7 @@
       </c>
       <c r="D401" s="8" t="inlineStr">
         <is>
-          <t>REST inventory of the 147 controllers and ~830 actions: classify (view-only MVC, form post, JSON endpoint, API candidate) and map each to a target resource</t>
+          <t>REST inventory of the 147 controllers and 1,062 actions: classify (view-only MVC, form post, JSON endpoint, API candidate) and map each to a target resource</t>
         </is>
       </c>
       <c r="E401" s="10" t="inlineStr">
@@ -47763,7 +47763,11 @@
           <t>Done when: a table (controller, actions, kind, target resource, wave, owner) is committed under docs/audits; the 22 JSON-returning controllers each have a target shape; rows #85 and #12 reference it.</t>
         </is>
       </c>
-      <c r="K401" s="8" t="n"/>
+      <c r="K401" s="8" t="inlineStr">
+        <is>
+          <t>Done in the PR of branch feature/SCRUM-432-rest-inventory-hamid: tools/rest-inventory/rest_inventory.py (static scan, matches the attribute counts 163 GET / 668 POST exactly), docs/audits/rest-inventory.csv (1,062 actions with verb, kind, permission signal, target resource, wave) and REST_INVENTORY_2026-10-28.md (totals, findings, 30 heaviest controllers classified by hand, target shape of every JSON endpoint: 170 actions in 57 controllers, covering the 22 earlier counted). Findings: 0 PUT/PATCH/DELETE, 476 verb-named actions, 2 preference changes via GET, 269 actions without a permission signal beyond sign-in (security review list, not proof of a hole). QA pending: owner review of the permission-signal list.</t>
+        </is>
+      </c>
       <c r="L401" s="10" t="inlineStr">
         <is>
           <t>M0</t>

</xml_diff>

<commit_message>
SCRUM-432: REST inventory of the controllers (hamid) (#73)
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -13550,7 +13550,7 @@
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>Server-side paging above ~1,000 rows regressed twice on a comparable platform; one query contract from the start is required.</t>
+          <t>Server-side paging above ~1,000 rows regressed twice on a comparable platform; one query contract from the start is required. 2026-10-28: REST inventory done, see docs/audits/REST_INVENTORY_2026-10-28.md and rest-inventory.csv (#432).</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
@@ -20123,7 +20123,7 @@
       </c>
       <c r="H86" s="8" t="inlineStr">
         <is>
-          <t>98 controllers and 91 view folders (Asset, Contract, Crew, Permit, WorkOrder, DocumentRegister, VDR, ...).</t>
+          <t>98 controllers and 91 view folders (Asset, Contract, Crew, Permit, WorkOrder, DocumentRegister, VDR, ...). 2026-10-28: REST inventory done, see docs/audits/REST_INVENTORY_2026-10-28.md and rest-inventory.csv (#432).</t>
         </is>
       </c>
       <c r="I86" s="8" t="inlineStr">
@@ -47730,7 +47730,7 @@
       </c>
       <c r="D401" s="8" t="inlineStr">
         <is>
-          <t>REST inventory of the 147 controllers and ~830 actions: classify (view-only MVC, form post, JSON endpoint, API candidate) and map each to a target resource</t>
+          <t>REST inventory of the 147 controllers and 1,062 actions: classify (view-only MVC, form post, JSON endpoint, API candidate) and map each to a target resource</t>
         </is>
       </c>
       <c r="E401" s="10" t="inlineStr">
@@ -47763,7 +47763,11 @@
           <t>Done when: a table (controller, actions, kind, target resource, wave, owner) is committed under docs/audits; the 22 JSON-returning controllers each have a target shape; rows #85 and #12 reference it.</t>
         </is>
       </c>
-      <c r="K401" s="8" t="n"/>
+      <c r="K401" s="8" t="inlineStr">
+        <is>
+          <t>Done in the PR of branch feature/SCRUM-432-rest-inventory-hamid: tools/rest-inventory/rest_inventory.py (static scan, matches the attribute counts 163 GET / 668 POST exactly), docs/audits/rest-inventory.csv (1,062 actions with verb, kind, permission signal, target resource, wave) and REST_INVENTORY_2026-10-28.md (totals, findings, 30 heaviest controllers classified by hand, target shape of every JSON endpoint: 170 actions in 57 controllers, covering the 22 earlier counted). Findings: 0 PUT/PATCH/DELETE, 476 verb-named actions, 2 preference changes via GET, 269 actions without a permission signal beyond sign-in (security review list, not proof of a hole). QA pending: owner review of the permission-signal list.</t>
+        </is>
+      </c>
       <c r="L401" s="10" t="inlineStr">
         <is>
           <t>M0</t>

</xml_diff>

<commit_message>
SCRUM-433: component manifests generated from the code, with options validation (hamid)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -23357,7 +23357,7 @@
       </c>
       <c r="H122" s="8" t="inlineStr">
         <is>
-          <t>Dependencies: QuestPDF, Hangfire, Fido2, ZXing.Net, HtmlSanitizer, FluentFTP, Serilog and the front end. Some have commercial or copyleft terms (for example revenue thresholds for QuestPDF and the Hangfire Core licence); this must be verified formally, not guessed.</t>
+          <t>Dependencies: QuestPDF, Hangfire, Fido2, ZXing.Net, HtmlSanitizer, FluentFTP, Serilog and the front end. Some have commercial or copyleft terms (for example revenue thresholds for QuestPDF and the Hangfire Core licence); this must be verified formally, not guessed. 2026-10-28 (#433): LateApexEarlySpeed.Json.Schema 4.2.2 added to PEMS.UI: BSD-3-Clause (checked in the package nuspec), JSON Schema 2020-12 validation on System.Text.Json. JsonSchema.Net 9.x rejected: Open Source Maintenance Fee EULA, not a plain open-source licence; needs owner approval before any use. Schema generation uses the built-in System.Text.Json JsonSchemaExporter (no package).</t>
         </is>
       </c>
       <c r="I122" s="8" t="inlineStr">
@@ -43886,7 +43886,7 @@
       </c>
       <c r="H357" s="8" t="inlineStr">
         <is>
-          <t>A direct API call, an import or a bulk write bypasses whatever the page checks, and PEMS has no single validator to call. Validation must be authoritative on the server; the client only improves feedback.</t>
+          <t>A direct API call, an import or a bulk write bypasses whatever the page checks, and PEMS has no single validator to call. Validation must be authoritative on the server; the client only improves feedback. 2026-10-28: a JSON Schema validator (LateApexEarlySpeed.Json.Schema) already validates component options in PEMS.UI (#433); reuse it for definition payloads (ADR-0010).</t>
         </is>
       </c>
       <c r="I357" s="8" t="inlineStr">
@@ -47852,7 +47852,11 @@
           <t>Done when: a generator produces one JSON manifest per component from the code (no hand-written schema); a stored options JSON that violates the schema is rejected with a field error list; the manifest of Button, Badge, Field, Table, Form, Empty/Error/Loading state exists and a test fails when a component has no manifest.</t>
         </is>
       </c>
-      <c r="K402" s="8" t="n"/>
+      <c r="K402" s="8" t="inlineStr">
+        <is>
+          <t>Done in the PR of branch feature/SCRUM-433-component-manifest-hamid: [PemsComponent] now carries Category and Icon and is on all nine registered components (button, badge, skeleton, field, table, form, empty-state, error-state, loading-state); ComponentManifestGenerator builds one manifest per component from the code with the built-in JsonSchemaExporter (TranslatableText as string or language map, unknown properties rejected, required from C# required/EditorRequired); ComponentManifestCatalog validates stored options JSON with LateApexEarlySpeed.Json.Schema (BSD-3-Clause) and returns a field error list (JSON Pointer, constraint code, message key) and converts valid options to component parameters; approved snapshots in PEMS.UI.Tests/Manifests. PEMS.UI.Tests 124/124 (25 new); mutation checks: removing the attribute fails 3, making Label optional fails 3. QA pending: owner confirms the library licence choice.</t>
+        </is>
+      </c>
       <c r="L402" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-433: component manifests generated from the code, with options validation (hamid) (#74)
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -23357,7 +23357,7 @@
       </c>
       <c r="H122" s="8" t="inlineStr">
         <is>
-          <t>Dependencies: QuestPDF, Hangfire, Fido2, ZXing.Net, HtmlSanitizer, FluentFTP, Serilog and the front end. Some have commercial or copyleft terms (for example revenue thresholds for QuestPDF and the Hangfire Core licence); this must be verified formally, not guessed.</t>
+          <t>Dependencies: QuestPDF, Hangfire, Fido2, ZXing.Net, HtmlSanitizer, FluentFTP, Serilog and the front end. Some have commercial or copyleft terms (for example revenue thresholds for QuestPDF and the Hangfire Core licence); this must be verified formally, not guessed. 2026-10-28 (#433): LateApexEarlySpeed.Json.Schema 4.2.2 added to PEMS.UI: BSD-3-Clause (checked in the package nuspec), JSON Schema 2020-12 validation on System.Text.Json. JsonSchema.Net 9.x rejected: Open Source Maintenance Fee EULA, not a plain open-source licence; needs owner approval before any use. Schema generation uses the built-in System.Text.Json JsonSchemaExporter (no package).</t>
         </is>
       </c>
       <c r="I122" s="8" t="inlineStr">
@@ -43886,7 +43886,7 @@
       </c>
       <c r="H357" s="8" t="inlineStr">
         <is>
-          <t>A direct API call, an import or a bulk write bypasses whatever the page checks, and PEMS has no single validator to call. Validation must be authoritative on the server; the client only improves feedback.</t>
+          <t>A direct API call, an import or a bulk write bypasses whatever the page checks, and PEMS has no single validator to call. Validation must be authoritative on the server; the client only improves feedback. 2026-10-28: a JSON Schema validator (LateApexEarlySpeed.Json.Schema) already validates component options in PEMS.UI (#433); reuse it for definition payloads (ADR-0010).</t>
         </is>
       </c>
       <c r="I357" s="8" t="inlineStr">
@@ -47852,7 +47852,11 @@
           <t>Done when: a generator produces one JSON manifest per component from the code (no hand-written schema); a stored options JSON that violates the schema is rejected with a field error list; the manifest of Button, Badge, Field, Table, Form, Empty/Error/Loading state exists and a test fails when a component has no manifest.</t>
         </is>
       </c>
-      <c r="K402" s="8" t="n"/>
+      <c r="K402" s="8" t="inlineStr">
+        <is>
+          <t>Done in the PR of branch feature/SCRUM-433-component-manifest-hamid: [PemsComponent] now carries Category and Icon and is on all nine registered components (button, badge, skeleton, field, table, form, empty-state, error-state, loading-state); ComponentManifestGenerator builds one manifest per component from the code with the built-in JsonSchemaExporter (TranslatableText as string or language map, unknown properties rejected, required from C# required/EditorRequired); ComponentManifestCatalog validates stored options JSON with LateApexEarlySpeed.Json.Schema (BSD-3-Clause) and returns a field error list (JSON Pointer, constraint code, message key) and converts valid options to component parameters; approved snapshots in PEMS.UI.Tests/Manifests. PEMS.UI.Tests 124/124 (25 new); mutation checks: removing the attribute fails 3, making Label optional fails 3. QA pending: owner confirms the library licence choice.</t>
+        </is>
+      </c>
       <c r="L402" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-428: leave the plan workbook to its owner; rule in the guideline (saber)
The plan workbook and backlog.csv go back to main's version in this PR;
the #428 row update moves to the Jira comment. Guideline chapter 01 (Git):
feature branches do not edit the binary workbook (owner decision
2026-10-28), plus a learnings entry.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Summary" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licensing Design" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capability Checklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lessons" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supportability Matrix" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Old to New Map" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$U$350</definedName>
@@ -12367,7 +12367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U414"/>
+  <dimension ref="A1:U413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -48828,103 +48828,6 @@
       <c r="U413" s="10" t="inlineStr">
         <is>
           <t>Hamid</t>
-        </is>
-      </c>
-    </row>
-    <row r="414">
-      <c r="A414" s="10" t="n">
-        <v>428</v>
-      </c>
-      <c r="B414" s="10" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="C414" s="8" t="inlineStr">
-        <is>
-          <t>Domain: HR, Projects, Finance &amp; Procurement</t>
-        </is>
-      </c>
-      <c r="D414" s="8" t="inlineStr">
-        <is>
-          <t>Pick registered part numbers from the part catalogue in material requisition items</t>
-        </is>
-      </c>
-      <c r="E414" s="10" t="inlineStr">
-        <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="F414" s="10" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G414" s="10" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="H414" s="8" t="inlineStr">
-        <is>
-          <t>Owner request 2026-10-27: after the part catalogue registers a part number it must be selectable in procurement. SCRUM-428; batch 427 -&gt; 40 -&gt; 57 -&gt; 428 -&gt; 429.</t>
-        </is>
-      </c>
-      <c r="I414" s="8" t="inlineStr">
-        <is>
-          <t>Server-side resolution of each MR item part number against completed catalogue requests and Material Master (exact, normalised), nullable links on MaterialRequisitionItem (migration), lookup endpoint on the reused SearchExistingPartsAsync, pems-select url/create options, MR form and details.</t>
-        </is>
-      </c>
-      <c r="J414" s="8" t="inlineStr">
-        <is>
-          <t>Done when: a registered part is found in the MR item lookup, its description and unit fill in, the link is stored; a typed unregistered part stays free text, marked not catalogued.</t>
-        </is>
-      </c>
-      <c r="K414" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-28 SCRUM-428: built on feature/SCRUM-428-mr-registered-parts-saber; MrRegisteredPartTests + related 83/83; browser QA on PEMSDB_QA407 (lookup by MPN, fill, typed part, details badges). PO lines (gap analysis proposal 1) will carry the same link.</t>
-        </is>
-      </c>
-      <c r="L414" s="10" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
-      </c>
-      <c r="M414" s="10" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="N414" s="10" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="O414" s="10" t="inlineStr">
-        <is>
-          <t>#427</t>
-        </is>
-      </c>
-      <c r="P414" s="10" t="n"/>
-      <c r="Q414" s="10" t="n"/>
-      <c r="R414" s="8" t="inlineStr">
-        <is>
-          <t>Domain modules</t>
-        </is>
-      </c>
-      <c r="S414" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="T414" s="10" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="U414" s="10" t="inlineStr">
-        <is>
-          <t>Member A</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SCRUM-435: REST API walking skeleton and the disciplines pilot resource (hamid)
/api/v1 plumbing in PEMS.Web/Api (problem+json, ETag/If-Match, Idempotency-Key, list contract, permission policies,
antiforgery header, API-aware 401/403, OpenAPI 3.1 with an approved snapshot) and /api/v1/disciplines (GET, POST, PUT,
PATCH, DELETE) on the existing master-data service. Migration DisciplineRowVersion adds the concurrency token.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -48026,7 +48026,11 @@
           <t>Done when: GET/POST/PUT/PATCH/DELETE on the pilot resource follow #431 and are covered by tests; the OpenAPI document is served offline and lints clean; an endpoint without authorization fails a test; the browser and an integration token can both call it.</t>
         </is>
       </c>
-      <c r="K404" s="8" t="n"/>
+      <c r="K404" s="8" t="inlineStr">
+        <is>
+          <t>Done in the PR of branch feature/SCRUM-435-api-skeleton-hamid: PEMS.Web/Api with RFC 9457 problem+json (errors list), ETag/If-Match (412/428), Idempotency-Key (in memory), list contract (sort, filter[f], q, fields, offset paging capped at 10,000 rows), allowedActions, [ApiPermission(module, action)] policies over the permission matrix, 401/403 problems for /api, OpenAPI 3.1 at /api/v1/openapi.json (Microsoft.AspNetCore.OpenApi, MIT, signed-in users only, approved snapshot). Pilot resource /api/v1/disciplines: GET list/one, POST 201+Location, PUT, PATCH (merge patch), DELETE (409 when in use) on the same service as the master-data page; migration DisciplineRowVersion. 46 new tests (contract, policy gate, antiforgery gate, OpenAPI snapshot); unsafe verbs validate the X-CSRF-TOKEN antiforgery header. NOT done / QA pending: integration bearer token (issuing and validation stays with #195), durable Idempotency-Key store (#434), cursor paging (first export endpoint), SQL Server run of the row-version concurrency and the DELETE 409 path, a request through the real pipeline (cookie + antiforgery header) in a browser, external OpenAPI lint (Spectral) not available offline.</t>
+        </is>
+      </c>
       <c r="L404" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>

<commit_message>
SCRUM-435: REST API walking skeleton and the disciplines pilot resource (hamid) (#77)
/api/v1 plumbing in PEMS.Web/Api (problem+json, ETag/If-Match, Idempotency-Key, list contract, permission policies,
antiforgery header, API-aware 401/403, OpenAPI 3.1 with an approved snapshot) and /api/v1/disciplines (GET, POST, PUT,
PATCH, DELETE) on the existing master-data service. Migration DisciplineRowVersion adds the concurrency token.


Claude-Session: https://claude.ai/code/session_01D5zM1tCqx8B75BdCP689YP

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plan/PEMS_Backlog_Roadmap.xlsx
+++ b/plan/PEMS_Backlog_Roadmap.xlsx
@@ -48026,7 +48026,11 @@
           <t>Done when: GET/POST/PUT/PATCH/DELETE on the pilot resource follow #431 and are covered by tests; the OpenAPI document is served offline and lints clean; an endpoint without authorization fails a test; the browser and an integration token can both call it.</t>
         </is>
       </c>
-      <c r="K404" s="8" t="n"/>
+      <c r="K404" s="8" t="inlineStr">
+        <is>
+          <t>Done in the PR of branch feature/SCRUM-435-api-skeleton-hamid: PEMS.Web/Api with RFC 9457 problem+json (errors list), ETag/If-Match (412/428), Idempotency-Key (in memory), list contract (sort, filter[f], q, fields, offset paging capped at 10,000 rows), allowedActions, [ApiPermission(module, action)] policies over the permission matrix, 401/403 problems for /api, OpenAPI 3.1 at /api/v1/openapi.json (Microsoft.AspNetCore.OpenApi, MIT, signed-in users only, approved snapshot). Pilot resource /api/v1/disciplines: GET list/one, POST 201+Location, PUT, PATCH (merge patch), DELETE (409 when in use) on the same service as the master-data page; migration DisciplineRowVersion. 46 new tests (contract, policy gate, antiforgery gate, OpenAPI snapshot); unsafe verbs validate the X-CSRF-TOKEN antiforgery header. NOT done / QA pending: integration bearer token (issuing and validation stays with #195), durable Idempotency-Key store (#434), cursor paging (first export endpoint), SQL Server run of the row-version concurrency and the DELETE 409 path, a request through the real pipeline (cookie + antiforgery header) in a browser, external OpenAPI lint (Spectral) not available offline.</t>
+        </is>
+      </c>
       <c r="L404" s="10" t="inlineStr">
         <is>
           <t>M1</t>

</xml_diff>